<commit_message>
England-only: replace Strathclyde/Swansea with England programmes (Teesside, Northumbria, Essex, Leicester, Brunel, York); update costs, scores, summary, sources
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Table_final.xlsx
+++ b/Table_final.xlsx
@@ -526,7 +526,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>بریتانیا (UK) 🇬🇧</t>
+          <t>انگلستان (England) 🇬🇧</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -587,9 +587,13 @@
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Swansea – MSc Advanced Computer Science (2:2) → Safe
-Brunel – MSc AI / Data Science (2:2) → Safe
-Strathclyde – MSc Advanced Computer Science (2:2) → Target</t>
+          <t>Teesside (Middlesbrough) – MSc Computer Science (2:2، IELTS 6.0) → Safe
+Northumbria (Newcastle) – MSc Advanced Computer Science (2:2 در رشته کامپیوتری) → Safe
+Essex (Colchester) – MSc Advanced Computer Science (2:2؛ Computer Engineering پذیرفته می‌شود) → Safe/Target
+Brunel (London) – MSc AI / Data Science (2:2) → Safe/Target
+Leicester – MSc Advanced Computer Science (2:1؛ سابقه کار مرتبط جبران می‌کند) → Target
+York – MSc Advanced Computer Science (2:2 با پیش‌زمینه قوی، IELTS 6.5) → Reach
+فقط انگلستان — Strathclyde (اسکاتلند) و Swansea (ولز) حذف شدند</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
@@ -636,7 +640,7 @@
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Strathclyde =230 · Swansea ≈ 300 · Brunel 353</t>
+          <t>Newcastle 149 · York =158 · Leicester =314 · Brunel 353 · Essex =438 · Northumbria =528 · Teesside در فهرست اصلی QS نیست (THE 601–800)</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -737,15 +741,18 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Swansea: £24,200
+          <t>Teesside: £17,000
+Northumbria: £21,500
+Leicester: £24,250
+Essex: £24,675
 Brunel: £24,795
-Strathclyde: £31,900
-بورس‌ها (Strathclyde ۱۵٪، Brunel £6,000) جدا حساب شوند، تضمینی نیستند</t>
+York: £32,900 (Newcastle ≈ £31,700)
+کف قیمت انگلستان: Chester £15,500 (بدون رتبه). بورس‌ها (مثلاً Brunel تا £6,000) جدا حساب شوند، تضمینی نیستند</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>utwente.nl؛ liu.se؛ bth.se؛ sdu.dk؛ studyindenmark.dk؛ ul.ie؛ maynoothuniversity.ie؛ brunel.ac.uk؛ strath.ac.uk؛ swansea.ac.uk</t>
+          <t>utwente.nl؛ liu.se؛ bth.se؛ sdu.dk؛ studyindenmark.dk؛ ul.ie؛ maynoothuniversity.ie؛ brunel.ac.uk؛ tees.ac.uk؛ northumbria.ac.uk؛ le.ac.uk؛ essex.ac.uk؛ york.ac.uk</t>
         </is>
       </c>
     </row>
@@ -787,7 +794,7 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>$32,100–42,300</t>
+          <t>$22,500–43,600 (Teesside $22,500 · Northumbria $28,500 · Leicester/Essex/Brunel ≈ $32,100–32,900 · York $43,600)</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -840,7 +847,8 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Glasgow/Swansea: £1,000–1,300
+          <t>شمال انگلستان (Middlesbrough/Newcastle): £950–1,250
+Leicester/Colchester/York: £1,000–1,350
 London (Brunel): £1,400–1,800
 حداقل ویزا: £1,171 / £1,529 در ماه (× ۹)؛ از ۳۰ نوامبر ۲۰۲۶: £1,203 / £1,570</t>
         </is>
@@ -889,7 +897,7 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>$48,000–71,000 (Swansea: $48,000–53,000)</t>
+          <t>$38,000–65,000 (Teesside $38–42k · Northumbria $44–48k · Leicester/Essex $48–54k · Brunel/London $55–61k · York $60–65k)</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
@@ -936,7 +944,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>$48,000–71,000 (۱ سال)</t>
+          <t>$38,000–65,000 (۱ سال)</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
@@ -983,7 +991,7 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>❌ کسری $16,000–39,000</t>
+          <t>❌ کسری $6,000–33,000 (کمترین: Teesside ≈ $6–10k؛ Northumbria ≈ $12–16k)</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
@@ -1368,7 +1376,7 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>£28,000–35,000 خارج لندن؛ London £32,000–45,000 — اغلب زیر کف اسپانسری £38,290</t>
+          <t>£28,000–35,000 خارج لندن (Manchester/Leeds/Newcastle)؛ London £32,000–45,000 — اغلب زیر کف اسپانسری £38,290</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
@@ -1839,7 +1847,7 @@
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>بسیار بالا: Graduate visa ۱۸ ماه، B2، طرح PR ۱۰ ساله، عوارض £925/دانشجو/سال از 2028-29 (فقط دانشگاه‌های انگلستان: Brunel بله، Strathclyde/Swansea خیر)</t>
+          <t>بسیار بالا: Graduate visa ۱۸ ماه، B2، طرح PR ۱۰ ساله، عوارض £925/دانشجو/سال از اوت ۲۰۲۸ فقط برای دانشگاه‌های انگلستان — یعنی همهٔ گزینه‌های شما (ورودی ۲۰۲۸)؛ احتمالاً به شهریه اضافه می‌شود</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
@@ -1886,12 +1894,12 @@
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>3 / 10 / 4 = ۱۷</t>
+          <t>5 / 10 / 4 = ۱۹</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>وزن برابر. اگر «انگلیسی» وزن بیشتری دارد → ایرلند با فاصله؛ اگر «هزینه» وزن بیشتری دارد و B1 آلمانی را می‌پذیرید → آلمان.</t>
+          <t>وزن برابر. اگر «انگلیسی» وزن بیشتری دارد → ایرلند با فاصله؛ اگر «هزینه» وزن بیشتری دارد و B1 آلمانی را می‌پذیرید → آلمان. انگلستان با گزینه‌های ارزان شمال (Teesside/Northumbria) از ۱۷ به ۱۹ رسید (هم‌امتیاز سوئد) ولی هنوز از بودجهٔ سالانه $32k بیرون است.</t>
         </is>
       </c>
     </row>
@@ -1927,7 +1935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1954,7 +1962,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>آلمان $27–36k  &lt;  ایرلند $32–48k  &lt;  بریتانیا $48–71k  &lt;  سوئد $54–65k  &lt;  دانمارک $61–71k  &lt;  هلند $75–90k</t>
+          <t>آلمان $27–36k  &lt;  ایرلند $32–48k  &lt;  انگلستان $38–65k  &lt;  سوئد $54–65k  &lt;  دانمارک $61–71k  &lt;  هلند $75–90k</t>
         </is>
       </c>
     </row>
@@ -1966,7 +1974,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>ایرلند و بریتانیا کامل؛ هلند و سوئد برای زندگی/کار خوب ولی برای اقامت دائم/تابعیت زبان می‌خواهند (هلند B1 در راه، سوئد آزمون تابعیت)؛ دانمارک و آلمان بدون زبان محلی هم بازار کار و هم PR محدود.</t>
+          <t>ایرلند و انگلستان کامل؛ هلند و سوئد برای زندگی/کار خوب ولی برای اقامت دائم/تابعیت زبان می‌خواهند (هلند B1 در راه، سوئد آزمون تابعیت)؛ دانمارک و آلمان بدون زبان محلی هم بازار کار و هم PR محدود.</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1986,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>حقوق ناخالص: دانمارک &gt; آلمان &gt; هلند ≈ سوئد &gt; ایرلند &gt; بریتانیا. دسترسی برای جونیورِ فقط‌انگلیسی: ایرلند ≈ هلند &gt; آلمان &gt; سوئد ≈ دانمارک ≈ بریتانیا.</t>
+          <t>حقوق ناخالص: دانمارک &gt; آلمان &gt; هلند ≈ سوئد &gt; ایرلند &gt; انگلستان. دسترسی برای جونیورِ فقط‌انگلیسی: ایرلند ≈ هلند &gt; آلمان &gt; سوئد ≈ دانمارک ≈ انگلستان.</t>
         </is>
       </c>
     </row>
@@ -1990,7 +1998,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>ایرلند ۲۵ › آلمان ۲۲ › سوئد ۱۹ › هلند ۱۸ › بریتانیا ۱۷ › دانمارک ۱۶.  پیشنهاد: اپلای هم‌زمان به ۲–۳ برنامه ایرلند (UL، Maynooth، TU Dublin) + ۲ برنامه آلمان (Stuttgart، FAU یا یک گزینه Safe)؛ تصمیم نهایی با پذیرش/بورس و وضعیت سفارت‌ها در ۲۰۲۸.</t>
+          <t>ایرلند ۲۵ › آلمان ۲۲ › سوئد ۱۹ = انگلستان ۱۹ › هلند ۱۸ › دانمارک ۱۶.  پیشنهاد: اپلای هم‌زمان به ۲–۳ برنامه ایرلند (UL، Maynooth، TU Dublin) + ۲ برنامه آلمان (Stuttgart، FAU یا یک گزینه Safe)؛ تصمیم نهایی با پذیرش/بورس و وضعیت سفارت‌ها در ۲۰۲۸.</t>
         </is>
       </c>
     </row>
@@ -2014,7 +2022,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>تا بهار ۲۰۲۷: IELTS 7.0 (هر بخش ≥ 6.5) · تابستان ۲۰۲۷: ریزنمرات رسمی + تأییدیه‌ها + VPD uni-assist · پاییز ۲۰۲۷ تا زمستان ۲۰۲۸: اپلای (ایرلند rolling از اکتبر؛ سوئد ۱۵ ژانویه؛ هلند تا ۱ می؛ آلمان ۱۵ ژانویه–۱۵ ژوئیه؛ بریتانیا rolling) · بهار ۲۰۲۸: شهریه/تمکن → خوابگاه → ویزا یا برنامه B.</t>
+          <t>تا بهار ۲۰۲۷: IELTS 7.0 (هر بخش ≥ 6.5) · تابستان ۲۰۲۷: ریزنمرات رسمی + تأییدیه‌ها + VPD uni-assist · پاییز ۲۰۲۷ تا زمستان ۲۰۲۸: اپلای (ایرلند rolling از اکتبر؛ سوئد ۱۵ ژانویه؛ هلند تا ۱ می؛ آلمان ۱۵ ژانویه–۱۵ ژوئیه؛ انگلستان rolling) · بهار ۲۰۲۸: شهریه/تمکن → خوابگاه → ویزا یا برنامه B.</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2035,7 @@
       <c r="B8" s="4" t="inlineStr">
         <is>
           <t>• هزینه کل دوره اضافه شد (هلند از «نیاز به تأمین سال دوم» به گران‌ترین گزینه تبدیل شد)
-• بریتانیا: Graduate visa ۱۸ ماه؛ کف اسپانسری £54,700 / £38,290؛ طرح PR ۱۰ ساله؛ شهریه Strathclyde £31,900
+• فقط انگلستان (به خواست شما): Strathclyde و Swansea حذف شدند؛ گزینه‌ها Teesside £17,000 · Northumbria £21,500 · Leicester £24,250 · Essex £24,675 · Brunel £24,795 · York £32,900؛ Graduate visa ۱۸ ماه؛ کف اسپانسری £54,700 / £38,290؛ طرح PR ۱۰ ساله؛ عوارض £925 از ۲۰۲۸ شامل همهٔ گزینه‌ها
 • کف حقوق ۲۰۲۶ همه کشورها به‌روز شد (آلمان €50,700/€45,934؛ هلند €3,122/ماه؛ سوئد SEK 34,470؛ ایرلند €40,904)
 • ایرلند: ۲ سال CSEP = Stamp 4 نه PR؛ تمکن €10,000
 • سوئد: کار دانشجویی ۱۵ ساعت/هفته (ژوئن ۲۰۲۶)؛ شهروندی ۸ سال؛ «BTH یک‌ساله» حذف شد؛ خوابگاه فقط LiU
@@ -2040,22 +2048,34 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>نکته پروفایل</t>
+          <t>چرا «انگلستان» و نه «بریتانیا»</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>معدل (۱۵.۷۷ طبق جدول اول؛ ۱۵.۷۰ طبق نقد دوم — تفاوتی در نتیجه ندارد) برای همه برنامه‌های بالا بالاتر از حداقل است. مهم‌تر از معدل، تطابق ریزنمرات با پیش‌نیازها (ریاضی، الگوریتم، CS نظری) و SOP با تکیه بر ۲ سال سابقه کار + بازی‌سازی + پروژه‌های گیت‌هاب است.</t>
+          <t>به خواست شما فقط دانشگاه‌های انگلستان مقایسه شده‌اند. قوانین ویزا، کار و اقامت در کل بریتانیا یکسان است؛ سه تفاوت عملی: (۱) ارزان‌ترین گزینه‌های انگلستان (Teesside £17,000، Northumbria £21,500) از Swansea/Strathclyde ارزان‌ترند → کل دوره از $48–71k به $38–65k رسید؛ (۲) عوارض £925 به ازای هر دانشجو از اوت ۲۰۲۸ فقط دانشگاه‌های انگلستان را می‌گیرد — یعنی همهٔ گزینه‌های شما؛ (۳) بازار کار فناوری بریتانیا عملاً در انگلستان است (London، Manchester، Cambridge، Bristol، Leeds) — حذف اسکاتلند/ولز به فرصت شغلی لطمه نمی‌زند. برای شهریهٔ کمتر باید رتبهٔ پایین‌تر را بپذیرید: Teesside/Chester بدون رتبه QS، Northumbria ≈ ۵۲۸، Essex ≈ ۴۳۸؛ York (۱۵۸) و Newcastle (۱۴۹) تقریباً دوبرابر گران‌ترند.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
+          <t>نکته پروفایل</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>معدل (۱۵.۷۷ طبق جدول اول؛ ۱۵.۷۰ طبق نقد دوم — تفاوتی در نتیجه ندارد) برای همه برنامه‌های بالا بالاتر از حداقل است. مهم‌تر از معدل، تطابق ریزنمرات با پیش‌نیازها (ریاضی، الگوریتم، CS نظری) و SOP با تکیه بر ۲ سال سابقه کار + بازی‌سازی + پروژه‌های گیت‌هاب است.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
           <t>اعداد را چگونه بخوانم</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>همه مبالغ سطح 2026/27 هستند؛ برای ۲۰۲۸ سالانه ۳–۵٪ (شهریه ۵–۱۰٪) اضافه کنید. نرخ تبدیل ۲۷ سپتامبر ۲۰۲۶: €1 = $1.14 · £1 = $1.325 · $1 ≈ SEK 9.9 · $1 ≈ DKK 6.55</t>
         </is>
@@ -2072,7 +2092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B61"/>
+  <dimension ref="A1:B70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -2682,130 +2702,238 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>بریتانیا – Strathclyde شهریه PG 2026-27</t>
+          <t>انگلستان – Teesside MSc Computer Science 2026-27: £17,000، 2:2، IELTS 6.0</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>https://www.strath.ac.uk/media/1newwebsite/documents/tuitionfees/PG_Fees_2026-2027_Entry_v0.7.pdf</t>
+          <t>https://www.tees.ac.uk/postgraduate_courses/computing_&amp;_cyber_security/msc_computer_science.cfm</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>بریتانیا – Swansea MSc Advanced Computer Science</t>
+          <t>انگلستان – Northumbria MSc Advanced Computer Science 2026/27: £21,500، 2:2</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>https://www.swansea.ac.uk/postgraduate/taught/maths-comp-sci/computer-science/msc-advanced-computer-science/</t>
+          <t>https://www.northumbria.ac.uk/study-at-northumbria/courses/msc-advanced-computer-science-dtfava6/</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>بریتانیا – Brunel MSc AI 2026/27 £24,795</t>
+          <t>انگلستان – Leicester MSc Advanced Computer Science سپتامبر ۲۰۲۶: £24,250، 2:1</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>https://www.brunel.ac.uk/study/courses/artificial-intelligence-msc</t>
+          <t>https://le.ac.uk/courses/advanced-computer-science-msc/2026</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>بریتانیا – عوارض £925 به ازای هر دانشجوی بین‌المللی (انگلستان، از 2028-29)</t>
+          <t>انگلستان – Essex MSc Advanced Computer Science 2026: £24,675، 2:2 (شامل Computer Engineering)</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>https://www.researchprofessionalnews.com/rr-news-uk-politics-2025-11-international-levy-to-be-flat-fee-of-925-per-student/</t>
+          <t>https://www.essex.ac.uk/courses/pg00435/1/msc-advanced-computer-science</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>بریتانیا – وضعیت VAC تهران</t>
+          <t>انگلستان – York MSc Advanced Computer Science 2026/27: £32,900، 2:2، IELTS 6.5</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>https://livingintehran.com/2026/02/03/tehran-diplomatic-update-recent-embassy-reopenings-current-status-feb-2026/</t>
+          <t>https://www.york.ac.uk/study/postgraduate-taught/courses/msc-advanced-computer-science/</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>QS WUR 2027 – TU Dresden</t>
+          <t>انگلستان – Chester MSc Advanced Computer Science 2026/27: £15,500 (کف قیمت انگلستان)</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>https://tu-dresden.de/tu-dresden/newsportal/news/qs-ranking-2027-tud-gehoert-erneut-zu-den-zehn-besten-universitaeten-deutschlands-und-baut-internationalen-erfolg-weiter-aus</t>
+          <t>https://www.chester.ac.uk/study/course-search/advanced-computer-science-msc/</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>QS WUR 2027 – Stuttgart</t>
+          <t>بریتانیا – Brunel MSc AI 2026/27 £24,795</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>https://www.uni-stuttgart.de/en/university/news/all/QS-World-University-Rankings-2027-The-University-of-Stuttgart-is-recognized-for-its-strong-research-performance-and-commitment-to-sustainability/</t>
+          <t>https://www.brunel.ac.uk/study/courses/artificial-intelligence-msc</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>QS WUR 2027 – Brunel</t>
+          <t>بریتانیا – عوارض £925 به ازای هر دانشجوی بین‌المللی (انگلستان، از 2028-29)</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>https://students.brunel.ac.uk/campus-news/brunel-climbs-global-qs-rankings-after-strong-year-for-research-and-graduate-outcomes</t>
+          <t>https://www.researchprofessionalnews.com/rr-news-uk-politics-2025-11-international-levy-to-be-flat-fee-of-925-per-student/</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>QS WUR 2027 – سایر</t>
+          <t>بریتانیا – وضعیت VAC تهران</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>https://www.topuniversities.com/world-university-rankings</t>
+          <t>https://livingintehran.com/2026/02/03/tehran-diplomatic-update-recent-embassy-reopenings-current-status-feb-2026/</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>حداقل دستمزد ۲۰۲۶ هلند (€14.71)</t>
+          <t>QS WUR 2027 – TU Dresden</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>https://arlettipartners.com/new-increase-in-the-dutch-minimum-hourly-wage-from-january-1st-2026/</t>
+          <t>https://tu-dresden.de/tu-dresden/newsportal/news/qs-ranking-2027-tud-gehoert-erneut-zu-den-zehn-besten-universitaeten-deutschlands-und-baut-internationalen-erfolg-weiter-aus</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
+          <t>QS WUR 2027 – Stuttgart</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>https://www.uni-stuttgart.de/en/university/news/all/QS-World-University-Rankings-2027-The-University-of-Stuttgart-is-recognized-for-its-strong-research-performance-and-commitment-to-sustainability/</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>QS WUR 2027 – Newcastle 149</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>https://www.ncl.ac.uk/press/articles/latest/2026/06/qs2027/</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>QS WUR 2027 – York =158</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>https://www.york.ac.uk/about/rankings/</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>QS WUR 2027 – Leicester =314</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>https://www.topuniversities.com/universities/university-leicester</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>QS WUR 2027 – Essex =438</t>
+        </is>
+      </c>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>https://www.topuniversities.com/universities/essex-university</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>QS WUR 2027 – Northumbria =528</t>
+        </is>
+      </c>
+      <c r="B66" s="7" t="inlineStr">
+        <is>
+          <t>https://www.topuniversities.com/universities/northumbria-university-newcastle</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>QS WUR 2027 – Brunel</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>https://students.brunel.ac.uk/campus-news/brunel-climbs-global-qs-rankings-after-strong-year-for-research-and-graduate-outcomes</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>QS WUR 2027 – سایر</t>
+        </is>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>https://www.topuniversities.com/world-university-rankings</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>حداقل دستمزد ۲۰۲۶ هلند (€14.71)</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>https://arlettipartners.com/new-increase-in-the-dutch-minimum-hourly-wage-from-january-1st-2026/</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
           <t>نرخ ارز (xe.com، ۲۷ سپتامبر ۲۰۲۶)</t>
         </is>
       </c>
-      <c r="B61" s="7" t="inlineStr">
+      <c r="B70" s="7" t="inlineStr">
         <is>
           <t>https://www.xe.com/</t>
         </is>
@@ -2873,6 +3001,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B59" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B60" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B70" r:id="rId69"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Accuracy audit: FAU non-EU tuition from 2027, ITU €16,500, Radboud €19,714, Chalmers ≈SEK 175k, AAU 150 ECTS, Surrey/Newcastle/Sheffield fixes; +8 sources; MD section 9
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Table_final.xlsx
+++ b/Table_final.xlsx
@@ -607,7 +607,7 @@
       <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Stuttgart (اشتوتگارت) – MSc Computer Science (انگلیسی، بدون NC، IELTS 7) → Target
-FAU (Erlangen/Nürnberg) – MSc Artificial Intelligence (انگلیسی، B2) → Target
+FAU (Erlangen/Nürnberg) – MSc Artificial Intelligence (انگلیسی، B2؛ ⚠️ از تابستان ۲۰۲۷ شهریهٔ €4,000/ترم برای غیر-EU) → Target
 TU Darmstadt (دارمشتات) – MSc Computer Science (انگلیسی، IELTS 7) → Target/Reach
 TU Dresden (درسدن) – MSc Computer Science (انگلیسی، IELTS 7، ارزیابی استعداد) → Reach
 Safe: RPTU Kaiserslautern، Passau، Saarland (Saarbrücken)، TU Chemnitz، OVGU Magdeburg</t>
@@ -632,7 +632,7 @@
         <is>
           <t>AAU (Aalborg) – MSc Computer Science (IT) (انگلیسی؛ نه برنامه Computer Science دانمارکی‌زبان) → Target
 SDU (Odense) – MSc Computer Science → Target
-(پذیرش بر اساس داشتن ≥ ۱۰۰ ECTS دروس کامپیوتر)</t>
+(AAU رسماً حداقل ۱۵۰ ECTS دروس مرتبط با CS می‌خواهد و از ۲۰۲۷ سابقهٔ کار را هم در رتبه‌بندی حساب می‌کند؛ SDU هم واحدهای CS ریزنمرات را ارزیابی می‌کند)</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -769,13 +769,14 @@
       <c r="C5" s="4" t="inlineStr">
         <is>
           <t>€0 + سهم ترمی €150–400 (≈ €300–800 در سال)
-Stuttgart: €1,500 در ترم = €3,000 در سال (بادن-وورتمبرگ)</t>
+Stuttgart: €1,500 در ترم = €3,000 در سال (بادن-وورتمبرگ)
+⚠️ FAU: از ترم تابستان ۲۰۲۷ برای ورودی‌های جدید غیر-EU €4,000 در ترم (AI/CS) = €8,000 در سال (BayHIG §13)؛ Passau فعلاً بدون شهریه</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Twente: €21,700
-Radboud: ≈ €19,700 (2025/26) → 2026/27 ≈ €20,500</t>
+Radboud: €19,714 (2026/27، رسمی)</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -787,7 +788,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>AAU: €14,910 (7,455 در ترم)
+          <t>AAU: ≈ €14,910 (2025/26: 7,455 در ترم؛ نرخ ۲۰۲۶ هنوز روی سایت AAU نیست)
 SDU: €17,300 (نرخ رسمی برای ورودی سپتامبر ۲۰۲۶ به بعد — رقم قدیمی €13,900 دیگر معتبر نیست)</t>
         </is>
       </c>
@@ -828,7 +829,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>$350–900 (Stuttgart ≈ $3,400)</t>
+          <t>$350–900 (Stuttgart ≈ $3,400؛ FAU از ۲۰۲۷ ≈ $9,300)</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -931,7 +932,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>$13,000–18,000 (Stuttgart تا $20,500)</t>
+          <t>$13,000–18,000 (Stuttgart تا $20,500؛ FAU از ۲۰۲۷ تا ≈ $26,000)</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -978,7 +979,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>$27,000–36,000 (۲ سال؛ Stuttgart تا $41,000) — ارزان‌ترین</t>
+          <t>$27,000–36,000 (۲ سال؛ Stuttgart تا $41,000؛ FAU از ۲۰۲۷ تا ≈ $53,000) — ارزان‌ترین</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -2001,7 +2002,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q109"/>
+  <dimension ref="A1:Q110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3697,7 +3698,7 @@
       </c>
       <c r="P20" s="4" t="inlineStr">
         <is>
-          <t>Guildford قطب بازی‌سازی و امنیت بریتانیا (نزدیک لندن)؛ رقم 2025/26 + برآورد 2026/27</t>
+          <t>Guildford قطب بازی‌سازی و امنیت بریتانیا (نزدیک لندن)؛ رقم AI برآورد است (Cyber همین دانشگاه: £26,900 برای سپتامبر ۲۰۲۷ رسمی)</t>
         </is>
       </c>
       <c r="Q20" s="8" t="inlineStr">
@@ -3747,12 +3748,12 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>£25,900</t>
+          <t>£25,900 (ورودی فوریه ۲۰۲۷) / £26,900 (سپتامبر ۲۰۲۷)</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>$34,300</t>
+          <t>$34,300–35,600</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
@@ -3779,7 +3780,11 @@
           <t>4/5 — کمبود ساختاری (Bitkom: جزو ۳ کمبود اصلی آلمان)؛ اما ۳۱٪ تیم‌ها هیچ نیروی جونیور ندارند → کارآموزی/گواهی لازم است</t>
         </is>
       </c>
-      <c r="P21" s="4" t="inlineStr"/>
+      <c r="P21" s="4" t="inlineStr">
+        <is>
+          <t>صفحهٔ رسمی الان ورودی ۲۰۲۷ را نشان می‌دهد (رقم رسمی)؛ برای ۲۰۲۸ ≈ £27,900 انتظار داشته باشید</t>
+        </is>
+      </c>
       <c r="Q21" s="8" t="inlineStr">
         <is>
           <t>https://www.surrey.ac.uk/postgraduate/cyber-security-msc</t>
@@ -3995,7 +4000,7 @@
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>£32,300</t>
+          <t>£32,300 (2026)</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -4005,7 +4010,7 @@
       </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
-          <t>2:1 (2:2 با سابقه بررسی می‌شود)</t>
+          <t>2:2 در رشتهٔ کامپیوتری/ریاضی‌محور (طبق QS TopUniversities و IDP — صفحهٔ رسمی را چک کنید)</t>
         </is>
       </c>
       <c r="L24" s="4" t="inlineStr">
@@ -4018,9 +4023,9 @@
           <t>149</t>
         </is>
       </c>
-      <c r="N24" s="12" t="inlineStr">
-        <is>
-          <t>Reach</t>
+      <c r="N24" s="11" t="inlineStr">
+        <is>
+          <t>Target/Reach</t>
         </is>
       </c>
       <c r="O24" s="4" t="inlineStr">
@@ -4165,12 +4170,12 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>£34,340</t>
+          <t>≈ £32,900–34,340 (2026؛ MSc AI for Engineering همین دانشگاه رسماً £32,905)</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>$45,500</t>
+          <t>$43,600–45,500</t>
         </is>
       </c>
       <c r="K26" s="4" t="inlineStr">
@@ -4200,7 +4205,7 @@
       </c>
       <c r="P26" s="4" t="inlineStr">
         <is>
-          <t>رتبهٔ بالا، شهریه و شرط ورود بالا</t>
+          <t>رتبهٔ بالا، شهریه و شرط ورود بالا؛ رقم دقیق MSc AI را از صفحهٔ رسمی بگیرید</t>
         </is>
       </c>
       <c r="Q26" s="8" t="inlineStr">
@@ -5096,7 +5101,7 @@
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>€28,000</t>
+          <t>≈ €28,000 (IDP/collegedunia 2025–26؛ صفحهٔ رسمی چک شود)</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -5436,12 +5441,12 @@
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>€0 + ≈ €130 سهم ترم (≈ €260/سال)</t>
+          <t>€4,000 در ترم برای غیر-EU از ترم تابستان ۲۰۲۷ (€8,000/سال) + €82 سهم ترم</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>$300</t>
+          <t>$9,300</t>
         </is>
       </c>
       <c r="K41" s="4" t="inlineStr">
@@ -5471,7 +5476,7 @@
       </c>
       <c r="P41" s="4" t="inlineStr">
         <is>
-          <t>Siemens/adidas/Schaeffler در منطقه</t>
+          <t>⚠️ FAU طبق BayHIG §13 از تابستان ۲۰۲۷ برای ورودی‌های جدید غیر-EU شهریه می‌گیرد (AI و CS: €4,000/ترم) — ورودی ۲۰۲۸ مشمول است؛ دیگر «رایگان» نیست. Siemens/adidas/Schaeffler در منطقه</t>
         </is>
       </c>
       <c r="Q41" s="8" t="inlineStr">
@@ -5521,12 +5526,12 @@
       </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>€0 + ≈ €130 سهم ترم</t>
+          <t>€2,000 در ترم از تابستان ۲۰۲۷ (€4,000/سال) + €82 سهم ترم</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
         <is>
-          <t>$300</t>
+          <t>$4,700</t>
         </is>
       </c>
       <c r="K42" s="4" t="inlineStr">
@@ -5556,7 +5561,7 @@
       </c>
       <c r="P42" s="4" t="inlineStr">
         <is>
-          <t>رباتیک/خودران؛ صفحهٔ رسمی سپتامبر ۲۰۲۶</t>
+          <t>رباتیک/خودران؛ ⚠️ مشمول شهریهٔ جدید FAU از ۲۰۲۷ (صفحهٔ رسمی شهریه، ۲۰۲۶)</t>
         </is>
       </c>
       <c r="Q42" s="8" t="inlineStr">
@@ -6064,7 +6069,7 @@
       </c>
       <c r="P48" s="4" t="inlineStr">
         <is>
-          <t>کاملاً انگلیسی؛ شهر کوچک و ارزان</t>
+          <t>کاملاً انگلیسی؛ شهر کوچک و ارزان؛ Passau رسماً اعلام کرده «فعلاً» شهریهٔ غیر-EU نمی‌گیرد (برخلاف FAU/TUM) ولی طبق قانون باواریا می‌تواند — قبل از اپلای چک کنید</t>
         </is>
       </c>
       <c r="Q48" s="8" t="inlineStr">
@@ -6959,12 +6964,12 @@
       </c>
       <c r="I59" s="4" t="inlineStr">
         <is>
-          <t>€19,714 (2025/26) → ≈ €20,500</t>
+          <t>€19,714 (2026/27 — نرخ رسمی دانشکدهٔ علوم)</t>
         </is>
       </c>
       <c r="J59" s="4" t="inlineStr">
         <is>
-          <t>$23,400</t>
+          <t>$22,500</t>
         </is>
       </c>
       <c r="K59" s="4" t="inlineStr">
@@ -7044,12 +7049,12 @@
       </c>
       <c r="I60" s="4" t="inlineStr">
         <is>
-          <t>€19,714 (2025/26) → ≈ €20,500</t>
+          <t>€19,714 (2026/27 — نرخ رسمی دانشکدهٔ علوم)</t>
         </is>
       </c>
       <c r="J60" s="4" t="inlineStr">
         <is>
-          <t>$23,400</t>
+          <t>$22,500</t>
         </is>
       </c>
       <c r="K60" s="4" t="inlineStr">
@@ -8392,12 +8397,12 @@
       </c>
       <c r="I76" s="4" t="inlineStr">
         <is>
-          <t>SEK 190,000</t>
+          <t>≈ SEK 180,000–190,000 (کل دوره ≈ 360k–380k)</t>
         </is>
       </c>
       <c r="J76" s="4" t="inlineStr">
         <is>
-          <t>$19,200</t>
+          <t>$18,200–19,200</t>
         </is>
       </c>
       <c r="K76" s="4" t="inlineStr">
@@ -8427,7 +8432,7 @@
       </c>
       <c r="P76" s="4" t="inlineStr">
         <is>
-          <t>Stockholm گران (اتاق SEK 7–10k)</t>
+          <t>Stockholm گران (اتاق SEK 7–10k)؛ رقم دقیق روی kth.se فقط در سامانهٔ اپلای نمایش داده می‌شود</t>
         </is>
       </c>
       <c r="Q76" s="8" t="inlineStr">
@@ -8477,12 +8482,12 @@
       </c>
       <c r="I77" s="4" t="inlineStr">
         <is>
-          <t>SEK 190,000</t>
+          <t>≈ SEK 180,000–190,000</t>
         </is>
       </c>
       <c r="J77" s="4" t="inlineStr">
         <is>
-          <t>$19,200</t>
+          <t>$18,200–19,200</t>
         </is>
       </c>
       <c r="K77" s="4" t="inlineStr">
@@ -8643,12 +8648,12 @@
       </c>
       <c r="I79" s="4" t="inlineStr">
         <is>
-          <t>SEK 160,000</t>
+          <t>≈ SEK 175,000 (2026/27؛ 2025/26: 160,000)</t>
         </is>
       </c>
       <c r="J79" s="4" t="inlineStr">
         <is>
-          <t>$16,200</t>
+          <t>$17,700</t>
         </is>
       </c>
       <c r="K79" s="4" t="inlineStr">
@@ -8678,7 +8683,7 @@
       </c>
       <c r="P79" s="4" t="inlineStr">
         <is>
-          <t>Volvo، Ericsson، Zenseact؛ مهلت ۱۵ ژانویه</t>
+          <t>Volvo، Ericsson، Zenseact؛ مهلت ۱۵ ژانویه؛ ⚠️ طبق صفحهٔ شهریهٔ Chalmers دانشگاه‌های سوئد فعلاً نمی‌توانند از ایران پول دریافت کنند (تحریم بانکی) — پرداخت از کشور ثالث</t>
         </is>
       </c>
       <c r="Q79" s="8" t="inlineStr">
@@ -8728,12 +8733,12 @@
       </c>
       <c r="I80" s="4" t="inlineStr">
         <is>
-          <t>SEK 160,000</t>
+          <t>≈ SEK 175,000 (2026/27)</t>
         </is>
       </c>
       <c r="J80" s="4" t="inlineStr">
         <is>
-          <t>$16,200</t>
+          <t>$17,700</t>
         </is>
       </c>
       <c r="K80" s="4" t="inlineStr">
@@ -8809,12 +8814,12 @@
       </c>
       <c r="I81" s="4" t="inlineStr">
         <is>
-          <t>SEK 160,000</t>
+          <t>≈ SEK 175,000 (2026/27)</t>
         </is>
       </c>
       <c r="J81" s="4" t="inlineStr">
         <is>
-          <t>$16,200</t>
+          <t>$17,700</t>
         </is>
       </c>
       <c r="K81" s="4" t="inlineStr">
@@ -9396,22 +9401,22 @@
       </c>
       <c r="I88" s="4" t="inlineStr">
         <is>
-          <t>€14,910 (€7,455 در ترم)</t>
+          <t>≈ €14,910 (2025/26: €7,455 در ترم؛ نرخ ۲۰۲۶ روی سایت AAU منتشر نشده — mastersportal: €15,340)</t>
         </is>
       </c>
       <c r="J88" s="4" t="inlineStr">
         <is>
-          <t>$17,000</t>
+          <t>$17,000–17,500</t>
         </is>
       </c>
       <c r="K88" s="4" t="inlineStr">
         <is>
-          <t>کارشناسی CS/SE</t>
+          <t>رسمی: حداقل ۱۵۰ ECTS دروس مرتبط با CS (برنامه‌نویسی ۱۵، مهندسی نرم‌افزار ۵، الگوریتم ۵، پایگاه داده ۵، ریاضیات گسسته ۵)؛ از ورودی ۲۰۲۷ سابقهٔ کار و انگیزه‌نامه هم در رتبه‌بندی حساب می‌شود</t>
         </is>
       </c>
       <c r="L88" s="4" t="inlineStr">
         <is>
-          <t>6.5</t>
+          <t>6.5 (هر بخش ≥ 6.0)</t>
         </is>
       </c>
       <c r="M88" s="4">
@@ -9430,7 +9435,7 @@
       </c>
       <c r="P88" s="4" t="inlineStr">
         <is>
-          <t>گزینهٔ Target جدول اصلی؛ PBL (پروژه‌محور)</t>
+          <t>گزینهٔ Target جدول اصلی؛ PBL (پروژه‌محور)؛ ظرفیت محدود</t>
         </is>
       </c>
       <c r="Q88" s="8" t="inlineStr">
@@ -9480,12 +9485,12 @@
       </c>
       <c r="I89" s="4" t="inlineStr">
         <is>
-          <t>€14,910</t>
+          <t>≈ €14,910–15,340</t>
         </is>
       </c>
       <c r="J89" s="4" t="inlineStr">
         <is>
-          <t>$17,000</t>
+          <t>$17,000–17,500</t>
         </is>
       </c>
       <c r="K89" s="4" t="inlineStr">
@@ -9560,12 +9565,12 @@
       </c>
       <c r="I90" s="4" t="inlineStr">
         <is>
-          <t>€14,910</t>
+          <t>≈ €14,910–15,340</t>
         </is>
       </c>
       <c r="J90" s="4" t="inlineStr">
         <is>
-          <t>$17,000</t>
+          <t>$17,000–17,500</t>
         </is>
       </c>
       <c r="K90" s="4" t="inlineStr">
@@ -9644,12 +9649,12 @@
       </c>
       <c r="I91" s="4" t="inlineStr">
         <is>
-          <t>€14,910</t>
+          <t>≈ €14,910–15,340</t>
         </is>
       </c>
       <c r="J91" s="4" t="inlineStr">
         <is>
-          <t>$17,000</t>
+          <t>$17,000–17,500</t>
         </is>
       </c>
       <c r="K91" s="4" t="inlineStr">
@@ -10144,12 +10149,12 @@
       </c>
       <c r="I97" s="4" t="inlineStr">
         <is>
-          <t>€13,400 (€6,700 در ترم)</t>
+          <t>€16,500 (€8,250 در ترم؛ ورودی ۲۰۲۶ — رسمی)</t>
         </is>
       </c>
       <c r="J97" s="4" t="inlineStr">
         <is>
-          <t>$15,300</t>
+          <t>$18,800</t>
         </is>
       </c>
       <c r="K97" s="4" t="inlineStr">
@@ -10184,7 +10189,7 @@
       </c>
       <c r="Q97" s="8" t="inlineStr">
         <is>
-          <t>https://studyindenmark.dk/portal/it-university-of-copenhagen-itu/kobenhavn/games</t>
+          <t>https://en.itu.dk/Programmes/MSc-Programmes/Applying-to-a-MSc-programme/Non-EU-EOES</t>
         </is>
       </c>
     </row>
@@ -10229,12 +10234,12 @@
       </c>
       <c r="I98" s="4" t="inlineStr">
         <is>
-          <t>€13,400</t>
+          <t>€16,500 (€8,250 در ترم)</t>
         </is>
       </c>
       <c r="J98" s="4" t="inlineStr">
         <is>
-          <t>$15,300</t>
+          <t>$18,800</t>
         </is>
       </c>
       <c r="K98" s="4" t="inlineStr">
@@ -10264,12 +10269,12 @@
       </c>
       <c r="P98" s="4" t="inlineStr">
         <is>
-          <t>ارزان‌ترین شهریهٔ کپنهاگ</t>
+          <t>ارزان‌تر از DTU/KU در کپنهاگ؛ رقم قدیمی €13,400 (پورتال studyindenmark) منسوخ است</t>
         </is>
       </c>
       <c r="Q98" s="8" t="inlineStr">
         <is>
-          <t>https://studyindenmark.dk/portal/it-university-of-copenhagen-itu/kobenhavn/computer-science</t>
+          <t>https://en.itu.dk/Programmes/MSc-Programmes/Applying-to-a-MSc-programme/Non-EU-EOES</t>
         </is>
       </c>
     </row>
@@ -10314,12 +10319,12 @@
       </c>
       <c r="I99" s="4" t="inlineStr">
         <is>
-          <t>€13,400</t>
+          <t>€16,500 (€8,250 در ترم)</t>
         </is>
       </c>
       <c r="J99" s="4" t="inlineStr">
         <is>
-          <t>$15,300</t>
+          <t>$18,800</t>
         </is>
       </c>
       <c r="K99" s="4" t="inlineStr">
@@ -10350,7 +10355,7 @@
       <c r="P99" s="4" t="inlineStr"/>
       <c r="Q99" s="8" t="inlineStr">
         <is>
-          <t>https://studyindenmark.dk/portal/it-university-of-copenhagen-itu/kobenhavn/data-science</t>
+          <t>https://en.itu.dk/Programmes/MSc-Programmes/Applying-to-a-MSc-programme/Non-EU-EOES</t>
         </is>
       </c>
     </row>
@@ -10717,15 +10722,23 @@
     <row r="109" ht="34" customHeight="1">
       <c r="B109" s="13" t="inlineStr">
         <is>
+          <t>بازبینی صحت اعداد (۲۷ سپتامبر ۲۰۲۶): ≈۷۰٪ شهریه‌ها مستقیماً از صفحهٔ رسمی 2026/27 است؛ ردیف‌های «≈» از منبع ثانویه یا سال قبل‌اند. اصلاح‌های این بازبینی: FAU از تابستان ۲۰۲۷ شهریه می‌گیرد (AI/CS €4,000/ترم)؛ ITU €16,500 (نه €13,400)؛ Radboud €19,714 رسمی؛ Chalmers ≈ SEK 175k (نه 160k)؛ KTH ≈ 180–190k؛ AAU شرط ≥ ۱۵۰ ECTS؛ Surrey Cyber ورودی ۲۰۲۷؛ Newcastle Games 2:2؛ Sheffield AI ≈ £32.9–34.3k. رتبه‌بندی Safe/Target/Reach، امتیاز بازار و ردهٔ هزینهٔ شهر ارزیابی‌اند، نه دادهٔ رسمی.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="34" customHeight="1">
+      <c r="B110" s="13" t="inlineStr">
+        <is>
           <t>حذف‌شده‌ها: Essex MSc Computer Games (برای 2025/26 و 2026/27 تعلیق شده)، Hull AI &amp; Data Science (سه رقم متناقض شهریه)، UCD/TCD (2:1 و ≈ €30k → Reach، بررسی نشد)، KU Copenhagen (شهریه تأیید نشد)، NCI/DBS ایرلند (کالج خصوصی، اعتبار کمتر).</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:Q103"/>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="B107:Q107"/>
     <mergeCell ref="B108:Q108"/>
+    <mergeCell ref="B110:Q110"/>
     <mergeCell ref="B105:Q105"/>
     <mergeCell ref="B106:Q106"/>
     <mergeCell ref="B109:Q109"/>
@@ -11064,7 +11077,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>متوسط: مدرک‌های ارزان و Safe زیاد است (Maynooth €17k، Skövde، Brunel، ITU) ولی رقابت جونیور بالاست؛ اگر می‌روید، Data Engineering را انتخاب کنید</t>
+          <t>متوسط: مدرک‌های ارزان و Safe زیاد است (Maynooth €17k، Skövde، Brunel، ITU €16.5k) ولی رقابت جونیور بالاست؛ اگر می‌روید، Data Engineering را انتخاب کنید</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -11273,7 +11286,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>ایرلند ۲۵ › آلمان ۲۲ › سوئد ۱۹ = انگلستان ۱۹ › هلند ۱۸ › دانمارک ۱۶.  پیشنهاد: اپلای هم‌زمان به ۲–۳ برنامه ایرلند (UL، Maynooth، TU Dublin) + ۲ برنامه آلمان (Stuttgart، FAU یا یک گزینه Safe)؛ تصمیم نهایی با پذیرش/بورس و وضعیت سفارت‌ها در ۲۰۲۸.</t>
+          <t>ایرلند ۲۵ › آلمان ۲۲ › سوئد ۱۹ = انگلستان ۱۹ › هلند ۱۸ › دانمارک ۱۶.  پیشنهاد: اپلای هم‌زمان به ۲–۳ برنامه ایرلند (UL، Maynooth، TU Dublin) + ۲ برنامه آلمان (Stuttgart + یک گزینه Safe مثل Passau/Saarland؛ FAU فقط اگر شهریهٔ جدید €8,000/سال را می‌پذیرید)؛ تصمیم نهایی با پذیرش/بورس و وضعیت سفارت‌ها در ۲۰۲۸.</t>
         </is>
       </c>
     </row>
@@ -11367,7 +11380,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B112"/>
+  <dimension ref="A1:B120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -11569,12 +11582,12 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>هلند – Radboud Computing Science شهریه</t>
+          <t>هلند – Radboud شهریهٔ رسمی 2026/27 غیر-EEA €19,714 (Data Science and AI؛ دانشکدهٔ علوم)</t>
         </is>
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>https://www.mastersportal.com/studies/8984/computing-science.html</t>
+          <t>https://www.ru.nl/en/education/masters/data-science-and-ai/tuition</t>
         </is>
       </c>
     </row>
@@ -12541,7 +12554,7 @@
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>سوئد – KTH Machine Learning: SEK 190,000</t>
+          <t>سوئد – KTH Machine Learning: ≈ SEK 180,000–190,000 (کل دوره 360k طبق راهنمای ۲۰۲۶؛ kth.se رقم را فقط در سامانه نشان می‌دهد)</t>
         </is>
       </c>
       <c r="B98" s="15" t="inlineStr">
@@ -12577,12 +12590,12 @@
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>دانمارک – ITU شهریه €6,700 در ترم (Games / CS / Data Science)</t>
+          <t>دانمارک – ITU شهریهٔ رسمی ورودی ۲۰۲۶: €8,250 در ترم = €16,500 در سال (رقم قدیمی €6,700 منسوخ)</t>
         </is>
       </c>
       <c r="B101" s="15" t="inlineStr">
         <is>
-          <t>https://studyindenmark.dk/portal/it-university-of-copenhagen-itu/kobenhavn/games</t>
+          <t>https://en.itu.dk/Programmes/MSc-Programmes/Applying-to-a-MSc-programme/Non-EU-EOES</t>
         </is>
       </c>
     </row>
@@ -12715,6 +12728,102 @@
       <c r="B112" s="15" t="inlineStr">
         <is>
           <t>https://collegedunia.com/uk/university/862-nottingham-trent-university-nottingham/ranking</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="4" t="inlineStr">
+        <is>
+          <t>آلمان – FAU: شهریهٔ غیر-EU از ترم تابستان ۲۰۲۷ (AI/CS €4,000، Autonomy Tech €2,000 در ترم؛ BayHIG §13)</t>
+        </is>
+      </c>
+      <c r="B113" s="15" t="inlineStr">
+        <is>
+          <t>https://www.fau.eu/studying/international-students/application-and-enrollment-for-international-applicants/tuition-fees-for-students-from-non-eu-states/</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="4" t="inlineStr">
+        <is>
+          <t>آلمان – Passau: «فعلاً» بدون شهریه برای غیر-EU (اعلام رسمی)</t>
+        </is>
+      </c>
+      <c r="B114" s="15" t="inlineStr">
+        <is>
+          <t>https://www.uni-passau.de/en/study/news/news/no-tuition-fees-for-international-students-at-the-university-of-passau</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="4" t="inlineStr">
+        <is>
+          <t>دانمارک – Aarhus نرخ رسمی 2026/27: Computer Science / Data Science / Computer Engineering €17,300</t>
+        </is>
+      </c>
+      <c r="B115" s="15" t="inlineStr">
+        <is>
+          <t>https://masters.au.dk/tuitionfees/current-tuition-fee-rates</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="4" t="inlineStr">
+        <is>
+          <t>دانمارک – AAU Computer Science (IT): شرط رسمی ≥ ۱۵۰ ECTS دروس CS؛ معیار رتبه‌بندی ۲۰۲۷ شامل سابقهٔ کار</t>
+        </is>
+      </c>
+      <c r="B116" s="15" t="inlineStr">
+        <is>
+          <t>https://www.en.aau.dk/education/master/computer-science-it</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="4" t="inlineStr">
+        <is>
+          <t>سوئد – Chalmers شهریهٔ استاندارد 2026/27 ≈ SEK 175,000 (collegedunia به نقل از صفحهٔ شهریهٔ Chalmers)</t>
+        </is>
+      </c>
+      <c r="B117" s="15" t="inlineStr">
+        <is>
+          <t>https://collegedunia.com/sweden/university/769-chalmers-university-of-technology-gothenburg/programs?stream_id=48&amp;degree_type=Master</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="4" t="inlineStr">
+        <is>
+          <t>انگلستان – Surrey MSc Cyber Security ورودی ۲۰۲۷: £25,900 (فوریه) / £26,900 (سپتامبر)</t>
+        </is>
+      </c>
+      <c r="B118" s="15" t="inlineStr">
+        <is>
+          <t>https://www.surrey.ac.uk/postgraduate/cyber-security-msc</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="4" t="inlineStr">
+        <is>
+          <t>انگلستان – Newcastle MSc Computer Game Engineering £32,300، شرط 2:2 (QS TopUniversities)</t>
+        </is>
+      </c>
+      <c r="B119" s="15" t="inlineStr">
+        <is>
+          <t>https://www.topuniversities.com/universities/newcastle-university/postgrad/msc-computer-game-engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="4" t="inlineStr">
+        <is>
+          <t>هلند – TU/e شهریهٔ رسمی 2026/27 €21,700 (2027/28: €22,400)</t>
+        </is>
+      </c>
+      <c r="B120" s="15" t="inlineStr">
+        <is>
+          <t>https://www.tue.nl/en/education/become-a-tue-student/tuition-fees</t>
         </is>
       </c>
     </row>
@@ -12831,6 +12940,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B110" r:id="rId109"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B111" r:id="rId110"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B112" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B113" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B114" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B115" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B116" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B117" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B118" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B119" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B120" r:id="rId119"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Retarget to September 2027 intake: dated action-plan sheet, deadlines, IELTS/TOEFL-not-in-Iran and exit-permit notes, 2027/28 fees where official; MD sections 5 & 10; +14 sources
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Table_final.xlsx
+++ b/Table_final.xlsx
@@ -1,17 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="جدول نهایی ۲۰۲۶" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="برنامه‌ها" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="حوزه‌ها و بازار کار" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="جمع‌بندی" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="منابع" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="جدول نهایی ۲۰۲۶" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="برنامه‌ها" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="حوزه‌ها و بازار کار" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="برنامهٔ زمانی ۲۰۲۷" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="جمع‌بندی" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="منابع" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'برنامه‌ها'!$A$1:$Q$103</definedName>
@@ -122,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="2"/>
@@ -162,6 +163,9 @@
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1771,7 +1775,7 @@
       </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
-          <t>سایت برنامه‌ها — IELTS معمولاً ۲ سال اعتبار دارد؛ زمان امتحان را با اقدام ۲۰۲۸ هماهنگ کنید</t>
+          <t>سایت برنامه‌ها — ⚠️ IELTS از ۳۱ ژانویه ۲۰۲۶ و TOEFL از ۱۴۰۵ در ایران برگزار نمی‌شوند؛ آزمون را در استانبول/ایروان/دبی/تفلیس بدهید (نتیجهٔ کامپیوتری ۳–۵ روزه). برای مهلت ۱۵ ژانویهٔ ۲۰۲۷ (سوئد/دانمارک/Stuttgart) نتیجه باید تا اوایل ژانویه در دست باشد</t>
         </is>
       </c>
     </row>
@@ -1907,7 +1911,7 @@
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>بسیار بالا: Graduate visa ۱۸ ماه، B2، طرح PR ۱۰ ساله، عوارض £925/دانشجو/سال از اوت ۲۰۲۸ فقط برای دانشگاه‌های انگلستان — یعنی همهٔ گزینه‌های شما (ورودی ۲۰۲۸)؛ احتمالاً به شهریه اضافه می‌شود</t>
+          <t>بسیار بالا: Graduate visa ۱۸ ماه، B2، طرح PR ۱۰ ساله، عوارض £925/دانشجو/سال از اوت ۲۰۲۸ فقط برای دانشگاه‌های انگلستان — دورهٔ یک‌سالهٔ شما (سپتامبر ۲۰۲۷ تا سپتامبر ۲۰۲۸) عملاً از آن رد می‌شود، ولی بعضی دانشگاه‌ها ممکن است از ۲۰۲۷ در شهریه پیش‌خور کنند</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
@@ -1973,7 +1977,7 @@
     <row r="32">
       <c r="B32" t="inlineStr">
         <is>
-          <t>همه ارقام سطح 2026/27 و از منابع رسمی (شیت «منابع»)؛ برای ورودی ۲۰۲۸ سالانه ۳–۵٪ (شهریه ۵–۱۰٪) اضافه کنید. ردیف‌های ۱۳، ۱۴، ۱۷–۱۹، ۲۶ برآورد/ارزیابی هستند و در ستون منبع مشخص شده‌اند.</t>
+          <t>همه ارقام سطح 2026/27 و از منابع رسمی (شیت «منابع»)؛ برای ورودی سپتامبر ۲۰۲۷ نرخ 2027/28 را بگیرید (تا بهار ۲۰۲۷ منتشر می‌شود؛ فعلاً +۳–۵٪). ردیف‌های ۱۳، ۱۴، ۱۷–۱۹، ۲۶ برآورد/ارزیابی هستند و در ستون منبع مشخص شده‌اند.</t>
         </is>
       </c>
     </row>
@@ -2067,7 +2071,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>شهریهٔ سالانه 2026/27 (ارز محلی)</t>
+          <t>شهریهٔ سالانه (2026/27؛ اگر نرخ 2027/28 منتشر شده، ذکر شده) — ارز محلی</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
@@ -3748,12 +3752,12 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>£25,900 (ورودی فوریه ۲۰۲۷) / £26,900 (سپتامبر ۲۰۲۷)</t>
+          <t>£26,900 (ورودی سپتامبر ۲۰۲۷ — رسمی؛ فوریه ۲۰۲۷: £25,900)</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>$34,300–35,600</t>
+          <t>$35,600</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
@@ -3782,7 +3786,7 @@
       </c>
       <c r="P21" s="4" t="inlineStr">
         <is>
-          <t>صفحهٔ رسمی الان ورودی ۲۰۲۷ را نشان می‌دهد (رقم رسمی)؛ برای ۲۰۲۸ ≈ £27,900 انتظار داشته باشید</t>
+          <t>رقم رسمی دقیقاً برای سال ورود شما (سپتامبر ۲۰۲۷)</t>
         </is>
       </c>
       <c r="Q21" s="8" t="inlineStr">
@@ -5476,7 +5480,7 @@
       </c>
       <c r="P41" s="4" t="inlineStr">
         <is>
-          <t>⚠️ FAU طبق BayHIG §13 از تابستان ۲۰۲۷ برای ورودی‌های جدید غیر-EU شهریه می‌گیرد (AI و CS: €4,000/ترم) — ورودی ۲۰۲۸ مشمول است؛ دیگر «رایگان» نیست. Siemens/adidas/Schaeffler در منطقه</t>
+          <t>⚠️ FAU طبق BayHIG §13 از تابستان ۲۰۲۷ برای ورودی‌های جدید غیر-EU شهریه می‌گیرد (AI و CS: €4,000/ترم) — ورودی اکتبر ۲۰۲۷ شما مشمول است؛ دیگر «رایگان» نیست. Siemens/adidas/Schaeffler در منطقه</t>
         </is>
       </c>
       <c r="Q41" s="8" t="inlineStr">
@@ -7721,12 +7725,12 @@
       </c>
       <c r="I68" s="4" t="inlineStr">
         <is>
-          <t>€21,700</t>
+          <t>€22,400 (2027/28 رسمی؛ 2026/27: €21,700)</t>
         </is>
       </c>
       <c r="J68" s="4" t="inlineStr">
         <is>
-          <t>$24,700</t>
+          <t>$25,500</t>
         </is>
       </c>
       <c r="K68" s="4" t="inlineStr">
@@ -7806,12 +7810,12 @@
       </c>
       <c r="I69" s="4" t="inlineStr">
         <is>
-          <t>€21,700</t>
+          <t>€22,400 (2027/28 رسمی؛ 2026/27: €21,700)</t>
         </is>
       </c>
       <c r="J69" s="4" t="inlineStr">
         <is>
-          <t>$24,700</t>
+          <t>$25,500</t>
         </is>
       </c>
       <c r="K69" s="4" t="inlineStr">
@@ -8895,12 +8899,12 @@
       </c>
       <c r="I82" s="4" t="inlineStr">
         <is>
-          <t>SEK 145,000 (کل ۲۹۰k؛ ورودی ۲۰۲۷: ۲۹۴k)</t>
+          <t>SEK 147,000 (ورودی ۲۰۲۷: کل دوره SEK 294,000 رسمی)</t>
         </is>
       </c>
       <c r="J82" s="4" t="inlineStr">
         <is>
-          <t>$14,600–14,800</t>
+          <t>$14,800</t>
         </is>
       </c>
       <c r="K82" s="4" t="inlineStr">
@@ -10701,7 +10705,7 @@
     <row r="106" ht="34" customHeight="1">
       <c r="B106" s="13" t="inlineStr">
         <is>
-          <t>شهریهٔ دلاری با نرخ نرخ تبدیل ۲۷ سپتامبر ۲۰۲۶: €1 = $1.14 · £1 = $1.325 · $1 ≈ SEK 9.9 · $1 ≈ DKK 6.55 و گرد شده به $100. برای ورودی ۲۰۲۸ شهریه‌ها را ۵–۱۰٪ در سال بالاتر فرض کنید. آلمان: عدد فقط سهم ترم (Semesterbeitrag) است که بلیت حمل‌ونقل را هم شامل می‌شود.</t>
+          <t>شهریهٔ دلاری با نرخ نرخ تبدیل ۲۷ سپتامبر ۲۰۲۶: €1 = $1.14 · £1 = $1.325 · $1 ≈ SEK 9.9 · $1 ≈ DKK 6.55 و گرد شده به $100. برای ورودی سپتامبر ۲۰۲۷ نرخ 2027/28 ملاک است (تا بهار ۲۰۲۷ منتشر می‌شود؛ فعلاً +۳–۵٪؛ TU/e و Surrey و Gothenburg همین حالا رسمی‌اند). آلمان: عدد فقط سهم ترم (Semesterbeitrag) است که بلیت حمل‌ونقل را هم شامل می‌شود.</t>
         </is>
       </c>
     </row>
@@ -11223,153 +11227,648 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="130" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="110" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>موضوع</t>
+          <t>تاریخ / مهلت</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>جمع‌بندی</t>
+          <t>اقدام</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>کشور / برنامه</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>جزئیات</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>منبع</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>رتبه‌بندی هزینه کل تا فارغ‌التحصیلی</t>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>همین هفته (اکتبر ۲۰۲۶)</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>آلمان $27–36k  &lt;  ایرلند $32–48k  &lt;  انگلستان $38–65k  &lt;  سوئد $54–65k  &lt;  دانمارک $63–76k  &lt;  هلند $75–90k</t>
+          <t>تعیین تکلیف نظام‌وظیفه</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>همه</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>اگر کارت پایان خدمت یا معافیت دائم ندارید: خروج تحصیلی مشمولانِ بدون غیبت فقط با مجوز سامانهٔ «سخا»، وثیقهٔ ۲۰۰ میلیون تومان (از خرداد/تیر ۱۴۰۵؛ قبلاً ۸۰ میلیون) و پذیرش از دانشگاه مورد تأیید وزارت علوم ممکن است؛ مدت مجوز = طول دوره. این را قبل از هر هزینه‌ای روشن کنید.</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>sakha.epolice.ir؛ زومیت/فرارو تیر ۱۴۰۵</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>فقط با انگلیسی (تحصیل + کار + اداری + اقامت)</t>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>اکتبر ۲۰۲۶</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>ایرلند و انگلستان کامل؛ هلند و سوئد برای زندگی/کار خوب ولی برای اقامت دائم/تابعیت زبان می‌خواهند (هلند B1 در راه، سوئد آزمون تابعیت)؛ دانمارک و آلمان بدون زبان محلی هم بازار کار و هم PR محدود.</t>
+          <t>رزرو آزمون زبان — خارج از ایران</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>همه</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>IELTS از ۳۱ ژانویه ۲۰۲۶ و TOEFL از ۱۴۰۵ در ایران برگزار نمی‌شوند. IELTS Academic کامپیوتری در استانبول/ایروان/دبی/تفلیس برای نوامبر تا اوایل دسامبر ۲۰۲۶ رزرو کنید (نتیجه ۳–۵ روزه؛ ≈ $250–300 + سفر). هدف 7.0 با هر بخش ≥ 6.5 (Stuttgart C1، Saarland 7.0). Duolingo فقط بعضی دانشگاه‌های انگلستان/ایرلند را باز می‌کند، نه سوئد/دانمارک/هلند/آلمان.</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>اعلام IDP (دسامبر ۲۰۲۵)؛ وضعیت ETS/سنجش شهریور ۱۴۰۵</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>بازار کار و حقوق جونیور</t>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>اکتبر ۲۰۲۶</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>حقوق ناخالص: دانمارک &gt; آلمان &gt; هلند ≈ سوئد &gt; ایرلند &gt; انگلستان. دسترسی برای جونیورِ فقط‌انگلیسی: ایرلند ≈ هلند &gt; آلمان &gt; سوئد ≈ دانمارک ≈ انگلستان.</t>
+          <t>مدارک پایه</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>همه</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>ریزنمرات و دانشنامهٔ انگلیسی رسمی (دانشگاه سمنان + تأییدیه‌ها)؛ گواهی رتبه/میانگین کلاس اگر می‌دهند؛ ۲ توصیه‌نامه (استاد + کارفرما)؛ SOP با تکیه بر ۲ سال IT + Unity؛ CV؛ گیت‌هاب مرتب؛ گواهی سابقهٔ کار (AAU از ورودی ۲۰۲۷ برایش امتیاز می‌دهد).</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>نتیجه با وزن برابر برای ۳ معیار</t>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>۱۴–۱۶ اکتبر ۲۰۲۶</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>ایرلند ۲۵ › آلمان ۲۲ › سوئد ۱۹ = انگلستان ۱۹ › هلند ۱۸ › دانمارک ۱۶.  پیشنهاد: اپلای هم‌زمان به ۲–۳ برنامه ایرلند (UL، Maynooth، TU Dublin) + ۲ برنامه آلمان (Stuttgart + یک گزینه Safe مثل Passau/Saarland؛ FAU فقط اگر شهریهٔ جدید €8,000/سال را می‌پذیرید)؛ تصمیم نهایی با پذیرش/بورس و وضعیت سفارت‌ها در ۲۰۲۸.</t>
+          <t>باز شدن پورتال‌ها</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>ایرلند، هلند، سوئد</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Maynooth (۱۴ اکتبر)، UL (۱۵ اکتبر)، فرم بورس UTS Twente (۱۵ اکتبر)، سوئد universityadmissions.se (۱۶ اکتبر — تا ۴ برنامه با یک درخواست، SEK 900).</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>maynoothuniversity.ie؛ ul.ie؛ utwente.nl؛ universityadmissions.se</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>ریسک شماره یک</t>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>نوامبر ۲۰۲۶</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>دسترسی به سفارت‌ها از داخل ایران (ردیف ۲۳): در سپتامبر ۲۰۲۶ هیچ‌کدام از ۶ کشور خدمات عادی ویزای دانشجویی در تهران ندارند. از الان هزینه «برنامه B» (اقدام از ترکیه/ارمنستان/امارات) را در بودجه ببینید.</t>
+          <t>VPD از uni-assist</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>آلمان</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>برای TU Darmstadt، TU Dresden، Saarland، RPTU، Chemnitz، OVGU و Passau (uni-assist) ۴–۶ هفته زمان و €75 هزینه؛ Stuttgart مستقیم در C@MPUS اپلای می‌گیرد (۱۵ نوامبر – ۱۵ ژانویه).</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>uni-assist.de؛ uni-stuttgart.de</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>برنامه زمانی ورودی سپتامبر ۲۰۲۸</t>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>نوامبر – اوایل دسامبر ۲۰۲۶</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>تا بهار ۲۰۲۷: IELTS 7.0 (هر بخش ≥ 6.5) · تابستان ۲۰۲۷: ریزنمرات رسمی + تأییدیه‌ها + VPD uni-assist · پاییز ۲۰۲۷ تا زمستان ۲۰۲۸: اپلای (ایرلند rolling از اکتبر؛ سوئد ۱۵ ژانویه؛ هلند تا ۱ می؛ آلمان ۱۵ ژانویه–۱۵ ژوئیه؛ انگلستان rolling) · بهار ۲۰۲۸: شهریه/تمکن → خوابگاه → ویزا یا برنامه B.</t>
+          <t>آزمون IELTS</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>همه</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>نتیجه باید تا اوایل ژانویه ۲۰۲۷ در دست باشد (سوئد، دانمارک، Stuttgart). یک تاریخ ذخیره در دسامبر رزرو کنید.</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>تغییرات اصلی نسبت به جدول اول</t>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>اواسط دسامبر ۲۰۲۶</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>• هزینه کل دوره اضافه شد (هلند از «نیاز به تأمین سال دوم» به گران‌ترین گزینه تبدیل شد)
-• فقط انگلستان (به خواست شما): Strathclyde و Swansea حذف شدند؛ گزینه‌ها Teesside £17,000 · Northumbria £21,500 · Leicester £24,250 · Essex £24,675 · Brunel £24,795 · York £32,900؛ Graduate visa ۱۸ ماه؛ کف اسپانسری £54,700 / £38,290؛ طرح PR ۱۰ ساله؛ عوارض £925 از ۲۰۲۸ شامل همهٔ گزینه‌ها
-• کف حقوق ۲۰۲۶ همه کشورها به‌روز شد (آلمان €50,700/€45,934؛ هلند €3,122/ماه؛ سوئد SEK 34,470؛ ایرلند €40,904)
-• ایرلند: ۲ سال CSEP = Stamp 4 نه PR؛ تمکن €10,000
-• سوئد: کار دانشجویی ۱۵ ساعت/هفته (ژوئن ۲۰۲۶)؛ شهروندی ۸ سال؛ «BTH یک‌ساله» حذف شد؛ خوابگاه فقط LiU
-• QS 2027؛ شهریه‌های واقعی 2026/27؛ «۷۵٪ قبولی» حذف شد
-• «۱۰۰٪ انگلیسی» برای هلند/سوئد/دانمارک تعدیل شد؛ دانمارک PD2/PD3 تفکیک شد
-• ردیف ویزا برای وضعیت ۲۰۲۶ بازنویسی شد؛ ردیف‌های IELTS، تمکن مالی، پس‌انداز، شهروندی و امتیاز اضافه شد</t>
+          <t>پورتال AAU باز می‌شود</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>دانمارک</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>برای شهریه‌پردازها مهلت ۱۵ ژانویه است (۱ مارس فقط برای EU).</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>en.aau.dk/how-and-when-to-apply</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>چرا «انگلستان» و نه «بریتانیا»</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>به خواست شما فقط دانشگاه‌های انگلستان مقایسه شده‌اند. قوانین ویزا، کار و اقامت در کل بریتانیا یکسان است؛ سه تفاوت عملی: (۱) ارزان‌ترین گزینه‌های انگلستان (Teesside £17,000، Northumbria £21,500) از Swansea/Strathclyde ارزان‌ترند → کل دوره از $48–71k به $38–65k رسید؛ (۲) عوارض £925 به ازای هر دانشجو از اوت ۲۰۲۸ فقط دانشگاه‌های انگلستان را می‌گیرد — یعنی همهٔ گزینه‌های شما؛ (۳) بازار کار فناوری بریتانیا عملاً در انگلستان است (London، Manchester، Cambridge، Bristol، Leeds) — حذف اسکاتلند/ولز به فرصت شغلی لطمه نمی‌زند. برای شهریهٔ کمتر باید رتبهٔ پایین‌تر را بپذیرید: Teesside/Chester بدون رتبه QS، Northumbria ≈ ۵۲۸، Essex ≈ ۴۳۸؛ York (۱۵۸) و Newcastle (۱۴۹) تقریباً دوبرابر گران‌ترند.</t>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>۱۵ ژانویه ۲۰۲۷</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>⛔ مهلت اصلی ۱: سوئد + دانمارک + Stuttgart</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>سوئد، دانمارک، آلمان</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>سوئد (همهٔ دانشگاه‌ها: Linköping، Halmstad، BTH، Chalmers، KTH، Uppsala، Umeå، Skövde)؛ AAU (fee-paying)، Aarhus، DTU (الگوی ۱۵ ژانویه برای غیر-EU)؛ Stuttgart MSc Computer Science / INFOTECH.</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>umu.se و uu.se key dates؛ en.aau.dk؛ uni-stuttgart.de</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>نکته پروفایل</t>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>۳۱ ژانویه ۲۰۲۷</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>معدل (۱۵.۷۷ طبق جدول اول؛ ۱۵.۷۰ طبق نقد دوم — تفاوتی در نتیجه ندارد) برای همه برنامه‌های بالا بالاتر از حداقل است. مهم‌تر از معدل، تطابق ریزنمرات با پیش‌نیازها (ریاضی، الگوریتم، CS نظری) و SOP با تکیه بر ۲ سال سابقه کار + بازی‌سازی + پروژه‌های گیت‌هاب است.</t>
+          <t>مهلت بورس Radboud</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>هلند</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Radboud Scholarship Programme (≈۳۳ نفر؛ شهریه به €2,694 می‌رسد) — اپلای اصلی هم باید تا این تاریخ کامل باشد.</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>ru.nl deadlines</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>اعداد را چگونه بخوانم</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>همه مبالغ سطح 2026/27 هستند؛ برای ۲۰۲۸ سالانه ۳–۵٪ (شهریه ۵–۱۰٪) اضافه کنید. نرخ تبدیل ۲۷ سپتامبر ۲۰۲۶: €1 = $1.14 · £1 = $1.325 · $1 ≈ SEK 9.9 · $1 ≈ DKK 6.55</t>
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>۱ فوریه ۲۰۲۷</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>⛔ مهلت اصلی ۲</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>سوئد، دانمارک، هلند</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>سوئد: مدارک + SEK 900 روی universityadmissions.se؛ SDU (غیر-EU)؛ Twente: برای بورس UTS (۱ آوریل) اپلای را تا اوایل فوریه بفرستید.</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>universityadmissions.se؛ sdu.dk/datalogi؛ utwente.nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>فوریه – مارس ۲۰۲۷</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>اپلای ایرلند و انگلستان</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>ایرلند، انگلستان</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>همه rolling هستند ولی زود اپلای کنید: بورس‌ها (Brunel، DCU، Northumbria) و ظرفیت‌ها زود پر می‌شود؛ TU Dublin بین‌المللی ≈ ۳۱ می، Maynooth غیر-EU ≈ ۱۵ می تا ژوئن، UL غیر-EU ویزایی ۱ ژوئیه.</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>studyinireland.app؛ ul.ie/gps/applications-faq</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>۳۰ مارس – ۱ آوریل ۲۰۲۷</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>نتایج سوئد</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>سوئد</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>پاسخ به پیشنهاد در مهلت؛ قسط اول شهریه قبل از درخواست اقامت تحصیلی.</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>universityadmissions.se</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>۱ آوریل ۲۰۲۷</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>⛔ مهلت اصلی ۳</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>هلند، آلمان</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Radboud غیر-EU (اپلای اصلی)؛ بورس UTS Twente؛ پنجرهٔ Passau AI Engineering باز می‌شود (۱ آوریل – ۳۱ می).</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>ru.nl؛ utwente.nl؛ uni-passau.de</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>۱۵ آوریل ۲۰۲۷</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>دور دوم سوئد (فقط پشتیبان)</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>سوئد</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>۱۵ مارس – ۱۵ آوریل؛ مدارک تا ۲۱ ژوئن؛ نتیجه ۹ ژوئیه — برای اقامت و خوابگاه دیر است.</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>umu.se key dates</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>۱ می ۲۰۲۷</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>⛔ مهلت Twente (غیر-EEA)</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>هلند</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>MSc Computer Science / Embedded Systems / Interaction Technology.</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>utwente.nl (به نقل از collegedunia، اوت ۲۰۲۶)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>۱۵ – ۳۱ می ۲۰۲۷</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>مهلت‌های ایرلند و آلمان</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>ایرلند، آلمان</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Maynooth غیر-EU ≈ ۱۵ می؛ TU Dublin بین‌المللی ≈ ۳۱ می؛ Passau AI Eng ۳۱ می؛ بقیهٔ آلمان (TU Darmstadt، TU Dresden، Saarland، RPTU، Chemnitz، OVGU، FAU) بیشتر بین ۱۵ می تا ۱۵ ژوئیه — هر کدام را جدا چک کنید.</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>studyinireland.app؛ uni-passau.de؛ سایت دانشگاه‌ها</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>می – ژوئن ۲۰۲۷</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>💰 پول باید نقد و قابل انتقال باشد</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>همه</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>SDU: یک سال شهریه پیش‌پرداخت (€17,300)؛ سوئد: قسط ترم اول + تمکن SEK 10,656 × ماه‌ها؛ هلند: شهریه + €13,569 زندگی به حساب دانشگاه (Radboud تا ۱ ژوئن)؛ آلمان: حساب مسدود €11,904 (Fintiba ایران را نمی‌پذیرد → Expatrio/Coracle) + Stuttgart €1,500؛ ایرلند: €10,000 + حداقل €6,000 شهریه؛ انگلستان: ودیعه → CAS + £1,203 × ۹ ماه. انتقال از کشور ثالث/صرافی ۳–۶٪ هزینه.</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>ردیف ۲۵ جدول اصلی</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>۱ ژوئن ۲۰۲۷</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>مهلت ثبت‌نام/ویزای Radboud</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>هلند</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>برای شروع سپتامبر (غیر-EU)؛ درخواست MVV را دانشگاه از طرف شما به IND می‌دهد.</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>ru.nl deadlines</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>۱ ژوئیه ۲۰۲۷</t>
+        </is>
+      </c>
+      <c r="B20" s="15" t="inlineStr">
+        <is>
+          <t>⛔ مهلت UL (غیر-EU ویزایی)</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>ایرلند</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>الگوی ۲۰۲۶: ۱ ژوئیه ساعت ۱۲؛ بعد از آن بررسی نمی‌شود.</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>ul.ie/gps/applications-faq</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>ژوئن – ژوئیه ۲۰۲۷</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>🛂 ویزا / برنامهٔ B</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>همه</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>وضعیت تهران (سپتامبر ۲۰۲۶): آلمان حالت اضطراری، هلند از باکو، دانمارک «از ایران ممکن نیست»، ایرلند کنسول بسته، انگلستان VFS متناوب؛ سوئد بدون بیومتریک (آنلاین). یعنی برای DE/DK/IE/UK سفر به ترکیه/ارمنستان/امارات را (۲–۶ هفته) در بودجه و تقویم بگذارید.</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>ردیف ۲۳ جدول اصلی</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>ژوئیه ۲۰۲۷</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>خوابگاه</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>همه</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Twente/Radboud اتاق رزروشده برای بین‌المللی‌ها (مهلت‌دار)؛ Linköping یک پیشنهاد اتاق برای شهریه‌پردازها؛ آلمان لیست Studierendenwerk بلافاصله بعد از پذیرش؛ ایرلند/انگلستان خوابگاه دانشگاه زود پر می‌شود.</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>ردیف‌های ۹–۱۰ جدول اصلی</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>اوت – اکتبر ۲۰۲۷</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>شروع</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>همه</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>سوئد ≈ ۳۰ اوت؛ دانمارک ۱ سپتامبر؛ هلند اوایل سپتامبر؛ ایرلند/انگلستان اواسط تا اواخر سپتامبر؛ آلمان ترم زمستان از ۱ اکتبر (کلاس‌ها ≈ اواسط اکتبر).</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="60" customHeight="1">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>جمع‌بندی: ورودی سپتامبر ۲۰۲۷ شدنی است، فقط اگر (۱) IELTS تا دسامبر ۲۰۲۶ خارج از ایران گرفته شود، (۲) پول سال اول تا می ۲۰۲۷ نقد و قابل انتقال باشد، (۳) وضعیت نظام‌وظیفه/مجوز خروج روشن باشد. سوئد، دانمارک و Stuttgart با مهلت ۱۵ ژانویه سخت‌ترین‌اند؛ ایرلند، انگلستان، هلند و بیشتر آلمان تا بهار ۲۰۲۷ وقت دارند — اگر IELTS به ژانویه نرسید، تمرکز را روی این‌ها بگذارید. مهلت‌های علامت «≈» از منابع ثانویه‌اند؛ تاریخ دقیق را از صفحهٔ برنامه بگیرید.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A25:E25"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11380,7 +11879,176 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B120"/>
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="130" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>موضوع</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>جمع‌بندی</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>رتبه‌بندی هزینه کل تا فارغ‌التحصیلی</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>آلمان $27–36k  &lt;  ایرلند $32–48k  &lt;  انگلستان $38–65k  &lt;  سوئد $54–65k  &lt;  دانمارک $63–76k  &lt;  هلند $75–90k</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>فقط با انگلیسی (تحصیل + کار + اداری + اقامت)</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>ایرلند و انگلستان کامل؛ هلند و سوئد برای زندگی/کار خوب ولی برای اقامت دائم/تابعیت زبان می‌خواهند (هلند B1 در راه، سوئد آزمون تابعیت)؛ دانمارک و آلمان بدون زبان محلی هم بازار کار و هم PR محدود.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>بازار کار و حقوق جونیور</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>حقوق ناخالص: دانمارک &gt; آلمان &gt; هلند ≈ سوئد &gt; ایرلند &gt; انگلستان. دسترسی برای جونیورِ فقط‌انگلیسی: ایرلند ≈ هلند &gt; آلمان &gt; سوئد ≈ دانمارک ≈ انگلستان.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>نتیجه با وزن برابر برای ۳ معیار</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>ایرلند ۲۵ › آلمان ۲۲ › سوئد ۱۹ = انگلستان ۱۹ › هلند ۱۸ › دانمارک ۱۶.  پیشنهاد: اپلای هم‌زمان به ۲–۳ برنامه ایرلند (UL، Maynooth، TU Dublin) + ۲ برنامه آلمان (Stuttgart + یک گزینه Safe مثل Passau/Saarland؛ FAU فقط اگر شهریهٔ جدید €8,000/سال را می‌پذیرید)؛ تصمیم نهایی با پذیرش/بورس و وضعیت سفارت‌ها در بهار ۲۰۲۷.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>ریسک شماره یک</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>دسترسی به سفارت‌ها از داخل ایران (ردیف ۲۳): در سپتامبر ۲۰۲۶ هیچ‌کدام از ۶ کشور خدمات عادی ویزای دانشجویی در تهران ندارند. از الان هزینه «برنامه B» (اقدام از ترکیه/ارمنستان/امارات) را در بودجه ببینید.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>برنامه زمانی ورودی سپتامبر ۲۰۲۷ (فشرده — جزئیات در شیت «برنامهٔ زمانی ۲۰۲۷»)</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>اکتبر ۲۰۲۶: نظام‌وظیفه + رزرو IELTS خارج از ایران + مدارک · ۱۶ اکتبر: باز شدن سوئد · نوامبر–دسامبر: IELTS + VPD uni-assist · ۱۵ ژانویه ۲۰۲۷: مهلت سوئد / AAU / Stuttgart · ۱ فوریه: مدارک سوئد + SDU · فوریه–مارس: ایرلند و انگلستان · ۱ آوریل: Radboud · ۱ می: Twente · ۳۱ می: Passau / TU Dublin · می–ژوئن: پول + ویزا یا برنامهٔ B · ۱ ژوئیه: UL · اوت–اکتبر: شروع.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>سه پیش‌نیاز عملی ورودی ۲۰۲۷</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>(۱) آزمون زبان: IELTS و TOEFL در ایران برگزار نمی‌شوند → سفر به ترکیه/ارمنستان/امارات/گرجستان تا دسامبر ۲۰۲۶. (۲) نظام‌وظیفه: بدون کارت/معافیت، خروج تحصیلی فقط با مجوز سخا + وثیقهٔ ۲۰۰ میلیون تومان + پذیرش از دانشگاه مورد تأیید وزارت علوم. (۳) نقدینگی: شهریه/تمکن سال اول باید تا می–ژوئن ۲۰۲۷ قابل انتقال باشد (SDU یک سال کامل پیش‌پرداخت). اگر یکی از این سه تا ژانویه ۲۰۲۷ حل نشود، هدف واقع‌بینانه ایرلند/انگلستان/هلند/آلمان با مهلت‌های بهار ۲۰۲۷ است — یا ورودی ۲۰۲۸.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>تغییرات اصلی نسبت به جدول اول</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>• هزینه کل دوره اضافه شد (هلند از «نیاز به تأمین سال دوم» به گران‌ترین گزینه تبدیل شد)
+• فقط انگلستان (به خواست شما): Strathclyde و Swansea حذف شدند؛ گزینه‌ها Teesside £17,000 · Northumbria £21,500 · Leicester £24,250 · Essex £24,675 · Brunel £24,795 · York £32,900؛ Graduate visa ۱۸ ماه؛ کف اسپانسری £54,700 / £38,290؛ طرح PR ۱۰ ساله؛ عوارض £925 از ۲۰۲۸ شامل همهٔ گزینه‌ها
+• کف حقوق ۲۰۲۶ همه کشورها به‌روز شد (آلمان €50,700/€45,934؛ هلند €3,122/ماه؛ سوئد SEK 34,470؛ ایرلند €40,904)
+• ایرلند: ۲ سال CSEP = Stamp 4 نه PR؛ تمکن €10,000
+• سوئد: کار دانشجویی ۱۵ ساعت/هفته (ژوئن ۲۰۲۶)؛ شهروندی ۸ سال؛ «BTH یک‌ساله» حذف شد؛ خوابگاه فقط LiU
+• QS 2027؛ شهریه‌های واقعی 2026/27؛ «۷۵٪ قبولی» حذف شد
+• «۱۰۰٪ انگلیسی» برای هلند/سوئد/دانمارک تعدیل شد؛ دانمارک PD2/PD3 تفکیک شد
+• ردیف ویزا برای وضعیت ۲۰۲۶ بازنویسی شد؛ ردیف‌های IELTS، تمکن مالی، پس‌انداز، شهروندی و امتیاز اضافه شد</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>چرا «انگلستان» و نه «بریتانیا»</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>به خواست شما فقط دانشگاه‌های انگلستان مقایسه شده‌اند. قوانین ویزا، کار و اقامت در کل بریتانیا یکسان است؛ سه تفاوت عملی: (۱) ارزان‌ترین گزینه‌های انگلستان (Teesside £17,000، Northumbria £21,500) از Swansea/Strathclyde ارزان‌ترند → کل دوره از $48–71k به $38–65k رسید؛ (۲) عوارض £925 به ازای هر دانشجو از اوت ۲۰۲۸ فقط دانشگاه‌های انگلستان را می‌گیرد — یعنی همهٔ گزینه‌های شما؛ (۳) بازار کار فناوری بریتانیا عملاً در انگلستان است (London، Manchester، Cambridge، Bristol، Leeds) — حذف اسکاتلند/ولز به فرصت شغلی لطمه نمی‌زند. برای شهریهٔ کمتر باید رتبهٔ پایین‌تر را بپذیرید: Teesside/Chester بدون رتبه QS، Northumbria ≈ ۵۲۸، Essex ≈ ۴۳۸؛ York (۱۵۸) و Newcastle (۱۴۹) تقریباً دوبرابر گران‌ترند.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>نکته پروفایل</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>معدل (۱۵.۷۷ طبق جدول اول؛ ۱۵.۷۰ طبق نقد دوم — تفاوتی در نتیجه ندارد) برای همه برنامه‌های بالا بالاتر از حداقل است. مهم‌تر از معدل، تطابق ریزنمرات با پیش‌نیازها (ریاضی، الگوریتم، CS نظری) و SOP با تکیه بر ۲ سال سابقه کار + بازی‌سازی + پروژه‌های گیت‌هاب است.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>اعداد را چگونه بخوانم</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>مبالغ سطح 2026/27 هستند؛ نرخ 2027/28 (سال ورود شما) بین اکتبر ۲۰۲۶ تا بهار ۲۰۲۷ منتشر می‌شود — جایی که رسمی بود (TU/e €22,400، Surrey £26,900، Gothenburg SEK 294k کل) در جدول آمده؛ برای بقیه فعلاً ۳–۵٪ اضافه کنید. نرخ تبدیل ۲۷ سپتامبر ۲۰۲۶: €1 = $1.14 · £1 = $1.325 · $1 ≈ SEK 9.9 · $1 ≈ DKK 6.55</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -11405,7 +12073,7 @@
           <t>آلمان – EU Blue Card 2026 (€50,700 / €45,934.20)</t>
         </is>
       </c>
-      <c r="B2" s="15" t="inlineStr">
+      <c r="B2" s="16" t="inlineStr">
         <is>
           <t>https://www.make-it-in-germany.com/en/visa-residence/types/eu-blue-card</t>
         </is>
@@ -11417,7 +12085,7 @@
           <t>آلمان – Sperrkonto €992/ماه (2026)</t>
         </is>
       </c>
-      <c r="B3" s="15" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>https://www.make-it-in-germany.com/en/study-training/study/financing</t>
         </is>
@@ -11429,7 +12097,7 @@
           <t>آلمان – Niederlassungserlaubnis §18c (فارغ‌التحصیلان، ۲ سال، B1)</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>https://www.make-it-in-germany.com/en/visa-residence/living-permanently/permanent-residence</t>
         </is>
@@ -11441,7 +12109,7 @@
           <t>آلمان – Stuttgart MSc Computer Science (انگلیسی، IELTS 7، €1,500/ترم)</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>https://www.uni-stuttgart.de/en/study/study-programs/Computer-Science-M.Sc./</t>
         </is>
@@ -11453,7 +12121,7 @@
           <t>آلمان – FAU MSc Artificial Intelligence (انگلیسی، B2)</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="16" t="inlineStr">
         <is>
           <t>https://www.ai.study.fau.eu/prospective-students/living-studying-in-germany/language-proficiency/</t>
         </is>
@@ -11465,7 +12133,7 @@
           <t>آلمان – TU Darmstadt MSc Computer Science</t>
         </is>
       </c>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>https://www.informatik.tu-darmstadt.de/studium_fb20/im_studium/studiengaenge_liste/computer_science_msc.en.jsp</t>
         </is>
@@ -11477,7 +12145,7 @@
           <t>آلمان – TU Dresden MSc Computer Science admission</t>
         </is>
       </c>
-      <c r="B8" s="15" t="inlineStr">
+      <c r="B8" s="16" t="inlineStr">
         <is>
           <t>https://tu-dresden.de/ing/informatik/studium/studienangebot/master-studiengaenge/m-sc-computer-science/admission?set_language=en</t>
         </is>
@@ -11489,7 +12157,7 @@
           <t>آلمان – TLScontact Tehran (لیست انتظار دانشجویی)</t>
         </is>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>https://visas-de.tlscontact.com/en-us/country/ir/vac/irTHR2de</t>
         </is>
@@ -11501,7 +12169,7 @@
           <t>آلمان – وضعیت سفارت تهران (Iran International، اوت ۲۰۲۶)</t>
         </is>
       </c>
-      <c r="B10" s="15" t="inlineStr">
+      <c r="B10" s="16" t="inlineStr">
         <is>
           <t>https://www.iranintl.com/en/202608115899</t>
         </is>
@@ -11513,7 +12181,7 @@
           <t>آلمان – Fintiba: ساکنان ایران پذیرفته نمی‌شوند</t>
         </is>
       </c>
-      <c r="B11" s="15" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
         <is>
           <t>https://www.simplegermany.com/best-blocked-account-germany/</t>
         </is>
@@ -11525,7 +12193,7 @@
           <t>آلمان – حقوق توسعه‌دهنده (StepStone)</t>
         </is>
       </c>
-      <c r="B12" s="15" t="inlineStr">
+      <c r="B12" s="16" t="inlineStr">
         <is>
           <t>https://www.stepstone.de/gehalt/Software-Entwickler-in.html</t>
         </is>
@@ -11537,7 +12205,7 @@
           <t>هلند – IND مبالغ ۲۰۲۶ (HSM €3,122 / €4,357؛ دانشجو €1,130.77)</t>
         </is>
       </c>
-      <c r="B13" s="15" t="inlineStr">
+      <c r="B13" s="16" t="inlineStr">
         <is>
           <t>https://ind.nl/en/required-amounts-income-requirements</t>
         </is>
@@ -11549,7 +12217,7 @@
           <t>هلند – Twente شهریه 2026/27 €21,700</t>
         </is>
       </c>
-      <c r="B14" s="15" t="inlineStr">
+      <c r="B14" s="16" t="inlineStr">
         <is>
           <t>https://www.utwente.nl/en/education/master/programmes/computer-science/finance/</t>
         </is>
@@ -11561,7 +12229,7 @@
           <t>هلند – Twente حداقل معدل برای مدرک ایرانی (۱۵/۲۰)</t>
         </is>
       </c>
-      <c r="B15" s="15" t="inlineStr">
+      <c r="B15" s="16" t="inlineStr">
         <is>
           <t>https://www.utwente.nl/en/education/master/programmes/european-studies/admission/international/</t>
         </is>
@@ -11573,7 +12241,7 @@
           <t>هلند – Twente QS 2027 = 223</t>
         </is>
       </c>
-      <c r="B16" s="15" t="inlineStr">
+      <c r="B16" s="16" t="inlineStr">
         <is>
           <t>https://www.utwente.nl/en/about-us/impact-ambitions/rankings/</t>
         </is>
@@ -11585,7 +12253,7 @@
           <t>هلند – Radboud شهریهٔ رسمی 2026/27 غیر-EEA €19,714 (Data Science and AI؛ دانشکدهٔ علوم)</t>
         </is>
       </c>
-      <c r="B17" s="15" t="inlineStr">
+      <c r="B17" s="16" t="inlineStr">
         <is>
           <t>https://www.ru.nl/en/education/masters/data-science-and-ai/tuition</t>
         </is>
@@ -11597,7 +12265,7 @@
           <t>هلند – MVV در ایران (سفارت در باکو)</t>
         </is>
       </c>
-      <c r="B18" s="15" t="inlineStr">
+      <c r="B18" s="16" t="inlineStr">
         <is>
           <t>https://www.netherlandsworldwide.nl/visa-the-netherlands/mvv-long-stay/apply-iran</t>
         </is>
@@ -11609,7 +12277,7 @@
           <t>هلند – B1 برای PR/تابعیت (تصمیم کابینه ۲۰۲۶)</t>
         </is>
       </c>
-      <c r="B19" s="15" t="inlineStr">
+      <c r="B19" s="16" t="inlineStr">
         <is>
           <t>https://thedutchdaily.nl/dutch-citizenship-b1-language-requirement-confirmed-2026/</t>
         </is>
@@ -11621,7 +12289,7 @@
           <t>سوئد – قوانین جدید اقامت تحصیلی از ۱۱ ژوئن ۲۰۲۶ (۱۵ ساعت/هفته)</t>
         </is>
       </c>
-      <c r="B20" s="15" t="inlineStr">
+      <c r="B20" s="16" t="inlineStr">
         <is>
           <t>https://www.migrationsverket.se/nyheter/news-archive/2026-05-25-new-rules-for-residence-permits-for-studies-in-higher-education.html</t>
         </is>
@@ -11633,7 +12301,7 @@
           <t>سوئد – قوانین جدید مجوز کار از ۱ ژوئن ۲۰۲۶ (SEK 34,470)</t>
         </is>
       </c>
-      <c r="B21" s="15" t="inlineStr">
+      <c r="B21" s="16" t="inlineStr">
         <is>
           <t>https://www.migrationsverket.se/nyheter/news-archive/2026-04-17-new-rules-for-work-permits-from-1-june-2026.html</t>
         </is>
@@ -11645,7 +12313,7 @@
           <t>سوئد – گروه‌های معاف (فارغ‌التحصیلان ۷۵٪)</t>
         </is>
       </c>
-      <c r="B22" s="15" t="inlineStr">
+      <c r="B22" s="16" t="inlineStr">
         <is>
           <t>https://eiglaw.com/sweden-publishes-exempt-occupations-for-new-salary-rule/</t>
         </is>
@@ -11657,7 +12325,7 @@
           <t>سوئد – مجوز ۱۲ ماهه جست‌وجوی کار و تمکن SEK 10,656</t>
         </is>
       </c>
-      <c r="B23" s="15" t="inlineStr">
+      <c r="B23" s="16" t="inlineStr">
         <is>
           <t>https://www.migrationsverket.se/en/you-want-to-extend/study/look-for-work-after-completing-your-studies-in-sweden.html</t>
         </is>
@@ -11669,7 +12337,7 @@
           <t>سوئد – Linköping MSc CS شهریه SEK 332,000 (کل)</t>
         </is>
       </c>
-      <c r="B24" s="15" t="inlineStr">
+      <c r="B24" s="16" t="inlineStr">
         <is>
           <t>https://liu.se/en/education/program/6mics</t>
         </is>
@@ -11681,7 +12349,7 @@
           <t>سوئد – BTH MSc Software Engineering 120 credits (SEK 70,000/ترم)</t>
         </is>
       </c>
-      <c r="B25" s="15" t="inlineStr">
+      <c r="B25" s="16" t="inlineStr">
         <is>
           <t>https://www.bth.se/english/education/programmes/masters-programme-in-software-engineering-120-credits</t>
         </is>
@@ -11693,7 +12361,7 @@
           <t>سوئد – BTH برنامه ۶۰ واحدی (از راه دور، نیمه‌وقت، ۲ سال سابقه)</t>
         </is>
       </c>
-      <c r="B26" s="15" t="inlineStr">
+      <c r="B26" s="16" t="inlineStr">
         <is>
           <t>https://www.bth.se/english/education/programmes/masters-programme-in-software-engineering-60-credits</t>
         </is>
@@ -11705,7 +12373,7 @@
           <t>سوئد – Halmstad MSc Information Technology شهریه</t>
         </is>
       </c>
-      <c r="B27" s="15" t="inlineStr">
+      <c r="B27" s="16" t="inlineStr">
         <is>
           <t>https://www.mastersportal.com/studies/22787/information-technology.html</t>
         </is>
@@ -11717,7 +12385,7 @@
           <t>سوئد – Halmstad مسکن (بدون تضمین)</t>
         </is>
       </c>
-      <c r="B28" s="15" t="inlineStr">
+      <c r="B28" s="16" t="inlineStr">
         <is>
           <t>https://www.hh.se/english/education/student-life/find-accommodation.html</t>
         </is>
@@ -11729,7 +12397,7 @@
           <t>سوئد – شهروندی ۸ ساله از ژوئن ۲۰۲۶</t>
         </is>
       </c>
-      <c r="B29" s="15" t="inlineStr">
+      <c r="B29" s="16" t="inlineStr">
         <is>
           <t>https://www.imidaily.com/europe/sweden-passes-law-curtailing-naturalization-8-year-wait-income-floor/</t>
         </is>
@@ -11741,7 +12409,7 @@
           <t>سوئد – اطلاعیه مهاجرتی سفارت تهران</t>
         </is>
       </c>
-      <c r="B30" s="15" t="inlineStr">
+      <c r="B30" s="16" t="inlineStr">
         <is>
           <t>https://www.swedenabroad.se/globalassets/ambassader/iran-teheran/documents/migration-issues/new-folder/english-versin.pdf</t>
         </is>
@@ -11753,7 +12421,7 @@
           <t>دانمارک – Pay Limit Scheme 2026</t>
         </is>
       </c>
-      <c r="B31" s="15" t="inlineStr">
+      <c r="B31" s="16" t="inlineStr">
         <is>
           <t>https://www.nyidanmark.dk/pl-PL/You-want-to-apply/Work/Pay-limit-scheme</t>
         </is>
@@ -11765,7 +12433,7 @@
           <t>دانمارک – برنامه‌های آموزش عالی: ۹۰ ساعت/ماه، ۶ ماه یا ۳ سال جست‌وجوی کار</t>
         </is>
       </c>
-      <c r="B32" s="15" t="inlineStr">
+      <c r="B32" s="16" t="inlineStr">
         <is>
           <t>https://www.nyidanmark.dk/en-GB/You-want-to-apply/Study/Higher-Education</t>
         </is>
@@ -11777,7 +12445,7 @@
           <t>دانمارک – مجوز ۳ ساله جست‌وجوی کار</t>
         </is>
       </c>
-      <c r="B33" s="15" t="inlineStr">
+      <c r="B33" s="16" t="inlineStr">
         <is>
           <t>https://www.nyidanmark.dk/de-DE/You-want-to-apply/Study/Study---job-seeking/Study---3-years-job-seeking</t>
         </is>
@@ -11789,7 +12457,7 @@
           <t>دانمارک – اقامت دائم</t>
         </is>
       </c>
-      <c r="B34" s="15" t="inlineStr">
+      <c r="B34" s="16" t="inlineStr">
         <is>
           <t>https://www.nyidanmark.dk/de-DE/You-want-to-apply/Permanent-residence-permit/Permanent-residence</t>
         </is>
@@ -11801,7 +12469,7 @@
           <t>دانمارک – تمکن DKK 7,426 (2026)</t>
         </is>
       </c>
-      <c r="B35" s="15" t="inlineStr">
+      <c r="B35" s="16" t="inlineStr">
         <is>
           <t>https://nyidanmark.dk/en-GB/Words-and-concepts/SIRI/Self-support---SIRI</t>
         </is>
@@ -11813,7 +12481,7 @@
           <t>دانمارک – AAU Computer Science (IT) شهریه €7,455/ترم</t>
         </is>
       </c>
-      <c r="B36" s="15" t="inlineStr">
+      <c r="B36" s="16" t="inlineStr">
         <is>
           <t>https://studyindenmark.dk/portal/aalborg-university-aau/aalborg/computer-science-it-msc</t>
         </is>
@@ -11825,7 +12493,7 @@
           <t>دانمارک – SDU شهریهٔ رسمی از ورودی ۲۰۲۶: Science/Engineering €17,300 در سال</t>
         </is>
       </c>
-      <c r="B37" s="15" t="inlineStr">
+      <c r="B37" s="16" t="inlineStr">
         <is>
           <t>https://www.sdu.dk/en/uddannelse/fees_and_funding/tuition</t>
         </is>
@@ -11837,7 +12505,7 @@
           <t>دانمارک – SDU MSc Computer Science (ظرفیت محدود، €17,300)</t>
         </is>
       </c>
-      <c r="B38" s="15" t="inlineStr">
+      <c r="B38" s="16" t="inlineStr">
         <is>
           <t>https://www.sdu.dk/en/uddannelse/kandidat/datalogi/adgangskrav</t>
         </is>
@@ -11849,7 +12517,7 @@
           <t>دانمارک – سفارت تهران (درخواست از ایران ممکن نیست)</t>
         </is>
       </c>
-      <c r="B39" s="15" t="inlineStr">
+      <c r="B39" s="16" t="inlineStr">
         <is>
           <t>https://iran.um.dk/en</t>
         </is>
@@ -11861,7 +12529,7 @@
           <t>دانمارک – IDA حقوق شروع ۲۰۲۶</t>
         </is>
       </c>
-      <c r="B40" s="15" t="inlineStr">
+      <c r="B40" s="16" t="inlineStr">
         <is>
           <t>https://studerende.ida.dk/snart-nyuddannet/loen/softwareingenioer-loen-saa-meget-kommer-du-til-at-tjene/</t>
         </is>
@@ -11873,7 +12541,7 @@
           <t>ایرلند – کف حقوق مجوز کار از ۱ مارس ۲۰۲۶ (€40,904 / €36,848 / €36,605)</t>
         </is>
       </c>
-      <c r="B41" s="15" t="inlineStr">
+      <c r="B41" s="16" t="inlineStr">
         <is>
           <t>https://kodlyons.ie/critical-skills-employment-permit-changes/</t>
         </is>
@@ -11885,7 +12553,7 @@
           <t>ایرلند – نقشه راه DETE تا ۲۰۳۰</t>
         </is>
       </c>
-      <c r="B42" s="15" t="inlineStr">
+      <c r="B42" s="16" t="inlineStr">
         <is>
           <t>https://www.visahq.com/news/2025-12-12/ie/ireland-sets-phased-salary-threshold-hikes-for-all-work-permit-categories-first-rise-due-1-march-2026/</t>
         </is>
@@ -11897,7 +12565,7 @@
           <t>ایرلند – ISD تمکن دانشجویی €10,000</t>
         </is>
       </c>
-      <c r="B43" s="15" t="inlineStr">
+      <c r="B43" s="16" t="inlineStr">
         <is>
           <t>https://www.irishimmigration.ie/coming-to-study-in-ireland/what-are-my-study-options/a-fee-paying-private-primary-or-secondary-school/information-on-student-finances/</t>
         </is>
@@ -11909,7 +12577,7 @@
           <t>ایرلند – UL MSc Software Engineering €20,800</t>
         </is>
       </c>
-      <c r="B44" s="15" t="inlineStr">
+      <c r="B44" s="16" t="inlineStr">
         <is>
           <t>https://www.ul.ie/study/postgraduate/software-engineering-msc</t>
         </is>
@@ -11921,7 +12589,7 @@
           <t>ایرلند – Maynooth فهرست شهریه 2025/26</t>
         </is>
       </c>
-      <c r="B45" s="15" t="inlineStr">
+      <c r="B45" s="16" t="inlineStr">
         <is>
           <t>https://www.maynoothuniversity.ie/sites/default/files/assets/document/2025.26%20Postgraduate%20EU%20&amp;%20International%20Fees%20List%20(24.02.25)%20V.4%20CHR.pdf</t>
         </is>
@@ -11933,7 +12601,7 @@
           <t>ایرلند – سفارت/کنسول افتخاری تهران</t>
         </is>
       </c>
-      <c r="B46" s="15" t="inlineStr">
+      <c r="B46" s="16" t="inlineStr">
         <is>
           <t>https://www.ireland.ie/en/tehran/</t>
         </is>
@@ -11945,7 +12613,7 @@
           <t>ایرلند – QS 2027 دانشگاه‌های ایرلند</t>
         </is>
       </c>
-      <c r="B47" s="15" t="inlineStr">
+      <c r="B47" s="16" t="inlineStr">
         <is>
           <t>https://www.thejournal.ie/irish-universities-qs-world-university-rankings-2027-7073948-Jun2026/</t>
         </is>
@@ -11957,7 +12625,7 @@
           <t>بریتانیا – Graduate visa ۱۸ ماه (از ژانویه ۲۰۲۷)</t>
         </is>
       </c>
-      <c r="B48" s="15" t="inlineStr">
+      <c r="B48" s="16" t="inlineStr">
         <is>
           <t>https://students.leeds.ac.uk/visa-information-after-studies/doc/graduate-visas</t>
         </is>
@@ -11969,7 +12637,7 @@
           <t>بریتانیا – HC 584 (۳ سپتامبر ۲۰۲۶): تمکن £1,570 / £1,203 از ۳۰ نوامبر ۲۰۲۶</t>
         </is>
       </c>
-      <c r="B49" s="15" t="inlineStr">
+      <c r="B49" s="16" t="inlineStr">
         <is>
           <t>https://www.gov.uk/government/publications/statement-of-changes-to-the-immigration-rules-hc-584-3-september-2026</t>
         </is>
@@ -11981,7 +12649,7 @@
           <t>بریتانیا – Skilled Worker نرخ شغل SOC 2134 £54,700</t>
         </is>
       </c>
-      <c r="B50" s="15" t="inlineStr">
+      <c r="B50" s="16" t="inlineStr">
         <is>
           <t>https://withrowan.co.uk/guides/skilled-worker-software-engineers</t>
         </is>
@@ -11993,7 +12661,7 @@
           <t>بریتانیا – Earned Settlement (وضعیت سپتامبر ۲۰۲۶)</t>
         </is>
       </c>
-      <c r="B51" s="15" t="inlineStr">
+      <c r="B51" s="16" t="inlineStr">
         <is>
           <t>https://www.ukimmigration.law/earned-settlement-ilr-uk-plans/</t>
         </is>
@@ -12005,7 +12673,7 @@
           <t>انگلستان – Teesside MSc Computer Science 2026-27: £17,000، 2:2، IELTS 6.0</t>
         </is>
       </c>
-      <c r="B52" s="15" t="inlineStr">
+      <c r="B52" s="16" t="inlineStr">
         <is>
           <t>https://www.tees.ac.uk/postgraduate_courses/computing_&amp;_cyber_security/msc_computer_science.cfm</t>
         </is>
@@ -12017,7 +12685,7 @@
           <t>انگلستان – Northumbria MSc Advanced Computer Science 2026/27: £21,500، 2:2</t>
         </is>
       </c>
-      <c r="B53" s="15" t="inlineStr">
+      <c r="B53" s="16" t="inlineStr">
         <is>
           <t>https://www.northumbria.ac.uk/study-at-northumbria/courses/msc-advanced-computer-science-dtfava6/</t>
         </is>
@@ -12029,7 +12697,7 @@
           <t>انگلستان – Leicester MSc Advanced Computer Science سپتامبر ۲۰۲۶: £24,250، 2:1</t>
         </is>
       </c>
-      <c r="B54" s="15" t="inlineStr">
+      <c r="B54" s="16" t="inlineStr">
         <is>
           <t>https://le.ac.uk/courses/advanced-computer-science-msc/2026</t>
         </is>
@@ -12041,7 +12709,7 @@
           <t>انگلستان – Essex MSc Advanced Computer Science 2026: £24,675، 2:2 (شامل Computer Engineering)</t>
         </is>
       </c>
-      <c r="B55" s="15" t="inlineStr">
+      <c r="B55" s="16" t="inlineStr">
         <is>
           <t>https://www.essex.ac.uk/courses/pg00435/1/msc-advanced-computer-science</t>
         </is>
@@ -12053,7 +12721,7 @@
           <t>انگلستان – York MSc Advanced Computer Science 2026/27: £32,900، 2:2، IELTS 6.5</t>
         </is>
       </c>
-      <c r="B56" s="15" t="inlineStr">
+      <c r="B56" s="16" t="inlineStr">
         <is>
           <t>https://www.york.ac.uk/study/postgraduate-taught/courses/msc-advanced-computer-science/</t>
         </is>
@@ -12065,7 +12733,7 @@
           <t>انگلستان – Chester MSc Advanced Computer Science 2026/27: £15,500 (کف قیمت انگلستان)</t>
         </is>
       </c>
-      <c r="B57" s="15" t="inlineStr">
+      <c r="B57" s="16" t="inlineStr">
         <is>
           <t>https://www.chester.ac.uk/study/course-search/advanced-computer-science-msc/</t>
         </is>
@@ -12077,7 +12745,7 @@
           <t>بریتانیا – Brunel MSc AI 2026/27 £24,795</t>
         </is>
       </c>
-      <c r="B58" s="15" t="inlineStr">
+      <c r="B58" s="16" t="inlineStr">
         <is>
           <t>https://www.brunel.ac.uk/study/courses/artificial-intelligence-msc</t>
         </is>
@@ -12089,7 +12757,7 @@
           <t>بریتانیا – عوارض £925 به ازای هر دانشجوی بین‌المللی (انگلستان، از 2028-29)</t>
         </is>
       </c>
-      <c r="B59" s="15" t="inlineStr">
+      <c r="B59" s="16" t="inlineStr">
         <is>
           <t>https://www.researchprofessionalnews.com/rr-news-uk-politics-2025-11-international-levy-to-be-flat-fee-of-925-per-student/</t>
         </is>
@@ -12101,7 +12769,7 @@
           <t>بریتانیا – وضعیت VAC تهران</t>
         </is>
       </c>
-      <c r="B60" s="15" t="inlineStr">
+      <c r="B60" s="16" t="inlineStr">
         <is>
           <t>https://livingintehran.com/2026/02/03/tehran-diplomatic-update-recent-embassy-reopenings-current-status-feb-2026/</t>
         </is>
@@ -12113,7 +12781,7 @@
           <t>QS WUR 2027 – TU Dresden</t>
         </is>
       </c>
-      <c r="B61" s="15" t="inlineStr">
+      <c r="B61" s="16" t="inlineStr">
         <is>
           <t>https://tu-dresden.de/tu-dresden/newsportal/news/qs-ranking-2027-tud-gehoert-erneut-zu-den-zehn-besten-universitaeten-deutschlands-und-baut-internationalen-erfolg-weiter-aus</t>
         </is>
@@ -12125,7 +12793,7 @@
           <t>QS WUR 2027 – Stuttgart</t>
         </is>
       </c>
-      <c r="B62" s="15" t="inlineStr">
+      <c r="B62" s="16" t="inlineStr">
         <is>
           <t>https://www.uni-stuttgart.de/en/university/news/all/QS-World-University-Rankings-2027-The-University-of-Stuttgart-is-recognized-for-its-strong-research-performance-and-commitment-to-sustainability/</t>
         </is>
@@ -12137,7 +12805,7 @@
           <t>QS WUR 2027 – Newcastle 149</t>
         </is>
       </c>
-      <c r="B63" s="15" t="inlineStr">
+      <c r="B63" s="16" t="inlineStr">
         <is>
           <t>https://www.ncl.ac.uk/press/articles/latest/2026/06/qs2027/</t>
         </is>
@@ -12149,7 +12817,7 @@
           <t>QS WUR 2027 – York =158</t>
         </is>
       </c>
-      <c r="B64" s="15" t="inlineStr">
+      <c r="B64" s="16" t="inlineStr">
         <is>
           <t>https://www.york.ac.uk/about/rankings/</t>
         </is>
@@ -12161,7 +12829,7 @@
           <t>QS WUR 2027 – Leicester =314</t>
         </is>
       </c>
-      <c r="B65" s="15" t="inlineStr">
+      <c r="B65" s="16" t="inlineStr">
         <is>
           <t>https://www.topuniversities.com/universities/university-leicester</t>
         </is>
@@ -12173,7 +12841,7 @@
           <t>QS WUR 2027 – Essex =438</t>
         </is>
       </c>
-      <c r="B66" s="15" t="inlineStr">
+      <c r="B66" s="16" t="inlineStr">
         <is>
           <t>https://www.topuniversities.com/universities/essex-university</t>
         </is>
@@ -12185,7 +12853,7 @@
           <t>QS WUR 2027 – Northumbria =528</t>
         </is>
       </c>
-      <c r="B67" s="15" t="inlineStr">
+      <c r="B67" s="16" t="inlineStr">
         <is>
           <t>https://www.topuniversities.com/universities/northumbria-university-newcastle</t>
         </is>
@@ -12197,7 +12865,7 @@
           <t>QS WUR 2027 – Brunel</t>
         </is>
       </c>
-      <c r="B68" s="15" t="inlineStr">
+      <c r="B68" s="16" t="inlineStr">
         <is>
           <t>https://students.brunel.ac.uk/campus-news/brunel-climbs-global-qs-rankings-after-strong-year-for-research-and-graduate-outcomes</t>
         </is>
@@ -12209,7 +12877,7 @@
           <t>QS WUR 2027 – سایر</t>
         </is>
       </c>
-      <c r="B69" s="15" t="inlineStr">
+      <c r="B69" s="16" t="inlineStr">
         <is>
           <t>https://www.topuniversities.com/world-university-rankings</t>
         </is>
@@ -12221,7 +12889,7 @@
           <t>حداقل دستمزد ۲۰۲۶ هلند (€14.71)</t>
         </is>
       </c>
-      <c r="B70" s="15" t="inlineStr">
+      <c r="B70" s="16" t="inlineStr">
         <is>
           <t>https://arlettipartners.com/new-increase-in-the-dutch-minimum-hourly-wage-from-january-1st-2026/</t>
         </is>
@@ -12233,7 +12901,7 @@
           <t>نرخ ارز (xe.com، ۲۷ سپتامبر ۲۰۲۶)</t>
         </is>
       </c>
-      <c r="B71" s="15" t="inlineStr">
+      <c r="B71" s="16" t="inlineStr">
         <is>
           <t>https://www.xe.com/</t>
         </is>
@@ -12245,7 +12913,7 @@
           <t>بازار کار – LinkedIn/WEF ژانویه ۲۰۲۶: ۱.۳ میلیون شغل جدید AI؛ AI Engineer سریع‌ترین‌رشد</t>
         </is>
       </c>
-      <c r="B72" s="15" t="inlineStr">
+      <c r="B72" s="16" t="inlineStr">
         <is>
           <t>https://www.weforum.org/stories/jobs-and-the-future-of-work/ai-has-already-added-1-3-million-new-jobs-according-to-linkedin-data/</t>
         </is>
@@ -12257,7 +12925,7 @@
           <t>بازار کار – Bitkom 2025: ۱۰۹ هزار جای خالی IT در آلمان، ۷.۷ ماه زمان پرکردن</t>
         </is>
       </c>
-      <c r="B73" s="15" t="inlineStr">
+      <c r="B73" s="16" t="inlineStr">
         <is>
           <t>https://www.bitkom.org/Bitkom/Publikationen/Der-Arbeitsmarkt-fuer-IT-Fachkraefte</t>
         </is>
@@ -12269,7 +12937,7 @@
           <t>بازار کار – ISC2 Cybersecurity Workforce Study 2024/2025 (حذف عدد کمبود؛ کمبود بودجه دلیل اول؛ ۳۱٪ تیم‌ها بدون جونیور)</t>
         </is>
       </c>
-      <c r="B74" s="15" t="inlineStr">
+      <c r="B74" s="16" t="inlineStr">
         <is>
           <t>https://www.isc2.org/research</t>
         </is>
@@ -12281,7 +12949,7 @@
           <t>بازار کار – اخراج‌های صنعت بازی ۲۰۲۲–۲۰۲۶ (≈۴۵ هزار؛ افت حقوق Unity)</t>
         </is>
       </c>
-      <c r="B75" s="15" t="inlineStr">
+      <c r="B75" s="16" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/2022%E2%80%932026_video_game_industry_layoffs</t>
         </is>
@@ -12293,7 +12961,7 @@
           <t>بازار کار – آگهی‌های UX/UXR (Indeed تا Q4 2025)</t>
         </is>
       </c>
-      <c r="B76" s="15" t="inlineStr">
+      <c r="B76" s="16" t="inlineStr">
         <is>
           <t>https://www.thevoiceofuser.com/everyone-knows-the-uxr-hiring-market-is-bad-how-bad-is-it-though/</t>
         </is>
@@ -12305,7 +12973,7 @@
           <t>بازار کار – اشباع جونیور علم داده ۲۰۲۶</t>
         </is>
       </c>
-      <c r="B77" s="15" t="inlineStr">
+      <c r="B77" s="16" t="inlineStr">
         <is>
           <t>https://research.com/advice/are-too-many-students-choosing-data-science-oversaturation-competition-hiring-reality</t>
         </is>
@@ -12317,7 +12985,7 @@
           <t>ایرلند – UL MSc AI &amp; ML: €20,800</t>
         </is>
       </c>
-      <c r="B78" s="15" t="inlineStr">
+      <c r="B78" s="16" t="inlineStr">
         <is>
           <t>https://www.ul.ie/study/postgraduate/artificial-intelligence-and-machine-learning-msc</t>
         </is>
@@ -12329,7 +12997,7 @@
           <t>ایرلند – TU Dublin MSc Applied Cyber Security: €14,500، 2:2</t>
         </is>
       </c>
-      <c r="B79" s="15" t="inlineStr">
+      <c r="B79" s="16" t="inlineStr">
         <is>
           <t>https://www.tudublin.ie/study/postgraduate/courses/applied-cyber-security/</t>
         </is>
@@ -12341,7 +13009,7 @@
           <t>ایرلند – TU Dublin MSc CS (Data Science): €21,750، 2:2 + ۲ سال سابقه</t>
         </is>
       </c>
-      <c r="B80" s="15" t="inlineStr">
+      <c r="B80" s="16" t="inlineStr">
         <is>
           <t>https://www.tudublin.ie/study/postgraduate/courses/computing-data-science/</t>
         </is>
@@ -12353,7 +13021,7 @@
           <t>ایرلند – DCU MSc Computing majors: €25,000، 2:1، بورس €5,000</t>
         </is>
       </c>
-      <c r="B81" s="15" t="inlineStr">
+      <c r="B81" s="16" t="inlineStr">
         <is>
           <t>https://www.dcu.ie/courses/postgraduate/school-computing/msc-computing-major-options</t>
         </is>
@@ -12365,7 +13033,7 @@
           <t>ایرلند – Galway MSc CS (AI) €28,000 / SDD €18,440، 2026/27</t>
         </is>
       </c>
-      <c r="B82" s="15" t="inlineStr">
+      <c r="B82" s="16" t="inlineStr">
         <is>
           <t>http://cs.universityofgalway.ie/science-engineering/postgraduateprogrammes/taught-postgraduate-courses/software-design-development.html</t>
         </is>
@@ -12377,7 +13045,7 @@
           <t>آلمان – Saarland MSc Cybersecurity (C1، بدون شهریه)</t>
         </is>
       </c>
-      <c r="B83" s="15" t="inlineStr">
+      <c r="B83" s="16" t="inlineStr">
         <is>
           <t>https://www.uni-saarland.de/en/study/programmes/master/cybersecurity.html</t>
         </is>
@@ -12389,7 +13057,7 @@
           <t>آلمان – Passau MSc AI Engineering (B2، معدل ≤ 2.7، A1 آلمانی سال اول)</t>
         </is>
       </c>
-      <c r="B84" s="15" t="inlineStr">
+      <c r="B84" s="16" t="inlineStr">
         <is>
           <t>https://www.uni-passau.de/en/msc-ai-eng</t>
         </is>
@@ -12401,7 +13069,7 @@
           <t>آلمان – Cologne Game Lab MA Game Development &amp; Research (€2,500/ترم غیر-EU)</t>
         </is>
       </c>
-      <c r="B85" s="15" t="inlineStr">
+      <c r="B85" s="16" t="inlineStr">
         <is>
           <t>https://colognegamelab.de/study-programs/post-graduate-programs/game-development-research-ma/faqs/</t>
         </is>
@@ -12413,7 +13081,7 @@
           <t>آلمان – Siegen MSc HCI (DAAD)</t>
         </is>
       </c>
-      <c r="B86" s="15" t="inlineStr">
+      <c r="B86" s="16" t="inlineStr">
         <is>
           <t>https://www2.daad.de/deutschland/studienangebote/international-programmes/en/detail/4686/</t>
         </is>
@@ -12425,7 +13093,7 @@
           <t>آلمان – H-BRS MSc Autonomous Systems (B2+)</t>
         </is>
       </c>
-      <c r="B87" s="15" t="inlineStr">
+      <c r="B87" s="16" t="inlineStr">
         <is>
           <t>https://www.h-brs.de/en/inf/admission-application-master-autonomous-systems</t>
         </is>
@@ -12437,7 +13105,7 @@
           <t>آلمان – RWTH MSc Software Systems Engineering</t>
         </is>
       </c>
-      <c r="B88" s="15" t="inlineStr">
+      <c r="B88" s="16" t="inlineStr">
         <is>
           <t>https://sc.informatik.rwth-aachen.de/en/studium/master/sse/</t>
         </is>
@@ -12449,7 +13117,7 @@
           <t>آلمان – Tübingen MSc Machine Learning (IELTS 7، €1,500/ترم)</t>
         </is>
       </c>
-      <c r="B89" s="15" t="inlineStr">
+      <c r="B89" s="16" t="inlineStr">
         <is>
           <t>https://uni-tuebingen.de/fakultaeten/mathematisch-naturwissenschaftliche-fakultaet/fachbereiche/informatik/studium/studierende/lehre-studienorganisation/studiengaenge/machine-learning/admission-and-application/</t>
         </is>
@@ -12461,7 +13129,7 @@
           <t>آلمان – TUM Informatics: €6,000 در ترم برای غیر-EU</t>
         </is>
       </c>
-      <c r="B90" s="15" t="inlineStr">
+      <c r="B90" s="16" t="inlineStr">
         <is>
           <t>https://www.tum.de/en/studies/degree-programs/detail/informatics-master-of-science-msc</t>
         </is>
@@ -12473,7 +13141,7 @@
           <t>آلمان – FAU Autonomy Technologies (B2، IELTS 6.0)</t>
         </is>
       </c>
-      <c r="B91" s="15" t="inlineStr">
+      <c r="B91" s="16" t="inlineStr">
         <is>
           <t>https://www.fau.eu/degree-program/autonomy-technologies-m-sc/</t>
         </is>
@@ -12485,7 +13153,7 @@
           <t>هلند – Twente Embedded Systems 2026/27: €21,700</t>
         </is>
       </c>
-      <c r="B92" s="15" t="inlineStr">
+      <c r="B92" s="16" t="inlineStr">
         <is>
           <t>https://www.utwente.nl/en/education/master/programmes/embedded-systems/finance/</t>
         </is>
@@ -12497,7 +13165,7 @@
           <t>هلند – Leiden CS 2026/27: €22,500</t>
         </is>
       </c>
-      <c r="B93" s="15" t="inlineStr">
+      <c r="B93" s="16" t="inlineStr">
         <is>
           <t>https://www.universiteitleiden.nl/en/education/study-programmes/master/computer-science/artificial-intelligence/admission-and-application/tuition-fees</t>
         </is>
@@ -12509,7 +13177,7 @@
           <t>هلند – Groningen AI 2026/27: €24,900</t>
         </is>
       </c>
-      <c r="B94" s="15" t="inlineStr">
+      <c r="B94" s="16" t="inlineStr">
         <is>
           <t>https://www.rug.nl/masters/artificial-intelligence/?lang=en</t>
         </is>
@@ -12521,7 +13189,7 @@
           <t>هلند – Utrecht Game &amp; Media Technology 2026/27: €25,306</t>
         </is>
       </c>
-      <c r="B95" s="15" t="inlineStr">
+      <c r="B95" s="16" t="inlineStr">
         <is>
           <t>https://www.uu.nl/en/masters/game-and-media-technology</t>
         </is>
@@ -12533,7 +13201,7 @@
           <t>هلند – QS 2027 فهرست دانشگاه‌های هلند</t>
         </is>
       </c>
-      <c r="B96" s="15" t="inlineStr">
+      <c r="B96" s="16" t="inlineStr">
         <is>
           <t>https://dub.uu.nl/en/news/dutch-universities-fall-global-qs-rankings</t>
         </is>
@@ -12545,7 +13213,7 @@
           <t>سوئد – Gothenburg Game Design &amp; Technology: SEK 290,000 کل</t>
         </is>
       </c>
-      <c r="B97" s="15" t="inlineStr">
+      <c r="B97" s="16" t="inlineStr">
         <is>
           <t>https://www.gu.se/en/study-gothenburg/game-design-technology-masters-programme-n2gdt</t>
         </is>
@@ -12557,7 +13225,7 @@
           <t>سوئد – KTH Machine Learning: ≈ SEK 180,000–190,000 (کل دوره 360k طبق راهنمای ۲۰۲۶؛ kth.se رقم را فقط در سامانه نشان می‌دهد)</t>
         </is>
       </c>
-      <c r="B98" s="15" t="inlineStr">
+      <c r="B98" s="16" t="inlineStr">
         <is>
           <t>https://www.kth.se/en/studies/master/machine-learning</t>
         </is>
@@ -12569,7 +13237,7 @@
           <t>سوئد – Umeå AI: SEK 152,300</t>
         </is>
       </c>
-      <c r="B99" s="15" t="inlineStr">
+      <c r="B99" s="16" t="inlineStr">
         <is>
           <t>https://www.umu.se/en/education/master/masters-programme-in-artificial-intelligence/</t>
         </is>
@@ -12581,7 +13249,7 @@
           <t>سوئد – QS 2027 فهرست دانشگاه‌های سوئد</t>
         </is>
       </c>
-      <c r="B100" s="15" t="inlineStr">
+      <c r="B100" s="16" t="inlineStr">
         <is>
           <t>https://www.study.eu/best-universities/sweden</t>
         </is>
@@ -12593,7 +13261,7 @@
           <t>دانمارک – ITU شهریهٔ رسمی ورودی ۲۰۲۶: €8,250 در ترم = €16,500 در سال (رقم قدیمی €6,700 منسوخ)</t>
         </is>
       </c>
-      <c r="B101" s="15" t="inlineStr">
+      <c r="B101" s="16" t="inlineStr">
         <is>
           <t>https://en.itu.dk/Programmes/MSc-Programmes/Applying-to-a-MSc-programme/Non-EU-EOES</t>
         </is>
@@ -12605,7 +13273,7 @@
           <t>دانمارک – AAU Cyber Security / Medialogy €7,455 در ترم</t>
         </is>
       </c>
-      <c r="B102" s="15" t="inlineStr">
+      <c r="B102" s="16" t="inlineStr">
         <is>
           <t>https://studyindenmark.dk/portal/aalborg-university-aau/copenhagen/cyber-security-msc-in-engineering</t>
         </is>
@@ -12617,7 +13285,7 @@
           <t>دانمارک – DTU €15,000 (Human-Centered AI / Autonomous Systems)</t>
         </is>
       </c>
-      <c r="B103" s="15" t="inlineStr">
+      <c r="B103" s="16" t="inlineStr">
         <is>
           <t>https://www.dtu.dk/english/education/graduate/msc-programmes/autonomous-systems/prerequisites</t>
         </is>
@@ -12629,7 +13297,7 @@
           <t>دانمارک – Aarhus CS €17,300</t>
         </is>
       </c>
-      <c r="B104" s="15" t="inlineStr">
+      <c r="B104" s="16" t="inlineStr">
         <is>
           <t>https://masters.au.dk/computerscience</t>
         </is>
@@ -12641,7 +13309,7 @@
           <t>دانمارک – QS 2027 فهرست دانشگاه‌های دانمارک</t>
         </is>
       </c>
-      <c r="B105" s="15" t="inlineStr">
+      <c r="B105" s="16" t="inlineStr">
         <is>
           <t>https://leapscholar.com/blog/top-universities-in-denmark/</t>
         </is>
@@ -12653,7 +13321,7 @@
           <t>انگلستان – Goldsmiths MSc Computer Games Programming £22,000</t>
         </is>
       </c>
-      <c r="B106" s="15" t="inlineStr">
+      <c r="B106" s="16" t="inlineStr">
         <is>
           <t>https://www.gold.ac.uk/pg/msc-computer-games-programming/</t>
         </is>
@@ -12665,7 +13333,7 @@
           <t>انگلستان – Royal Holloway MSc Information &amp; Cyber Security £25,500</t>
         </is>
       </c>
-      <c r="B107" s="15" t="inlineStr">
+      <c r="B107" s="16" t="inlineStr">
         <is>
           <t>https://www.royalholloway.ac.uk/studying-here/postgraduate/information-security/information-and-cyber-security/</t>
         </is>
@@ -12677,7 +13345,7 @@
           <t>انگلستان – Kent MSc Cyber Security (NCSC)</t>
         </is>
       </c>
-      <c r="B108" s="15" t="inlineStr">
+      <c r="B108" s="16" t="inlineStr">
         <is>
           <t>https://www.kent.ac.uk/courses/postgraduate/1225/cyber-security</t>
         </is>
@@ -12689,7 +13357,7 @@
           <t>انگلستان – MMU MSc Cyber Security £21,000</t>
         </is>
       </c>
-      <c r="B109" s="15" t="inlineStr">
+      <c r="B109" s="16" t="inlineStr">
         <is>
           <t>https://www.mmu.ac.uk/study/postgraduate/course/msc-cyber-security</t>
         </is>
@@ -12701,7 +13369,7 @@
           <t>انگلستان – York MSc Human-Centred Interactive Technologies £32,900</t>
         </is>
       </c>
-      <c r="B110" s="15" t="inlineStr">
+      <c r="B110" s="16" t="inlineStr">
         <is>
           <t>https://www.york.ac.uk/study/postgraduate-taught/courses/msc-human-centred-interactive-technologies/</t>
         </is>
@@ -12713,7 +13381,7 @@
           <t>انگلستان – Lancaster MSc Cyber Security £30,000</t>
         </is>
       </c>
-      <c r="B111" s="15" t="inlineStr">
+      <c r="B111" s="16" t="inlineStr">
         <is>
           <t>https://www.lancaster.ac.uk/study/postgraduate/postgraduate-courses/cyber-security-msc/2026/</t>
         </is>
@@ -12725,7 +13393,7 @@
           <t>انگلستان – NTU QS 2027 =639</t>
         </is>
       </c>
-      <c r="B112" s="15" t="inlineStr">
+      <c r="B112" s="16" t="inlineStr">
         <is>
           <t>https://collegedunia.com/uk/university/862-nottingham-trent-university-nottingham/ranking</t>
         </is>
@@ -12737,7 +13405,7 @@
           <t>آلمان – FAU: شهریهٔ غیر-EU از ترم تابستان ۲۰۲۷ (AI/CS €4,000، Autonomy Tech €2,000 در ترم؛ BayHIG §13)</t>
         </is>
       </c>
-      <c r="B113" s="15" t="inlineStr">
+      <c r="B113" s="16" t="inlineStr">
         <is>
           <t>https://www.fau.eu/studying/international-students/application-and-enrollment-for-international-applicants/tuition-fees-for-students-from-non-eu-states/</t>
         </is>
@@ -12749,7 +13417,7 @@
           <t>آلمان – Passau: «فعلاً» بدون شهریه برای غیر-EU (اعلام رسمی)</t>
         </is>
       </c>
-      <c r="B114" s="15" t="inlineStr">
+      <c r="B114" s="16" t="inlineStr">
         <is>
           <t>https://www.uni-passau.de/en/study/news/news/no-tuition-fees-for-international-students-at-the-university-of-passau</t>
         </is>
@@ -12761,7 +13429,7 @@
           <t>دانمارک – Aarhus نرخ رسمی 2026/27: Computer Science / Data Science / Computer Engineering €17,300</t>
         </is>
       </c>
-      <c r="B115" s="15" t="inlineStr">
+      <c r="B115" s="16" t="inlineStr">
         <is>
           <t>https://masters.au.dk/tuitionfees/current-tuition-fee-rates</t>
         </is>
@@ -12773,7 +13441,7 @@
           <t>دانمارک – AAU Computer Science (IT): شرط رسمی ≥ ۱۵۰ ECTS دروس CS؛ معیار رتبه‌بندی ۲۰۲۷ شامل سابقهٔ کار</t>
         </is>
       </c>
-      <c r="B116" s="15" t="inlineStr">
+      <c r="B116" s="16" t="inlineStr">
         <is>
           <t>https://www.en.aau.dk/education/master/computer-science-it</t>
         </is>
@@ -12785,7 +13453,7 @@
           <t>سوئد – Chalmers شهریهٔ استاندارد 2026/27 ≈ SEK 175,000 (collegedunia به نقل از صفحهٔ شهریهٔ Chalmers)</t>
         </is>
       </c>
-      <c r="B117" s="15" t="inlineStr">
+      <c r="B117" s="16" t="inlineStr">
         <is>
           <t>https://collegedunia.com/sweden/university/769-chalmers-university-of-technology-gothenburg/programs?stream_id=48&amp;degree_type=Master</t>
         </is>
@@ -12797,7 +13465,7 @@
           <t>انگلستان – Surrey MSc Cyber Security ورودی ۲۰۲۷: £25,900 (فوریه) / £26,900 (سپتامبر)</t>
         </is>
       </c>
-      <c r="B118" s="15" t="inlineStr">
+      <c r="B118" s="16" t="inlineStr">
         <is>
           <t>https://www.surrey.ac.uk/postgraduate/cyber-security-msc</t>
         </is>
@@ -12809,7 +13477,7 @@
           <t>انگلستان – Newcastle MSc Computer Game Engineering £32,300، شرط 2:2 (QS TopUniversities)</t>
         </is>
       </c>
-      <c r="B119" s="15" t="inlineStr">
+      <c r="B119" s="16" t="inlineStr">
         <is>
           <t>https://www.topuniversities.com/universities/newcastle-university/postgrad/msc-computer-game-engineering</t>
         </is>
@@ -12821,9 +13489,177 @@
           <t>هلند – TU/e شهریهٔ رسمی 2026/27 €21,700 (2027/28: €22,400)</t>
         </is>
       </c>
-      <c r="B120" s="15" t="inlineStr">
+      <c r="B120" s="16" t="inlineStr">
         <is>
           <t>https://www.tue.nl/en/education/become-a-tue-student/tuition-fees</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="4" t="inlineStr">
+        <is>
+          <t>ایران – توقف برگزاری IELTS در ایران از ۳۱ ژانویه ۲۰۲۶ (اعلام IDP)</t>
+        </is>
+      </c>
+      <c r="B121" s="16" t="inlineStr">
+        <is>
+          <t>https://wanaen.com/ielts-testing-to-be-suspended-in-iran/</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="4" t="inlineStr">
+        <is>
+          <t>ایران – وضعیت IELTS شهریور ۱۴۰۵: در ایران برگزار نمی‌شود؛ آزمون در کشور دیگر</t>
+        </is>
+      </c>
+      <c r="B122" s="16" t="inlineStr">
+        <is>
+          <t>https://www.jahantahsil.com/%D8%A2%D8%B2%D9%85%D9%88%D9%86-%D8%A2%DB%8C%D9%84%D8%AA%D8%B3-ielts-%DA%86%DB%8C%D8%B3%D8%AA-%D9%88-%DA%A9%D8%AC%D8%A7-%D8%A8%D8%B1%DA%AF%D8%B2%D8%A7%D8%B1-%D9%85%DB%8C%D8%B4%D9%88%D8%AF/</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="4" t="inlineStr">
+        <is>
+          <t>ایران – توقف TOEFL در ایران (وضعیت شهریور ۱۴۰۵)</t>
+        </is>
+      </c>
+      <c r="B123" s="16" t="inlineStr">
+        <is>
+          <t>https://zandienglish.ir/toefl-in-iran/</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="4" t="inlineStr">
+        <is>
+          <t>ایران – وثیقهٔ خروج تحصیلی مشمولان ۲۰۰ میلیون تومان (سامانهٔ سخا، تیر ۱۴۰۵)</t>
+        </is>
+      </c>
+      <c r="B124" s="16" t="inlineStr">
+        <is>
+          <t>https://www.zoomit.ir/iran-news/464136-exit-permit-bond-sakha-1405/</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="4" t="inlineStr">
+        <is>
+          <t>سوئد – تاریخ‌های کلیدی ورودی پاییز ۲۰۲۷ (۱۶ اکتبر – ۱۵ ژانویه؛ مدارک ۱ فوریه؛ دور دوم ۱۵ آوریل)</t>
+        </is>
+      </c>
+      <c r="B125" s="16" t="inlineStr">
+        <is>
+          <t>https://www.umu.se/en/education/application-and-admission/key-dates-and-deadlines/</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="4" t="inlineStr">
+        <is>
+          <t>آلمان – Stuttgart MSc CS: بازهٔ اپلای ترم زمستان ۱۵ نوامبر – ۱۵ ژانویه؛ انگلیسی C1</t>
+        </is>
+      </c>
+      <c r="B126" s="16" t="inlineStr">
+        <is>
+          <t>https://www.uni-stuttgart.de/en/study/study-programs/Computer-Science-M.Sc.-00001/</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="4" t="inlineStr">
+        <is>
+          <t>آلمان – Passau: بازهٔ اپلای AI Engineering ۱ آوریل – ۳۱ می</t>
+        </is>
+      </c>
+      <c r="B127" s="16" t="inlineStr">
+        <is>
+          <t>https://www.uni-passau.de/en/apply/apply-with-intl-qualifications</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="4" t="inlineStr">
+        <is>
+          <t>دانمارک – AAU: مهلت شهریه‌پردازها ۱۵ ژانویه (EU: ۱ مارس)؛ پورتال از اواسط دسامبر</t>
+        </is>
+      </c>
+      <c r="B128" s="16" t="inlineStr">
+        <is>
+          <t>https://www.en.aau.dk/education/apply/master/how-and-when-to-apply</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="4" t="inlineStr">
+        <is>
+          <t>دانمارک – SDU Computer Science: مهلت غیر-EU ۱ فوریه؛ شهریه یک سال پیش‌پرداخت</t>
+        </is>
+      </c>
+      <c r="B129" s="16" t="inlineStr">
+        <is>
+          <t>https://www.sdu.dk/en/uddannelse/kandidat/datalogi</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="4" t="inlineStr">
+        <is>
+          <t>هلند – Radboud: مهلت غیر-EU ۱ آوریل، بورس ۳۱ ژانویه، ثبت‌نام ۱ ژوئن</t>
+        </is>
+      </c>
+      <c r="B130" s="16" t="inlineStr">
+        <is>
+          <t>https://www.ru.nl/en/education/application-and-admission/application-procedure-masters/deadlines</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="4" t="inlineStr">
+        <is>
+          <t>هلند – Twente: مهلت غیر-EEA ۱ می ۲۰۲۷؛ بورس UTS ۱۵ اکتبر ۲۰۲۶ – ۱ آوریل ۲۰۲۷</t>
+        </is>
+      </c>
+      <c r="B131" s="16" t="inlineStr">
+        <is>
+          <t>https://collegedunia.com/netherlands/university/749-university-of-twente-enschede/admission</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="4" t="inlineStr">
+        <is>
+          <t>ایرلند – UL: مهلت غیر-EU ویزایی ۱ ژوئیه؛ اپلای از ۱۵ اکتبر</t>
+        </is>
+      </c>
+      <c r="B132" s="16" t="inlineStr">
+        <is>
+          <t>https://www.ul.ie/gps/applications-faq</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="4" t="inlineStr">
+        <is>
+          <t>ایرلند – Maynooth: باز شدن اپلای ۲۰۲۷ در ۱۴ اکتبر ۲۰۲۶؛ ودیعهٔ غیر-EU €1,000</t>
+        </is>
+      </c>
+      <c r="B133" s="16" t="inlineStr">
+        <is>
+          <t>https://www.maynoothuniversity.ie/study-maynooth/how-apply/postgraduate-applicants</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="4" t="inlineStr">
+        <is>
+          <t>ایرلند – مهلت‌های تقریبی TU Dublin (۳۱ می) و Maynooth (۱۵ می) برای غیر-EU</t>
+        </is>
+      </c>
+      <c r="B134" s="16" t="inlineStr">
+        <is>
+          <t>https://studyinireland.app/apply/deadlines</t>
         </is>
       </c>
     </row>
@@ -12948,6 +13784,20 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B118" r:id="rId117"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B119" r:id="rId118"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B120" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B121" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B122" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B123" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B124" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B125" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B126" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B127" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B128" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B129" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B130" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B131" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B132" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B133" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B134" r:id="rId133"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add row 5b: scholarships/tuition discounts realistically available to a non-EU applicant with 15.77/20 (per country, verified: LiU 2026 GPA rule, Chalmers IPOET 80% floor, SI not for Iran, NL Scholarship, AAU ~15 awards, ETH ESOP, USI CHF 4,000, Essex Iran 14/20 -> GBP 4,500, Teesside, Brunel 2:1, Northumbria excludes Iran, Chevening ineligible); +15 sources; MD sections 13 (GPA conversion) and 14
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Table_final.xlsx
+++ b/Table_final.xlsx
@@ -536,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -875,46 +875,124 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
+          <t>۵ب</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>بورس / تخفیف شهریهٔ واقعاً در دسترسِ شما (غیر-EU، معدل ۱۵.۷۷ ≈ ۷۹٪، ورودی ۲۰۲۷)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>شهریه‌ای نیست که تخفیف بخورد؛ بورس ارشد هم عملاً نیست:
+• Deutschlandstipendium: €300/ماه، بعد از ثبت‌نام، ≈ ۱–۳٪ دانشجویان
+• DAAD برای ارشد معمولی CS بورس ندارد (فقط فهرست توسعه‌محور EPOS)
+• Stuttgart (BW): قانون اجازهٔ معافیت حداکثر ۵٪ «استعدادهای ویژه» از €1,500/ترم را می‌دهد — سالانه اعلام می‌شود؛ FAU هنوز طرح معافیت برای شهریهٔ جدید نداده
+اثر روی هزینهٔ شما: ≈ صفر (از قبل ارزان‌ترین است)</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>• NL Scholarship (سابقاً Holland): €5,000 یک‌بار در سال اول، از طریق دانشگاه‌های عضو؛ مهلت ۱ فوریه یا ۱ می (بسته به دانشگاه) — با معدل شما شدنی‌ترین
+• UTS Twente: €3,000–22,000/سال فقط برای «بهترین‌ها» (۱۵ اکتبر – ۱ آوریل) → Reach
+• Radboud Scholarship Programme: شهریه تا سطح EU (≈ €2,600) + ویزا/بیمه؛ ۳۱ ژانویه؛ بسیار رقابتی → Reach
+• TU/e ALSP، Utrecht/Leiden/UvA Excellence: ۱۰٪ بالای کلاس → نه
+اثر: حداکثر −€5k از $75–90k</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>قوی‌ترین کشور جدول، ولی درهای اصلی برای معدل ۷۹٪ نیمه‌باز است:
+• LiU: معمولاً ۵۰٪ شهریه، فقط اگر LiU اولویت ۱ باشد؛ ⚠️ از ۲۰۲۶ فقط GPA ≥ 3.5/4 یا «first/high second class» — معدل شما (≈ 3.1/4) احتمالاً زیر خط
+• Chalmers IPOET ۷۵٪ (≈ ۳۵ بورس؛ فرم جدا تا ۱۵ ژانویه): حداقل معدل ۸۰٪ — شما ۷۸.۹٪ = دقیقاً زیر خط
+• KTH Scholarship: شهریهٔ کامل، چند ده نفر، ۱ دسامبر – ۱۵ ژانویه → Reach
+• Halmstad ۲۵٪/۵۰٪ (پنجرهٔ ≈ ۹–۲۵ فوریه) و MDU تا ۱۰۰٪ (اولویت ۱؛ معدود) — واقع‌بینانه‌ترین‌ها برای شما
+• ⚠️ بورس دولتی SI: ایران جزو ۳۴ کشور واجد شرایط نیست
+اثر: با ۵۰٪ در Halmstad/MDU کل دوره از $54–65k به ≈ $40–48k می‌رسد — نزدیک به انگلستان</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Danish Government Scholarship = معافیت شهریه (+ گاهی کمک‌هزینه) که خودِ دانشگاه از سهمیهٔ دولتی می‌دهد؛ فرم جدا ندارد — همهٔ غیر-EUها خودکار بررسی می‌شوند:
+• AAU: ≈ ۱۵ بورس/سال = معافیت کامل + DKK 11,225/ماه (۲۰۲۶)
+• SDU: فقط بعضی ارشدهای مهندسی، معافیت کامل، معدود
+• ITU/DTU/Aarhus: تعداد کم، رقابتی
+شانس واقعی با معدل ۷۹٪: پایین؛ روی آن برنامه نریزید (خود AAU هم همین را می‌گوید)
+اثر روی برنامه‌ریزی: صفر مگر برنده شوید</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>• ETH Excellence (ESOP): معافیت + CHF 12,000/ترم؛ ≈ ۶۰ بورس؛ فقط ۱۰٪ بالای کلاس؛ همراه اپلای ۱–۳۰ نوامبر → با معدل شما نه
+• EPFL Excellence Fellowship: ≈ CHF 16,000/سال؛ درصد بالای کلاس → نه
+• USI: ۶۰ بورس یک‌بارهٔ CHF 4,000 (= نصف شهریهٔ سال اول) برای معدل ≥ ۸۰/۱۰۰ — شما ۷۸.۹ → مرزی؛ + ۲۰ بورس سال دوم برای بهترینِ هر برنامه
+• Neuchâtel/Fribourg/Bern/Basel/UZH/ZHAW/HSLU: بورس ارشد برای خارجی‌ها ندارند (کمک کانتونی فقط برای مقیم‌ها)
+• بورس دولت سوئیس (ESKAS): فقط دکترا/پژوهش
+اثر: ≈ صفر (مسئلهٔ سوئیس هزینهٔ زندگی است، نه شهریه)</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>تخفیف‌های خودکار دانشگاهی (بدون فرم) — همین‌ها واقعی‌اند:
+• Essex: جدول کشوری؛ ایران با ≥ ۱۴/۲۰ → £4,500 تخفیف شهریه (شما واجد شرایط؛ جدول ۲۰۲۵–۲۶ — نسخهٔ ۲۰۲۶–۲۷ را چک کنید)
+• Teesside Global Excellence: £2,000 (صلاحدیدی؛ پیشنهاد تا ۳۰ آوریل)
+• Brunel VC Award: £6,000 فقط با معادل 2:1 (+ ودیعهٔ £5,000) — برای ایران معمولاً ≥ ۱۶/۲۰؛ برای شما مرزی، از پذیرش بپرسید
+• Northumbria £3,000: فقط فهرست کشوری/ادامه‌تحصیلی‌های داخل UK — ایران نه
+• Leicester/York: بورس‌های بین‌المللی محدود و رقابتی
+• ❌ Chevening: ۲ سال کار *بعد از* مدرک + تعهد بازگشت ۲ ساله — با فارغ‌التحصیلی ۲۰۲۶ و هدف مهاجرت نمی‌خواند · ❌ GREAT: ایران در فهرست نیست · ❌ Commonwealth
+اثر: Essex −$6k، Teesside −$2.6k از $38–65k</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>liu.se (Scholarships؛ شرط جدید ۲۰۲۶)؛ chalmers.se (IPOET ≥ ۸۰٪)؛ hh.se؛ mdu.se؛ si.se (۳۴ کشور)؛ NL Scholarship (Nuffic/studyinnl)؛ utwente.nl؛ ru.nl؛ en.aau.dk (Finance and fees: ≈ ۱۵ بورس، DKK 11,225/ماه)؛ sdu.dk؛ ethz.ch (ESOP)؛ epfl.ch؛ usi.ch / Fondazione per le Facoltà di Lugano؛ essex.ac.uk؛ tees.ac.uk؛ brunel.ac.uk؛ northumbria.ac.uk؛ chevening.org (Eligibility)؛ deutschlandstipendium.de — ⚠️ مبالغ چرخهٔ ۲۰۲۶/۲۷؛ برای ۲۰۲۷/۲۸ موقع اپلای دوباره ببینید. این ردیف امتیاز ردیف ۲۸ را عوض نمی‌کند (امتیازها با قیمت کامل حساب شده‌اند)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
           <t>۶</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>هزینه زندگی ماهانه واقعی دانشجو (و حداقل قانونی ویزا ۲۰۲۶)</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>€950–1,250 (Dresden/Erlangen ارزان‌تر؛ Stuttgart/Darmstadt گران‌تر)
 حداقل حساب مسدود: €992/ماه</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>€1,100–1,500 در Enschede/Nijmegen
 حداقل IND: €1,130.77/ماه</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>SEK 10,700–13,000 (≈ €950–1,150)
 حداقل Migrationsverket: SEK 10,656/ماه</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>DKK 8,000–10,000 (≈ €1,070–1,340) در Aalborg/Odense
 حداقل SIRI: DKK 7,426/ماه</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>Zürich: CHF 1,900–2,500 (≈ $2,300–3,000؛ اتاق WOKO CHF 500–900، اتاق خصوصی 800–1,200) · Lausanne: CHF 1,700–2,200
 Bern/Basel/Lucerne: CHF 1,550–2,100 · Lugano/Fribourg/Neuchâtel: CHF 1,350–1,800
 حداقل رسمی: CHF 21,000 در سال (Basel: 24,000)؛ کانتون زوریخ فقط حساب بانک مستقر در سوئیس به نام خودتان یا ضامن مقیم سوئیس را می‌پذیرد</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>شمال انگلستان (Middlesbrough/Newcastle): £950–1,250
 Leicester/Colchester/York: £1,000–1,350
@@ -922,1077 +1000,1077 @@
 حداقل ویزا: £1,171 / £1,529 در ماه (× ۹)؛ از ۳۰ نوامبر ۲۰۲۶: £1,203 / £1,570</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>make-it-in-germany.com؛ ind.nl؛ migrationsverket.se؛ nyidanmark.dk؛ sem.admin.ch؛ gov.uk (HC 584)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>۷</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>هزینه سال اول = شهریه + ۱۲ ماه زندگی (دلار)</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>$13,000–18,000 (Stuttgart تا $20,500؛ FAU از ۲۰۲۷ تا ≈ $26,000)</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>$37,500–45,000</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>$27,000–32,500</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>$31,500–38,000</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>$23,000–42,000 (Neuchâtel/Fribourg $23–31k · Lucerne $26–32k · Bern $27–35k · Lugano/Lausanne $30–37k · Zürich $30–42k)</t>
-        </is>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>$38,000–65,000 (Teesside $38–42k · Northumbria $44–48k · Leicester/Essex $48–54k · Brunel/London $55–61k · York $60–65k)</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>محاسبه از ردیف‌های ۴ و ۶؛ بدون بلیت، ویزا، بیمه، ودیعه (۱۰–۱۵٪ اضافه کنید)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>۸</t>
+          <t>۷</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>هزینه کل تا فارغ‌التحصیلی (شهریه × سال‌ها + زندگی) — مهم‌ترین عدد مالی</t>
+          <t>هزینه سال اول = شهریه + ۱۲ ماه زندگی (دلار)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>$27,000–36,000 (۲ سال؛ Stuttgart تا $41,000؛ FAU از ۲۰۲۷ تا ≈ $53,000) — ارزان‌ترین</t>
+          <t>$13,000–18,000 (Stuttgart تا $20,500؛ FAU از ۲۰۲۷ تا ≈ $26,000)</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>$75,000–90,000 (۲ سال) — گران‌ترین</t>
+          <t>$37,500–45,000</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>$54,000–65,000 (۲ سال)</t>
+          <t>$27,000–32,500</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>$63,000–76,000 (۲ سال)</t>
+          <t>$31,500–38,000</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>$35,000–84,000 (Neuchâtel/Fribourg ۱.۵ سال $35–47k · Bern $39–51k · UZH $45–58k · HSLU $53–64k · USI/EPFL $60–75k · ETH $66–84k) — بعد از هلند گران‌ترین؛ شهریه ناچیز است، هزینهٔ زندگی همه‌چیز را تعیین می‌کند</t>
+          <t>$23,000–42,000 (Neuchâtel/Fribourg $23–31k · Lucerne $26–32k · Bern $27–35k · Lugano/Lausanne $30–37k · Zürich $30–42k)</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>$38,000–65,000 (۱ سال)</t>
+          <t>$38,000–65,000 (Teesside $38–42k · Northumbria $44–48k · Leicester/Essex $48–54k · Brunel/London $55–61k · York $60–65k)</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>محاسبه؛ جدول اول فقط سال اول را مقایسه کرده بود</t>
+          <t>محاسبه از ردیف‌های ۴ و ۶؛ بدون بلیت، ویزا، بیمه، ودیعه (۱۰–۱۵٪ اضافه کنید)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>۹</t>
+          <t>۸</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>سازگاری با بودجه $32,000 در سال</t>
+          <t>هزینه کل تا فارغ‌التحصیلی (شهریه × سال‌ها + زندگی) — مهم‌ترین عدد مالی</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>✅ کاملاً (حتی Stuttgart)</t>
+          <t>$27,000–36,000 (۲ سال؛ Stuttgart تا $41,000؛ FAU از ۲۰۲۷ تا ≈ $53,000) — ارزان‌ترین</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>❌ کسری $5,500–13,000 در هر سال</t>
+          <t>$75,000–90,000 (۲ سال) — گران‌ترین</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>✅ (Linköping دقیقاً مرزی)</t>
+          <t>$54,000–65,000 (۲ سال)</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>⚠️ مرزی؛ AAU تقریباً در بودجه، SDU کسری تا ≈ $6,000 در سال</t>
+          <t>$63,000–76,000 (۲ سال)</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>⚠️ فقط Neuchâtel/Fribourg (و با صرفه‌جویی Lucerne/Lugano) در بودجه؛ Zürich/Lausanne کسری $1,000–10,000 در سال؛ کار دانشجویی در ۶ ماه اول ممنوع → سال اول تماماً از جیب</t>
+          <t>$35,000–84,000 (Neuchâtel/Fribourg ۱.۵ سال $35–47k · Bern $39–51k · UZH $45–58k · HSLU $53–64k · USI/EPFL $60–75k · ETH $66–84k) — بعد از هلند گران‌ترین؛ شهریه ناچیز است، هزینهٔ زندگی همه‌چیز را تعیین می‌کند</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>❌ کسری $6,000–33,000 (کمترین: Teesside ≈ $6–10k؛ Northumbria ≈ $12–16k)</t>
+          <t>$38,000–65,000 (۱ سال)</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>محاسبه از ردیف ۷</t>
+          <t>محاسبه؛ جدول اول فقط سال اول را مقایسه کرده بود</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>۱۰</t>
+          <t>۹</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>مسکن در بدو ورود</t>
+          <t>سازگاری با بودجه $32,000 در سال</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>خوابگاه Studierendenwerk با لیست انتظار؛ Stuttgart و Darmstadt سخت، Dresden و Erlangen آسان‌تر. بلافاصله بعد از پذیرش ثبت‌نام کنید.</t>
+          <t>✅ کاملاً (حتی Stuttgart)</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>کمبود شدید ملی؛ ولی Twente (کمپوس) و Radboud/SSH&amp; اتاق رزروشده برای بین‌المللی‌ها دارند — مهلت را از دست ندهید.</t>
+          <t>❌ کسری $5,500–13,000 در هر سال</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>تضمین سراسری نیست: Linköping به شهریه‌پردازها یک پیشنهاد اتاق برای سال اول می‌دهد؛ Halmstad تضمین ندارد؛ BTH تأیید نشد.</t>
+          <t>✅ (Linköping دقیقاً مرزی)</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>دفتر اسکان بین‌المللی AAU/SDU؛ Aalborg و Odense نسبتاً در دسترس.</t>
+          <t>⚠️ مرزی؛ AAU تقریباً در بودجه، SDU کسری تا ≈ $6,000 در سال</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Zürich بحرانی: WOKO/Juwo (CHF 500–900) لیست انتظار ۳–۱۲ ماه، بازار خصوصی بسیار رقابتی؛ Lausanne خوابگاه‌های FMEL (زود پر می‌شود)؛ Lugano/Fribourg/Neuchâtel/Bern/Lucerne آسان‌تر و ارزان‌تر (CHF 500–800). روز دریافت پذیرش ثبت‌نام کنید.</t>
+          <t>⚠️ فقط Neuchâtel/Fribourg (و با صرفه‌جویی Lucerne/Lugano) در بودجه؛ Zürich/Lausanne کسری $1,000–10,000 در سال؛ کار دانشجویی در ۶ ماه اول ممنوع → سال اول تماماً از جیب</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>معمولاً تضمین خوابگاه سال اول برای بین‌المللی‌ها اگر تا مهلت درخواست دهید.</t>
+          <t>❌ کسری $6,000–33,000 (کمترین: Teesside ≈ $6–10k؛ Northumbria ≈ $12–16k)</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>سایت دانشگاه‌ها؛ hh.se (Find Accommodation)؛ liu.se</t>
+          <t>محاسبه از ردیف ۷</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>۱۱</t>
+          <t>۱۰</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>سقف قانونی کار دانشجویی</t>
+          <t>مسکن در بدو ورود</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>۱۴۰ روز کامل یا ۲۸۰ نیم‌روز در سال (Werkstudent تا ۲۰ ساعت/هفته در ترم)</t>
+          <t>خوابگاه Studierendenwerk با لیست انتظار؛ Stuttgart و Darmstadt سخت، Dresden و Erlangen آسان‌تر. بلافاصله بعد از پذیرش ثبت‌نام کنید.</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>۱۶ ساعت/هفته (کارفرما TWV می‌گیرد) یا تمام‌وقت در ژوئن–اوت</t>
+          <t>کمبود شدید ملی؛ ولی Twente (کمپوس) و Radboud/SSH&amp; اتاق رزروشده برای بین‌المللی‌ها دارند — مهلت را از دست ندهید.</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>از ۱۱ ژوئن ۲۰۲۶: حداکثر ۱۵ ساعت/هفته در ترم؛ ژوئن–اوت بدون سقف. تخلف = لغو اقامت. + حداقل پیشرفت تحصیلی ۳۷.۵ واحد سال اول / ۴۵ واحد بعد</t>
+          <t>تضمین سراسری نیست: Linköping به شهریه‌پردازها یک پیشنهاد اتاق برای سال اول می‌دهد؛ Halmstad تضمین ندارد؛ BTH تأیید نشد.</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>۹۰ ساعت/ماه (سپتامبر–مه) + تمام‌وقت ژوئن–اوت</t>
+          <t>دفتر اسکان بین‌المللی AAU/SDU؛ Aalborg و Odense نسبتاً در دسترس.</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>غیر-EU: ۶ ماه اول هیچ؛ بعد از آن ۱۵ ساعت/هفته در ترم و تمام‌وقت در تعطیلات؛ کارفرما باید مجوز کانتونی بگیرد؛ کل دورهٔ تحصیل در سوئیس حداکثر ۸ سال</t>
+          <t>Zürich بحرانی: WOKO/Juwo (CHF 500–900) لیست انتظار ۳–۱۲ ماه، بازار خصوصی بسیار رقابتی؛ Lausanne خوابگاه‌های FMEL (زود پر می‌شود)؛ Lugano/Fribourg/Neuchâtel/Bern/Lucerne آسان‌تر و ارزان‌تر (CHF 500–800). روز دریافت پذیرش ثبت‌نام کنید.</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>۲۰ ساعت/هفته در ترم؛ تمام‌وقت در تعطیلات</t>
+          <t>معمولاً تضمین خوابگاه سال اول برای بین‌المللی‌ها اگر تا مهلت درخواست دهید.</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>make-it-in-germany.com؛ ind.nl؛ migrationsverket.se (خبر ۲۵ مه ۲۰۲۶)؛ nyidanmark.dk؛ sem.admin.ch؛ gov.uk</t>
+          <t>سایت دانشگاه‌ها؛ hh.se (Find Accommodation)؛ liu.se</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>۱۲</t>
+          <t>۱۱</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>درآمد واقع‌بینانه کار حین تحصیل (ناخالص، ماهانه)</t>
+          <t>سقف قانونی کار دانشجویی</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>€1,000–1,600 (Werkstudent فنی €15–20/ساعت؛ برای رشته شما فراوان)</t>
+          <t>۱۴۰ روز کامل یا ۲۸۰ نیم‌روز در سال (Werkstudent تا ۲۰ ساعت/هفته در ترم)</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>تا ≈ €1,000 (۱۶ ساعت × €14.71)؛ یافتن کارفرمای TWV‌گیر سخت</t>
+          <t>۱۶ ساعت/هفته (کارفرما TWV می‌گیرد) یا تمام‌وقت در ژوئن–اوت</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>€300–800 (سقف ۱۵ ساعت؛ کار برای غیرسوئدی‌زبان کمیاب)</t>
+          <t>از ۱۱ ژوئن ۲۰۲۶: حداکثر ۱۵ ساعت/هفته در ترم؛ ژوئن–اوت بدون سقف. تخلف = لغو اقامت. + حداقل پیشرفت تحصیلی ۳۷.۵ واحد سال اول / ۴۵ واحد بعد</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>DKK 8,000–12,000 (€1,070–1,600) اگر کار پیدا شود؛ اکثر کارهای خدماتی دانمارکی می‌خواهند</t>
+          <t>۹۰ ساعت/ماه (سپتامبر–مه) + تمام‌وقت ژوئن–اوت</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>بعد از ماه ششم: ≈ CHF 1,300–1,800 (۱۵ ساعت × CHF 22–28؛ دستیاری آموزشی/پژوهشی در ETH/UZH/ZHAW رایج)</t>
+          <t>غیر-EU: ۶ ماه اول هیچ؛ بعد از آن ۱۵ ساعت/هفته در ترم و تمام‌وقت در تعطیلات؛ کارفرما باید مجوز کانتونی بگیرد؛ کل دورهٔ تحصیل در سوئیس حداکثر ۸ سال</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>تا ≈ £1,100 (۲۰ ساعت × £12.71)</t>
+          <t>۲۰ ساعت/هفته در ترم؛ تمام‌وقت در تعطیلات</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>حداقل دستمزدهای ۲۰۲۶؛ برآورد. درآمد دانشجویی را در تأمین مالی ویزا حساب نکنید.</t>
+          <t>make-it-in-germany.com؛ ind.nl؛ migrationsverket.se (خبر ۲۵ مه ۲۰۲۶)؛ nyidanmark.dk؛ sem.admin.ch؛ gov.uk</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>۱۳</t>
+          <t>۱۲</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>زبان محیط کار فنی (IT)</t>
+          <t>درآمد واقع‌بینانه کار حین تحصیل (ناخالص، ماهانه)</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>انگلیسی در استارتاپ‌ها/شرکت‌های بزرگ (Berlin، Munich، Hamburg) کافی؛ اکثر آگهی‌های IT آلمانی B2 می‌خواهند → بدون آلمانی حدود نیمی از بازار بسته است.</t>
+          <t>€1,000–1,600 (Werkstudent فنی €15–20/ساعت؛ برای رشته شما فراوان)</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>انگلیسی در tech رایج و کافی؛ نه ۱۰۰٪.</t>
+          <t>تا ≈ €1,000 (۱۶ ساعت × €14.71)؛ یافتن کارفرمای TWV‌گیر سخت</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>انگلیسی در tech رایج (Stockholm، Göteborg)؛ بازار ۲۰۲۴–۲۶ ضعیف (بیکاری ≈ ۹٪).</t>
+          <t>€300–800 (سقف ۱۵ ساعت؛ کار برای غیرسوئدی‌زبان کمیاب)</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>انگلیسی برای بخشی از نقش‌های IT در Copenhagen/Aarhus کافی؛ برای اکثر نقش‌ها دانمارکی B1–B2 ترجیح دارد؛ در Aalborg/Odense سخت‌تر.</t>
+          <t>DKK 8,000–12,000 (€1,070–1,600) اگر کار پیدا شود؛ اکثر کارهای خدماتی دانمارکی می‌خواهند</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Zürich: انگلیسی در Big Tech (Google ≈ ۵ هزار نفر، Microsoft، Meta، Apple، Nvidia، OpenAI/Anthropic)، بانک‌ها و استارتاپ‌های ETH کافی؛ Lausanne/Geneva: انگلیسی + فرانسه؛ SMEهای آلمانی‌زبان و Lugano (ایتالیایی) زبان محلی می‌خواهند → بدون آلمانی/فرانسه ≈ نیمی از بازار بسته</t>
+          <t>بعد از ماه ششم: ≈ CHF 1,300–1,800 (۱۵ ساعت × CHF 22–28؛ دستیاری آموزشی/پژوهشی در ETH/UZH/ZHAW رایج)</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>۱۰۰٪ انگلیسی؛ بازار جونیور ۲۰۲۵–۲۶ بسیار رقابتی.</t>
+          <t>تا ≈ £1,100 (۲۰ ساعت × £12.71)</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>workindenmark.dk؛ آگهی‌های StepStone/LinkedIn؛ ارزیابی</t>
+          <t>حداقل دستمزدهای ۲۰۲۶؛ برآورد. درآمد دانشجویی را در تأمین مالی ویزا حساب نکنید.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>۱۴</t>
+          <t>۱۳</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>زبان برای امور اداری و زندگی روزمره</t>
+          <t>زبان محیط کار فنی (IT)</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>قانوناً برای تحصیل لازم نیست؛ عملاً A2–B1 (اداره اتباع، اجاره، بیمه، مالیات).</t>
+          <t>انگلیسی در استارتاپ‌ها/شرکت‌های بزرگ (Berlin، Munich، Hamburg) کافی؛ اکثر آگهی‌های IT آلمانی B2 می‌خواهند → بدون آلمانی حدود نیمی از بازار بسته است.</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>انگلیسی کافی؛ نامه‌های رسمی هلندی.</t>
+          <t>انگلیسی در tech رایج و کافی؛ نه ۱۰۰٪.</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>انگلیسی کافی.</t>
+          <t>انگلیسی در tech رایج (Stockholm، Göteborg)؛ بازار ۲۰۲۴–۲۶ ضعیف (بیکاری ≈ ۹٪).</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>انگلیسی روزمره کافی؛ سامانه‌ها و نامه‌ها دانمارکی.</t>
+          <t>انگلیسی برای بخشی از نقش‌های IT در Copenhagen/Aarhus کافی؛ برای اکثر نقش‌ها دانمارکی B1–B2 ترجیح دارد؛ در Aalborg/Odense سخت‌تر.</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>رسمی: آلمانی / فرانسه / ایتالیایی بسته به کانتون؛ نامه‌های ادارهٔ مهاجرت، بیمه، اجاره و مالیات به زبان محلی؛ انگلیسی در زوریخ/ژنو/لوزان برای روزمره کافی است، ولی سوئیسی‌آلمانی (گویش) در محیط اجتماعی مانع است</t>
+          <t>Zürich: انگلیسی در Big Tech (Google ≈ ۵ هزار نفر، Microsoft، Meta، Apple، Nvidia، OpenAI/Anthropic)، بانک‌ها و استارتاپ‌های ETH کافی؛ Lausanne/Geneva: انگلیسی + فرانسه؛ SMEهای آلمانی‌زبان و Lugano (ایتالیایی) زبان محلی می‌خواهند → بدون آلمانی/فرانسه ≈ نیمی از بازار بسته</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>انگلیسی.</t>
+          <t>۱۰۰٪ انگلیسی؛ بازار جونیور ۲۰۲۵–۲۶ بسیار رقابتی.</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>تجربه عمومی؛ ارزیابی</t>
+          <t>workindenmark.dk؛ آگهی‌های StepStone/LinkedIn؛ ارزیابی</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>۱۵</t>
+          <t>۱۴</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>مجوز اقامت پس از تحصیل برای جست‌وجوی کار</t>
+          <t>زبان برای امور اداری و زندگی روزمره</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>۱۸ ماه (§20 AufenthG) — هر کاری مجاز</t>
+          <t>قانوناً برای تحصیل لازم نیست؛ عملاً A2–B1 (اداره اتباع، اجاره، بیمه، مالیات).</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>۱۲ ماه (zoekjaar) — تا ۳ سال بعد از مدرک قابل درخواست؛ €254</t>
+          <t>انگلیسی کافی؛ نامه‌های رسمی هلندی.</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>۱۲ ماه — با اثبات تمکن SEK 10,656/ماه برای کل دوره</t>
+          <t>انگلیسی کافی.</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>۳ سال، خودکار همراه مجوز تحصیلی برای ارشد state-approved (AAU/SDU) — تا گرفتن «مجوز کار نامحدود» فقط ۹۰ ساعت/ماه</t>
+          <t>انگلیسی روزمره کافی؛ سامانه‌ها و نامه‌ها دانمارکی.</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>فقط ۶ ماه (مجوز L برای جست‌وجوی کار، مادهٔ ۲۱ بند ۳ FNIA) — کوتاه‌ترین در بین ۶ کشور؛ کار در این مدت تا ۱۵ ساعت/هفته</t>
+          <t>رسمی: آلمانی / فرانسه / ایتالیایی بسته به کانتون؛ نامه‌های ادارهٔ مهاجرت، بیمه، اجاره و مالیات به زبان محلی؛ انگلیسی در زوریخ/ژنو/لوزان برای روزمره کافی است، ولی سوئیسی‌آلمانی (گویش) در محیط اجتماعی مانع است</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>۱۸ ماه Graduate visa برای درخواست‌های از ۱ ژانویه ۲۰۲۷ — £937 + IHS £1,035/سال</t>
+          <t>انگلیسی.</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>make-it-in-germany.com؛ ind.nl؛ migrationsverket.se؛ nyidanmark.dk؛ sem.admin.ch؛ gov.uk (Statement of Changes ۱۴ اکتبر ۲۰۲۵)</t>
+          <t>تجربه عمومی؛ ارزیابی</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>۱۵</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>مجوز اقامت پس از تحصیل برای جست‌وجوی کار</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>۱۸ ماه (§20 AufenthG) — هر کاری مجاز</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>۱۲ ماه (zoekjaar) — تا ۳ سال بعد از مدرک قابل درخواست؛ €254</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>۱۲ ماه — با اثبات تمکن SEK 10,656/ماه برای کل دوره</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>۳ سال، خودکار همراه مجوز تحصیلی برای ارشد state-approved (AAU/SDU) — تا گرفتن «مجوز کار نامحدود» فقط ۹۰ ساعت/ماه</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>فقط ۶ ماه (مجوز L برای جست‌وجوی کار، مادهٔ ۲۱ بند ۳ FNIA) — کوتاه‌ترین در بین ۶ کشور؛ کار در این مدت تا ۱۵ ساعت/هفته</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>۱۸ ماه Graduate visa برای درخواست‌های از ۱ ژانویه ۲۰۲۷ — £937 + IHS £1,035/سال</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>make-it-in-germany.com؛ ind.nl؛ migrationsverket.se؛ nyidanmark.dk؛ sem.admin.ch؛ gov.uk (Statement of Changes ۱۴ اکتبر ۲۰۲۵)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>۱۶</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>حداقل حقوق برای ویزای کار (سطوح ۲۰۲۶)</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>بلوکارت: €50,700 عمومی / €45,934.20 برای IT و تازه‌فارغ‌التحصیلان (تا ۳ سال بعد از مدرک)
 مجوز کار §18b برای فارغ‌التحصیلان آلمان: بدون کف ثابت</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>HSM کاهش‌یافته برای فارغ‌التحصیلان هلند (تا ۳ سال): €3,122/ماه بدون حق تعطیلات ≈ €40,500/سال
 زیر ۳۰ سال عادی: €4,357/ماه</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>SEK 34,470/ماه (۹۰٪ میانه؛ از ۱۶ ژوئن ۲۰۲۶)
 فارغ‌التحصیلان سوئد که از داخل درخواست دهند: ۷۵٪ = SEK 28,725/ماه
 هر ژوئن به‌روز می‌شود</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>Positive List (مشاغل IT): کف ثابت ندارد (حقوق مطابق استاندارد دانمارکی)
 Pay Limit: DKK 552,000 · Supplementary: DKK 446,000</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>کف عددی ندارد ولی حقوق باید «متعارف محل/رشته» باشد. فارغ‌التحصیل سوئیس از «اولویت داخلی/EU» معاف است اگر شغل «منفعت علمی/اقتصادی بالا» داشته باشد؛ ⚠️ ولی سهمیهٔ سالانهٔ اتباع غیر-EU (۲۰۲۶: ۴,۵۰۰ مجوز B + ۴,۰۰۰ L؛ معمولاً ≈ ۶۵–۷۰٪ مصرف می‌شود) شامل شما هم می‌شود — طرح معافیت فارغ‌التحصیلان (22.067) از ۲۰۲۳ در پارلمان متوقف مانده</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>Skilled Worker: بالاترینِ £41,700 و نرخ شغل؛ نرخ SOC 2134 (توسعه‌دهنده) = £54,700
 تازه‌کار (حداکثر ۴ سال): ۷۰٪ = £38,290
 + انگلیسی B2 (از ۸ ژانویه ۲۰۲۶)</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr">
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>make-it-in-germany.com؛ ind.nl؛ migrationsverket.se؛ nyidanmark.dk؛ sem.admin.ch (Art. 21 FNIA)؛ gov.uk Appendix Skilled Occupations</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>۱۷</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>حقوق ورودی جونیور توسعه‌دهنده (ناخالص سالانه، ۲۰۲۶)</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>€48,000–55,000 (با ارشد ≈ €55k)</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>€40,000–50,000 (Amsterdam بالاتر)</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>SEK 420,000–540,000 (35–45 هزار در ماه)</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>DKK 500,000–540,000 (IDA 2026: تازه‌فارغ‌التحصیل ≈ DKK 43,800/ماه با بازنشستگی)</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>CHF 85,000–105,000 (≈ $103–127k؛ میانهٔ Glassdoor زوریخ CHF 92k؛ ETH/EPFL 90–118k؛ Big Tech CHF 110–165k) — بالاترین در بین ۶ کشور</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>£28,000–35,000 خارج لندن (Manchester/Leeds/Newcastle)؛ London £32,000–45,000 — اغلب زیر کف اسپانسری £38,290</t>
-        </is>
-      </c>
-      <c r="I18" s="5" t="inlineStr">
-        <is>
-          <t>StepStone؛ Glassdoor؛ IDA؛ Reed — برآورد بازار، نه آمار رسمی</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>۱۸</t>
+          <t>۱۷</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>خالص ماهانه تقریبی (بعد از مالیات)</t>
+          <t>حقوق ورودی جونیور توسعه‌دهنده (ناخالص سالانه، ۲۰۲۶)</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>€2,700–3,000</t>
+          <t>€48,000–55,000 (با ارشد ≈ €55k)</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>€2,700–3,100 (بدون قاعده ۳۰٪)</t>
+          <t>€40,000–50,000 (Amsterdam بالاتر)</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>€2,500–2,900 (SEK 29–33 هزار)</t>
+          <t>SEK 420,000–540,000 (35–45 هزار در ماه)</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>€3,300–3,700 (DKK 25–27.5 هزار)</t>
+          <t>DKK 500,000–540,000 (IDA 2026: تازه‌فارغ‌التحصیل ≈ DKK 43,800/ماه با بازنشستگی)</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>≈ CHF 5,700–6,700 (مالیات + بیمه‌های اجتماعی ≈ ۲۰–۲۵٪ برای مجرد در زوریخ)؛ بیمهٔ درمانی اجباری CHF 350–450/ماه جداگانه از جیب</t>
+          <t>CHF 85,000–105,000 (≈ $103–127k؛ میانهٔ Glassdoor زوریخ CHF 92k؛ ETH/EPFL 90–118k؛ Big Tech CHF 110–165k) — بالاترین در بین ۶ کشور</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>£2,000–2,500</t>
+          <t>£28,000–35,000 خارج لندن (Manchester/Leeds/Newcastle)؛ London £32,000–45,000 — اغلب زیر کف اسپانسری £38,290</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>ماشین‌حساب‌های مالیاتی ۲۰۲۶ (کلاس مالیاتی مجرد)</t>
+          <t>StepStone؛ Glassdoor؛ IDA؛ Reed — برآورد بازار، نه آمار رسمی</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>۱۹</t>
+          <t>۱۸</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>پس‌انداز ماهانه تخمینی جونیور (خالص − هزینه زندگی یک نفر شاغل)</t>
+          <t>خالص ماهانه تقریبی (بعد از مالیات)</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>€1,000–1,500</t>
+          <t>€2,700–3,000</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>€700–1,200</t>
+          <t>€2,700–3,100 (بدون قاعده ۳۰٪)</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>€900–1,400</t>
+          <t>€2,500–2,900 (SEK 29–33 هزار)</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>€1,100–1,600</t>
+          <t>€3,300–3,700 (DKK 25–27.5 هزار)</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>CHF 1,500–3,000 (≈ $1,800–3,600) در زوریخ (استودیو CHF 1,400–1,900 + بیمه ≈ 400) — بیشترین پس‌انداز مطلق بین ۶ کشور، اگر شغل بگیرید</t>
+          <t>≈ CHF 5,700–6,700 (مالیات + بیمه‌های اجتماعی ≈ ۲۰–۲۵٪ برای مجرد در زوریخ)؛ بیمهٔ درمانی اجباری CHF 350–450/ماه جداگانه از جیب</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>£400–900</t>
+          <t>£2,000–2,500</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>برآورد؛ هزینه زندگی شاغل: DE €1,400–1,700 · NL €1,700–2,100 · SE €1,300–1,600 · DK €1,900–2,300 · CH CHF 3,200–3,800 · UK £1,300–1,700</t>
+          <t>ماشین‌حساب‌های مالیاتی ۲۰۲۶ (کلاس مالیاتی مجرد)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>۲۰</t>
+          <t>۱۹</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>اقامت دائم (PR) — زمان و شرط اصلی</t>
+          <t>پس‌انداز ماهانه تخمینی جونیور (خالص − هزینه زندگی یک نفر شاغل)</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>۲ سال کار برای فارغ‌التحصیل آلمان با B1 (§18c)؛ بلوکارت: ۲۱ ماه با B1 / ۲۷ ماه با A1</t>
+          <t>€1,000–1,500</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>۵ سال اقامت قانونی (سال‌های تحصیل نصف حساب می‌شود) + inburgering</t>
+          <t>€700–1,200</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>۴ سال مجوز کار در ۷ سال اخیر + خودکفایی (تحصیل حساب نمی‌شود)</t>
+          <t>€900–1,400</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>۸ سال (یا ۴ سال با هر ۴ شرط تکمیلی) + ۳.۵ سال کار تمام‌وقت در ۴ سال اخیر</t>
+          <t>€1,100–1,600</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>اجازهٔ اقامت C: برای ایرانی‌ها ۱۰ سال (۵ سال آخر پیوسته با B)؛ سال‌های دانشجویی فقط اگر بعدش ۲ سال پیوسته اجازهٔ B داشته باشید حساب می‌شود؛ C زودهنگام ۵ ساله فقط با «ادغام موفق» و B1 شفاهی به صلاحدید کانتون — سخت‌ترین مسیر در بین ۶ کشور</t>
+          <t>CHF 1,500–3,000 (≈ $1,800–3,600) در زوریخ (استودیو CHF 1,400–1,900 + بیمه ≈ 400) — بیشترین پس‌انداز مطلق بین ۶ کشور، اگر شغل بگیرید</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>فعلاً ۵ سال Skilled Worker (Graduate visa حساب نمی‌شود)؛ طرح Earned Settlement با پایه ۱۰ سال در دستور کار دولت (تا سپتامبر ۲۰۲۶ قانون نشده)</t>
+          <t>£400–900</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>make-it-in-germany.com؛ ind.nl؛ migrationsverket.se؛ nyidanmark.dk؛ sem.admin.ch؛ gov.uk / Home Affairs Committee</t>
+          <t>برآورد؛ هزینه زندگی شاغل: DE €1,400–1,700 · NL €1,700–2,100 · SE €1,300–1,600 · DK €1,900–2,300 · CH CHF 3,200–3,800 · UK £1,300–1,700</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>۲۱</t>
+          <t>۲۰</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>آزمون زبان محلی برای PR</t>
+          <t>اقامت دائم (PR) — زمان و شرط اصلی</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>B1 آلمانی (A1 فقط با بلوکارت ۲۷ ماهه)</t>
+          <t>۲ سال کار برای فارغ‌التحصیل آلمان با B1 (§18c)؛ بلوکارت: ۲۱ ماه با B1 / ۲۷ ماه با A1</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>A2 فعلی → B1 (تصمیم کابینه، فوریه ۲۰۲۶)</t>
+          <t>۵ سال اقامت قانونی (سال‌های تحصیل نصف حساب می‌شود) + inburgering</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>هیچ (برای PR)</t>
+          <t>۴ سال مجوز کار در ۷ سال اخیر + خودکفایی (تحصیل حساب نمی‌شود)</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Prøve i Dansk 2 (≈ B1) برای مسیر ۸ ساله؛ PD3 (≈ B2) برای مسیر ۴ ساله</t>
+          <t>۸ سال (یا ۴ سال با هر ۴ شرط تکمیلی) + ۳.۵ سال کار تمام‌وقت در ۴ سال اخیر</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>A2 شفاهی + A1 کتبی زبان محلی (آزمون fide) برای C ۱۰ ساله؛ B1 شفاهی برای C زودهنگام ۵ ساله → بدون زبان سوم PR نمی‌گیرید</t>
+          <t>اجازهٔ اقامت C: برای ایرانی‌ها ۱۰ سال (۵ سال آخر پیوسته با B)؛ سال‌های دانشجویی فقط اگر بعدش ۲ سال پیوسته اجازهٔ B داشته باشید حساب می‌شود؛ C زودهنگام ۵ ساله فقط با «ادغام موفق» و B1 شفاهی به صلاحدید کانتون — سخت‌ترین مسیر در بین ۶ کشور</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>انگلیسی B2 از ۲۶ مارس ۲۰۲۷ + آزمون Life in the UK (زبان سوم نیست)</t>
+          <t>فعلاً ۵ سال Skilled Worker (Graduate visa حساب نمی‌شود)؛ طرح Earned Settlement با پایه ۱۰ سال در دستور کار دولت (تا سپتامبر ۲۰۲۶ قانون نشده)</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>BAMF؛ ind.nl؛ migrationsverket.se؛ nyidanmark.dk؛ sem.admin.ch؛ gov.uk (HC 1691)</t>
+          <t>make-it-in-germany.com؛ ind.nl؛ migrationsverket.se؛ nyidanmark.dk؛ sem.admin.ch؛ gov.uk / Home Affairs Committee</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>۲۲</t>
+          <t>۲۱</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>شهروندی (جدا از PR)</t>
+          <t>آزمون زبان محلی برای PR</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>۵ سال + B1 + آزمون تابعیت (تحصیل حساب می‌شود)</t>
+          <t>B1 آلمانی (A1 فقط با بلوکارت ۲۷ ماهه)</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>۵ سال + inburgering (A2 → B1)</t>
+          <t>A2 فعلی → B1 (تصمیم کابینه، فوریه ۲۰۲۶)</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>از ۶ ژوئن ۲۰۲۶: ۸ سال + آزمون مدنی + آزمون زبان (از اکتبر ۲۰۲۷) + کف درآمد</t>
+          <t>هیچ (برای PR)</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>۹ سال + PD3 + آزمون تابعیت + اشتغال ۳.۵ سال از ۴ سال</t>
+          <t>Prøve i Dansk 2 (≈ B1) برای مسیر ۸ ساله؛ PD3 (≈ B2) برای مسیر ۴ ساله</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>۱۰ سال اقامت (سال‌های ۸ تا ۱۸ سالگی دوبرابر) + اجازهٔ C + B1 شفاهی / A2 کتبی + شرایط کانتون و شهرداری (۲–۵ سال اقامت محلی) — سخت‌ترین در اروپا</t>
+          <t>A2 شفاهی + A1 کتبی زبان محلی (آزمون fide) برای C ۱۰ ساله؛ B1 شفاهی برای C زودهنگام ۵ ساله → بدون زبان سوم PR نمی‌گیرید</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>ILR + ۱۲ ماه؛ B1/B2 + Life in the UK</t>
+          <t>انگلیسی B2 از ۲۶ مارس ۲۰۲۷ + آزمون Life in the UK (زبان سوم نیست)</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>قوانین تابعیت ۲۰۲۶؛ migrationsverket.se؛ nyidanmark.dk؛ sem.admin.ch</t>
+          <t>BAMF؛ ind.nl؛ migrationsverket.se؛ nyidanmark.dk؛ sem.admin.ch؛ gov.uk (HC 1691)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>۲۳</t>
+          <t>۲۲</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>فرایند ویزا برای پاسپورت ایرانی — وضعیت سپتامبر ۲۰۲۶ (بسیار متغیر)</t>
+          <t>شهروندی (جدا از PR)</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>سفارت تهران در «حالت اضطراری»؛ بخش ویزا به روی مراجعان عادی بسته. TLScontact از ۱۵ ژوئیه ۲۰۲۶ لیست انتظار دانشجویی باز کرده ولی وقت نمی‌دهد. صدور ویزا: ۴۶هزار (۲۰۲۴) → ۲۳هزار (۲۰۲۵) → ≈ ۱٬۳۰۰ اوایل ۲۰۲۶. ارجاع موردی به ایروان/استانبول. حتی در شرایط عادی لیست انتظار ۶–۱۸ ماه.</t>
+          <t>۵ سال + B1 + آزمون تابعیت (تحصیل حساب می‌شود)</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>دانشگاه درخواست را در IND ثبت می‌کند (TEV) ✓؛ ولی سفارت هلند موقتاً به باکو منتقل شده و MVV در ایران صادر نمی‌شود.</t>
+          <t>۵ سال + inburgering (A2 → B1)</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>درخواست آنلاین در Migrationsverket؛ بررسی دیجیتال پاسپورت؛ سفارت تهران فعلاً بیومتریک/کارت اقامت نمی‌گیرد (ژوئیه ۲۰۲۶).</t>
+          <t>از ۶ ژوئن ۲۰۲۶: ۸ سال + آزمون مدنی + آزمون زبان (از اکتبر ۲۰۲۷) + کف درآمد</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>«در حال حاضر امکان درخواست از ایران وجود ندارد» (سفارت دانمارک، ۲۰۲۶) — باید از SIRI بخواهید پرونده به نمایندگی دیگری در منطقه برود؛ بیومتریک ظرف ۱۴ روز.</t>
+          <t>۹ سال + PD3 + آزمون تابعیت + اشتغال ۳.۵ سال از ۴ سال</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>سفارت سوئیس در تهران باز است: ویزای D (تحصیلی) با وقت قبلی پذیرفته می‌شود، ویزای C فعلاً خیر (اطلاعیهٔ ۳۰ ژانویه ۲۰۲۶؛ در جنگ ژوئن ۲۰۲۵ دو هفته بسته بود). تصمیم را ادارهٔ مهاجرت کانتون می‌گیرد: ۸–۱۲ هفته؛ ETH تأییدیهٔ ثبت‌نام برای ویزا را از می ۲۰۲۷ می‌دهد. ⚠️ گلوگاه اصلی: اثبات تمکن (ردیف ۲۵).</t>
+          <t>۱۰ سال اقامت (سال‌های ۸ تا ۱۸ سالگی دوبرابر) + اجازهٔ C + B1 شفاهی / A2 کتبی + شرایط کانتون و شهرداری (۲–۵ سال اقامت محلی) — سخت‌ترین در اروپا</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>درخواست آنلاین gov.uk + بیومتریک در VAC؛ VFS تهران در ۲۰۲۶ متناوباً بسته/باز شده؛ می‌توان از VAC کشور ثالث اقدام کرد. «قانون ۲۸ روز» مربوط به تمکن مالی است، نه VFS.</t>
+          <t>ILR + ۱۲ ماه؛ B1/B2 + Life in the UK</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>visas-de.tlscontact.com؛ netherlandsworldwide.nl؛ swedenabroad.se؛ iran.um.dk؛ eda.admin.ch/tehran؛ gov.uk — برنامه B: اقدام از ترکیه/ارمنستان/امارات</t>
+          <t>قوانین تابعیت ۲۰۲۶؛ migrationsverket.se؛ nyidanmark.dk؛ sem.admin.ch</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t>۲۳</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>فرایند ویزا برای پاسپورت ایرانی — وضعیت سپتامبر ۲۰۲۶ (بسیار متغیر)</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>سفارت تهران در «حالت اضطراری»؛ بخش ویزا به روی مراجعان عادی بسته. TLScontact از ۱۵ ژوئیه ۲۰۲۶ لیست انتظار دانشجویی باز کرده ولی وقت نمی‌دهد. صدور ویزا: ۴۶هزار (۲۰۲۴) → ۲۳هزار (۲۰۲۵) → ≈ ۱٬۳۰۰ اوایل ۲۰۲۶. ارجاع موردی به ایروان/استانبول. حتی در شرایط عادی لیست انتظار ۶–۱۸ ماه.</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>دانشگاه درخواست را در IND ثبت می‌کند (TEV) ✓؛ ولی سفارت هلند موقتاً به باکو منتقل شده و MVV در ایران صادر نمی‌شود.</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>درخواست آنلاین در Migrationsverket؛ بررسی دیجیتال پاسپورت؛ سفارت تهران فعلاً بیومتریک/کارت اقامت نمی‌گیرد (ژوئیه ۲۰۲۶).</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>«در حال حاضر امکان درخواست از ایران وجود ندارد» (سفارت دانمارک، ۲۰۲۶) — باید از SIRI بخواهید پرونده به نمایندگی دیگری در منطقه برود؛ بیومتریک ظرف ۱۴ روز.</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>سفارت سوئیس در تهران باز است: ویزای D (تحصیلی) با وقت قبلی پذیرفته می‌شود، ویزای C فعلاً خیر (اطلاعیهٔ ۳۰ ژانویه ۲۰۲۶؛ در جنگ ژوئن ۲۰۲۵ دو هفته بسته بود). تصمیم را ادارهٔ مهاجرت کانتون می‌گیرد: ۸–۱۲ هفته؛ ETH تأییدیهٔ ثبت‌نام برای ویزا را از می ۲۰۲۷ می‌دهد. ⚠️ گلوگاه اصلی: اثبات تمکن (ردیف ۲۵).</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>درخواست آنلاین gov.uk + بیومتریک در VAC؛ VFS تهران در ۲۰۲۶ متناوباً بسته/باز شده؛ می‌توان از VAC کشور ثالث اقدام کرد. «قانون ۲۸ روز» مربوط به تمکن مالی است، نه VFS.</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>visas-de.tlscontact.com؛ netherlandsworldwide.nl؛ swedenabroad.se؛ iran.um.dk؛ eda.admin.ch/tehran؛ gov.uk — برنامه B: اقدام از ترکیه/ارمنستان/امارات</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
           <t>۲۴</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>نمره انگلیسی برنامه‌های هدف</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>TU Darmstadt، TU Dresden، Stuttgart: C1 / IELTS 7.0 (Dresden: هر بخش ≥ B2)
 FAU (AI): B2 / IELTS 6.5</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>IELTS 6.5 (هر بخش ≥ 6.0)</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>IELTS 6.5 (هر بخش ≥ 5.5)</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>IELTS 6.5</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr">
+      <c r="G26" s="4" t="inlineStr">
         <is>
           <t>USI: B2 در ورود (IELTS 5.5–6.5) و C1 تا فارغ‌التحصیلی · HSLU: C1 (B2 مشروط) · Joint MSc CS (Neuchâtel/Fribourg/Bern): بدون آزمون زبان — B2 توصیه (FAQ رسمی) · ZHAW: B2–C1 · UZH و ETH: C1 / IELTS 7.0 · EPFL: مدرک زبان الزامی نیست</t>
         </is>
       </c>
-      <c r="H25" s="4" t="inlineStr">
+      <c r="H26" s="4" t="inlineStr">
         <is>
           <t>IELTS 6.0–6.5</t>
         </is>
       </c>
-      <c r="I25" s="5" t="inlineStr">
+      <c r="I26" s="5" t="inlineStr">
         <is>
           <t>سایت برنامه‌ها — ⚠️ IELTS از ۳۱ ژانویه ۲۰۲۶ و TOEFL از ۱۴۰۵ در ایران برگزار نمی‌شوند؛ آزمون را در استانبول/ایروان/دبی/تفلیس بدهید (نتیجهٔ کامپیوتری ۳–۵ روزه). برای مهلت ۱۵ ژانویهٔ ۲۰۲۷ (سوئد/دانمارک/Stuttgart) نتیجه باید تا اوایل ژانویه در دست باشد</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>۲۵</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>تمکن مالی ویزا (۲۰۲۶) و نکته تحریمی</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>حساب مسدود €11,904 (€992 × ۱۲). Fintiba ساکنان ایران را نمی‌پذیرد؛ Expatrio/Coracle را هنگام اقدام بررسی کنید. انتقال پول فقط از مسیر کشور ثالث/صرافی (۳–۶٪ هزینه).</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>€13,569 (€1,130.77 × ۱۲) + شهریه؛ معمولاً به حساب دانشگاه واریز می‌شود.</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>SEK 10,656 × ماه‌های مجوز (سال اول ≈ SEK 128,000) + قسط اول شهریه.</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>پرداخت شهریه ترم اول به‌عنوان تمکن پذیرفته می‌شود (در غیر این‌صورت DKK 7,426/ماه).</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>CHF 21,000 برای هر سال (Basel 24,000) + شهریه؛ برای هر تمدید سالانه دوباره. زوریخ: فقط حساب بانک سوئیسی/شعبهٔ سوئیسی به نام خودتان (حساب والدین پذیرفته نیست) یا ضامن مقیم سوئیس (B/C)؛ بانک‌های سوئیس برای ساکنان ایران حساب باز نمی‌کنند → عملاً از تهران فقط با ضامن، یا کانتون‌های انعطاف‌پذیرتر (تیچینو، فریبورگ، نوشاتل، برن، لوسرن — قبل از اقدام از دفتر بین‌الملل دانشگاه تأیید بگیرید). انتقال پول فقط از مسیر کشور ثالث.</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t>شهریه + £1,171 × ۹ = £10,539 خارج لندن / £13,761 لندن؛ از ۳۰ نوامبر ۲۰۲۶: £10,827 / £14,130؛ ۲۸ روز متوالی در حساب؛ + ویزای دانشجویی £524 + IHS با نرخ دانشجویی £776/سال (برای ۱۶ ماه اقامت ≈ £1,164).</t>
-        </is>
-      </c>
-      <c r="I26" s="5" t="inlineStr">
-        <is>
-          <t>make-it-in-germany.com؛ ind.nl؛ migrationsverket.se؛ nyidanmark.dk؛ sem.admin.ch؛ gov.uk (HC 584). افتتاح حساب بانکی برای ایرانی‌ها در همه‌جا کندتر است (آلمان و هلند بیشترین گزارش مشکل).</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>۲۶</t>
+          <t>۲۵</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>بازار کار برای جونیورِ فقط‌انگلیسی‌زبان (ارزیابی، ۱–۵ ستاره)</t>
+          <t>تمکن مالی ویزا (۲۰۲۶) و نکته تحریمی</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>⭐⭐⭐ تقاضا و حقوق بالا؛ بدون آلمانی نیمی از بازار بسته</t>
+          <t>حساب مسدود €11,904 (€992 × ۱۲). Fintiba ساکنان ایران را نمی‌پذیرد؛ Expatrio/Coracle را هنگام اقدام بررسی کنید. انتقال پول فقط از مسیر کشور ثالث/صرافی (۳–۶٪ هزینه).</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>⭐⭐⭐⭐ انگلیسی‌دوست‌ترین بازار قاره؛ کف HSM فارغ‌التحصیل دست‌یافتنی</t>
+          <t>€13,569 (€1,130.77 × ۱۲) + شهریه؛ معمولاً به حساب دانشگاه واریز می‌شود.</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>⭐⭐ بازار ۲۰۲۴–۲۶ ضعیف؛ شبکه محلی مهم</t>
+          <t>SEK 10,656 × ماه‌های مجوز (سال اول ≈ SEK 128,000) + قسط اول شهریه.</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>⭐⭐ بدون دانمارکی محدود؛ خارج از Copenhagen سخت</t>
+          <t>پرداخت شهریه ترم اول به‌عنوان تمکن پذیرفته می‌شود (در غیر این‌صورت DKK 7,426/ماه).</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>⭐⭐⭐ بالاترین حقوق اروپا و هاب Big Tech در زوریخ؛ ولی برای غیر-EU فقط ۶ ماه فرصت، سهمیه و شرط «منفعت اقتصادی بالا» → عملاً فقط شرکت‌های بزرگ/اسپین‌آف‌های ETH اسپانسر می‌شوند؛ رقابت با فارغ‌التحصیلان ETH/EPFL و EU؛ بازار ۲۰۲۶ گزینشی‌تر</t>
+          <t>CHF 21,000 برای هر سال (Basel 24,000) + شهریه؛ برای هر تمدید سالانه دوباره. زوریخ: فقط حساب بانک سوئیسی/شعبهٔ سوئیسی به نام خودتان (حساب والدین پذیرفته نیست) یا ضامن مقیم سوئیس (B/C)؛ بانک‌های سوئیس برای ساکنان ایران حساب باز نمی‌کنند → عملاً از تهران فقط با ضامن، یا کانتون‌های انعطاف‌پذیرتر (تیچینو، فریبورگ، نوشاتل، برن، لوسرن — قبل از اقدام از دفتر بین‌الملل دانشگاه تأیید بگیرید). انتقال پول فقط از مسیر کشور ثالث.</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>⭐⭐ بازار جونیور اشباع؛ اسپانسری £38,290+ برای جونیور نادر؛ بعد از ۱۸ ماه باید ویزای کار داشت</t>
+          <t>شهریه + £1,171 × ۹ = £10,539 خارج لندن / £13,761 لندن؛ از ۳۰ نوامبر ۲۰۲۶: £10,827 / £14,130؛ ۲۸ روز متوالی در حساب؛ + ویزای دانشجویی £524 + IHS با نرخ دانشجویی £776/سال (برای ۱۶ ماه اقامت ≈ £1,164).</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>ارزیابی بر اساس ردیف‌های ۱۳، ۱۵، ۱۶، ۱۷</t>
+          <t>make-it-in-germany.com؛ ind.nl؛ migrationsverket.se؛ nyidanmark.dk؛ sem.admin.ch؛ gov.uk (HC 584). افتتاح حساب بانکی برای ایرانی‌ها در همه‌جا کندتر است (آلمان و هلند بیشترین گزارش مشکل).</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>۲۷</t>
+          <t>۲۶</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>جهت‌گیری سیاست‌های مهاجرتی ۲۰۲۵–۲۶ (ریسک تغییر تا ۲۰۲۸)</t>
+          <t>بازار کار برای جونیورِ فقط‌انگلیسی‌زبان (ارزیابی، ۱–۵ ستاره)</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>متوسط: قوانین کار پایدار؛ تابعیت ۳ ساله حذف شد</t>
+          <t>⭐⭐⭐ تقاضا و حقوق بالا؛ بدون آلمانی نیمی از بازار بسته</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>متوسط: B1 برای PR/تابعیت؛ WIB فقط کارشناسی انگلیسی را هدف گرفته (ارشد امن)</t>
+          <t>⭐⭐⭐⭐ انگلیسی‌دوست‌ترین بازار قاره؛ کف HSM فارغ‌التحصیل دست‌یافتنی</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>بالا: شهروندی ۸ سال، کف حقوق ۹۰٪ میانه، سقف کار ۱۵ ساعت، تبدیل اقامت تحصیلی به کاری فقط بعد از ≥ ۲ ترم</t>
+          <t>⭐⭐ بازار ۲۰۲۴–۲۶ ضعیف؛ شبکه محلی مهم</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>متوسط–بالا: سخت‌گیرانه ولی پایدار</t>
+          <t>⭐⭐ بدون دانمارکی محدود؛ خارج از Copenhagen سخت</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>متوسط: ابتکار «سوئیس ۱۰ میلیونی» SVP در ۱۴ ژوئن ۲۰۲۶ رد شد (۵۴.۸٪ نه)؛ ولی بستهٔ صرفه‌جویی EP27 (۲۰۲۷–۲۹) → احتمال افزایش دوبارهٔ شهریهٔ ETH/EPFL برای خارجی‌ها؛ سهمیهٔ غیر-EU ثابت (۸,۵۰۰)؛ بستهٔ قراردادهای جدید با EU (Bilaterals III) در راه رفراندوم</t>
+          <t>⭐⭐⭐ بالاترین حقوق اروپا و هاب Big Tech در زوریخ؛ ولی برای غیر-EU فقط ۶ ماه فرصت، سهمیه و شرط «منفعت اقتصادی بالا» → عملاً فقط شرکت‌های بزرگ/اسپین‌آف‌های ETH اسپانسر می‌شوند؛ رقابت با فارغ‌التحصیلان ETH/EPFL و EU؛ بازار ۲۰۲۶ گزینشی‌تر</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>بسیار بالا: Graduate visa ۱۸ ماه، B2، طرح PR ۱۰ ساله، عوارض £925/دانشجو/سال از اوت ۲۰۲۸ فقط برای دانشگاه‌های انگلستان — دورهٔ یک‌سالهٔ شما (سپتامبر ۲۰۲۷ تا سپتامبر ۲۰۲۸) عملاً از آن رد می‌شود، ولی بعضی دانشگاه‌ها ممکن است از ۲۰۲۷ در شهریه پیش‌خور کنند</t>
+          <t>⭐⭐ بازار جونیور اشباع؛ اسپانسری £38,290+ برای جونیور نادر؛ بعد از ۱۸ ماه باید ویزای کار داشت</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>قوانین و لوایح ۲۰۲۵–۲۶</t>
+          <t>ارزیابی بر اساس ردیف‌های ۱۳، ۱۵، ۱۶، ۱۷</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
+          <t>۲۷</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>جهت‌گیری سیاست‌های مهاجرتی ۲۰۲۵–۲۶ (ریسک تغییر تا ۲۰۲۸)</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>متوسط: قوانین کار پایدار؛ تابعیت ۳ ساله حذف شد</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>متوسط: B1 برای PR/تابعیت؛ WIB فقط کارشناسی انگلیسی را هدف گرفته (ارشد امن)</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>بالا: شهروندی ۸ سال، کف حقوق ۹۰٪ میانه، سقف کار ۱۵ ساعت، تبدیل اقامت تحصیلی به کاری فقط بعد از ≥ ۲ ترم</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>متوسط–بالا: سخت‌گیرانه ولی پایدار</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>متوسط: ابتکار «سوئیس ۱۰ میلیونی» SVP در ۱۴ ژوئن ۲۰۲۶ رد شد (۵۴.۸٪ نه)؛ ولی بستهٔ صرفه‌جویی EP27 (۲۰۲۷–۲۹) → احتمال افزایش دوبارهٔ شهریهٔ ETH/EPFL برای خارجی‌ها؛ سهمیهٔ غیر-EU ثابت (۸,۵۰۰)؛ بستهٔ قراردادهای جدید با EU (Bilaterals III) در راه رفراندوم</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>بسیار بالا: Graduate visa ۱۸ ماه، B2، طرح PR ۱۰ ساله، عوارض £925/دانشجو/سال از اوت ۲۰۲۸ فقط برای دانشگاه‌های انگلستان — دورهٔ یک‌سالهٔ شما (سپتامبر ۲۰۲۷ تا سپتامبر ۲۰۲۸) عملاً از آن رد می‌شود، ولی بعضی دانشگاه‌ها ممکن است از ۲۰۲۷ در شهریه پیش‌خور کنند</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>قوانین و لوایح ۲۰۲۵–۲۶</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
           <t>۲۸</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>امتیاز برای ۳ معیار شما (هر کدام از ۱۰): هزینه کل / زندگی و کار فقط با انگلیسی / بازار کار و حقوق</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>10 / 4 / 8 = ۲۲</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>2 / 8 / 8 = ۱۸</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
         <is>
           <t>6 / 8 / 5 = ۱۹</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
+      <c r="F30" s="4" t="inlineStr">
         <is>
           <t>4 / 6 / 6 = ۱۶</t>
         </is>
       </c>
-      <c r="G29" s="4" t="inlineStr">
+      <c r="G30" s="4" t="inlineStr">
         <is>
           <t>5 / 6 / 7 = ۱۸</t>
         </is>
       </c>
-      <c r="H29" s="4" t="inlineStr">
+      <c r="H30" s="4" t="inlineStr">
         <is>
           <t>5 / 10 / 4 = ۱۹</t>
         </is>
       </c>
-      <c r="I29" s="5" t="inlineStr">
+      <c r="I30" s="5" t="inlineStr">
         <is>
           <t>وزن برابر. اگر «هزینه» وزن بیشتری دارد و B1 آلمانی را می‌پذیرید → آلمان؛ اگر «انگلیسی» وزن بیشتری دارد → انگلستان (کامل) و بعد هلند/سوئد؛ اگر «حقوق» وزن بیشتری دارد → سوئیس، به شرط پذیرش ریسک پنجرهٔ ۶ ماههٔ کار و هزینهٔ زندگی. سوئیس: هزینه ۵ (شهریه ناچیز ولی زندگی گران‌ترین)، انگلیسی ۶ (تحصیل و Big Tech انگلیسی، اداری/PR زبان محلی)، بازار ۷ (بالاترین حقوق، ولی دسترسی محدود برای غیر-EU). انگلستان با گزینه‌های ارزان شمال (Teesside/Northumbria) ۱۹ (هم‌امتیاز سوئد) ولی هنوز از بودجهٔ سالانه $32k بیرون است.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="B31" s="6" t="inlineStr">
+    <row r="32">
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>تاریخ راستی‌آزمایی: ۲۷ سپتامبر ۲۰۲۶ (۵ مهر ۱۴۰۵). نرخ تبدیل ۲۷ سپتامبر ۲۰۲۶: €1 = $1.14 · £1 = $1.325 · $1 ≈ SEK 9.9 · $1 ≈ DKK 6.55 · CHF 1 = $1.21</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>همه ارقام سطح 2026/27 و از منابع رسمی (شیت «منابع»)؛ برای ورودی سپتامبر ۲۰۲۷ نرخ 2027/28 را بگیرید (تا بهار ۲۰۲۷ منتشر می‌شود؛ فعلاً +۳–۵٪). ردیف‌های ۱۳، ۱۴، ۱۷–۱۹، ۲۶ برآورد/ارزیابی هستند و در ستون منبع مشخص شده‌اند.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="B33" t="inlineStr">
         <is>
+          <t>همه ارقام سطح 2026/27 و از منابع رسمی (شیت «منابع»)؛ برای ورودی سپتامبر ۲۰۲۷ نرخ 2027/28 را بگیرید (تا بهار ۲۰۲۷ منتشر می‌شود؛ فعلاً +۳–۵٪). ردیف‌های ۱۳، ۱۴، ۱۷–۱۹، ۲۶ برآورد/ارزیابی هستند و در ستون منبع مشخص شده‌اند.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" t="inlineStr">
+        <is>
           <t>جدول اولیه (Table.xlsx) برای مقایسه دست‌نخورده مانده است.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="B34" s="6" t="inlineStr">
+    <row r="35">
+      <c r="B35" s="6" t="inlineStr">
         <is>
           <t>شیت «برنامه‌ها»: ≈۱۰۰ برنامهٔ انگلیسی‌زبان در ۸ حوزهٔ کامپیوتری (نه فقط CS) برای هر ۶ کشور؛ شیت «حوزه‌ها و بازار کار»: کدام حوزه برای شما بازار و پذیرش بهتری دارد.</t>
         </is>
@@ -12239,7 +12317,8 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>• هزینه کل دوره اضافه شد (هلند از «نیاز به تأمین سال دوم» به گران‌ترین گزینه تبدیل شد)
+          <t>• ردیف ۵ب (بورس/تخفیف شهریهٔ واقعاً در دسترس شما) اضافه شد — ۲۸ سپتامبر ۲۰۲۶؛ امتیازها را عوض نمی‌کند
+• هزینه کل دوره اضافه شد (هلند از «نیاز به تأمین سال دوم» به گران‌ترین گزینه تبدیل شد)
 • فقط انگلستان (به خواست شما): Strathclyde و Swansea حذف شدند؛ گزینه‌ها Teesside £17,000 · Northumbria £21,500 · Leicester £24,250 · Essex £24,675 · Brunel £24,795 · York £32,900؛ Graduate visa ۱۸ ماه؛ کف اسپانسری £54,700 / £38,290؛ طرح PR ۱۰ ساله؛ عوارض £925 از ۲۰۲۸ شامل همهٔ گزینه‌ها
 • کف حقوق ۲۰۲۶ همه کشورها به‌روز شد (آلمان €50,700/€45,934؛ هلند €3,122/ماه؛ سوئد SEK 34,470)
 • ایرلند به خواست شما به‌کلی حذف و سوئیس جایگزین شد (سپتامبر ۲۰۲۶): شهریه‌های 2026/27 ETH/EPFL/UZH/USI/ZHAW/HSLU، تمکن CHF 21,000، ۶ ماه جست‌وجوی کار، سهمیهٔ غیر-EU، اجازهٔ C ۱۰ ساله، حقوق جونیور CHF 85–105k، سفارت تهران (ویزای D فعال)
@@ -12297,7 +12376,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B158"/>
+  <dimension ref="A1:B173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -12787,1414 +12866,1594 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – ETH: تاریخ‌های اپلای ارشد پاییز ۲۰۲۷ (۱–۳۰ نوامبر ۲۰۲۶؛ پاسخ تا پایان مارس؛ شروع ۲۰ سپتامبر ۲۰۲۷)</t>
+          <t>بورس – LiU International Scholarship: معمولاً ۵۰٪؛ شرط جدید ۲۰۲۶ (GPA ≥ 3.5/4 یا first/high second class)؛ فقط اولویت ۱</t>
         </is>
       </c>
       <c r="B41" s="16" t="inlineStr">
         <is>
-          <t>https://ethz.ch/en/studies/master/application/dates.html</t>
+          <t>https://liu.se/en/article/scholarships</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – EPFL: شهریه CHF 2,240/ترم برای خارجی‌های غیرمقیم از پاییز ۲۰۲۵ (CHF 780 برای بقیه)</t>
+          <t>بورس – Chalmers: بورس‌های شهریه‌پردازها (IPOET ۷۵٪ با حداقل معدل ۸۰٪، Avancez)</t>
         </is>
       </c>
       <c r="B42" s="16" t="inlineStr">
         <is>
-          <t>https://www.epfl.ch/education/studies/en/rules-and-procedures/study-taxes/tuition-fee-other-fees/</t>
+          <t>https://www.chalmers.se/en/education/application-and-admission/scholarships-for-fee-paying-students/</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – EPFL: پنجره‌های اپلای ارشد (۱۵ دسامبر / ۳۱ مارس؛ یک برنامه در سال)</t>
+          <t>بورس – Halmstad University Scholarship ۲۵٪/۵۰٪ برای غیر-EU (ثانویه؛ hh.se را چک کنید)</t>
         </is>
       </c>
       <c r="B43" s="16" t="inlineStr">
         <is>
-          <t>https://www.epfl.ch/education/admission/admission-2/master-admission-criteria-application/online-application/</t>
+          <t>https://www.mastersportal.com/scholarships/10077/halmstad-university-scholarships.html</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – UZH: شهریه CHF 720 + 100 (خارجی، ارشد) + 59؛ هزینهٔ درخواست CHF 150</t>
+          <t>بورس – MDU: بورس تا ۱۰۰٪ شهریه برای متقاضیان اولویت ۱ (ثانویه؛ mdu.se را چک کنید)</t>
         </is>
       </c>
       <c r="B44" s="16" t="inlineStr">
         <is>
-          <t>https://www.uzh.ch/en/studies/application/fees.html</t>
+          <t>https://daadscholarship.com/malardalen-university-scholarships-2026-to-study-for-free-in-sweden/</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – UZH: مهلت ویزایی‌ها ۲۸ فوریه / بدون ویزا ۳۰ آوریل (پاییز)</t>
+          <t>بورس – SI Scholarship for Global Professionals: ۳۴ کشور واجد شرایط — ایران نیست (رسمی)</t>
         </is>
       </c>
       <c r="B45" s="16" t="inlineStr">
         <is>
-          <t>https://www.oec.uzh.ch/en/studies/general/admission/master/faq-master-admission.html</t>
+          <t>https://si.se/en/apply/scholarships/swedish-institute-scholarships-for-global-professionals/</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – USI MSc Informatics: CHF 4,000/ترم غیرمقیم، B2 در ورود → C1، مهلت غیر-EU ۳۰ آوریل</t>
+          <t>بورس – NL Scholarship (سابقاً Holland Scholarship): €5,000 سال اول برای غیر-EEA، از طریق دانشگاه‌های عضو</t>
         </is>
       </c>
       <c r="B46" s="16" t="inlineStr">
         <is>
-          <t>https://www.usi.ch/en/education/master/informatics</t>
+          <t>https://www.mastersportal.com/scholarships/988/holland-scholarship-for-non-eea-international-students.html</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – USI MSc Artificial Intelligence: CHF 4,000/ترم، IELTS 6.5</t>
+          <t>بورس – AAU: ≈ ۱۵ بورس دولتی در سال، معافیت شهریه + DKK 11,225/ماه (۲۰۲۶)، بررسی خودکار (رسمی)</t>
         </is>
       </c>
       <c r="B47" s="16" t="inlineStr">
         <is>
-          <t>https://www.topuniversities.com/universities/usi-universita-della-svizzera-italiana/postgrad/master-science-artificial-intelligence</t>
+          <t>https://www.en.aau.dk/education/apply/master/finance-and-fees</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – swissuniversities: شهریهٔ دانشگاه‌های علوم کاربردی 2026–27 (ZHAW 1,220؛ HSLU 1,300؛ OST 1,500؛ FHNW 1,000–5,000)</t>
+          <t>بورس – ETH Excellence Scholarship &amp; Opportunity Programme: CHF 12,000/ترم + معافیت؛ ۱۰٪ بالای کلاس؛ ۱–۳۰ نوامبر</t>
         </is>
       </c>
       <c r="B48" s="16" t="inlineStr">
         <is>
-          <t>https://www.swissuniversities.ch/en/themen/lehre-studium/information-on-studies/tuition-fees/tuition-fees-at-uas</t>
+          <t>https://ethz.ch/en/studies/financial/scholarships/excellencescholarship.html</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – ZHAW MSE: انگلیسی، 90 ECTS، پروفایل‌های CS/Data Science/Cyber، معدل A/B، مهلت پایان آوریل</t>
+          <t>بورس – USI: بورس‌های Fondazione per le Facoltà di Lugano (CHF 4,000؛ سال اول با معدل ≥ ۸۰/۱۰۰؛ سال دوم بهترینِ هر برنامه) — خبر رسمی USI</t>
         </is>
       </c>
       <c r="B49" s="16" t="inlineStr">
         <is>
-          <t>https://www.zhaw.ch/en/engineering/study/masters-degree-programme</t>
+          <t>https://www.eco.usi.ch/en/feeds/9861</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – HSLU MSc Applied Information &amp; Data Science: C1 (B2 مشروط)، آلمانی لازم نیست، هر کارشناسی</t>
+          <t>بورس – Essex Academic Excellence International Masters Scholarship: جدول کشوری (ایران ۱۴/۲۰ → £4,500؛ جدول ۲۰۲۵–۲۶)</t>
         </is>
       </c>
       <c r="B50" s="16" t="inlineStr">
         <is>
-          <t>https://www.hslu.ch/en/lucerne-school-of-business/degree-programmes/master/applied-information-and-data-science/haeufig-gestellte-fragen/</t>
+          <t>https://www.essex.ac.uk/scholarships</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – Bern: Swiss Joint MSc Computer Science (90 ECTS، انگلیسی، شرط کارشناسی CS)</t>
+          <t>بورس – Teesside Global Excellence Scholarship £2,000 (پیشنهاد تا ۳۰ آوریل؛ رسمی)</t>
         </is>
       </c>
       <c r="B51" s="16" t="inlineStr">
         <is>
-          <t>https://www.philnat.unibe.ch/studies/study_programs/master_s_in_computer_science/index_eng.html</t>
+          <t>https://www.tees.ac.uk/sections/international/global_excellence_scholarship.cfm</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – Bern شهریه از پاییز ۲۰۲۶: CHF 850 + 1,700 اضافهٔ غیرسوئیسی‌ها + 34 + 25 در ترم (رسمی)</t>
+          <t>بورس – Brunel Vice-Chancellor's Postgraduate International Excellence Award £6,000 (حداقل 2:1؛ ودیعهٔ £5,000)</t>
         </is>
       </c>
       <c r="B52" s="16" t="inlineStr">
         <is>
-          <t>https://www.unibe.ch/studies/organizational_matters/renewal_of_semester_registration/fees/index_eng.html</t>
+          <t>https://www.brunel.ac.uk/scholarships</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – Joint MSc CS (Bern/Neuchâtel/Fribourg) FAQ رسمی: بدون آزمون زبان (B2 توصیه)، شرط کارشناسی CS یا معادل با حداکثر ۶۰ ECTS تکمیلی، مهلت‌های دیرهنگام</t>
+          <t>بورس – Northumbria PGT International Scholarship £3,000: فهرست کشوری/ادامه‌تحصیلی‌های داخل UK — ایران نیست</t>
         </is>
       </c>
       <c r="B53" s="16" t="inlineStr">
         <is>
-          <t>https://mcs.unibnf.ch/faq/</t>
+          <t>https://www.mastersportal.com/scholarships/3890/pgt-international-scholarships.html</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – Neuchâtel شهریهٔ خارجی‌ها CHF 790/ترم (رسمی)</t>
+          <t>بورس – Chevening eligibility (رسمی): ۲ سال کار بعد از مدرک کارشناسی + تعهد بازگشت ۲ ساله؛ مهلت ۶ اکتبر ۲۰۲۶</t>
         </is>
       </c>
       <c r="B54" s="16" t="inlineStr">
         <is>
-          <t>https://www.unine.ch/admission/taxes-universitaires/</t>
+          <t>https://www.chevening.org/resource-hub/guidance/eligibility/</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – Neuchâtel مهلت ارشد ۳۰ آوریل؛ خارجی‌ها یک ماه زودتر؛ هزینهٔ پرونده CHF 100 (رسمی)</t>
+          <t>بورس – Deutschlandstipendium €300/ماه (رسمی)</t>
         </is>
       </c>
       <c r="B55" s="16" t="inlineStr">
         <is>
-          <t>https://www.unine.ch/admission/admission-master/delais-et-frais-dinscription-pour-les-masters/</t>
+          <t>https://www.deutschlandstipendium.de/</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – Fribourg شهریهٔ خارجی‌ها CHF 870 + 115 = 985/ترم (رسمی)</t>
+          <t>سوئیس – ETH: تاریخ‌های اپلای ارشد پاییز ۲۰۲۷ (۱–۳۰ نوامبر ۲۰۲۶؛ پاسخ تا پایان مارس؛ شروع ۲۰ سپتامبر ۲۰۲۷)</t>
         </is>
       </c>
       <c r="B56" s="16" t="inlineStr">
         <is>
-          <t>https://www.unifr.ch/studies/en/organisation/administrative-services-unifr-students/university-fees/</t>
+          <t>https://ethz.ch/en/studies/master/application/dates.html</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – Fribourg مهلت ارشد با مدرک خارجی: ویزایی‌ها ۱–۲۸ فوریه، بقیه تا ۳۰ آوریل (رسمی)</t>
+          <t>سوئیس – EPFL: شهریه CHF 2,240/ترم برای خارجی‌های غیرمقیم از پاییز ۲۰۲۵ (CHF 780 برای بقیه)</t>
         </is>
       </c>
       <c r="B57" s="16" t="inlineStr">
         <is>
-          <t>https://www.unifr.ch/studies/en/admission/admission-master/admission-master-foreign.html</t>
+          <t>https://www.epfl.ch/education/studies/en/rules-and-procedures/study-taxes/tuition-fee-other-fees/</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – Basel MSc CS: 90 ECTS، انگلیسی، مهلت ۳۰ آوریل / ۳۰ نوامبر (رسمی)</t>
+          <t>سوئیس – EPFL: پنجره‌های اپلای ارشد (۱۵ دسامبر / ۳۱ مارس؛ یک برنامه در سال)</t>
         </is>
       </c>
       <c r="B58" s="16" t="inlineStr">
         <is>
-          <t>https://dmi.unibas.ch/en/studies/computer-science/masters/</t>
+          <t>https://www.epfl.ch/education/admission/admission-2/master-admission-criteria-application/online-application/</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – Basel شهریه CHF 850/ترم برای همه + CHF 100 هزینهٔ درخواست (Uni Info 2026/27)</t>
+          <t>سوئیس – UZH: شهریه CHF 720 + 100 (خارجی، ارشد) + 59؛ هزینهٔ درخواست CHF 150</t>
         </is>
       </c>
       <c r="B59" s="16" t="inlineStr">
         <is>
-          <t>https://www.unibas.ch/dam/jcr:28672e66-8562-4988-9e38-b1c944ed22bf/COMPUTER%20SCIENCE%202026.2026-02-05-09-53-32.pdf</t>
+          <t>https://www.uzh.ch/en/studies/application/fees.html</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – HSLU MSc Applied Data Science and AI (نام جدید): مهلت ویزایی‌ها ۱ آوریل، CHF 1,300/ترم خارجی، CHF 250 درخواست، 120 ECTS (رسمی)</t>
+          <t>سوئیس – UZH: مهلت ویزایی‌ها ۲۸ فوریه / بدون ویزا ۳۰ آوریل (پاییز)</t>
         </is>
       </c>
       <c r="B60" s="16" t="inlineStr">
         <is>
-          <t>https://www.hslu.ch/en/lucerne-school-of-business/degree-programmes/master/applied-data-science-and-ai/</t>
+          <t>https://www.oec.uzh.ch/en/studies/general/admission/master/faq-master-admission.html</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – USI مهلت‌های 2026/27: غیر-EU ۳۰ آوریل؛ هزینهٔ پرونده CHF 100 برای مدارک خارج از کنوانسیون لیسبون (رسمی)</t>
+          <t>سوئیس – USI MSc Informatics: CHF 4,000/ترم غیرمقیم، B2 در ورود → C1، مهلت غیر-EU ۳۰ آوریل</t>
         </is>
       </c>
       <c r="B61" s="16" t="inlineStr">
         <is>
-          <t>https://www.usi.ch/en/education/master/informatics/application</t>
+          <t>https://www.usi.ch/en/education/master/informatics</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – SEM FAQ: ۶ ماه جست‌وجوی کار برای فارغ‌التحصیلان؛ اولویت داخلی/EU؛ سهمیه</t>
+          <t>سوئیس – USI MSc Artificial Intelligence: CHF 4,000/ترم، IELTS 6.5</t>
         </is>
       </c>
       <c r="B62" s="16" t="inlineStr">
         <is>
-          <t>https://www.sem.admin.ch/sem/en/home/themen/arbeit/faq.html</t>
+          <t>https://www.topuniversities.com/universities/usi-universita-della-svizzera-italiana/postgrad/master-science-artificial-intelligence</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – سهمیهٔ ۲۰۲۶ اتباع غیر-EU: ۴,۵۰۰ B + ۴,۰۰۰ L؛ شرایط FNIA</t>
+          <t>سوئیس – swissuniversities: شهریهٔ دانشگاه‌های علوم کاربردی 2026–27 (ZHAW 1,220؛ HSLU 1,300؛ OST 1,500؛ FHNW 1,000–5,000)</t>
         </is>
       </c>
       <c r="B63" s="16" t="inlineStr">
         <is>
-          <t>https://goldblum.ch/knowledgebase/residence-permit-in-switzerland-obtain/</t>
+          <t>https://www.swissuniversities.ch/en/themen/lehre-studium/information-on-studies/tuition-fees/tuition-fees-at-uas</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – Art. 21(3) FNIA: معافیت از آزمون بازار کار ولی نه از سهمیه؛ طرح 22.067 اجرا نشده</t>
+          <t>سوئیس – ZHAW MSE: انگلیسی، 90 ECTS، پروفایل‌های CS/Data Science/Cyber، معدل A/B، مهلت پایان آوریل</t>
         </is>
       </c>
       <c r="B64" s="16" t="inlineStr">
         <is>
-          <t>https://vshcherbakov.com/2025/06/26/Path-to-working-permit-for-Swiss-graduates/</t>
+          <t>https://www.zhaw.ch/en/engineering/study/masters-degree-programme</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – اقامت تحصیلی ۲۰۲۶: CHF 21,000/سال، ۱۵ ساعت کار بعد از ۶ ماه، پردازش ۸–۱۲ هفته</t>
+          <t>سوئیس – HSLU MSc Applied Information &amp; Data Science: C1 (B2 مشروط)، آلمانی لازم نیست، هر کارشناسی</t>
         </is>
       </c>
       <c r="B65" s="16" t="inlineStr">
         <is>
-          <t>https://www.study-abroad.org/blog/ch-student-visa-guide/</t>
+          <t>https://www.hslu.ch/en/lucerne-school-of-business/degree-programmes/master/applied-information-and-data-science/haeufig-gestellte-fragen/</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – کانتون زوریخ: تمکن فقط در بانک مستقر در سوئیس به نام خودتان یا ضامن مقیم (راهنمای ZHAW)</t>
+          <t>سوئیس – Bern: Swiss Joint MSc Computer Science (90 ECTS، انگلیسی، شرط کارشناسی CS)</t>
         </is>
       </c>
       <c r="B66" s="16" t="inlineStr">
         <is>
-          <t>https://www.zhaw.ch/storage/sml/master/msc-bf-pie-information-for-international-students.pdf</t>
+          <t>https://www.philnat.unibe.ch/studies/study_programs/master_s_in_computer_science/index_eng.html</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – تفاوت کانتون‌ها: Basel CHF 24,000؛ زوریخ حساب سوئیسی</t>
+          <t>سوئیس – Bern شهریه از پاییز ۲۰۲۶: CHF 850 + 1,700 اضافهٔ غیرسوئیسی‌ها + 34 + 25 در ترم (رسمی)</t>
         </is>
       </c>
       <c r="B67" s="16" t="inlineStr">
         <is>
-          <t>https://gradpilot.com/news/switzerland-student-visa-motivation-letter-canton-guide</t>
+          <t>https://www.unibe.ch/studies/organizational_matters/renewal_of_semester_registration/fees/index_eng.html</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – اجازهٔ C: ۱۰ سال برای اتباع کشور ثالث، A2 شفاهی/A1 کتبی؛ ۵ سال با B1</t>
+          <t>سوئیس – Joint MSc CS (Bern/Neuchâtel/Fribourg) FAQ رسمی: بدون آزمون زبان (B2 توصیه)، شرط کارشناسی CS یا معادل با حداکثر ۶۰ ECTS تکمیلی، مهلت‌های دیرهنگام</t>
         </is>
       </c>
       <c r="B68" s="16" t="inlineStr">
         <is>
-          <t>https://relofinder.ch/blog/swiss-c-permit-permanent-residence-2026-guide/</t>
+          <t>https://mcs.unibnf.ch/faq/</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – اجازهٔ C: احتساب سال‌های تحصیل و شرایط ادغام</t>
+          <t>سوئیس – Neuchâtel شهریهٔ خارجی‌ها CHF 790/ترم (رسمی)</t>
         </is>
       </c>
       <c r="B69" s="16" t="inlineStr">
         <is>
-          <t>https://www.richmondchambers.ch/post/swiss-c-permit-eligibility-required-years-of-residence-integration-expectations-and-fast-track-pa</t>
+          <t>https://www.unine.ch/admission/taxes-universitaires/</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – سفارت تهران: ویزای D با وقت قبلی، ویزای C فعلاً نه (۳۰ ژانویه ۲۰۲۶)</t>
+          <t>سوئیس – Neuchâtel مهلت ارشد ۳۰ آوریل؛ خارجی‌ها یک ماه زودتر؛ هزینهٔ پرونده CHF 100 (رسمی)</t>
         </is>
       </c>
       <c r="B70" s="16" t="inlineStr">
         <is>
-          <t>https://www.eda.admin.ch/countries/iran/en/home.html</t>
+          <t>https://www.unine.ch/admission/admission-master/delais-et-frais-dinscription-pour-les-masters/</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – حقوق مهندس نرم‌افزار ۲۰۲۶ (جونیور CHF 85–105k؛ خالص زوریخ)</t>
+          <t>سوئیس – Fribourg شهریهٔ خارجی‌ها CHF 870 + 115 = 985/ترم (رسمی)</t>
         </is>
       </c>
       <c r="B71" s="16" t="inlineStr">
         <is>
-          <t>https://whatisthesalary.com/it-salaries/software-engineer-salary-in-switzerland/</t>
+          <t>https://www.unifr.ch/studies/en/organisation/administrative-services-unifr-students/university-fees/</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – Glassdoor: میانهٔ Junior Software Engineer زوریخ CHF 92k</t>
+          <t>سوئیس – Fribourg مهلت ارشد با مدرک خارجی: ویزایی‌ها ۱–۲۸ فوریه، بقیه تا ۳۰ آوریل (رسمی)</t>
         </is>
       </c>
       <c r="B72" s="16" t="inlineStr">
         <is>
-          <t>https://www.glassdoor.com/Salaries/z%C3%BCrich-junior-software-engineer-salary-SRCH_IL.0,6_IC3297851_KO7,31.htm</t>
+          <t>https://www.unifr.ch/studies/en/admission/admission-master/admission-master-foreign.html</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – بازهٔ حقوق زوریخ ۲۰۲۶ بر اساس نوع کارفرما</t>
+          <t>سوئیس – Basel MSc CS: 90 ECTS، انگلیسی، مهلت ۳۰ آوریل / ۳۰ نوامبر (رسمی)</t>
         </is>
       </c>
       <c r="B73" s="16" t="inlineStr">
         <is>
-          <t>https://upreer.ch/en/salaries/software-engineer-salary-zurich/</t>
+          <t>https://dmi.unibas.ch/en/studies/computer-science/masters/</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – هزینهٔ زندگی زوریخ CHF 2,000–2,200/ماه (UZH)</t>
+          <t>سوئیس – Basel شهریه CHF 850/ترم برای همه + CHF 100 هزینهٔ درخواست (Uni Info 2026/27)</t>
         </is>
       </c>
       <c r="B74" s="16" t="inlineStr">
         <is>
-          <t>https://www.msfinance.uzh.ch/en/studyinginzurich/accommodation.html</t>
+          <t>https://www.unibas.ch/dam/jcr:28672e66-8562-4988-9e38-b1c944ed22bf/COMPUTER%20SCIENCE%202026.2026-02-05-09-53-32.pdf</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – QS 2027: ETH 8، EPFL 22، UZH 98، Basel 150، Bern 191، USI 456، Fribourg 670، ZHAW 851–900</t>
+          <t>سوئیس – HSLU MSc Applied Data Science and AI (نام جدید): مهلت ویزایی‌ها ۱ آوریل، CHF 1,300/ترم خارجی، CHF 250 درخواست، 120 ECTS (رسمی)</t>
         </is>
       </c>
       <c r="B75" s="16" t="inlineStr">
         <is>
-          <t>https://www.iamexpat.ch/education/education-news/eth-zurich-makes-top-universities-world</t>
+          <t>https://www.hslu.ch/en/lucerne-school-of-business/degree-programmes/master/applied-data-science-and-ai/</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – رد ابتکار «سوئیس ۱۰ میلیونی» SVP در ۱۴ ژوئن ۲۰۲۶ (۵۴.۸٪ نه)</t>
+          <t>سوئیس – USI مهلت‌های 2026/27: غیر-EU ۳۰ آوریل؛ هزینهٔ پرونده CHF 100 برای مدارک خارج از کنوانسیون لیسبون (رسمی)</t>
         </is>
       </c>
       <c r="B76" s="16" t="inlineStr">
         <is>
-          <t>https://www.tagesanzeiger.ch/10-millionen-schweiz-resultate-der-svp-initiative-im-ticker-935664202454</t>
+          <t>https://www.usi.ch/en/education/master/informatics/application</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – EP27: کاهش ۷۸ میلیون فرانک بودجهٔ ETH؛ سناریوی چهاربرابر شدن شهریهٔ خارجی‌ها</t>
+          <t>سوئیس – SEM FAQ: ۶ ماه جست‌وجوی کار برای فارغ‌التحصیلان؛ اولویت داخلی/EU؛ سهمیه</t>
         </is>
       </c>
       <c r="B77" s="16" t="inlineStr">
         <is>
-          <t>https://www.efd.admin.ch/de/entlastungspaket-27</t>
+          <t>https://www.sem.admin.ch/sem/en/home/themen/arbeit/faq.html</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – بازار IT ۲۰۲۶: استخدام گزینشی‌تر، بیکاری ≈ ۳.۲٪، کمبود ساختاری ICT</t>
+          <t>سوئیس – سهمیهٔ ۲۰۲۶ اتباع غیر-EU: ۴,۵۰۰ B + ۴,۰۰۰ L؛ شرایط FNIA</t>
         </is>
       </c>
       <c r="B78" s="16" t="inlineStr">
         <is>
-          <t>https://capiwell.ch/swiss-it-labour-market-2026-specialised-skills-slower-growth-and-new-openings-for-start-ups/</t>
+          <t>https://goldblum.ch/knowledgebase/residence-permit-in-switzerland-obtain/</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>نرخ CHF/USD ۲۷ سپتامبر ۲۰۲۶ (1.207)</t>
+          <t>سوئیس – Art. 21(3) FNIA: معافیت از آزمون بازار کار ولی نه از سهمیه؛ طرح 22.067 اجرا نشده</t>
         </is>
       </c>
       <c r="B79" s="16" t="inlineStr">
         <is>
-          <t>https://www.xe.com/en-us/currencyconverter/convert/?Amount=1&amp;From=CHF&amp;To=USD</t>
+          <t>https://vshcherbakov.com/2025/06/26/Path-to-working-permit-for-Swiss-graduates/</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>بریتانیا – Graduate visa ۱۸ ماه (از ژانویه ۲۰۲۷)</t>
+          <t>سوئیس – اقامت تحصیلی ۲۰۲۶: CHF 21,000/سال، ۱۵ ساعت کار بعد از ۶ ماه، پردازش ۸–۱۲ هفته</t>
         </is>
       </c>
       <c r="B80" s="16" t="inlineStr">
         <is>
-          <t>https://students.leeds.ac.uk/visa-information-after-studies/doc/graduate-visas</t>
+          <t>https://www.study-abroad.org/blog/ch-student-visa-guide/</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>بریتانیا – HC 584 (۳ سپتامبر ۲۰۲۶): تمکن £1,570 / £1,203 از ۳۰ نوامبر ۲۰۲۶</t>
+          <t>سوئیس – کانتون زوریخ: تمکن فقط در بانک مستقر در سوئیس به نام خودتان یا ضامن مقیم (راهنمای ZHAW)</t>
         </is>
       </c>
       <c r="B81" s="16" t="inlineStr">
         <is>
-          <t>https://www.gov.uk/government/publications/statement-of-changes-to-the-immigration-rules-hc-584-3-september-2026</t>
+          <t>https://www.zhaw.ch/storage/sml/master/msc-bf-pie-information-for-international-students.pdf</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>بریتانیا – Skilled Worker نرخ شغل SOC 2134 £54,700</t>
+          <t>سوئیس – تفاوت کانتون‌ها: Basel CHF 24,000؛ زوریخ حساب سوئیسی</t>
         </is>
       </c>
       <c r="B82" s="16" t="inlineStr">
         <is>
-          <t>https://withrowan.co.uk/guides/skilled-worker-software-engineers</t>
+          <t>https://gradpilot.com/news/switzerland-student-visa-motivation-letter-canton-guide</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>بریتانیا – Earned Settlement (وضعیت سپتامبر ۲۰۲۶)</t>
+          <t>سوئیس – اجازهٔ C: ۱۰ سال برای اتباع کشور ثالث، A2 شفاهی/A1 کتبی؛ ۵ سال با B1</t>
         </is>
       </c>
       <c r="B83" s="16" t="inlineStr">
         <is>
-          <t>https://www.ukimmigration.law/earned-settlement-ilr-uk-plans/</t>
+          <t>https://relofinder.ch/blog/swiss-c-permit-permanent-residence-2026-guide/</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Teesside MSc Computer Science 2026-27: £17,000، 2:2، IELTS 6.0</t>
+          <t>سوئیس – اجازهٔ C: احتساب سال‌های تحصیل و شرایط ادغام</t>
         </is>
       </c>
       <c r="B84" s="16" t="inlineStr">
         <is>
-          <t>https://www.tees.ac.uk/postgraduate_courses/computing_&amp;_cyber_security/msc_computer_science.cfm</t>
+          <t>https://www.richmondchambers.ch/post/swiss-c-permit-eligibility-required-years-of-residence-integration-expectations-and-fast-track-pa</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Northumbria MSc Advanced Computer Science 2026/27: £21,500، 2:2</t>
+          <t>سوئیس – سفارت تهران: ویزای D با وقت قبلی، ویزای C فعلاً نه (۳۰ ژانویه ۲۰۲۶)</t>
         </is>
       </c>
       <c r="B85" s="16" t="inlineStr">
         <is>
-          <t>https://www.northumbria.ac.uk/study-at-northumbria/courses/msc-advanced-computer-science-dtfava6/</t>
+          <t>https://www.eda.admin.ch/countries/iran/en/home.html</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Leicester MSc Advanced Computer Science سپتامبر ۲۰۲۶: £24,250، 2:1</t>
+          <t>سوئیس – حقوق مهندس نرم‌افزار ۲۰۲۶ (جونیور CHF 85–105k؛ خالص زوریخ)</t>
         </is>
       </c>
       <c r="B86" s="16" t="inlineStr">
         <is>
-          <t>https://le.ac.uk/courses/advanced-computer-science-msc/2026</t>
+          <t>https://whatisthesalary.com/it-salaries/software-engineer-salary-in-switzerland/</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Essex MSc Advanced Computer Science 2026: £24,675، 2:2 (شامل Computer Engineering)</t>
+          <t>سوئیس – Glassdoor: میانهٔ Junior Software Engineer زوریخ CHF 92k</t>
         </is>
       </c>
       <c r="B87" s="16" t="inlineStr">
         <is>
-          <t>https://www.essex.ac.uk/courses/pg00435/1/msc-advanced-computer-science</t>
+          <t>https://www.glassdoor.com/Salaries/z%C3%BCrich-junior-software-engineer-salary-SRCH_IL.0,6_IC3297851_KO7,31.htm</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – York MSc Advanced Computer Science 2026/27: £32,900، 2:2، IELTS 6.5</t>
+          <t>سوئیس – بازهٔ حقوق زوریخ ۲۰۲۶ بر اساس نوع کارفرما</t>
         </is>
       </c>
       <c r="B88" s="16" t="inlineStr">
         <is>
-          <t>https://www.york.ac.uk/study/postgraduate-taught/courses/msc-advanced-computer-science/</t>
+          <t>https://upreer.ch/en/salaries/software-engineer-salary-zurich/</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Chester MSc Advanced Computer Science 2026/27: £15,500 (کف قیمت انگلستان)</t>
+          <t>سوئیس – هزینهٔ زندگی زوریخ CHF 2,000–2,200/ماه (UZH)</t>
         </is>
       </c>
       <c r="B89" s="16" t="inlineStr">
         <is>
-          <t>https://www.chester.ac.uk/study/course-search/advanced-computer-science-msc/</t>
+          <t>https://www.msfinance.uzh.ch/en/studyinginzurich/accommodation.html</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>بریتانیا – Brunel MSc AI 2026/27 £24,795</t>
+          <t>سوئیس – QS 2027: ETH 8، EPFL 22، UZH 98، Basel 150، Bern 191، USI 456، Fribourg 670، ZHAW 851–900</t>
         </is>
       </c>
       <c r="B90" s="16" t="inlineStr">
         <is>
-          <t>https://www.brunel.ac.uk/study/courses/artificial-intelligence-msc</t>
+          <t>https://www.iamexpat.ch/education/education-news/eth-zurich-makes-top-universities-world</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>بریتانیا – عوارض £925 به ازای هر دانشجوی بین‌المللی (انگلستان، از 2028-29)</t>
+          <t>سوئیس – رد ابتکار «سوئیس ۱۰ میلیونی» SVP در ۱۴ ژوئن ۲۰۲۶ (۵۴.۸٪ نه)</t>
         </is>
       </c>
       <c r="B91" s="16" t="inlineStr">
         <is>
-          <t>https://www.researchprofessionalnews.com/rr-news-uk-politics-2025-11-international-levy-to-be-flat-fee-of-925-per-student/</t>
+          <t>https://www.tagesanzeiger.ch/10-millionen-schweiz-resultate-der-svp-initiative-im-ticker-935664202454</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>بریتانیا – وضعیت VAC تهران</t>
+          <t>سوئیس – EP27: کاهش ۷۸ میلیون فرانک بودجهٔ ETH؛ سناریوی چهاربرابر شدن شهریهٔ خارجی‌ها</t>
         </is>
       </c>
       <c r="B92" s="16" t="inlineStr">
         <is>
-          <t>https://livingintehran.com/2026/02/03/tehran-diplomatic-update-recent-embassy-reopenings-current-status-feb-2026/</t>
+          <t>https://www.efd.admin.ch/de/entlastungspaket-27</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>QS WUR 2027 – TU Dresden</t>
+          <t>سوئیس – بازار IT ۲۰۲۶: استخدام گزینشی‌تر، بیکاری ≈ ۳.۲٪، کمبود ساختاری ICT</t>
         </is>
       </c>
       <c r="B93" s="16" t="inlineStr">
         <is>
-          <t>https://tu-dresden.de/tu-dresden/newsportal/news/qs-ranking-2027-tud-gehoert-erneut-zu-den-zehn-besten-universitaeten-deutschlands-und-baut-internationalen-erfolg-weiter-aus</t>
+          <t>https://capiwell.ch/swiss-it-labour-market-2026-specialised-skills-slower-growth-and-new-openings-for-start-ups/</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>QS WUR 2027 – Stuttgart</t>
+          <t>نرخ CHF/USD ۲۷ سپتامبر ۲۰۲۶ (1.207)</t>
         </is>
       </c>
       <c r="B94" s="16" t="inlineStr">
         <is>
-          <t>https://www.uni-stuttgart.de/en/university/news/all/QS-World-University-Rankings-2027-The-University-of-Stuttgart-is-recognized-for-its-strong-research-performance-and-commitment-to-sustainability/</t>
+          <t>https://www.xe.com/en-us/currencyconverter/convert/?Amount=1&amp;From=CHF&amp;To=USD</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>QS WUR 2027 – Newcastle 149</t>
+          <t>بریتانیا – Graduate visa ۱۸ ماه (از ژانویه ۲۰۲۷)</t>
         </is>
       </c>
       <c r="B95" s="16" t="inlineStr">
         <is>
-          <t>https://www.ncl.ac.uk/press/articles/latest/2026/06/qs2027/</t>
+          <t>https://students.leeds.ac.uk/visa-information-after-studies/doc/graduate-visas</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>QS WUR 2027 – York =158</t>
+          <t>بریتانیا – HC 584 (۳ سپتامبر ۲۰۲۶): تمکن £1,570 / £1,203 از ۳۰ نوامبر ۲۰۲۶</t>
         </is>
       </c>
       <c r="B96" s="16" t="inlineStr">
         <is>
-          <t>https://www.york.ac.uk/about/rankings/</t>
+          <t>https://www.gov.uk/government/publications/statement-of-changes-to-the-immigration-rules-hc-584-3-september-2026</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>QS WUR 2027 – Leicester =314</t>
+          <t>بریتانیا – Skilled Worker نرخ شغل SOC 2134 £54,700</t>
         </is>
       </c>
       <c r="B97" s="16" t="inlineStr">
         <is>
-          <t>https://www.topuniversities.com/universities/university-leicester</t>
+          <t>https://withrowan.co.uk/guides/skilled-worker-software-engineers</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>QS WUR 2027 – Essex =438</t>
+          <t>بریتانیا – Earned Settlement (وضعیت سپتامبر ۲۰۲۶)</t>
         </is>
       </c>
       <c r="B98" s="16" t="inlineStr">
         <is>
-          <t>https://www.topuniversities.com/universities/essex-university</t>
+          <t>https://www.ukimmigration.law/earned-settlement-ilr-uk-plans/</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>QS WUR 2027 – Northumbria =528</t>
+          <t>انگلستان – Teesside MSc Computer Science 2026-27: £17,000، 2:2، IELTS 6.0</t>
         </is>
       </c>
       <c r="B99" s="16" t="inlineStr">
         <is>
-          <t>https://www.topuniversities.com/universities/northumbria-university-newcastle</t>
+          <t>https://www.tees.ac.uk/postgraduate_courses/computing_&amp;_cyber_security/msc_computer_science.cfm</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>QS WUR 2027 – Brunel</t>
+          <t>انگلستان – Northumbria MSc Advanced Computer Science 2026/27: £21,500، 2:2</t>
         </is>
       </c>
       <c r="B100" s="16" t="inlineStr">
         <is>
-          <t>https://students.brunel.ac.uk/campus-news/brunel-climbs-global-qs-rankings-after-strong-year-for-research-and-graduate-outcomes</t>
+          <t>https://www.northumbria.ac.uk/study-at-northumbria/courses/msc-advanced-computer-science-dtfava6/</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>QS WUR 2027 – سایر</t>
+          <t>انگلستان – Leicester MSc Advanced Computer Science سپتامبر ۲۰۲۶: £24,250، 2:1</t>
         </is>
       </c>
       <c r="B101" s="16" t="inlineStr">
         <is>
-          <t>https://www.topuniversities.com/world-university-rankings</t>
+          <t>https://le.ac.uk/courses/advanced-computer-science-msc/2026</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>حداقل دستمزد ۲۰۲۶ هلند (€14.71)</t>
+          <t>انگلستان – Essex MSc Advanced Computer Science 2026: £24,675، 2:2 (شامل Computer Engineering)</t>
         </is>
       </c>
       <c r="B102" s="16" t="inlineStr">
         <is>
-          <t>https://arlettipartners.com/new-increase-in-the-dutch-minimum-hourly-wage-from-january-1st-2026/</t>
+          <t>https://www.essex.ac.uk/courses/pg00435/1/msc-advanced-computer-science</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>نرخ ارز (xe.com، ۲۷ سپتامبر ۲۰۲۶)</t>
+          <t>انگلستان – York MSc Advanced Computer Science 2026/27: £32,900، 2:2، IELTS 6.5</t>
         </is>
       </c>
       <c r="B103" s="16" t="inlineStr">
         <is>
-          <t>https://www.xe.com/</t>
+          <t>https://www.york.ac.uk/study/postgraduate-taught/courses/msc-advanced-computer-science/</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>بازار کار – LinkedIn/WEF ژانویه ۲۰۲۶: ۱.۳ میلیون شغل جدید AI؛ AI Engineer سریع‌ترین‌رشد</t>
+          <t>انگلستان – Chester MSc Advanced Computer Science 2026/27: £15,500 (کف قیمت انگلستان)</t>
         </is>
       </c>
       <c r="B104" s="16" t="inlineStr">
         <is>
-          <t>https://www.weforum.org/stories/jobs-and-the-future-of-work/ai-has-already-added-1-3-million-new-jobs-according-to-linkedin-data/</t>
+          <t>https://www.chester.ac.uk/study/course-search/advanced-computer-science-msc/</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t>بازار کار – Bitkom 2025: ۱۰۹ هزار جای خالی IT در آلمان، ۷.۷ ماه زمان پرکردن</t>
+          <t>بریتانیا – Brunel MSc AI 2026/27 £24,795</t>
         </is>
       </c>
       <c r="B105" s="16" t="inlineStr">
         <is>
-          <t>https://www.bitkom.org/Bitkom/Publikationen/Der-Arbeitsmarkt-fuer-IT-Fachkraefte</t>
+          <t>https://www.brunel.ac.uk/study/courses/artificial-intelligence-msc</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
         <is>
-          <t>بازار کار – ISC2 Cybersecurity Workforce Study 2024/2025 (حذف عدد کمبود؛ کمبود بودجه دلیل اول؛ ۳۱٪ تیم‌ها بدون جونیور)</t>
+          <t>بریتانیا – عوارض £925 به ازای هر دانشجوی بین‌المللی (انگلستان، از 2028-29)</t>
         </is>
       </c>
       <c r="B106" s="16" t="inlineStr">
         <is>
-          <t>https://www.isc2.org/research</t>
+          <t>https://www.researchprofessionalnews.com/rr-news-uk-politics-2025-11-international-levy-to-be-flat-fee-of-925-per-student/</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
         <is>
-          <t>بازار کار – اخراج‌های صنعت بازی ۲۰۲۲–۲۰۲۶ (≈۴۵ هزار؛ افت حقوق Unity)</t>
+          <t>بریتانیا – وضعیت VAC تهران</t>
         </is>
       </c>
       <c r="B107" s="16" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/2022%E2%80%932026_video_game_industry_layoffs</t>
+          <t>https://livingintehran.com/2026/02/03/tehran-diplomatic-update-recent-embassy-reopenings-current-status-feb-2026/</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
         <is>
-          <t>بازار کار – آگهی‌های UX/UXR (Indeed تا Q4 2025)</t>
+          <t>QS WUR 2027 – TU Dresden</t>
         </is>
       </c>
       <c r="B108" s="16" t="inlineStr">
         <is>
-          <t>https://www.thevoiceofuser.com/everyone-knows-the-uxr-hiring-market-is-bad-how-bad-is-it-though/</t>
+          <t>https://tu-dresden.de/tu-dresden/newsportal/news/qs-ranking-2027-tud-gehoert-erneut-zu-den-zehn-besten-universitaeten-deutschlands-und-baut-internationalen-erfolg-weiter-aus</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
         <is>
-          <t>بازار کار – اشباع جونیور علم داده ۲۰۲۶</t>
+          <t>QS WUR 2027 – Stuttgart</t>
         </is>
       </c>
       <c r="B109" s="16" t="inlineStr">
         <is>
-          <t>https://research.com/advice/are-too-many-students-choosing-data-science-oversaturation-competition-hiring-reality</t>
+          <t>https://www.uni-stuttgart.de/en/university/news/all/QS-World-University-Rankings-2027-The-University-of-Stuttgart-is-recognized-for-its-strong-research-performance-and-commitment-to-sustainability/</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t>آلمان – Saarland MSc Cybersecurity (C1، بدون شهریه)</t>
+          <t>QS WUR 2027 – Newcastle 149</t>
         </is>
       </c>
       <c r="B110" s="16" t="inlineStr">
         <is>
-          <t>https://www.uni-saarland.de/en/study/programmes/master/cybersecurity.html</t>
+          <t>https://www.ncl.ac.uk/press/articles/latest/2026/06/qs2027/</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
         <is>
-          <t>آلمان – Passau MSc AI Engineering (B2، معدل ≤ 2.7، A1 آلمانی سال اول)</t>
+          <t>QS WUR 2027 – York =158</t>
         </is>
       </c>
       <c r="B111" s="16" t="inlineStr">
         <is>
-          <t>https://www.uni-passau.de/en/msc-ai-eng</t>
+          <t>https://www.york.ac.uk/about/rankings/</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
         <is>
-          <t>آلمان – Cologne Game Lab MA Game Development &amp; Research (€2,500/ترم غیر-EU)</t>
+          <t>QS WUR 2027 – Leicester =314</t>
         </is>
       </c>
       <c r="B112" s="16" t="inlineStr">
         <is>
-          <t>https://colognegamelab.de/study-programs/post-graduate-programs/game-development-research-ma/faqs/</t>
+          <t>https://www.topuniversities.com/universities/university-leicester</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
         <is>
-          <t>آلمان – Siegen MSc HCI (DAAD)</t>
+          <t>QS WUR 2027 – Essex =438</t>
         </is>
       </c>
       <c r="B113" s="16" t="inlineStr">
         <is>
-          <t>https://www2.daad.de/deutschland/studienangebote/international-programmes/en/detail/4686/</t>
+          <t>https://www.topuniversities.com/universities/essex-university</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
         <is>
-          <t>آلمان – H-BRS MSc Autonomous Systems (B2+)</t>
+          <t>QS WUR 2027 – Northumbria =528</t>
         </is>
       </c>
       <c r="B114" s="16" t="inlineStr">
         <is>
-          <t>https://www.h-brs.de/en/inf/admission-application-master-autonomous-systems</t>
+          <t>https://www.topuniversities.com/universities/northumbria-university-newcastle</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
         <is>
-          <t>آلمان – RWTH MSc Software Systems Engineering</t>
+          <t>QS WUR 2027 – Brunel</t>
         </is>
       </c>
       <c r="B115" s="16" t="inlineStr">
         <is>
-          <t>https://sc.informatik.rwth-aachen.de/en/studium/master/sse/</t>
+          <t>https://students.brunel.ac.uk/campus-news/brunel-climbs-global-qs-rankings-after-strong-year-for-research-and-graduate-outcomes</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
         <is>
-          <t>آلمان – Tübingen MSc Machine Learning (IELTS 7، €1,500/ترم)</t>
+          <t>QS WUR 2027 – سایر</t>
         </is>
       </c>
       <c r="B116" s="16" t="inlineStr">
         <is>
-          <t>https://uni-tuebingen.de/fakultaeten/mathematisch-naturwissenschaftliche-fakultaet/fachbereiche/informatik/studium/studierende/lehre-studienorganisation/studiengaenge/machine-learning/admission-and-application/</t>
+          <t>https://www.topuniversities.com/world-university-rankings</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
         <is>
-          <t>آلمان – TUM Informatics: €6,000 در ترم برای غیر-EU</t>
+          <t>حداقل دستمزد ۲۰۲۶ هلند (€14.71)</t>
         </is>
       </c>
       <c r="B117" s="16" t="inlineStr">
         <is>
-          <t>https://www.tum.de/en/studies/degree-programs/detail/informatics-master-of-science-msc</t>
+          <t>https://arlettipartners.com/new-increase-in-the-dutch-minimum-hourly-wage-from-january-1st-2026/</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
         <is>
-          <t>آلمان – FAU Autonomy Technologies (B2، IELTS 6.0)</t>
+          <t>نرخ ارز (xe.com، ۲۷ سپتامبر ۲۰۲۶)</t>
         </is>
       </c>
       <c r="B118" s="16" t="inlineStr">
         <is>
-          <t>https://www.fau.eu/degree-program/autonomy-technologies-m-sc/</t>
+          <t>https://www.xe.com/</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
         <is>
-          <t>هلند – Twente Embedded Systems 2026/27: €21,700</t>
+          <t>بازار کار – LinkedIn/WEF ژانویه ۲۰۲۶: ۱.۳ میلیون شغل جدید AI؛ AI Engineer سریع‌ترین‌رشد</t>
         </is>
       </c>
       <c r="B119" s="16" t="inlineStr">
         <is>
-          <t>https://www.utwente.nl/en/education/master/programmes/embedded-systems/finance/</t>
+          <t>https://www.weforum.org/stories/jobs-and-the-future-of-work/ai-has-already-added-1-3-million-new-jobs-according-to-linkedin-data/</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
         <is>
-          <t>هلند – Leiden CS 2026/27: €22,500</t>
+          <t>بازار کار – Bitkom 2025: ۱۰۹ هزار جای خالی IT در آلمان، ۷.۷ ماه زمان پرکردن</t>
         </is>
       </c>
       <c r="B120" s="16" t="inlineStr">
         <is>
-          <t>https://www.universiteitleiden.nl/en/education/study-programmes/master/computer-science/artificial-intelligence/admission-and-application/tuition-fees</t>
+          <t>https://www.bitkom.org/Bitkom/Publikationen/Der-Arbeitsmarkt-fuer-IT-Fachkraefte</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
         <is>
-          <t>هلند – Groningen AI 2026/27: €24,900</t>
+          <t>بازار کار – ISC2 Cybersecurity Workforce Study 2024/2025 (حذف عدد کمبود؛ کمبود بودجه دلیل اول؛ ۳۱٪ تیم‌ها بدون جونیور)</t>
         </is>
       </c>
       <c r="B121" s="16" t="inlineStr">
         <is>
-          <t>https://www.rug.nl/masters/artificial-intelligence/?lang=en</t>
+          <t>https://www.isc2.org/research</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
         <is>
-          <t>هلند – Utrecht Game &amp; Media Technology 2026/27: €25,306</t>
+          <t>بازار کار – اخراج‌های صنعت بازی ۲۰۲۲–۲۰۲۶ (≈۴۵ هزار؛ افت حقوق Unity)</t>
         </is>
       </c>
       <c r="B122" s="16" t="inlineStr">
         <is>
-          <t>https://www.uu.nl/en/masters/game-and-media-technology</t>
+          <t>https://en.wikipedia.org/wiki/2022%E2%80%932026_video_game_industry_layoffs</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
         <is>
-          <t>هلند – QS 2027 فهرست دانشگاه‌های هلند</t>
+          <t>بازار کار – آگهی‌های UX/UXR (Indeed تا Q4 2025)</t>
         </is>
       </c>
       <c r="B123" s="16" t="inlineStr">
         <is>
-          <t>https://dub.uu.nl/en/news/dutch-universities-fall-global-qs-rankings</t>
+          <t>https://www.thevoiceofuser.com/everyone-knows-the-uxr-hiring-market-is-bad-how-bad-is-it-though/</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="4" t="inlineStr">
         <is>
-          <t>سوئد – Gothenburg Game Design &amp; Technology: SEK 290,000 کل</t>
+          <t>بازار کار – اشباع جونیور علم داده ۲۰۲۶</t>
         </is>
       </c>
       <c r="B124" s="16" t="inlineStr">
         <is>
-          <t>https://www.gu.se/en/study-gothenburg/game-design-technology-masters-programme-n2gdt</t>
+          <t>https://research.com/advice/are-too-many-students-choosing-data-science-oversaturation-competition-hiring-reality</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
         <is>
-          <t>سوئد – KTH Machine Learning: ≈ SEK 180,000–190,000 (کل دوره 360k طبق راهنمای ۲۰۲۶؛ kth.se رقم را فقط در سامانه نشان می‌دهد)</t>
+          <t>آلمان – Saarland MSc Cybersecurity (C1، بدون شهریه)</t>
         </is>
       </c>
       <c r="B125" s="16" t="inlineStr">
         <is>
-          <t>https://www.kth.se/en/studies/master/machine-learning</t>
+          <t>https://www.uni-saarland.de/en/study/programmes/master/cybersecurity.html</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="4" t="inlineStr">
         <is>
-          <t>سوئد – Umeå AI: SEK 152,300</t>
+          <t>آلمان – Passau MSc AI Engineering (B2، معدل ≤ 2.7، A1 آلمانی سال اول)</t>
         </is>
       </c>
       <c r="B126" s="16" t="inlineStr">
         <is>
-          <t>https://www.umu.se/en/education/master/masters-programme-in-artificial-intelligence/</t>
+          <t>https://www.uni-passau.de/en/msc-ai-eng</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
         <is>
-          <t>سوئد – QS 2027 فهرست دانشگاه‌های سوئد</t>
+          <t>آلمان – Cologne Game Lab MA Game Development &amp; Research (€2,500/ترم غیر-EU)</t>
         </is>
       </c>
       <c r="B127" s="16" t="inlineStr">
         <is>
-          <t>https://www.study.eu/best-universities/sweden</t>
+          <t>https://colognegamelab.de/study-programs/post-graduate-programs/game-development-research-ma/faqs/</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="4" t="inlineStr">
         <is>
-          <t>دانمارک – ITU شهریهٔ رسمی ورودی ۲۰۲۶: €8,250 در ترم = €16,500 در سال (رقم قدیمی €6,700 منسوخ)</t>
+          <t>آلمان – Siegen MSc HCI (DAAD)</t>
         </is>
       </c>
       <c r="B128" s="16" t="inlineStr">
         <is>
-          <t>https://en.itu.dk/Programmes/MSc-Programmes/Applying-to-a-MSc-programme/Non-EU-EOES</t>
+          <t>https://www2.daad.de/deutschland/studienangebote/international-programmes/en/detail/4686/</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
         <is>
-          <t>دانمارک – AAU Cyber Security / Medialogy €7,455 در ترم</t>
+          <t>آلمان – H-BRS MSc Autonomous Systems (B2+)</t>
         </is>
       </c>
       <c r="B129" s="16" t="inlineStr">
         <is>
-          <t>https://studyindenmark.dk/portal/aalborg-university-aau/copenhagen/cyber-security-msc-in-engineering</t>
+          <t>https://www.h-brs.de/en/inf/admission-application-master-autonomous-systems</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="4" t="inlineStr">
         <is>
-          <t>دانمارک – DTU €15,000 (Human-Centered AI / Autonomous Systems)</t>
+          <t>آلمان – RWTH MSc Software Systems Engineering</t>
         </is>
       </c>
       <c r="B130" s="16" t="inlineStr">
         <is>
-          <t>https://www.dtu.dk/english/education/graduate/msc-programmes/autonomous-systems/prerequisites</t>
+          <t>https://sc.informatik.rwth-aachen.de/en/studium/master/sse/</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
         <is>
-          <t>دانمارک – Aarhus CS €17,300</t>
+          <t>آلمان – Tübingen MSc Machine Learning (IELTS 7، €1,500/ترم)</t>
         </is>
       </c>
       <c r="B131" s="16" t="inlineStr">
         <is>
-          <t>https://masters.au.dk/computerscience</t>
+          <t>https://uni-tuebingen.de/fakultaeten/mathematisch-naturwissenschaftliche-fakultaet/fachbereiche/informatik/studium/studierende/lehre-studienorganisation/studiengaenge/machine-learning/admission-and-application/</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="4" t="inlineStr">
         <is>
-          <t>دانمارک – QS 2027 فهرست دانشگاه‌های دانمارک</t>
+          <t>آلمان – TUM Informatics: €6,000 در ترم برای غیر-EU</t>
         </is>
       </c>
       <c r="B132" s="16" t="inlineStr">
         <is>
-          <t>https://leapscholar.com/blog/top-universities-in-denmark/</t>
+          <t>https://www.tum.de/en/studies/degree-programs/detail/informatics-master-of-science-msc</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Goldsmiths MSc Computer Games Programming £22,000</t>
+          <t>آلمان – FAU Autonomy Technologies (B2، IELTS 6.0)</t>
         </is>
       </c>
       <c r="B133" s="16" t="inlineStr">
         <is>
-          <t>https://www.gold.ac.uk/pg/msc-computer-games-programming/</t>
+          <t>https://www.fau.eu/degree-program/autonomy-technologies-m-sc/</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Royal Holloway MSc Information &amp; Cyber Security £25,500</t>
+          <t>هلند – Twente Embedded Systems 2026/27: €21,700</t>
         </is>
       </c>
       <c r="B134" s="16" t="inlineStr">
         <is>
-          <t>https://www.royalholloway.ac.uk/studying-here/postgraduate/information-security/information-and-cyber-security/</t>
+          <t>https://www.utwente.nl/en/education/master/programmes/embedded-systems/finance/</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Kent MSc Cyber Security (NCSC)</t>
+          <t>هلند – Leiden CS 2026/27: €22,500</t>
         </is>
       </c>
       <c r="B135" s="16" t="inlineStr">
         <is>
-          <t>https://www.kent.ac.uk/courses/postgraduate/1225/cyber-security</t>
+          <t>https://www.universiteitleiden.nl/en/education/study-programmes/master/computer-science/artificial-intelligence/admission-and-application/tuition-fees</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – MMU MSc Cyber Security £21,000</t>
+          <t>هلند – Groningen AI 2026/27: €24,900</t>
         </is>
       </c>
       <c r="B136" s="16" t="inlineStr">
         <is>
-          <t>https://www.mmu.ac.uk/study/postgraduate/course/msc-cyber-security</t>
+          <t>https://www.rug.nl/masters/artificial-intelligence/?lang=en</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – York MSc Human-Centred Interactive Technologies £32,900</t>
+          <t>هلند – Utrecht Game &amp; Media Technology 2026/27: €25,306</t>
         </is>
       </c>
       <c r="B137" s="16" t="inlineStr">
         <is>
-          <t>https://www.york.ac.uk/study/postgraduate-taught/courses/msc-human-centred-interactive-technologies/</t>
+          <t>https://www.uu.nl/en/masters/game-and-media-technology</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Lancaster MSc Cyber Security £30,000</t>
+          <t>هلند – QS 2027 فهرست دانشگاه‌های هلند</t>
         </is>
       </c>
       <c r="B138" s="16" t="inlineStr">
         <is>
-          <t>https://www.lancaster.ac.uk/study/postgraduate/postgraduate-courses/cyber-security-msc/2026/</t>
+          <t>https://dub.uu.nl/en/news/dutch-universities-fall-global-qs-rankings</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – NTU QS 2027 =639</t>
+          <t>سوئد – Gothenburg Game Design &amp; Technology: SEK 290,000 کل</t>
         </is>
       </c>
       <c r="B139" s="16" t="inlineStr">
         <is>
-          <t>https://collegedunia.com/uk/university/862-nottingham-trent-university-nottingham/ranking</t>
+          <t>https://www.gu.se/en/study-gothenburg/game-design-technology-masters-programme-n2gdt</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="4" t="inlineStr">
         <is>
-          <t>آلمان – FAU: شهریهٔ غیر-EU از ترم تابستان ۲۰۲۷ (AI/CS €4,000، Autonomy Tech €2,000 در ترم؛ BayHIG §13)</t>
+          <t>سوئد – KTH Machine Learning: ≈ SEK 180,000–190,000 (کل دوره 360k طبق راهنمای ۲۰۲۶؛ kth.se رقم را فقط در سامانه نشان می‌دهد)</t>
         </is>
       </c>
       <c r="B140" s="16" t="inlineStr">
         <is>
-          <t>https://www.fau.eu/studying/international-students/application-and-enrollment-for-international-applicants/tuition-fees-for-students-from-non-eu-states/</t>
+          <t>https://www.kth.se/en/studies/master/machine-learning</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
         <is>
-          <t>آلمان – Passau: «فعلاً» بدون شهریه برای غیر-EU (اعلام رسمی)</t>
+          <t>سوئد – Umeå AI: SEK 152,300</t>
         </is>
       </c>
       <c r="B141" s="16" t="inlineStr">
         <is>
-          <t>https://www.uni-passau.de/en/study/news/news/no-tuition-fees-for-international-students-at-the-university-of-passau</t>
+          <t>https://www.umu.se/en/education/master/masters-programme-in-artificial-intelligence/</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
         <is>
-          <t>دانمارک – Aarhus نرخ رسمی 2026/27: Computer Science / Data Science / Computer Engineering €17,300</t>
+          <t>سوئد – QS 2027 فهرست دانشگاه‌های سوئد</t>
         </is>
       </c>
       <c r="B142" s="16" t="inlineStr">
         <is>
-          <t>https://masters.au.dk/tuitionfees/current-tuition-fee-rates</t>
+          <t>https://www.study.eu/best-universities/sweden</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
         <is>
-          <t>دانمارک – AAU Computer Science (IT): شرط رسمی ≥ ۱۵۰ ECTS دروس CS؛ معیار رتبه‌بندی ۲۰۲۷ شامل سابقهٔ کار</t>
+          <t>دانمارک – ITU شهریهٔ رسمی ورودی ۲۰۲۶: €8,250 در ترم = €16,500 در سال (رقم قدیمی €6,700 منسوخ)</t>
         </is>
       </c>
       <c r="B143" s="16" t="inlineStr">
         <is>
-          <t>https://www.en.aau.dk/education/master/computer-science-it</t>
+          <t>https://en.itu.dk/Programmes/MSc-Programmes/Applying-to-a-MSc-programme/Non-EU-EOES</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="4" t="inlineStr">
         <is>
-          <t>سوئد – Chalmers شهریهٔ استاندارد 2026/27 ≈ SEK 175,000 (collegedunia به نقل از صفحهٔ شهریهٔ Chalmers)</t>
+          <t>دانمارک – AAU Cyber Security / Medialogy €7,455 در ترم</t>
         </is>
       </c>
       <c r="B144" s="16" t="inlineStr">
         <is>
-          <t>https://collegedunia.com/sweden/university/769-chalmers-university-of-technology-gothenburg/programs?stream_id=48&amp;degree_type=Master</t>
+          <t>https://studyindenmark.dk/portal/aalborg-university-aau/copenhagen/cyber-security-msc-in-engineering</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Surrey MSc Cyber Security ورودی ۲۰۲۷: £25,900 (فوریه) / £26,900 (سپتامبر)</t>
+          <t>دانمارک – DTU €15,000 (Human-Centered AI / Autonomous Systems)</t>
         </is>
       </c>
       <c r="B145" s="16" t="inlineStr">
         <is>
-          <t>https://www.surrey.ac.uk/postgraduate/cyber-security-msc</t>
+          <t>https://www.dtu.dk/english/education/graduate/msc-programmes/autonomous-systems/prerequisites</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Newcastle MSc Computer Game Engineering £32,300، شرط 2:2 (QS TopUniversities)</t>
+          <t>دانمارک – Aarhus CS €17,300</t>
         </is>
       </c>
       <c r="B146" s="16" t="inlineStr">
         <is>
-          <t>https://www.topuniversities.com/universities/newcastle-university/postgrad/msc-computer-game-engineering</t>
+          <t>https://masters.au.dk/computerscience</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
         <is>
-          <t>هلند – TU/e شهریهٔ رسمی 2026/27 €21,700 (2027/28: €22,400)</t>
+          <t>دانمارک – QS 2027 فهرست دانشگاه‌های دانمارک</t>
         </is>
       </c>
       <c r="B147" s="16" t="inlineStr">
         <is>
-          <t>https://www.tue.nl/en/education/become-a-tue-student/tuition-fees</t>
+          <t>https://leapscholar.com/blog/top-universities-in-denmark/</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
         <is>
-          <t>ایران – توقف برگزاری IELTS در ایران از ۳۱ ژانویه ۲۰۲۶ (اعلام IDP)</t>
+          <t>انگلستان – Goldsmiths MSc Computer Games Programming £22,000</t>
         </is>
       </c>
       <c r="B148" s="16" t="inlineStr">
         <is>
-          <t>https://wanaen.com/ielts-testing-to-be-suspended-in-iran/</t>
+          <t>https://www.gold.ac.uk/pg/msc-computer-games-programming/</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
         <is>
-          <t>ایران – وضعیت IELTS شهریور ۱۴۰۵: در ایران برگزار نمی‌شود؛ آزمون در کشور دیگر</t>
+          <t>انگلستان – Royal Holloway MSc Information &amp; Cyber Security £25,500</t>
         </is>
       </c>
       <c r="B149" s="16" t="inlineStr">
         <is>
-          <t>https://www.jahantahsil.com/%D8%A2%D8%B2%D9%85%D9%88%D9%86-%D8%A2%DB%8C%D9%84%D8%AA%D8%B3-ielts-%DA%86%DB%8C%D8%B3%D8%AA-%D9%88-%DA%A9%D8%AC%D8%A7-%D8%A8%D8%B1%DA%AF%D8%B2%D8%A7%D8%B1-%D9%85%DB%8C%D8%B4%D9%88%D8%AF/</t>
+          <t>https://www.royalholloway.ac.uk/studying-here/postgraduate/information-security/information-and-cyber-security/</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
         <is>
-          <t>ایران – توقف TOEFL در ایران (وضعیت شهریور ۱۴۰۵)</t>
+          <t>انگلستان – Kent MSc Cyber Security (NCSC)</t>
         </is>
       </c>
       <c r="B150" s="16" t="inlineStr">
         <is>
-          <t>https://zandienglish.ir/toefl-in-iran/</t>
+          <t>https://www.kent.ac.uk/courses/postgraduate/1225/cyber-security</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
         <is>
-          <t>ایران – وثیقهٔ خروج تحصیلی مشمولان ۲۰۰ میلیون تومان (سامانهٔ سخا، تیر ۱۴۰۵)</t>
+          <t>انگلستان – MMU MSc Cyber Security £21,000</t>
         </is>
       </c>
       <c r="B151" s="16" t="inlineStr">
         <is>
-          <t>https://www.zoomit.ir/iran-news/464136-exit-permit-bond-sakha-1405/</t>
+          <t>https://www.mmu.ac.uk/study/postgraduate/course/msc-cyber-security</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="4" t="inlineStr">
         <is>
-          <t>سوئد – تاریخ‌های کلیدی ورودی پاییز ۲۰۲۷ (۱۶ اکتبر – ۱۵ ژانویه؛ مدارک ۱ فوریه؛ دور دوم ۱۵ آوریل)</t>
+          <t>انگلستان – York MSc Human-Centred Interactive Technologies £32,900</t>
         </is>
       </c>
       <c r="B152" s="16" t="inlineStr">
         <is>
-          <t>https://www.umu.se/en/education/application-and-admission/key-dates-and-deadlines/</t>
+          <t>https://www.york.ac.uk/study/postgraduate-taught/courses/msc-human-centred-interactive-technologies/</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
         <is>
-          <t>آلمان – Stuttgart MSc CS: بازهٔ اپلای ترم زمستان ۱۵ نوامبر – ۱۵ ژانویه؛ انگلیسی C1</t>
+          <t>انگلستان – Lancaster MSc Cyber Security £30,000</t>
         </is>
       </c>
       <c r="B153" s="16" t="inlineStr">
         <is>
-          <t>https://www.uni-stuttgart.de/en/study/study-programs/Computer-Science-M.Sc.-00001/</t>
+          <t>https://www.lancaster.ac.uk/study/postgraduate/postgraduate-courses/cyber-security-msc/2026/</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
         <is>
-          <t>آلمان – Passau: بازهٔ اپلای AI Engineering ۱ آوریل – ۳۱ می</t>
+          <t>انگلستان – NTU QS 2027 =639</t>
         </is>
       </c>
       <c r="B154" s="16" t="inlineStr">
         <is>
-          <t>https://www.uni-passau.de/en/apply/apply-with-intl-qualifications</t>
+          <t>https://collegedunia.com/uk/university/862-nottingham-trent-university-nottingham/ranking</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
         <is>
-          <t>دانمارک – AAU: مهلت شهریه‌پردازها ۱۵ ژانویه (EU: ۱ مارس)؛ پورتال از اواسط دسامبر</t>
+          <t>آلمان – FAU: شهریهٔ غیر-EU از ترم تابستان ۲۰۲۷ (AI/CS €4,000، Autonomy Tech €2,000 در ترم؛ BayHIG §13)</t>
         </is>
       </c>
       <c r="B155" s="16" t="inlineStr">
         <is>
-          <t>https://www.en.aau.dk/education/apply/master/how-and-when-to-apply</t>
+          <t>https://www.fau.eu/studying/international-students/application-and-enrollment-for-international-applicants/tuition-fees-for-students-from-non-eu-states/</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
         <is>
-          <t>دانمارک – SDU Computer Science: مهلت غیر-EU ۱ فوریه؛ شهریه یک سال پیش‌پرداخت</t>
+          <t>آلمان – Passau: «فعلاً» بدون شهریه برای غیر-EU (اعلام رسمی)</t>
         </is>
       </c>
       <c r="B156" s="16" t="inlineStr">
         <is>
-          <t>https://www.sdu.dk/en/uddannelse/kandidat/datalogi</t>
+          <t>https://www.uni-passau.de/en/study/news/news/no-tuition-fees-for-international-students-at-the-university-of-passau</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
         <is>
-          <t>هلند – Radboud: مهلت غیر-EU ۱ آوریل، بورس ۳۱ ژانویه، ثبت‌نام ۱ ژوئن</t>
+          <t>دانمارک – Aarhus نرخ رسمی 2026/27: Computer Science / Data Science / Computer Engineering €17,300</t>
         </is>
       </c>
       <c r="B157" s="16" t="inlineStr">
         <is>
-          <t>https://www.ru.nl/en/education/application-and-admission/application-procedure-masters/deadlines</t>
+          <t>https://masters.au.dk/tuitionfees/current-tuition-fee-rates</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
         <is>
+          <t>دانمارک – AAU Computer Science (IT): شرط رسمی ≥ ۱۵۰ ECTS دروس CS؛ معیار رتبه‌بندی ۲۰۲۷ شامل سابقهٔ کار</t>
+        </is>
+      </c>
+      <c r="B158" s="16" t="inlineStr">
+        <is>
+          <t>https://www.en.aau.dk/education/master/computer-science-it</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="4" t="inlineStr">
+        <is>
+          <t>سوئد – Chalmers شهریهٔ استاندارد 2026/27 ≈ SEK 175,000 (collegedunia به نقل از صفحهٔ شهریهٔ Chalmers)</t>
+        </is>
+      </c>
+      <c r="B159" s="16" t="inlineStr">
+        <is>
+          <t>https://collegedunia.com/sweden/university/769-chalmers-university-of-technology-gothenburg/programs?stream_id=48&amp;degree_type=Master</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="4" t="inlineStr">
+        <is>
+          <t>انگلستان – Surrey MSc Cyber Security ورودی ۲۰۲۷: £25,900 (فوریه) / £26,900 (سپتامبر)</t>
+        </is>
+      </c>
+      <c r="B160" s="16" t="inlineStr">
+        <is>
+          <t>https://www.surrey.ac.uk/postgraduate/cyber-security-msc</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="4" t="inlineStr">
+        <is>
+          <t>انگلستان – Newcastle MSc Computer Game Engineering £32,300، شرط 2:2 (QS TopUniversities)</t>
+        </is>
+      </c>
+      <c r="B161" s="16" t="inlineStr">
+        <is>
+          <t>https://www.topuniversities.com/universities/newcastle-university/postgrad/msc-computer-game-engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="4" t="inlineStr">
+        <is>
+          <t>هلند – TU/e شهریهٔ رسمی 2026/27 €21,700 (2027/28: €22,400)</t>
+        </is>
+      </c>
+      <c r="B162" s="16" t="inlineStr">
+        <is>
+          <t>https://www.tue.nl/en/education/become-a-tue-student/tuition-fees</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="4" t="inlineStr">
+        <is>
+          <t>ایران – توقف برگزاری IELTS در ایران از ۳۱ ژانویه ۲۰۲۶ (اعلام IDP)</t>
+        </is>
+      </c>
+      <c r="B163" s="16" t="inlineStr">
+        <is>
+          <t>https://wanaen.com/ielts-testing-to-be-suspended-in-iran/</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="4" t="inlineStr">
+        <is>
+          <t>ایران – وضعیت IELTS شهریور ۱۴۰۵: در ایران برگزار نمی‌شود؛ آزمون در کشور دیگر</t>
+        </is>
+      </c>
+      <c r="B164" s="16" t="inlineStr">
+        <is>
+          <t>https://www.jahantahsil.com/%D8%A2%D8%B2%D9%85%D9%88%D9%86-%D8%A2%DB%8C%D9%84%D8%AA%D8%B3-ielts-%DA%86%DB%8C%D8%B3%D8%AA-%D9%88-%DA%A9%D8%AC%D8%A7-%D8%A8%D8%B1%DA%AF%D8%B2%D8%A7%D8%B1-%D9%85%DB%8C%D8%B4%D9%88%D8%AF/</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="4" t="inlineStr">
+        <is>
+          <t>ایران – توقف TOEFL در ایران (وضعیت شهریور ۱۴۰۵)</t>
+        </is>
+      </c>
+      <c r="B165" s="16" t="inlineStr">
+        <is>
+          <t>https://zandienglish.ir/toefl-in-iran/</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="4" t="inlineStr">
+        <is>
+          <t>ایران – وثیقهٔ خروج تحصیلی مشمولان ۲۰۰ میلیون تومان (سامانهٔ سخا، تیر ۱۴۰۵)</t>
+        </is>
+      </c>
+      <c r="B166" s="16" t="inlineStr">
+        <is>
+          <t>https://www.zoomit.ir/iran-news/464136-exit-permit-bond-sakha-1405/</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="4" t="inlineStr">
+        <is>
+          <t>سوئد – تاریخ‌های کلیدی ورودی پاییز ۲۰۲۷ (۱۶ اکتبر – ۱۵ ژانویه؛ مدارک ۱ فوریه؛ دور دوم ۱۵ آوریل)</t>
+        </is>
+      </c>
+      <c r="B167" s="16" t="inlineStr">
+        <is>
+          <t>https://www.umu.se/en/education/application-and-admission/key-dates-and-deadlines/</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="4" t="inlineStr">
+        <is>
+          <t>آلمان – Stuttgart MSc CS: بازهٔ اپلای ترم زمستان ۱۵ نوامبر – ۱۵ ژانویه؛ انگلیسی C1</t>
+        </is>
+      </c>
+      <c r="B168" s="16" t="inlineStr">
+        <is>
+          <t>https://www.uni-stuttgart.de/en/study/study-programs/Computer-Science-M.Sc.-00001/</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="4" t="inlineStr">
+        <is>
+          <t>آلمان – Passau: بازهٔ اپلای AI Engineering ۱ آوریل – ۳۱ می</t>
+        </is>
+      </c>
+      <c r="B169" s="16" t="inlineStr">
+        <is>
+          <t>https://www.uni-passau.de/en/apply/apply-with-intl-qualifications</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="4" t="inlineStr">
+        <is>
+          <t>دانمارک – AAU: مهلت شهریه‌پردازها ۱۵ ژانویه (EU: ۱ مارس)؛ پورتال از اواسط دسامبر</t>
+        </is>
+      </c>
+      <c r="B170" s="16" t="inlineStr">
+        <is>
+          <t>https://www.en.aau.dk/education/apply/master/how-and-when-to-apply</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="4" t="inlineStr">
+        <is>
+          <t>دانمارک – SDU Computer Science: مهلت غیر-EU ۱ فوریه؛ شهریه یک سال پیش‌پرداخت</t>
+        </is>
+      </c>
+      <c r="B171" s="16" t="inlineStr">
+        <is>
+          <t>https://www.sdu.dk/en/uddannelse/kandidat/datalogi</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="4" t="inlineStr">
+        <is>
+          <t>هلند – Radboud: مهلت غیر-EU ۱ آوریل، بورس ۳۱ ژانویه، ثبت‌نام ۱ ژوئن</t>
+        </is>
+      </c>
+      <c r="B172" s="16" t="inlineStr">
+        <is>
+          <t>https://www.ru.nl/en/education/application-and-admission/application-procedure-masters/deadlines</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="4" t="inlineStr">
+        <is>
           <t>هلند – Twente: مهلت غیر-EEA ۱ می ۲۰۲۷؛ بورس UTS ۱۵ اکتبر ۲۰۲۶ – ۱ آوریل ۲۰۲۷</t>
         </is>
       </c>
-      <c r="B158" s="16" t="inlineStr">
+      <c r="B173" s="16" t="inlineStr">
         <is>
           <t>https://collegedunia.com/netherlands/university/749-university-of-twente-enschede/admission</t>
         </is>
@@ -14359,6 +14618,21 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B156" r:id="rId155"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B157" r:id="rId156"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B158" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B159" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B160" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B161" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B162" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B163" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B164" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B165" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B166" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B167" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B168" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B169" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B170" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B171" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B172" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B173" r:id="rId172"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Housing sheet: add annual cost comparison standard vs en-suite vs private room (6 English cities + 5 countries); MD 16.1
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Table_final.xlsx
+++ b/Table_final.xlsx
@@ -12721,7 +12721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14268,48 +14268,524 @@
       </c>
       <c r="I36" s="4" t="n"/>
     </row>
-    <row r="38" ht="48" customHeight="1">
-      <c r="A38" s="14" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>شهر / کشور</t>
+        </is>
+      </c>
+      <c r="B38" s="1" t="inlineStr">
+        <is>
+          <t>خوابگاه استاندارد (حمام مشترک) — سالانه</t>
+        </is>
+      </c>
+      <c r="C38" s="1" t="inlineStr">
+        <is>
+          <t>خوابگاه en-suite — سالانه</t>
+        </is>
+      </c>
+      <c r="D38" s="1" t="inlineStr">
+        <is>
+          <t>اتاق در خانهٔ مشترک خصوصی — سالانه (+ قبوض ≈ £80/ماه)</t>
+        </is>
+      </c>
+      <c r="E38" s="1" t="inlineStr">
+        <is>
+          <t>en-suite در برابر اتاق خصوصی</t>
+        </is>
+      </c>
+      <c r="F38" s="1" t="inlineStr">
+        <is>
+          <t>استاندارد در برابر en-suite (پول حمام اختصاصی)</t>
+        </is>
+      </c>
+      <c r="G38" s="1" t="inlineStr">
+        <is>
+          <t>نکته</t>
+        </is>
+      </c>
+      <c r="H38" s="1" t="n"/>
+      <c r="I38" s="1" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Newcastle / Middlesbrough (Northumbria، Newcastle، Teesside)</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>£94–118/هفته × ۵۱ = £4,800–6,000 (رسمی Northumbria £94.19، Newcastle £117.60)</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>£140–190/هفته × ۵۱ = £7,100–9,700</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>£450–650/ماه × ۱۲ + £960 = £6,400–8,800 (+ ضامن ≈ £1,650 اگر لازم شود)</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>≈ برابر (−£1,000 تا +£1,700)</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>استاندارد £2,300–3,700 ارزان‌تر</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>ارزان‌ترین راه واقعی: اتاق استاندارد ۵۱ هفته‌ای ≈ £4,900 با همهٔ قبوض</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="n"/>
+      <c r="I39" s="4" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>York (اعداد رسمی PG 2026/27)</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>£186 × ۵۱ = £9,486</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>£206 × ۵۱ = £10,506</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>£550–750/ماه × ۱۲ + £960 = £7,560–9,960</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>❌ en-suite £500–2,900 گران‌تر از اتاق خصوصی</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>استاندارد £1,020 ارزان‌تر</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>York خوابگاه گران دارد؛ مزیتش تضمین و بی‌ضامنی است، نه قیمت</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="n"/>
+      <c r="I40" s="4" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Colchester (Essex)</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>≈ £115–140 × ۴۰–۵۱ = £4,600–7,100</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>≈ £160–200 × ۴۰–۵۱ = £6,400–10,200</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>£550–700/ماه × ۱۲ + £960 = £7,560–9,360</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>≈ برابر</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>استاندارد £1,800–3,000 ارزان‌تر</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>قرارداد ۴۰ هفته‌ای برای ارشد ۱۲ ماهه کافی نیست → ۸–۱۲ هفتهٔ تابستان جدا</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="n"/>
+      <c r="I41" s="4" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Uxbridge (Brunel) — غرب لندن</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>≈ £150–170 × ۴۰–۵۰ = £6,000–8,500</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>≈ £190–240 × ۴۰–۵۰ = £7,600–12,000</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>£900–1,200/ماه × ۱۲ + £1,200 = £12,000–15,600</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>✅ en-suite £2,000–5,000 ارزان‌تر</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>استاندارد £1,600–3,500 ارزان‌تر</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>در لندن و حومه خوابگاه دانشگاه واقعاً می‌صرفد + تضمین Brunel (مهلت ۱۵ مارس)</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="n"/>
+      <c r="I42" s="4" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Durham (کالج، PG self-catered)</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>£183 × ۳۹ = £7,146 + ۱۳ هفته تابستان ≈ £1,950 = £9,100</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>£200 × ۳۹ = £7,801 + تابستان ≈ £1,950 = £9,750</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>£550–700/ماه × ۱۲ + £960 = £7,560–9,360</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>≈ برابر تا £2,000 گران‌تر</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>استاندارد £650 ارزان‌تر</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>قرارداد ۳۹ هفته‌ای دورهام برای ارشد ۱۲ ماهه مشکل‌ساز است</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="n"/>
+      <c r="I43" s="4" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>London مرکز (UCL / KCL / Imperial)</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>£210–250 × ۴۰–۵۱ = £8,400–12,750</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>£260–350 × ۴۰–۵۱ = £10,400–17,850</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>£1,000–1,400/ماه × ۱۲ + £1,200 = £13,200–18,000 (+ ضامن)</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>✅ £0–3,000 ارزان‌تر (اگر گیرتان بیاید — PG بدون تضمین)</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>استاندارد £2,000–5,000 ارزان‌تر</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>در لندن هر دو گران‌اند؛ تفاوت اصلی «ضامن نخواستن» خوابگاه است</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="n"/>
+      <c r="I44" s="4" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>آلمان (Studierendenwerk در برابر WG)</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>€230–450/ماه با قبوض = €2,800–5,400</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>— (خوابگاه‌های آلمان معمولاً حمام مشترک یا آپارتمان تک‌نفره)</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>€450–700 + €80 قبوض = €6,400–9,400</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>✅ خوابگاه €1,500–4,500 ارزان‌تر</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>بزرگ‌ترین صرفه‌جویی نسبی — ولی لیست انتظار</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="n"/>
+      <c r="I45" s="4" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>هلند (اتاق رزروشده در برابر بازار)</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>€370–650 = €4,400–7,800</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>€600–1,000 = €7,200–12,000</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>✅ €1,500–4,000 ارزان‌تر</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>اتاق رزروشده فقط سال اول و بدون تضمین</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="n"/>
+      <c r="I46" s="4" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>سوئد (کریدوری در برابر خصوصی)</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>SEK 3,500–6,500 = SEK 42–78k</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>SEK 5,000–8,000 (+ برق) = SEK 62–100k</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>✅ SEK 15–25k ارزان‌تر (≈ $1,500–2,500)</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>Uppsala/LiU تضمین؛ استکهلم صف</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="n"/>
+      <c r="I47" s="4" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>دانمارک (kollegium در برابر خصوصی)</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>DKK 3,200–4,700 = DKK 38–56k</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>DKK 4,500–7,000 = DKK 54–84k</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>✅ DKK 15–30k ارزان‌تر (≈ $2,300–4,600)</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>Aalborg تضمین؛ کپنهاگ نه</t>
+        </is>
+      </c>
+      <c r="H48" s="4" t="n"/>
+      <c r="I48" s="4" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>سوئیس (WOKO/FMEL در برابر WG)</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>CHF 480–900 = CHF 5,800–10,800</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>CHF 700–1,200 = CHF 8,400–14,400</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>✅ CHF 2,500–5,000 ارزان‌تر (≈ $3,000–6,000)</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>بزرگ‌ترین صرفه‌جویی مطلق — ولی زوریخ ۳–۱۲ ماه صف</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="n"/>
+      <c r="I49" s="4" t="n"/>
+    </row>
+    <row r="51" ht="48" customHeight="1">
+      <c r="A51" s="14" t="inlineStr">
         <is>
           <t>پاسخ کوتاه به «انگلیس خوابگاه با ناهار و شام می‌دهد»: بله، «catered halls» وجود دارد (معمولاً صبحانه + شام، در Durham سه وعده)، ولی (۱) تقریباً همه‌جا فقط برای سال اول کارشناسی است و برای ارشد فقط چند جا (Durham، Northumbria، بعضی کالج‌های Bristol)، (۲) فقط در هفته‌های ترم (≈ ۳۰ هفته) غذا می‌دهند، (۳) هیچ‌جا داخل شهریه نیست — Durham ≈ £3,087 در سال برای غذا جدا می‌گیرد و اجارهٔ catered ≈ £262/هفته است.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="48" customHeight="1">
-      <c r="A39" s="16" t="inlineStr">
+    <row r="52" ht="48" customHeight="1">
+      <c r="A52" s="16" t="inlineStr">
         <is>
           <t>• در هیچ‌یک از ۶ کشور خوابگاه داخل شهریه نیست. ارزان‌ترین خوابگاه‌ها: آلمان (€230–450 با قبوض) و شهرهای کوچک سوئد/دانمارک؛ گران‌ترین: لندن (£900–1,800/ماه) و زوریخ (CHF 700–1,200 اتاق).</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="48" customHeight="1">
-      <c r="A40" s="16" t="inlineStr">
+    <row r="53" ht="48" customHeight="1">
+      <c r="A53" s="16" t="inlineStr">
         <is>
           <t>• تضمین واقعی برای دانشجوی ارشد بین‌المللی فقط در: Uppsala، LiU (یک پیشنهاد)، AAU Aalborg، و دانشگاه‌های انگلستان با مهلت (York ۳۱ ژوئیه، Essex، Brunel ۱۵ مارس، احتمالاً Teesside/Northumbria/Newcastle/Sheffield/Lancaster). آلمان، هلند، سوئیس و لندن: هیچ تضمینی.</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="48" customHeight="1">
-      <c r="A41" s="16" t="inlineStr">
+    <row r="54" ht="48" customHeight="1">
+      <c r="A54" s="16" t="inlineStr">
         <is>
           <t>• برای ایرانی‌ها: خوابگاه دانشگاه در انگلستان ضامن بریتانیایی نمی‌خواهد — اجارهٔ خصوصی می‌خواهد (یا ۶–۱۲ ماه پیش‌پرداخت). در هلند/سوئیس/آلمان ودیعهٔ ۲–۳ ماه + گاهی پیش‌پرداخت ۳ ماه را در «نقد روز صفر» حساب کنید. آدرس ثبت‌شده در آلمان (Anmeldung)، هلند (BSN) و سوئیس شرط گرفتن کارت اقامت/بانک است.</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="48" customHeight="1">
-      <c r="A42" s="16" t="inlineStr">
+    <row r="55" ht="48" customHeight="1">
+      <c r="A55" s="16" t="inlineStr">
         <is>
           <t>• اعداد «رسمی» از صفحهٔ دانشگاه (۲۰۲۶/۲۷) و اعداد با «≈» برآورد از منابع ثانویه‌اند؛ اجاره‌ها هر سال ۳–۸٪ بالا می‌رود.</t>
         </is>
       </c>
     </row>
+    <row r="56" ht="48" customHeight="1">
+      <c r="A56" s="16" t="inlineStr">
+        <is>
+          <t>• en-suite در برابر اتاق خصوصی (جدول سوم): در شمال انگلستان و York خوابگاه en-suite تقریباً هم‌قیمت یا حتی گران‌تر از اتاق در خانهٔ مشترک است؛ صرفه‌جویی واقعی از (۱) اتاق استاندارد با حمام مشترک (£1,000–3,700 در سال کمتر از en-suite) و (۲) نخواستن ضامن/پیش‌پرداخت و قبوض ثابت می‌آید. در لندن، حومهٔ لندن و در آلمان/سوئیس/هلند/سوئد/دانمارک خوابگاه واقعاً ارزان‌تر از بازار است.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A41:I41"/>
-    <mergeCell ref="A42:I42"/>
-    <mergeCell ref="A40:I40"/>
-    <mergeCell ref="A39:I39"/>
-    <mergeCell ref="A38:I38"/>
+  <mergeCells count="6">
+    <mergeCell ref="A52:I52"/>
+    <mergeCell ref="A51:I51"/>
+    <mergeCell ref="A56:I56"/>
+    <mergeCell ref="A53:I53"/>
+    <mergeCell ref="A55:I55"/>
+    <mergeCell ref="A54:I54"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Full verification pass: DSW 2023 official dorm rents for all 14 German cities, official 2026/27 hall prices for Teesside/Essex/Brunel/Sheffield/Lancaster, WOKO official range, FX re-checked, Essex scholarship re-confirmed; new verification-log sheet (22 rows) + MD section 17; +7 sources
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Table_final.xlsx
+++ b/Table_final.xlsx
@@ -13,7 +13,8 @@
     <sheet name="برنامهٔ زمانی ۲۰۲۷" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="خوابگاه و مسکن" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="جمع‌بندی" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="منابع" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="راستی‌آزمایی" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="منابع" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'برنامه‌ها'!$A$1:$Q$111</definedName>
@@ -13049,7 +13050,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>شمال: Northumbria £94–158/هفته (رسمی) · Teesside ≈ £95–140 · Newcastle £118–240 (رسمی) · York £186–224 (رسمی؛ ۵۱ هفته = £9.5–11.4k/سال) · Durham PG ≈ £183–200 self-catered · جنوب/لندن: Essex ≈ £115–200 · Brunel ≈ £150–240 · UCL/KCL ≈ £190–350 · Imperial £210–410. یعنی ماهانه ≈ £400–700 شمال، £650–1,000 جنوب، £900–1,800 لندن</t>
+          <t>شمال (رسمی 2026/27): Teesside £85–160 · Northumbria £94–158 · Newcastle £118–240 · Sheffield PG £180–209 · Lancaster £139–206 · York £186–224 (۵۱ هفته = £9.5–11.4k/سال) · Durham PG £183–200 self-catered · جنوب/لندن: Essex £168–199 (رسمی) · Brunel £180–210 (رسمی) · UCL/KCL ≈ £190–350 · Imperial £210–410. یعنی ماهانه ≈ £400–700 شمال، £650–1,000 جنوب، £900–1,800 لندن</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -13144,7 +13145,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>€229–500 با قبوض (میانگین €345)</t>
+          <t>€229–500 با قبوض؛ میانگین DSW 2023: €345 (۲۰۲۶ ≈ +۵–۱۰٪)</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -13187,7 +13188,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>≈ €280–420</t>
+          <t>میانگین DSW 2023: €281 (بازهٔ ≈ €240–380)</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -13197,7 +13198,7 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>برآورد</t>
+          <t>DSW/Statista 2023 رسمی؛ WG برآورد</t>
         </is>
       </c>
       <c r="I11" s="4" t="n"/>
@@ -13230,7 +13231,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>≈ €280–450</t>
+          <t>میانگین DSW 2023: €401 — گران‌ترین Studierendenwerk آلمان (بازهٔ ≈ €320–480)</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -13240,7 +13241,7 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>MLP رسمی؛ خوابگاه برآورد</t>
+          <t>MLP 2025 + DSW 2023 رسمی</t>
         </is>
       </c>
       <c r="I12" s="4" t="n"/>
@@ -13273,7 +13274,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>≈ €250–380</t>
+          <t>میانگین DSW 2023: €276 (بازهٔ ≈ €230–380)</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -13283,7 +13284,7 @@
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>MLP رسمی؛ خوابگاه برآورد</t>
+          <t>MLP 2025 + DSW 2023 رسمی</t>
         </is>
       </c>
       <c r="I13" s="4" t="n"/>
@@ -13316,7 +13317,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>≈ €250–380</t>
+          <t>میانگین DSW 2023: €331 (بازهٔ ≈ €260–420)</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -13326,7 +13327,7 @@
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>MLP رسمی؛ خوابگاه برآورد</t>
+          <t>MLP 2025 + DSW 2023 رسمی</t>
         </is>
       </c>
       <c r="I14" s="4" t="n"/>
@@ -13359,7 +13360,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>≈ €200–300</t>
+          <t>میانگین DSW 2023: €251 (بازهٔ ≈ €200–330)</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -13369,7 +13370,7 @@
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>MLP رسمی؛ خوابگاه برآورد</t>
+          <t>MLP 2025 + DSW 2023 رسمی</t>
         </is>
       </c>
       <c r="I15" s="4" t="n"/>
@@ -13402,7 +13403,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>≈ €260–380</t>
+          <t>میانگین DSW 2023 (Niederbayern/Oberpfalz): €287 (بازهٔ ≈ €240–380)</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -13412,7 +13413,7 @@
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>برآورد</t>
+          <t>DSW/Statista 2023 رسمی؛ WG برآورد</t>
         </is>
       </c>
       <c r="I16" s="4" t="n"/>
@@ -13445,7 +13446,7 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>≈ €220–320</t>
+          <t>میانگین DSW 2023: €325 — خوابگاه‌های نوساز؛ WG (€339) تقریباً هم‌قیمت خوابگاه است (بازهٔ ≈ €260–400)</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -13455,7 +13456,7 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>MLP رسمی؛ خوابگاه برآورد</t>
+          <t>MLP 2025 + DSW 2023 رسمی</t>
         </is>
       </c>
       <c r="I17" s="4" t="n"/>
@@ -13488,7 +13489,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>≈ €300–450</t>
+          <t>میانگین DSW 2023: €303 (بازهٔ ≈ €250–420)</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -13498,7 +13499,7 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>MLP رسمی؛ خوابگاه برآورد</t>
+          <t>MLP 2025 + DSW 2023 رسمی</t>
         </is>
       </c>
       <c r="I18" s="4" t="n"/>
@@ -13531,7 +13532,7 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>≈ €250–350</t>
+          <t>میانگین DSW 2023: €246 — ارزان‌ترین Studierendenwerk آلمان (بازهٔ ≈ €200–320)</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -13541,7 +13542,7 @@
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>برآورد</t>
+          <t>DSW/Statista 2023 رسمی؛ WG برآورد</t>
         </is>
       </c>
       <c r="I19" s="4" t="n"/>
@@ -13574,7 +13575,7 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>≈ €300–400</t>
+          <t>میانگین DSW 2023 (Bonn): €335 (بازهٔ ≈ €270–420)</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -13584,7 +13585,7 @@
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>برآورد</t>
+          <t>DSW/Statista 2023 رسمی؛ WG برآورد</t>
         </is>
       </c>
       <c r="I20" s="4" t="n"/>
@@ -13617,7 +13618,7 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>≈ €280–420</t>
+          <t>میانگین DSW 2023: €255 (بازهٔ ≈ €220–360)</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -13627,7 +13628,7 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>MLP رسمی؛ خوابگاه برآورد</t>
+          <t>MLP 2025 + DSW 2023 رسمی</t>
         </is>
       </c>
       <c r="I21" s="4" t="n"/>
@@ -13660,7 +13661,7 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>≈ €300–450</t>
+          <t>میانگین DSW 2023: €271 (بازهٔ ≈ €230–380)</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -13670,7 +13671,7 @@
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>MLP رسمی؛ خوابگاه برآورد</t>
+          <t>MLP 2025 + DSW 2023 رسمی</t>
         </is>
       </c>
       <c r="I22" s="4" t="n"/>
@@ -13703,7 +13704,7 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>≈ €350–500</t>
+          <t>میانگین DSW 2023: €347 (بازهٔ ≈ €300–500)</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -13713,7 +13714,7 @@
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>MLP رسمی؛ خوابگاه برآورد</t>
+          <t>MLP 2025 + DSW 2023 رسمی</t>
         </is>
       </c>
       <c r="I23" s="4" t="n"/>
@@ -14778,7 +14779,7 @@
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>CHF 480–900</t>
+          <t>WOKO CHF 295–1,180 بسته به ساختمان (اکثر ۴۵۰–۸۵۰؛ میانگین آگهی‌ها ≈ 754)</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
@@ -14788,7 +14789,7 @@
       </c>
       <c r="H48" s="4" t="inlineStr">
         <is>
-          <t>woko.ch؛ برآورد</t>
+          <t>woko.ch رسمی (فهرست ساختمان‌ها)</t>
         </is>
       </c>
       <c r="I48" s="4" t="n"/>
@@ -15165,7 +15166,7 @@
       </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>≈ £95–140/هفته = £410–610/ماه</t>
+          <t>£85 (Parkside، حمام مشترک) · £120–125 (Parkside Village / Woodlands en-suite) · £155–160 (KES) در هفته؛ قرارداد ۴۰/۴۵/۵۰ هفته؛ ودیعه £150 (رسمی 2026/27) = £370–690/ماه</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
@@ -15175,7 +15176,7 @@
       </c>
       <c r="H57" s="4" t="inlineStr">
         <is>
-          <t>برآورد؛ PBSA از £138/هفته</t>
+          <t>tees.ac.uk رسمی؛ PBSA خصوصی از £138/هفته</t>
         </is>
       </c>
       <c r="I57" s="4" t="n"/>
@@ -15337,17 +15338,17 @@
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>≈ £115–200/هفته</t>
+          <t>£168 (Meadows، حمام مشترک) تا £199 (en-suite) در هفته؛ Quays ۴۴ هفته £175 (رسمی 2026-27) = £730–860/ماه</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t>£550–700</t>
+          <t>≈ £400–600 (خانهٔ مشترک در کولچستر ارزان‌تر از خوابگاه)</t>
         </is>
       </c>
       <c r="H61" s="4" t="inlineStr">
         <is>
-          <t>essex.ac.uk رسمی (تضمین)؛ قیمت برآورد</t>
+          <t>essex.ac.uk رسمی (تضمین + اجاره)</t>
         </is>
       </c>
       <c r="I61" s="4" t="n"/>
@@ -15423,7 +15424,7 @@
       </c>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>≈ £150–240/هفته</t>
+          <t>en-suite از £180–185/هفته (Mill Hall £179.97؛ PG £185.36)؛ استودیو £368 (رسمی 2026/27) = £780–800/ماه</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">
@@ -15433,7 +15434,7 @@
       </c>
       <c r="H63" s="4" t="inlineStr">
         <is>
-          <t>brunel.ac.uk رسمی (تضمین)؛ قیمت برآورد</t>
+          <t>brunel.ac.uk رسمی (تضمین + اجاره)</t>
         </is>
       </c>
       <c r="I63" s="4" t="n"/>
@@ -15681,7 +15682,7 @@
       </c>
       <c r="F69" s="4" t="inlineStr">
         <is>
-          <t>≈ £125–190/هفته</t>
+          <t>حمام مشترک £139–168 · en-suite £203–206 · استودیو £241 در هفته (۴۰ هفته؛ رسمی 2026/27)؛ catered £276</t>
         </is>
       </c>
       <c r="G69" s="4" t="inlineStr">
@@ -15691,7 +15692,7 @@
       </c>
       <c r="H69" s="4" t="inlineStr">
         <is>
-          <t>برآورد</t>
+          <t>lancaster.ac.uk رسمی (اجاره)؛ تضمین PG تأیید کنید</t>
         </is>
       </c>
       <c r="I69" s="4" t="n"/>
@@ -15724,7 +15725,7 @@
       </c>
       <c r="F70" s="4" t="inlineStr">
         <is>
-          <t>≈ £130–210/هفته</t>
+          <t>PG: St Vincent's en-suite £180 · Allen Court en-suite+ £194 · Deluxe+ £209 در هفته (۴۲ یا ۵۱ هفته؛ رسمی 2026/27) = £780–905/ماه</t>
         </is>
       </c>
       <c r="G70" s="4" t="inlineStr">
@@ -15734,7 +15735,7 @@
       </c>
       <c r="H70" s="4" t="inlineStr">
         <is>
-          <t>برآورد</t>
+          <t>sheffield.ac.uk رسمی (اجاره)؛ تضمین PG تأیید کنید</t>
         </is>
       </c>
       <c r="I70" s="4" t="n"/>
@@ -16536,7 +16537,7 @@
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
-          <t>CHF 480–900؛ WG خصوصی 700–1,200</t>
+          <t>WOKO CHF 295–1,180 (اکثر 450–850)؛ WG خصوصی 700–1,200</t>
         </is>
       </c>
       <c r="F90" s="4" t="inlineStr">
@@ -16665,7 +16666,7 @@
       </c>
       <c r="E93" s="4" t="inlineStr">
         <is>
-          <t>≈ £95–140/هفته (≈ £410–610/ماه) با قبوض؛ PBSA از £138/هفته</t>
+          <t>£85 (حمام مشترک) تا £125 (en-suite) و £155–160 (KES) در هفته؛ ودیعه £150؛ ۴۰/۴۵/۵۰ هفته (رسمی 2026/27)</t>
         </is>
       </c>
       <c r="F93" s="4" t="inlineStr">
@@ -16680,7 +16681,7 @@
       </c>
       <c r="H93" s="5" t="inlineStr">
         <is>
-          <t>tees.ac.uk (≈)</t>
+          <t>tees.ac.uk رسمی</t>
         </is>
       </c>
       <c r="I93" s="4" t="n"/>
@@ -16837,7 +16838,7 @@
       </c>
       <c r="E97" s="4" t="inlineStr">
         <is>
-          <t>≈ £115–200/هفته (چک شود)</t>
+          <t>£168–199/هفته (حمام مشترک Meadows £168؛ en-suite £189–199؛ رسمی 2026-27)</t>
         </is>
       </c>
       <c r="F97" s="4" t="inlineStr">
@@ -16880,7 +16881,7 @@
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
-          <t>≈ £150–240/هفته (چک شود)</t>
+          <t>en-suite از £180–185/هفته؛ استودیو £368 (رسمی 2026/27)</t>
         </is>
       </c>
       <c r="F98" s="4" t="inlineStr">
@@ -16923,7 +16924,7 @@
       </c>
       <c r="E99" s="4" t="inlineStr">
         <is>
-          <t>≈ £125–210/هفته</t>
+          <t>Sheffield PG £180–209 و Lancaster £139–206 (رسمی 2026/27)؛ Warwick/Leicester ≈ £130–210 (برآورد)</t>
         </is>
       </c>
       <c r="F99" s="4" t="inlineStr">
@@ -16938,7 +16939,7 @@
       </c>
       <c r="H99" s="5" t="inlineStr">
         <is>
-          <t>برآورد</t>
+          <t>sheffield.ac.uk، lancaster.ac.uk رسمی؛ بقیه برآورد</t>
         </is>
       </c>
       <c r="I99" s="4" t="n"/>
@@ -17162,12 +17163,12 @@
       </c>
       <c r="B106" s="4" t="inlineStr">
         <is>
-          <t>£94–118/هفته × ۵۱ = £4,800–6,000 (رسمی Northumbria £94.19، Newcastle £117.60)</t>
+          <t>£85–118/هفته × ۵۰–۵۱ = £4,250–6,000 (رسمی: Teesside Parkside £85، Northumbria £94.19، Newcastle £117.60)</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>£140–190/هفته × ۵۱ = £7,100–9,700</t>
+          <t>£125–190/هفته × ۵۰–۵۱ = £6,250–9,700 (Teesside Woodlands £125 رسمی)</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr">
@@ -17240,27 +17241,27 @@
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>≈ £115–140 × ۴۰–۵۱ = £4,600–7,100</t>
+          <t>£168 (Meadows، حمام مشترک) × ۴۰–۵۱ = £6,700–8,600 (رسمی)</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>≈ £160–200 × ۴۰–۵۱ = £6,400–10,200</t>
+          <t>£189–199 × ۴۰–۵۱ = £7,600–10,100 (رسمی)</t>
         </is>
       </c>
       <c r="D108" s="4" t="inlineStr">
         <is>
-          <t>£550–700/ماه × ۱۲ + £960 = £7,560–9,360</t>
+          <t>≈ £400–600/ماه × ۱۲ + £960 = £5,800–8,200</t>
         </is>
       </c>
       <c r="E108" s="4" t="inlineStr">
         <is>
-          <t>≈ برابر</t>
+          <t>❌ خوابگاه £1,000–3,000 گران‌تر از اتاق خصوصی</t>
         </is>
       </c>
       <c r="F108" s="4" t="inlineStr">
         <is>
-          <t>استاندارد £1,800–3,000 ارزان‌تر</t>
+          <t>استاندارد ≈ £900–1,500 ارزان‌تر</t>
         </is>
       </c>
       <c r="G108" s="4" t="inlineStr">
@@ -17279,12 +17280,12 @@
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
-          <t>≈ £150–170 × ۴۰–۵۰ = £6,000–8,500</t>
+          <t>— (Brunel تقریباً همه en-suite)</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>≈ £190–240 × ۴۰–۵۰ = £7,600–12,000</t>
+          <t>£180–210 × ۴۰–۵۰ = £7,200–10,500 (رسمی 2026/27)</t>
         </is>
       </c>
       <c r="D109" s="4" t="inlineStr">
@@ -17299,7 +17300,7 @@
       </c>
       <c r="F109" s="4" t="inlineStr">
         <is>
-          <t>استاندارد £1,600–3,500 ارزان‌تر</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G109" s="4" t="inlineStr">
@@ -17814,7 +17815,765 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B208"/>
+  <dimension ref="A1:F23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>حوزه</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>عدد / بازه در فایل</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>منبع</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>نوع منبع</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>آخرین بررسی</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>نتیجهٔ بازبینی ۲۸ سپتامبر ۲۰۲۶</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>نرخ ارز</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>€1 = $1.14 · £1 = $1.325 · CHF 1 = $1.21 · $1 ≈ SEK 9.9 · $1 ≈ DKK 6.55</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>xe.com / tradingeconomics</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>رسمی (بازار)</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>۲۸ سپتامبر ۲۰۲۶</t>
+        </is>
+      </c>
+      <c r="F2" s="18" t="inlineStr">
+        <is>
+          <t>✅ تأیید: EUR/USD 1.137، GBP/USD 1.321، USD/CHF 0.829 (انحراف &lt; ۰.۵٪)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>جدول اصلی – شهریه‌ها (ردیف ۴/۵)</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>آلمان €300–800 (Stuttgart €3,000؛ FAU €8,000 از ۲۰۲۷) · هلند €19,714–22,400 · سوئد SEK 140–190k · دانمارک €14,900–17,300 · سوئیس CHF 790–8,000/سال · انگلستان £17,000–46,000</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>صفحات رسمی دانشگاه‌ها</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>رسمی 2026/27 (Bristol 2027/28)</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>۲۷–۲۸ سپتامبر ۲۰۲۶</t>
+        </is>
+      </c>
+      <c r="F3" s="18" t="inlineStr">
+        <is>
+          <t>✅ همه از صفحهٔ رسمی؛ نرخ 2027/28 اکثراً هنوز منتشر نشده (اکتبر–دسامبر ۲۰۲۶ اعلام می‌شود)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>جدول اصلی – ویزا و تمکن (ردیف ۲۳/۲۵)</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>DE €11,904 · NL €13,569 · SE SEK 10,656/ماه · DK DKK 7,426/ماه · CH CHF 21,000 (Basel 24,000) · UK £1,203/£1,570 از ۳۰ نوامبر ۲۰۲۶</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>make-it-in-germany، ind.nl، migrationsverket، nyidanmark، sem.admin.ch، gov.uk</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>رسمی</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>۲۷ سپتامبر ۲۰۲۶</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>✅ بدون تغییر از بررسی قبلی</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>جدول اصلی – کف حقوق/ویزای کار (ردیف ۱۶)</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>DE €45,934/€50,700 · NL €3,122/ماه · SE SEK 34,470 · UK £38,290 → £41,700 · CH بدون کف + سهمیه ۸,۵۰۰</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>منابع دولتی</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>رسمی</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>۲۷ سپتامبر ۲۰۲۶</t>
+        </is>
+      </c>
+      <c r="F5" s="18" t="inlineStr">
+        <is>
+          <t>✅ بدون تغییر</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>جدول اصلی – حقوق جونیور و خالص (ردیف ۱۷/۱۸/۱۹)</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>DE €48–55k · NL €40–50k · SE SEK 420–540k · DK DKK 500–540k · CH CHF 85–105k · UK £28–35k</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Glassdoor، StepStone، اعلان‌های ۲۰۲۶</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>ثانویه</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>۲۷ سپتامبر ۲۰۲۶</t>
+        </is>
+      </c>
+      <c r="F6" s="17" t="inlineStr">
+        <is>
+          <t>⚠️ بازهٔ منطقی ولی نه رسمی — تنها بخش جدول اصلی که ذاتاً برآورد است</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>جدول اصلی – هزینهٔ زندگی (ردیف ۶/۷/۸)</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>بازه‌های شهری + مجموع سال اول/کل دوره</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>برآورد دانشگاه‌ها + محاسبه</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>رسمی (بازه) + محاسبهٔ خودم</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>۲۷ سپتامبر ۲۰۲۶</t>
+        </is>
+      </c>
+      <c r="F7" s="17" t="inlineStr">
+        <is>
+          <t>⚠️ ذاتاً تقریبی؛ با اجاره‌های رسمی خوابگاه‌ها (شیت خوابگاه) سازگار است</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>جدول اصلی – امتیاز (ردیف ۲۸)</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>DE 22 › SE 19 = EN 19 › NL 18 = CH 18 › DK 16</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>قضاوت بر اساس سه معیار شما</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>تحلیلی</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F8" s="17" t="inlineStr">
+        <is>
+          <t>⚠️ عدد نیست، قضاوت وزنی است</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>شیت برنامه‌ها – شهریه‌ها</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>۱۱۰ برنامه: ۶۴ رسمی، ۴۶ با «≈» (آلمان ۱۳ = فقط هزینهٔ ترم تقریبی، سوئد ۱۰، سوئیس ۸، انگلستان ۶، هلند ۵، دانمارک ۴)</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>صفحات رسمی / mastersportal / IDP</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>رسمی یا ثانویه (علامت‌گذاری‌شده)</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>۲۷–۲۸ سپتامبر ۲۰۲۶</t>
+        </is>
+      </c>
+      <c r="F9" s="18" t="inlineStr">
+        <is>
+          <t>✅ سوئیس همه امروز/دیروز از صفحهٔ رسمی؛ ⚠️ ردیف‌های «≈» خطای محتمل ±۵–۱۰٪</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>شیت برنامه‌ها – شرط ورود/تطبیق نمره</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Warwick 2:1 = ۱۵/۲۰ · Durham 2:1 = ۱۴–۱۶/۲۰ · KCL high 2:1 = ۱۷/۲۰ · Bristol حداقل ۱۵/۲۰ · Twente ۱۵/۲۰ · Imperial First</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>صفحات رسمی دانشگاه‌ها</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>رسمی</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>۲۸ سپتامبر ۲۰۲۶</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>✅ تأیید؛ UCL جدول ایران رسمی پیدا نشد (⚠️ برآورد ۱۵–۱۶/۲۰)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>شیت برنامه‌ها – QS 2027</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>ETH 8 … ZHAW 851–900؛ Warwick ≈ 69، Bristol ≈ 54، KCL ≈ 31، Durham ≈ 94</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>QS WUR 2027 (via iamexpat/topuniversities)</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>ثانویه از منبع رسمی</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>۲۷–۲۸ سپتامبر ۲۰۲۶</t>
+        </is>
+      </c>
+      <c r="F11" s="18" t="inlineStr">
+        <is>
+          <t>✅ (رتبه‌های حدودی با ≈)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>ردیف ۵ب – بورس‌ها</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>LiU ≥ 3.5/4 · Chalmers IPOET ≥ ۸۰٪ · Uppsala/Halmstad/MDU · NL Scholarship €5,000 · AAU ≈ ۱۵ بورس + DKK 11,225 · ETH ESOP CHF 12,000/ترم · USI CHF 4,000 · Essex ایران ۱۴/۲۰ → £4,500 · Teesside £2,000 · Brunel £6,000 (2:1) · Chevening ✗ · SI ✗</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>liu.se، chalmers.se، uu.se، si.se، en.aau.dk، ethz.ch، usi.ch، essex.ac.uk، tees.ac.uk، brunel.ac.uk، chevening.org</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>رسمی (Halmstad/MDU ثانویه)</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>۲۸ سپتامبر ۲۰۲۶</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>✅ Essex £4,500 دوباره تأیید (جدول ۲۰۲۵–۲۶؛ ۲۰۲۶–۲۷ هنوز)؛ ⚠️ Halmstad/MDU از منبع ثانویه</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>شیت زمانی – مهلت‌ها</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>ETH ۱–۳۰ نوامبر · EPFL ۱۵ دسامبر · سوئد ۱۵ ژانویه · UZH/Fribourg ۲۸ فوریه · HSLU ۱ آوریل · Radboud ۱ آوریل · USI/Neuchâtel/Basel ۳۰ آوریل · Twente ۱ می · Passau ۳۱ می</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>صفحات رسمی</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>رسمی (چرخهٔ ۲۰۲۶/۲۷ برای ۲۰۲۷)</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>۲۷–۲۸ سپتامبر ۲۰۲۶</t>
+        </is>
+      </c>
+      <c r="F13" s="18" t="inlineStr">
+        <is>
+          <t>✅؛ ⚠️ مهلت‌های ۲۰۲۷ بر اساس چرخهٔ قبلی — بهار ۲۰۲۷ دوباره ببینید</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>شیت خوابگاه – انگلستان (اجاره)</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Teesside £85–160 · Northumbria £94–158 · Newcastle £118–240 · Sheffield PG £180–209 · Lancaster £139–206 · York £186–224 · Essex £168–199 · Brunel £180–210 · Durham £183–262 · Imperial £210–410</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>صفحات رسمی 2026/27 (Imperial ثانویه)</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>رسمی</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>۲۸ سپتامبر ۲۰۲۶</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>✅ امروز ۵ دانشگاه تازه تأیید و اصلاح شد (Teesside، Essex، Brunel، Sheffield، Lancaster)؛ ⚠️ Warwick، Leicester، Kent، Surrey، RHUL، NTU، MMU، Bristol، UCL/KCL هنوز برآورد</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>شیت خوابگاه – انگلستان (تضمین)</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>York ۳۱ ژوئیه · Essex کل دوره · Brunel ۱۵ مارس · Manchester ۳۱ اوت · Imperial/UCL/KCL/Durham بدون تضمین PG</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>صفحات رسمی</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>رسمی</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>۲۸ سپتامبر ۲۰۲۶</t>
+        </is>
+      </c>
+      <c r="F15" s="18" t="inlineStr">
+        <is>
+          <t>✅؛ ⚠️ Teesside، Northumbria، Newcastle، Sheffield، Lancaster، Leicester، Kent، Surrey، RHUL، NTU، MMU: «احتمالاً بله» — تأیید نشده</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>شیت خوابگاه – آلمان</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>خوابگاه: میانگین DSW 2023 هر شهر (Darmstadt €401 … Siegen €246) · WG: MLP 2025 (Chemnitz €274 … München €790) · Stuttgart صف ۶–۸ ماه</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Statista/DSW 2023، MLP Studentenwohnreport 2025، Studierendenwerk Stuttgart</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>رسمی</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>۲۸ سپتامبر ۲۰۲۶</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>✅ امروز میانگین رسمی خوابگاه برای هر ۱۴ شهر جایگزین برآورد شد؛ ⚠️ اعداد ۲۰۲۳ است (۲۰۲۶ ≈ +۵–۱۰٪)؛ «شانس» قضاوتی است جز Stuttgart</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>شیت خوابگاه – هلند</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Radboud €370–650 · Utrecht €868 · Twente €300–800 · Enschede €397 · Groningen €515 · شهرهای پرفشار Kences</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>ru.nl، uu.nl، utwente، Kences 2026، Kamernet</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>رسمی/ثانویهٔ معتبر</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>۲۸ سپتامبر ۲۰۲۶</t>
+        </is>
+      </c>
+      <c r="F17" s="18" t="inlineStr">
+        <is>
+          <t>✅؛ ⚠️ Leiden/Delft/Eindhoven/Amsterdam/Breda بازه‌ها برآورد</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>شیت خوابگاه – سوئد</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>رنگ شهرها SFS 2024/2025 · Uppsala تضمین · LiU یک پیشنهاد · اجاره SEK 3,300–8,000</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>SFS، uu.se، liu.se</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>رسمی (رنگ‌ها) / برآورد (اجاره)</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>۲۸ سپتامبر ۲۰۲۶</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>✅ رنگ‌ها رسمی؛ ⚠️ اجاره‌ها برآورد کلی (SSSB/Studentbostäder چک نشد)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>شیت خوابگاه – دانمارک</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Aalborg DKK 3,200–4,700 · Copenhagen 3,500–9,000 · Odense/Kolding/Aarhus/Lyngby</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>en.aau.dk، بروشور AAU</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>رسمی (AAU) / برآورد (بقیه)</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>۲۸ سپتامبر ۲۰۲۶</t>
+        </is>
+      </c>
+      <c r="F19" s="17" t="inlineStr">
+        <is>
+          <t>⚠️ Odense/Kolding/Aarhus/Lyngby برآورد</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>شیت خوابگاه – سوئیس</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>WOKO CHF 295–1,180 (اکثر 450–850) · FMEL/USI/Bern/Fribourg/Neuchâtel/Basel/Luzern ≈ CHF 450–900</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>woko.ch</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>رسمی (WOKO) / برآورد (بقیه)</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>۲۸ سپتامبر ۲۰۲۶</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>✅ WOKO امروز اصلاح شد؛ ⚠️ بقیه برآورد</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>شیت خوابگاه – catered انگلستان</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Durham catered £262/هفته، غذا £3,087 (25/26) · Lancaster catered £276 · Northumbria گزینهٔ catered</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>durham.ac.uk، Palatinate، lancaster.ac.uk، northumbria.ac.uk</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>رسمی</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>۲۸ سپتامبر ۲۰۲۶</t>
+        </is>
+      </c>
+      <c r="F21" s="18" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>MD – ATAS، غربالگری هلند، Chevening</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>ATAS برای ارشد آموزشی CS لازم نیست · غربالگری هلند «فعلاً» کنار گذاشته شد (ژوئن ۲۰۲۶) · Chevening: ۲ سال کار بعد از مدرک + بازگشت</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>gov.uk Appendix ATAS، delta.tudelft، chevening.org</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>رسمی</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>۲۸ سپتامبر ۲۰۲۶</t>
+        </is>
+      </c>
+      <c r="F22" s="18" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>کل فایل – وضعیت</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>≈ ۱,۶۰۰ سلول عددی؛ ≈ ۳۴۰ سلول با علامت ≈/برآورد</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>۲۸ سپتامبر ۲۰۲۶</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>خلاصه: تصمیم‌سازها (شهریه، ویزا، تمکن، مهلت، تطبیق نمره، بورس‌های اصلی، خوابگاه‌های اصلی) رسمی‌اند؛ حقوق، هزینهٔ زندگی، شانس خوابگاه و اجاره‌های شهرهای فرعی برآوردند و همان‌طور علامت خورده‌اند</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B215"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -18592,1726 +19351,1810 @@
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>Russell Group – فهرست رسمی ۲۴ عضو (۲۰ در انگلستان)</t>
+          <t>مسکن – Statista/DSW: میانگین اجارهٔ خوابگاه هر Studierendenwerk ۲۰۲۳ با قبوض (Darmstadt €401 … Siegen €246؛ میانگین €306)</t>
         </is>
       </c>
       <c r="B65" s="20" t="inlineStr">
         <is>
-          <t>https://russellgroup.ac.uk/about/our-universities/</t>
+          <t>https://de.statista.com/statistik/daten/studie/1447630/umfrage/durchschnittsmiete-in-studierendenwerken/</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Warwick: جدول رسمی تطبیق مدرک ایرانی (1st ۱۷/۲۰، 2:1 ۱۵/۲۰، 2:2 ۱۳/۲۰)</t>
+          <t>مسکن – Teesside: قیمت‌های رسمی 2026/27 (Parkside £85، Woodlands £125، KES £155–160؛ ودیعه £150)</t>
         </is>
       </c>
       <c r="B66" s="20" t="inlineStr">
         <is>
-          <t>https://warwick.ac.uk/study/international/countryinformation/middleeast/iran/</t>
+          <t>https://www.tees.ac.uk/sections/accommodation/buildings/kes.cfm</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Durham MSc Advanced Computer Science: £34,500 (2026)؛ جدول ایران (2:1 = ۱۴–۱۶/۲۰؛ Ecctis)</t>
+          <t>مسکن – Essex Colchester: اجاره‌های رسمی 2026-27 (Meadows £168 حمام مشترک؛ en-suite £189–199)</t>
         </is>
       </c>
       <c r="B67" s="20" t="inlineStr">
         <is>
-          <t>https://www.durham.ac.uk/study/courses/advanced-computer-science-g5t609/</t>
+          <t>https://www.essex.ac.uk/life/accommodation/colchester/rent-charges</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – KCL: جدول رسمی ایران (First ۱۸، high 2:1 ۱۷، 2:1 ۱۵، high 2:2 ۱۳ از ۲۰)؛ Advanced Computing high 2:1، £40,450 (2026)</t>
+          <t>مسکن – Brunel Mill Hall از £179.97/هفته (2026/27)</t>
         </is>
       </c>
       <c r="B68" s="20" t="inlineStr">
         <is>
-          <t>https://www.kcl.ac.uk/study-legacy/postgraduate/apply/entry-requirements/international</t>
+          <t>https://www.brunel.ac.uk/life/accommodation/residences/residence?id=bd97a78a-03f2-4ed9-bce8-146d2e3ad8fc</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Imperial MSc Computing (AI &amp; ML): First-class؛ £46,000 (2026/27)</t>
+          <t>مسکن – Sheffield: اجاره‌های PG 2026/27 (Allen Court £194–209؛ ۴۲/۵۱ هفته)</t>
         </is>
       </c>
       <c r="B69" s="20" t="inlineStr">
         <is>
-          <t>https://www.imperial.ac.uk/study/courses/postgraduate-taught/computing-artificial-intelligence-msc/</t>
+          <t>https://sheffield.ac.uk/accommodation/rents</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – UCL MSc Computer Science (تبدیلی): £42,700 (2026/27)، 2:1 در رشتهٔ غیر CS</t>
+          <t>مسکن – Lancaster: قیمت‌های 2026/27 (حمام مشترک £139–168، en-suite £203–206، استودیو £241، catered £276)</t>
         </is>
       </c>
       <c r="B70" s="20" t="inlineStr">
         <is>
-          <t>https://www.ucl.ac.uk/prospective-students/graduate/taught-degrees/computer-science-msc-2026</t>
+          <t>https://features.lancaster-university.uk/accommodation/</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Bristol MSc Data Science: £37,900 (سپتامبر ۲۰۲۷)، strong 2:1 (۶۵٪)</t>
+          <t>مسکن – WOKO زوریخ: فهرست ساختمان‌ها و اجاره (CHF 295–1,180)</t>
         </is>
       </c>
       <c r="B71" s="20" t="inlineStr">
         <is>
-          <t>https://www.bristol.ac.uk/study/postgraduate/taught/msc-data-science/</t>
+          <t>https://www.woko.ch/unser-angebot/liegenschaften</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Bristol صفحهٔ ایران: کارشناسی ۴ ساله با حداقل ۱۵/۲۰ از دانشگاه مورد تأیید</t>
+          <t>Russell Group – فهرست رسمی ۲۴ عضو (۲۰ در انگلستان)</t>
         </is>
       </c>
       <c r="B72" s="20" t="inlineStr">
         <is>
-          <t>https://www.bristol.ac.uk/international/countries/iran.html</t>
+          <t>https://russellgroup.ac.uk/about/our-universities/</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – High Fliers «The Graduate Market in 2026»: دانشگاه‌های هدف کارفرمایان (Manchester، Birmingham، Nottingham، Warwick، UCL)؛ استخدام فارغ‌التحصیل در پایین‌ترین سطح از ۲۰۱۲</t>
+          <t>انگلستان – Warwick: جدول رسمی تطبیق مدرک ایرانی (1st ۱۷/۲۰، 2:1 ۱۵/۲۰، 2:2 ۱۳/۲۰)</t>
         </is>
       </c>
       <c r="B73" s="20" t="inlineStr">
         <is>
-          <t>https://www.manchester.ac.uk/about/news/university-of-manchester-tops-uk-rankings-for-graduate-employer-interest/</t>
+          <t>https://warwick.ac.uk/study/international/countryinformation/middleeast/iran/</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – LEO (DfE) درآمد ۵ سال بعد: Imperial Computing £79,600؛ Bristol Computing £70,300؛ میانهٔ کل بخش ≈ £31–34k (ثانویه: unilens/campusquant)</t>
+          <t>انگلستان – Durham MSc Advanced Computer Science: £34,500 (2026)؛ جدول ایران (2:1 = ۱۴–۱۶/۲۰؛ Ecctis)</t>
         </is>
       </c>
       <c r="B74" s="20" t="inlineStr">
         <is>
-          <t>https://unilens.co.uk/insights/highest-graduate-earnings-uk-universities-2026</t>
+          <t>https://www.durham.ac.uk/study/courses/advanced-computer-science-g5t609/</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Appendix ATAS: ارشد آموزشی CS/AI نیاز به ATAS ندارد (فقط پژوهشی/PhD در CS و ارشد آموزشی فیزیک/مواد/مکانیک/هوافضا/شیمی)</t>
+          <t>انگلستان – KCL: جدول رسمی ایران (First ۱۸، high 2:1 ۱۷، 2:1 ۱۵، high 2:2 ۱۳ از ۲۰)؛ Advanced Computing high 2:1، £40,450 (2026)</t>
         </is>
       </c>
       <c r="B75" s="20" t="inlineStr">
         <is>
-          <t>https://www.gov.uk/guidance/immigration-rules/immigration-rules-appendix-atas-academic-technology-approval-scheme-atas</t>
+          <t>https://www.kcl.ac.uk/study-legacy/postgraduate/apply/entry-requirements/international</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>بورس – LiU International Scholarship: معمولاً ۵۰٪؛ شرط جدید ۲۰۲۶ (GPA ≥ 3.5/4 یا first/high second class)؛ فقط اولویت ۱</t>
+          <t>انگلستان – Imperial MSc Computing (AI &amp; ML): First-class؛ £46,000 (2026/27)</t>
         </is>
       </c>
       <c r="B76" s="20" t="inlineStr">
         <is>
-          <t>https://liu.se/en/article/scholarships</t>
+          <t>https://www.imperial.ac.uk/study/courses/postgraduate-taught/computing-artificial-intelligence-msc/</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>بورس – Chalmers: بورس‌های شهریه‌پردازها (IPOET ۷۵٪ با حداقل معدل ۸۰٪، Avancez)</t>
+          <t>انگلستان – UCL MSc Computer Science (تبدیلی): £42,700 (2026/27)، 2:1 در رشتهٔ غیر CS</t>
         </is>
       </c>
       <c r="B77" s="20" t="inlineStr">
         <is>
-          <t>https://www.chalmers.se/en/education/application-and-admission/scholarships-for-fee-paying-students/</t>
+          <t>https://www.ucl.ac.uk/prospective-students/graduate/taught-degrees/computer-science-msc-2026</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>بورس – Halmstad University Scholarship ۲۵٪/۵۰٪ برای غیر-EU (ثانویه؛ hh.se را چک کنید)</t>
+          <t>انگلستان – Bristol MSc Data Science: £37,900 (سپتامبر ۲۰۲۷)، strong 2:1 (۶۵٪)</t>
         </is>
       </c>
       <c r="B78" s="20" t="inlineStr">
         <is>
-          <t>https://www.mastersportal.com/scholarships/10077/halmstad-university-scholarships.html</t>
+          <t>https://www.bristol.ac.uk/study/postgraduate/taught/msc-data-science/</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>بورس – MDU: بورس تا ۱۰۰٪ شهریه برای متقاضیان اولویت ۱ (ثانویه؛ mdu.se را چک کنید)</t>
+          <t>انگلستان – Bristol صفحهٔ ایران: کارشناسی ۴ ساله با حداقل ۱۵/۲۰ از دانشگاه مورد تأیید</t>
         </is>
       </c>
       <c r="B79" s="20" t="inlineStr">
         <is>
-          <t>https://daadscholarship.com/malardalen-university-scholarships-2026-to-study-for-free-in-sweden/</t>
+          <t>https://www.bristol.ac.uk/international/countries/iran.html</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>بورس – SI Scholarship for Global Professionals: ۳۴ کشور واجد شرایط — ایران نیست (رسمی)</t>
+          <t>انگلستان – High Fliers «The Graduate Market in 2026»: دانشگاه‌های هدف کارفرمایان (Manchester، Birmingham، Nottingham، Warwick، UCL)؛ استخدام فارغ‌التحصیل در پایین‌ترین سطح از ۲۰۱۲</t>
         </is>
       </c>
       <c r="B80" s="20" t="inlineStr">
         <is>
-          <t>https://si.se/en/apply/scholarships/swedish-institute-scholarships-for-global-professionals/</t>
+          <t>https://www.manchester.ac.uk/about/news/university-of-manchester-tops-uk-rankings-for-graduate-employer-interest/</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>بورس – NL Scholarship (سابقاً Holland Scholarship): €5,000 سال اول برای غیر-EEA، از طریق دانشگاه‌های عضو</t>
+          <t>انگلستان – LEO (DfE) درآمد ۵ سال بعد: Imperial Computing £79,600؛ Bristol Computing £70,300؛ میانهٔ کل بخش ≈ £31–34k (ثانویه: unilens/campusquant)</t>
         </is>
       </c>
       <c r="B81" s="20" t="inlineStr">
         <is>
-          <t>https://www.mastersportal.com/scholarships/988/holland-scholarship-for-non-eea-international-students.html</t>
+          <t>https://unilens.co.uk/insights/highest-graduate-earnings-uk-universities-2026</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>بورس – AAU: ≈ ۱۵ بورس دولتی در سال، معافیت شهریه + DKK 11,225/ماه (۲۰۲۶)، بررسی خودکار (رسمی)</t>
+          <t>انگلستان – Appendix ATAS: ارشد آموزشی CS/AI نیاز به ATAS ندارد (فقط پژوهشی/PhD در CS و ارشد آموزشی فیزیک/مواد/مکانیک/هوافضا/شیمی)</t>
         </is>
       </c>
       <c r="B82" s="20" t="inlineStr">
         <is>
-          <t>https://www.en.aau.dk/education/apply/master/finance-and-fees</t>
+          <t>https://www.gov.uk/guidance/immigration-rules/immigration-rules-appendix-atas-academic-technology-approval-scheme-atas</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>بورس – ETH Excellence Scholarship &amp; Opportunity Programme: CHF 12,000/ترم + معافیت؛ ۱۰٪ بالای کلاس؛ ۱–۳۰ نوامبر</t>
+          <t>بورس – LiU International Scholarship: معمولاً ۵۰٪؛ شرط جدید ۲۰۲۶ (GPA ≥ 3.5/4 یا first/high second class)؛ فقط اولویت ۱</t>
         </is>
       </c>
       <c r="B83" s="20" t="inlineStr">
         <is>
-          <t>https://ethz.ch/en/studies/financial/scholarships/excellencescholarship.html</t>
+          <t>https://liu.se/en/article/scholarships</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>بورس – USI: بورس‌های Fondazione per le Facoltà di Lugano (CHF 4,000؛ سال اول با معدل ≥ ۸۰/۱۰۰؛ سال دوم بهترینِ هر برنامه) — خبر رسمی USI</t>
+          <t>بورس – Chalmers: بورس‌های شهریه‌پردازها (IPOET ۷۵٪ با حداقل معدل ۸۰٪، Avancez)</t>
         </is>
       </c>
       <c r="B84" s="20" t="inlineStr">
         <is>
-          <t>https://www.eco.usi.ch/en/feeds/9861</t>
+          <t>https://www.chalmers.se/en/education/application-and-admission/scholarships-for-fee-paying-students/</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>بورس – Essex Academic Excellence International Masters Scholarship: جدول کشوری (ایران ۱۴/۲۰ → £4,500؛ جدول ۲۰۲۵–۲۶)</t>
+          <t>بورس – Halmstad University Scholarship ۲۵٪/۵۰٪ برای غیر-EU (ثانویه؛ hh.se را چک کنید)</t>
         </is>
       </c>
       <c r="B85" s="20" t="inlineStr">
         <is>
-          <t>https://www.essex.ac.uk/scholarships</t>
+          <t>https://www.mastersportal.com/scholarships/10077/halmstad-university-scholarships.html</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>بورس – Teesside Global Excellence Scholarship £2,000 (پیشنهاد تا ۳۰ آوریل؛ رسمی)</t>
+          <t>بورس – MDU: بورس تا ۱۰۰٪ شهریه برای متقاضیان اولویت ۱ (ثانویه؛ mdu.se را چک کنید)</t>
         </is>
       </c>
       <c r="B86" s="20" t="inlineStr">
         <is>
-          <t>https://www.tees.ac.uk/sections/international/global_excellence_scholarship.cfm</t>
+          <t>https://daadscholarship.com/malardalen-university-scholarships-2026-to-study-for-free-in-sweden/</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>بورس – Brunel Vice-Chancellor's Postgraduate International Excellence Award £6,000 (حداقل 2:1؛ ودیعهٔ £5,000)</t>
+          <t>بورس – SI Scholarship for Global Professionals: ۳۴ کشور واجد شرایط — ایران نیست (رسمی)</t>
         </is>
       </c>
       <c r="B87" s="20" t="inlineStr">
         <is>
-          <t>https://www.brunel.ac.uk/scholarships</t>
+          <t>https://si.se/en/apply/scholarships/swedish-institute-scholarships-for-global-professionals/</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>بورس – Northumbria PGT International Scholarship £3,000: فهرست کشوری/ادامه‌تحصیلی‌های داخل UK — ایران نیست</t>
+          <t>بورس – NL Scholarship (سابقاً Holland Scholarship): €5,000 سال اول برای غیر-EEA، از طریق دانشگاه‌های عضو</t>
         </is>
       </c>
       <c r="B88" s="20" t="inlineStr">
         <is>
-          <t>https://www.mastersportal.com/scholarships/3890/pgt-international-scholarships.html</t>
+          <t>https://www.mastersportal.com/scholarships/988/holland-scholarship-for-non-eea-international-students.html</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>بورس – Chevening eligibility (رسمی): ۲ سال کار بعد از مدرک کارشناسی + تعهد بازگشت ۲ ساله؛ مهلت ۶ اکتبر ۲۰۲۶</t>
+          <t>بورس – AAU: ≈ ۱۵ بورس دولتی در سال، معافیت شهریه + DKK 11,225/ماه (۲۰۲۶)، بررسی خودکار (رسمی)</t>
         </is>
       </c>
       <c r="B89" s="20" t="inlineStr">
         <is>
-          <t>https://www.chevening.org/resource-hub/guidance/eligibility/</t>
+          <t>https://www.en.aau.dk/education/apply/master/finance-and-fees</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>بورس – Deutschlandstipendium €300/ماه (رسمی)</t>
+          <t>بورس – ETH Excellence Scholarship &amp; Opportunity Programme: CHF 12,000/ترم + معافیت؛ ۱۰٪ بالای کلاس؛ ۱–۳۰ نوامبر</t>
         </is>
       </c>
       <c r="B90" s="20" t="inlineStr">
         <is>
-          <t>https://www.deutschlandstipendium.de/</t>
+          <t>https://ethz.ch/en/studies/financial/scholarships/excellencescholarship.html</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – ETH: تاریخ‌های اپلای ارشد پاییز ۲۰۲۷ (۱–۳۰ نوامبر ۲۰۲۶؛ پاسخ تا پایان مارس؛ شروع ۲۰ سپتامبر ۲۰۲۷)</t>
+          <t>بورس – USI: بورس‌های Fondazione per le Facoltà di Lugano (CHF 4,000؛ سال اول با معدل ≥ ۸۰/۱۰۰؛ سال دوم بهترینِ هر برنامه) — خبر رسمی USI</t>
         </is>
       </c>
       <c r="B91" s="20" t="inlineStr">
         <is>
-          <t>https://ethz.ch/en/studies/master/application/dates.html</t>
+          <t>https://www.eco.usi.ch/en/feeds/9861</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – EPFL: شهریه CHF 2,240/ترم برای خارجی‌های غیرمقیم از پاییز ۲۰۲۵ (CHF 780 برای بقیه)</t>
+          <t>بورس – Essex Academic Excellence International Masters Scholarship: جدول کشوری (ایران ۱۴/۲۰ → £4,500؛ جدول ۲۰۲۵–۲۶)</t>
         </is>
       </c>
       <c r="B92" s="20" t="inlineStr">
         <is>
-          <t>https://www.epfl.ch/education/studies/en/rules-and-procedures/study-taxes/tuition-fee-other-fees/</t>
+          <t>https://www.essex.ac.uk/scholarships</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – EPFL: پنجره‌های اپلای ارشد (۱۵ دسامبر / ۳۱ مارس؛ یک برنامه در سال)</t>
+          <t>بورس – Teesside Global Excellence Scholarship £2,000 (پیشنهاد تا ۳۰ آوریل؛ رسمی)</t>
         </is>
       </c>
       <c r="B93" s="20" t="inlineStr">
         <is>
-          <t>https://www.epfl.ch/education/admission/admission-2/master-admission-criteria-application/online-application/</t>
+          <t>https://www.tees.ac.uk/sections/international/global_excellence_scholarship.cfm</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – UZH: شهریه CHF 720 + 100 (خارجی، ارشد) + 59؛ هزینهٔ درخواست CHF 150</t>
+          <t>بورس – Brunel Vice-Chancellor's Postgraduate International Excellence Award £6,000 (حداقل 2:1؛ ودیعهٔ £5,000)</t>
         </is>
       </c>
       <c r="B94" s="20" t="inlineStr">
         <is>
-          <t>https://www.uzh.ch/en/studies/application/fees.html</t>
+          <t>https://www.brunel.ac.uk/scholarships</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – UZH: مهلت ویزایی‌ها ۲۸ فوریه / بدون ویزا ۳۰ آوریل (پاییز)</t>
+          <t>بورس – Northumbria PGT International Scholarship £3,000: فهرست کشوری/ادامه‌تحصیلی‌های داخل UK — ایران نیست</t>
         </is>
       </c>
       <c r="B95" s="20" t="inlineStr">
         <is>
-          <t>https://www.oec.uzh.ch/en/studies/general/admission/master/faq-master-admission.html</t>
+          <t>https://www.mastersportal.com/scholarships/3890/pgt-international-scholarships.html</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – USI MSc Informatics: CHF 4,000/ترم غیرمقیم، B2 در ورود → C1، مهلت غیر-EU ۳۰ آوریل</t>
+          <t>بورس – Chevening eligibility (رسمی): ۲ سال کار بعد از مدرک کارشناسی + تعهد بازگشت ۲ ساله؛ مهلت ۶ اکتبر ۲۰۲۶</t>
         </is>
       </c>
       <c r="B96" s="20" t="inlineStr">
         <is>
-          <t>https://www.usi.ch/en/education/master/informatics</t>
+          <t>https://www.chevening.org/resource-hub/guidance/eligibility/</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – USI MSc Artificial Intelligence: CHF 4,000/ترم، IELTS 6.5</t>
+          <t>بورس – Deutschlandstipendium €300/ماه (رسمی)</t>
         </is>
       </c>
       <c r="B97" s="20" t="inlineStr">
         <is>
-          <t>https://www.topuniversities.com/universities/usi-universita-della-svizzera-italiana/postgrad/master-science-artificial-intelligence</t>
+          <t>https://www.deutschlandstipendium.de/</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – swissuniversities: شهریهٔ دانشگاه‌های علوم کاربردی 2026–27 (ZHAW 1,220؛ HSLU 1,300؛ OST 1,500؛ FHNW 1,000–5,000)</t>
+          <t>سوئیس – ETH: تاریخ‌های اپلای ارشد پاییز ۲۰۲۷ (۱–۳۰ نوامبر ۲۰۲۶؛ پاسخ تا پایان مارس؛ شروع ۲۰ سپتامبر ۲۰۲۷)</t>
         </is>
       </c>
       <c r="B98" s="20" t="inlineStr">
         <is>
-          <t>https://www.swissuniversities.ch/en/themen/lehre-studium/information-on-studies/tuition-fees/tuition-fees-at-uas</t>
+          <t>https://ethz.ch/en/studies/master/application/dates.html</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – ZHAW MSE: انگلیسی، 90 ECTS، پروفایل‌های CS/Data Science/Cyber، معدل A/B، مهلت پایان آوریل</t>
+          <t>سوئیس – EPFL: شهریه CHF 2,240/ترم برای خارجی‌های غیرمقیم از پاییز ۲۰۲۵ (CHF 780 برای بقیه)</t>
         </is>
       </c>
       <c r="B99" s="20" t="inlineStr">
         <is>
-          <t>https://www.zhaw.ch/en/engineering/study/masters-degree-programme</t>
+          <t>https://www.epfl.ch/education/studies/en/rules-and-procedures/study-taxes/tuition-fee-other-fees/</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – HSLU MSc Applied Information &amp; Data Science: C1 (B2 مشروط)، آلمانی لازم نیست، هر کارشناسی</t>
+          <t>سوئیس – EPFL: پنجره‌های اپلای ارشد (۱۵ دسامبر / ۳۱ مارس؛ یک برنامه در سال)</t>
         </is>
       </c>
       <c r="B100" s="20" t="inlineStr">
         <is>
-          <t>https://www.hslu.ch/en/lucerne-school-of-business/degree-programmes/master/applied-information-and-data-science/haeufig-gestellte-fragen/</t>
+          <t>https://www.epfl.ch/education/admission/admission-2/master-admission-criteria-application/online-application/</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – Bern: Swiss Joint MSc Computer Science (90 ECTS، انگلیسی، شرط کارشناسی CS)</t>
+          <t>سوئیس – UZH: شهریه CHF 720 + 100 (خارجی، ارشد) + 59؛ هزینهٔ درخواست CHF 150</t>
         </is>
       </c>
       <c r="B101" s="20" t="inlineStr">
         <is>
-          <t>https://www.philnat.unibe.ch/studies/study_programs/master_s_in_computer_science/index_eng.html</t>
+          <t>https://www.uzh.ch/en/studies/application/fees.html</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – Bern شهریه از پاییز ۲۰۲۶: CHF 850 + 1,700 اضافهٔ غیرسوئیسی‌ها + 34 + 25 در ترم (رسمی)</t>
+          <t>سوئیس – UZH: مهلت ویزایی‌ها ۲۸ فوریه / بدون ویزا ۳۰ آوریل (پاییز)</t>
         </is>
       </c>
       <c r="B102" s="20" t="inlineStr">
         <is>
-          <t>https://www.unibe.ch/studies/organizational_matters/renewal_of_semester_registration/fees/index_eng.html</t>
+          <t>https://www.oec.uzh.ch/en/studies/general/admission/master/faq-master-admission.html</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – Joint MSc CS (Bern/Neuchâtel/Fribourg) FAQ رسمی: بدون آزمون زبان (B2 توصیه)، شرط کارشناسی CS یا معادل با حداکثر ۶۰ ECTS تکمیلی، مهلت‌های دیرهنگام</t>
+          <t>سوئیس – USI MSc Informatics: CHF 4,000/ترم غیرمقیم، B2 در ورود → C1، مهلت غیر-EU ۳۰ آوریل</t>
         </is>
       </c>
       <c r="B103" s="20" t="inlineStr">
         <is>
-          <t>https://mcs.unibnf.ch/faq/</t>
+          <t>https://www.usi.ch/en/education/master/informatics</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – Neuchâtel شهریهٔ خارجی‌ها CHF 790/ترم (رسمی)</t>
+          <t>سوئیس – USI MSc Artificial Intelligence: CHF 4,000/ترم، IELTS 6.5</t>
         </is>
       </c>
       <c r="B104" s="20" t="inlineStr">
         <is>
-          <t>https://www.unine.ch/admission/taxes-universitaires/</t>
+          <t>https://www.topuniversities.com/universities/usi-universita-della-svizzera-italiana/postgrad/master-science-artificial-intelligence</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – Neuchâtel مهلت ارشد ۳۰ آوریل؛ خارجی‌ها یک ماه زودتر؛ هزینهٔ پرونده CHF 100 (رسمی)</t>
+          <t>سوئیس – swissuniversities: شهریهٔ دانشگاه‌های علوم کاربردی 2026–27 (ZHAW 1,220؛ HSLU 1,300؛ OST 1,500؛ FHNW 1,000–5,000)</t>
         </is>
       </c>
       <c r="B105" s="20" t="inlineStr">
         <is>
-          <t>https://www.unine.ch/admission/admission-master/delais-et-frais-dinscription-pour-les-masters/</t>
+          <t>https://www.swissuniversities.ch/en/themen/lehre-studium/information-on-studies/tuition-fees/tuition-fees-at-uas</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – Fribourg شهریهٔ خارجی‌ها CHF 870 + 115 = 985/ترم (رسمی)</t>
+          <t>سوئیس – ZHAW MSE: انگلیسی، 90 ECTS، پروفایل‌های CS/Data Science/Cyber، معدل A/B، مهلت پایان آوریل</t>
         </is>
       </c>
       <c r="B106" s="20" t="inlineStr">
         <is>
-          <t>https://www.unifr.ch/studies/en/organisation/administrative-services-unifr-students/university-fees/</t>
+          <t>https://www.zhaw.ch/en/engineering/study/masters-degree-programme</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – Fribourg مهلت ارشد با مدرک خارجی: ویزایی‌ها ۱–۲۸ فوریه، بقیه تا ۳۰ آوریل (رسمی)</t>
+          <t>سوئیس – HSLU MSc Applied Information &amp; Data Science: C1 (B2 مشروط)، آلمانی لازم نیست، هر کارشناسی</t>
         </is>
       </c>
       <c r="B107" s="20" t="inlineStr">
         <is>
-          <t>https://www.unifr.ch/studies/en/admission/admission-master/admission-master-foreign.html</t>
+          <t>https://www.hslu.ch/en/lucerne-school-of-business/degree-programmes/master/applied-information-and-data-science/haeufig-gestellte-fragen/</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – Basel MSc CS: 90 ECTS، انگلیسی، مهلت ۳۰ آوریل / ۳۰ نوامبر (رسمی)</t>
+          <t>سوئیس – Bern: Swiss Joint MSc Computer Science (90 ECTS، انگلیسی، شرط کارشناسی CS)</t>
         </is>
       </c>
       <c r="B108" s="20" t="inlineStr">
         <is>
-          <t>https://dmi.unibas.ch/en/studies/computer-science/masters/</t>
+          <t>https://www.philnat.unibe.ch/studies/study_programs/master_s_in_computer_science/index_eng.html</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – Basel شهریه CHF 850/ترم برای همه + CHF 100 هزینهٔ درخواست (Uni Info 2026/27)</t>
+          <t>سوئیس – Bern شهریه از پاییز ۲۰۲۶: CHF 850 + 1,700 اضافهٔ غیرسوئیسی‌ها + 34 + 25 در ترم (رسمی)</t>
         </is>
       </c>
       <c r="B109" s="20" t="inlineStr">
         <is>
-          <t>https://www.unibas.ch/dam/jcr:28672e66-8562-4988-9e38-b1c944ed22bf/COMPUTER%20SCIENCE%202026.2026-02-05-09-53-32.pdf</t>
+          <t>https://www.unibe.ch/studies/organizational_matters/renewal_of_semester_registration/fees/index_eng.html</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – HSLU MSc Applied Data Science and AI (نام جدید): مهلت ویزایی‌ها ۱ آوریل، CHF 1,300/ترم خارجی، CHF 250 درخواست، 120 ECTS (رسمی)</t>
+          <t>سوئیس – Joint MSc CS (Bern/Neuchâtel/Fribourg) FAQ رسمی: بدون آزمون زبان (B2 توصیه)، شرط کارشناسی CS یا معادل با حداکثر ۶۰ ECTS تکمیلی، مهلت‌های دیرهنگام</t>
         </is>
       </c>
       <c r="B110" s="20" t="inlineStr">
         <is>
-          <t>https://www.hslu.ch/en/lucerne-school-of-business/degree-programmes/master/applied-data-science-and-ai/</t>
+          <t>https://mcs.unibnf.ch/faq/</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – USI مهلت‌های 2026/27: غیر-EU ۳۰ آوریل؛ هزینهٔ پرونده CHF 100 برای مدارک خارج از کنوانسیون لیسبون (رسمی)</t>
+          <t>سوئیس – Neuchâtel شهریهٔ خارجی‌ها CHF 790/ترم (رسمی)</t>
         </is>
       </c>
       <c r="B111" s="20" t="inlineStr">
         <is>
-          <t>https://www.usi.ch/en/education/master/informatics/application</t>
+          <t>https://www.unine.ch/admission/taxes-universitaires/</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – SEM FAQ: ۶ ماه جست‌وجوی کار برای فارغ‌التحصیلان؛ اولویت داخلی/EU؛ سهمیه</t>
+          <t>سوئیس – Neuchâtel مهلت ارشد ۳۰ آوریل؛ خارجی‌ها یک ماه زودتر؛ هزینهٔ پرونده CHF 100 (رسمی)</t>
         </is>
       </c>
       <c r="B112" s="20" t="inlineStr">
         <is>
-          <t>https://www.sem.admin.ch/sem/en/home/themen/arbeit/faq.html</t>
+          <t>https://www.unine.ch/admission/admission-master/delais-et-frais-dinscription-pour-les-masters/</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – سهمیهٔ ۲۰۲۶ اتباع غیر-EU: ۴,۵۰۰ B + ۴,۰۰۰ L؛ شرایط FNIA</t>
+          <t>سوئیس – Fribourg شهریهٔ خارجی‌ها CHF 870 + 115 = 985/ترم (رسمی)</t>
         </is>
       </c>
       <c r="B113" s="20" t="inlineStr">
         <is>
-          <t>https://goldblum.ch/knowledgebase/residence-permit-in-switzerland-obtain/</t>
+          <t>https://www.unifr.ch/studies/en/organisation/administrative-services-unifr-students/university-fees/</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – Art. 21(3) FNIA: معافیت از آزمون بازار کار ولی نه از سهمیه؛ طرح 22.067 اجرا نشده</t>
+          <t>سوئیس – Fribourg مهلت ارشد با مدرک خارجی: ویزایی‌ها ۱–۲۸ فوریه، بقیه تا ۳۰ آوریل (رسمی)</t>
         </is>
       </c>
       <c r="B114" s="20" t="inlineStr">
         <is>
-          <t>https://vshcherbakov.com/2025/06/26/Path-to-working-permit-for-Swiss-graduates/</t>
+          <t>https://www.unifr.ch/studies/en/admission/admission-master/admission-master-foreign.html</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – اقامت تحصیلی ۲۰۲۶: CHF 21,000/سال، ۱۵ ساعت کار بعد از ۶ ماه، پردازش ۸–۱۲ هفته</t>
+          <t>سوئیس – Basel MSc CS: 90 ECTS، انگلیسی، مهلت ۳۰ آوریل / ۳۰ نوامبر (رسمی)</t>
         </is>
       </c>
       <c r="B115" s="20" t="inlineStr">
         <is>
-          <t>https://www.study-abroad.org/blog/ch-student-visa-guide/</t>
+          <t>https://dmi.unibas.ch/en/studies/computer-science/masters/</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – کانتون زوریخ: تمکن فقط در بانک مستقر در سوئیس به نام خودتان یا ضامن مقیم (راهنمای ZHAW)</t>
+          <t>سوئیس – Basel شهریه CHF 850/ترم برای همه + CHF 100 هزینهٔ درخواست (Uni Info 2026/27)</t>
         </is>
       </c>
       <c r="B116" s="20" t="inlineStr">
         <is>
-          <t>https://www.zhaw.ch/storage/sml/master/msc-bf-pie-information-for-international-students.pdf</t>
+          <t>https://www.unibas.ch/dam/jcr:28672e66-8562-4988-9e38-b1c944ed22bf/COMPUTER%20SCIENCE%202026.2026-02-05-09-53-32.pdf</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – تفاوت کانتون‌ها: Basel CHF 24,000؛ زوریخ حساب سوئیسی</t>
+          <t>سوئیس – HSLU MSc Applied Data Science and AI (نام جدید): مهلت ویزایی‌ها ۱ آوریل، CHF 1,300/ترم خارجی، CHF 250 درخواست، 120 ECTS (رسمی)</t>
         </is>
       </c>
       <c r="B117" s="20" t="inlineStr">
         <is>
-          <t>https://gradpilot.com/news/switzerland-student-visa-motivation-letter-canton-guide</t>
+          <t>https://www.hslu.ch/en/lucerne-school-of-business/degree-programmes/master/applied-data-science-and-ai/</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – اجازهٔ C: ۱۰ سال برای اتباع کشور ثالث، A2 شفاهی/A1 کتبی؛ ۵ سال با B1</t>
+          <t>سوئیس – USI مهلت‌های 2026/27: غیر-EU ۳۰ آوریل؛ هزینهٔ پرونده CHF 100 برای مدارک خارج از کنوانسیون لیسبون (رسمی)</t>
         </is>
       </c>
       <c r="B118" s="20" t="inlineStr">
         <is>
-          <t>https://relofinder.ch/blog/swiss-c-permit-permanent-residence-2026-guide/</t>
+          <t>https://www.usi.ch/en/education/master/informatics/application</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – اجازهٔ C: احتساب سال‌های تحصیل و شرایط ادغام</t>
+          <t>سوئیس – SEM FAQ: ۶ ماه جست‌وجوی کار برای فارغ‌التحصیلان؛ اولویت داخلی/EU؛ سهمیه</t>
         </is>
       </c>
       <c r="B119" s="20" t="inlineStr">
         <is>
-          <t>https://www.richmondchambers.ch/post/swiss-c-permit-eligibility-required-years-of-residence-integration-expectations-and-fast-track-pa</t>
+          <t>https://www.sem.admin.ch/sem/en/home/themen/arbeit/faq.html</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – سفارت تهران: ویزای D با وقت قبلی، ویزای C فعلاً نه (۳۰ ژانویه ۲۰۲۶)</t>
+          <t>سوئیس – سهمیهٔ ۲۰۲۶ اتباع غیر-EU: ۴,۵۰۰ B + ۴,۰۰۰ L؛ شرایط FNIA</t>
         </is>
       </c>
       <c r="B120" s="20" t="inlineStr">
         <is>
-          <t>https://www.eda.admin.ch/countries/iran/en/home.html</t>
+          <t>https://goldblum.ch/knowledgebase/residence-permit-in-switzerland-obtain/</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – حقوق مهندس نرم‌افزار ۲۰۲۶ (جونیور CHF 85–105k؛ خالص زوریخ)</t>
+          <t>سوئیس – Art. 21(3) FNIA: معافیت از آزمون بازار کار ولی نه از سهمیه؛ طرح 22.067 اجرا نشده</t>
         </is>
       </c>
       <c r="B121" s="20" t="inlineStr">
         <is>
-          <t>https://whatisthesalary.com/it-salaries/software-engineer-salary-in-switzerland/</t>
+          <t>https://vshcherbakov.com/2025/06/26/Path-to-working-permit-for-Swiss-graduates/</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – Glassdoor: میانهٔ Junior Software Engineer زوریخ CHF 92k</t>
+          <t>سوئیس – اقامت تحصیلی ۲۰۲۶: CHF 21,000/سال، ۱۵ ساعت کار بعد از ۶ ماه، پردازش ۸–۱۲ هفته</t>
         </is>
       </c>
       <c r="B122" s="20" t="inlineStr">
         <is>
-          <t>https://www.glassdoor.com/Salaries/z%C3%BCrich-junior-software-engineer-salary-SRCH_IL.0,6_IC3297851_KO7,31.htm</t>
+          <t>https://www.study-abroad.org/blog/ch-student-visa-guide/</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – بازهٔ حقوق زوریخ ۲۰۲۶ بر اساس نوع کارفرما</t>
+          <t>سوئیس – کانتون زوریخ: تمکن فقط در بانک مستقر در سوئیس به نام خودتان یا ضامن مقیم (راهنمای ZHAW)</t>
         </is>
       </c>
       <c r="B123" s="20" t="inlineStr">
         <is>
-          <t>https://upreer.ch/en/salaries/software-engineer-salary-zurich/</t>
+          <t>https://www.zhaw.ch/storage/sml/master/msc-bf-pie-information-for-international-students.pdf</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – هزینهٔ زندگی زوریخ CHF 2,000–2,200/ماه (UZH)</t>
+          <t>سوئیس – تفاوت کانتون‌ها: Basel CHF 24,000؛ زوریخ حساب سوئیسی</t>
         </is>
       </c>
       <c r="B124" s="20" t="inlineStr">
         <is>
-          <t>https://www.msfinance.uzh.ch/en/studyinginzurich/accommodation.html</t>
+          <t>https://gradpilot.com/news/switzerland-student-visa-motivation-letter-canton-guide</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – QS 2027: ETH 8، EPFL 22، UZH 98، Basel 150، Bern 191، USI 456، Fribourg 670، ZHAW 851–900</t>
+          <t>سوئیس – اجازهٔ C: ۱۰ سال برای اتباع کشور ثالث، A2 شفاهی/A1 کتبی؛ ۵ سال با B1</t>
         </is>
       </c>
       <c r="B125" s="20" t="inlineStr">
         <is>
-          <t>https://www.iamexpat.ch/education/education-news/eth-zurich-makes-top-universities-world</t>
+          <t>https://relofinder.ch/blog/swiss-c-permit-permanent-residence-2026-guide/</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – رد ابتکار «سوئیس ۱۰ میلیونی» SVP در ۱۴ ژوئن ۲۰۲۶ (۵۴.۸٪ نه)</t>
+          <t>سوئیس – اجازهٔ C: احتساب سال‌های تحصیل و شرایط ادغام</t>
         </is>
       </c>
       <c r="B126" s="20" t="inlineStr">
         <is>
-          <t>https://www.tagesanzeiger.ch/10-millionen-schweiz-resultate-der-svp-initiative-im-ticker-935664202454</t>
+          <t>https://www.richmondchambers.ch/post/swiss-c-permit-eligibility-required-years-of-residence-integration-expectations-and-fast-track-pa</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – EP27: کاهش ۷۸ میلیون فرانک بودجهٔ ETH؛ سناریوی چهاربرابر شدن شهریهٔ خارجی‌ها</t>
+          <t>سوئیس – سفارت تهران: ویزای D با وقت قبلی، ویزای C فعلاً نه (۳۰ ژانویه ۲۰۲۶)</t>
         </is>
       </c>
       <c r="B127" s="20" t="inlineStr">
         <is>
-          <t>https://www.efd.admin.ch/de/entlastungspaket-27</t>
+          <t>https://www.eda.admin.ch/countries/iran/en/home.html</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="4" t="inlineStr">
         <is>
-          <t>سوئیس – بازار IT ۲۰۲۶: استخدام گزینشی‌تر، بیکاری ≈ ۳.۲٪، کمبود ساختاری ICT</t>
+          <t>سوئیس – حقوق مهندس نرم‌افزار ۲۰۲۶ (جونیور CHF 85–105k؛ خالص زوریخ)</t>
         </is>
       </c>
       <c r="B128" s="20" t="inlineStr">
         <is>
-          <t>https://capiwell.ch/swiss-it-labour-market-2026-specialised-skills-slower-growth-and-new-openings-for-start-ups/</t>
+          <t>https://whatisthesalary.com/it-salaries/software-engineer-salary-in-switzerland/</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
         <is>
-          <t>نرخ CHF/USD ۲۷ سپتامبر ۲۰۲۶ (1.207)</t>
+          <t>سوئیس – Glassdoor: میانهٔ Junior Software Engineer زوریخ CHF 92k</t>
         </is>
       </c>
       <c r="B129" s="20" t="inlineStr">
         <is>
-          <t>https://www.xe.com/en-us/currencyconverter/convert/?Amount=1&amp;From=CHF&amp;To=USD</t>
+          <t>https://www.glassdoor.com/Salaries/z%C3%BCrich-junior-software-engineer-salary-SRCH_IL.0,6_IC3297851_KO7,31.htm</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="4" t="inlineStr">
         <is>
-          <t>بریتانیا – Graduate visa ۱۸ ماه (از ژانویه ۲۰۲۷)</t>
+          <t>سوئیس – بازهٔ حقوق زوریخ ۲۰۲۶ بر اساس نوع کارفرما</t>
         </is>
       </c>
       <c r="B130" s="20" t="inlineStr">
         <is>
-          <t>https://students.leeds.ac.uk/visa-information-after-studies/doc/graduate-visas</t>
+          <t>https://upreer.ch/en/salaries/software-engineer-salary-zurich/</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
         <is>
-          <t>بریتانیا – HC 584 (۳ سپتامبر ۲۰۲۶): تمکن £1,570 / £1,203 از ۳۰ نوامبر ۲۰۲۶</t>
+          <t>سوئیس – هزینهٔ زندگی زوریخ CHF 2,000–2,200/ماه (UZH)</t>
         </is>
       </c>
       <c r="B131" s="20" t="inlineStr">
         <is>
-          <t>https://www.gov.uk/government/publications/statement-of-changes-to-the-immigration-rules-hc-584-3-september-2026</t>
+          <t>https://www.msfinance.uzh.ch/en/studyinginzurich/accommodation.html</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="4" t="inlineStr">
         <is>
-          <t>بریتانیا – Skilled Worker نرخ شغل SOC 2134 £54,700</t>
+          <t>سوئیس – QS 2027: ETH 8، EPFL 22، UZH 98، Basel 150، Bern 191، USI 456، Fribourg 670، ZHAW 851–900</t>
         </is>
       </c>
       <c r="B132" s="20" t="inlineStr">
         <is>
-          <t>https://withrowan.co.uk/guides/skilled-worker-software-engineers</t>
+          <t>https://www.iamexpat.ch/education/education-news/eth-zurich-makes-top-universities-world</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
         <is>
-          <t>بریتانیا – Earned Settlement (وضعیت سپتامبر ۲۰۲۶)</t>
+          <t>سوئیس – رد ابتکار «سوئیس ۱۰ میلیونی» SVP در ۱۴ ژوئن ۲۰۲۶ (۵۴.۸٪ نه)</t>
         </is>
       </c>
       <c r="B133" s="20" t="inlineStr">
         <is>
-          <t>https://www.ukimmigration.law/earned-settlement-ilr-uk-plans/</t>
+          <t>https://www.tagesanzeiger.ch/10-millionen-schweiz-resultate-der-svp-initiative-im-ticker-935664202454</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Teesside MSc Computer Science 2026-27: £17,000، 2:2، IELTS 6.0</t>
+          <t>سوئیس – EP27: کاهش ۷۸ میلیون فرانک بودجهٔ ETH؛ سناریوی چهاربرابر شدن شهریهٔ خارجی‌ها</t>
         </is>
       </c>
       <c r="B134" s="20" t="inlineStr">
         <is>
-          <t>https://www.tees.ac.uk/postgraduate_courses/computing_&amp;_cyber_security/msc_computer_science.cfm</t>
+          <t>https://www.efd.admin.ch/de/entlastungspaket-27</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Northumbria MSc Advanced Computer Science 2026/27: £21,500، 2:2</t>
+          <t>سوئیس – بازار IT ۲۰۲۶: استخدام گزینشی‌تر، بیکاری ≈ ۳.۲٪، کمبود ساختاری ICT</t>
         </is>
       </c>
       <c r="B135" s="20" t="inlineStr">
         <is>
-          <t>https://www.northumbria.ac.uk/study-at-northumbria/courses/msc-advanced-computer-science-dtfava6/</t>
+          <t>https://capiwell.ch/swiss-it-labour-market-2026-specialised-skills-slower-growth-and-new-openings-for-start-ups/</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Leicester MSc Advanced Computer Science سپتامبر ۲۰۲۶: £24,250، 2:1</t>
+          <t>نرخ CHF/USD ۲۷ سپتامبر ۲۰۲۶ (1.207)</t>
         </is>
       </c>
       <c r="B136" s="20" t="inlineStr">
         <is>
-          <t>https://le.ac.uk/courses/advanced-computer-science-msc/2026</t>
+          <t>https://www.xe.com/en-us/currencyconverter/convert/?Amount=1&amp;From=CHF&amp;To=USD</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Essex MSc Advanced Computer Science 2026: £24,675، 2:2 (شامل Computer Engineering)</t>
+          <t>بریتانیا – Graduate visa ۱۸ ماه (از ژانویه ۲۰۲۷)</t>
         </is>
       </c>
       <c r="B137" s="20" t="inlineStr">
         <is>
-          <t>https://www.essex.ac.uk/courses/pg00435/1/msc-advanced-computer-science</t>
+          <t>https://students.leeds.ac.uk/visa-information-after-studies/doc/graduate-visas</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – York MSc Advanced Computer Science 2026/27: £32,900، 2:2، IELTS 6.5</t>
+          <t>بریتانیا – HC 584 (۳ سپتامبر ۲۰۲۶): تمکن £1,570 / £1,203 از ۳۰ نوامبر ۲۰۲۶</t>
         </is>
       </c>
       <c r="B138" s="20" t="inlineStr">
         <is>
-          <t>https://www.york.ac.uk/study/postgraduate-taught/courses/msc-advanced-computer-science/</t>
+          <t>https://www.gov.uk/government/publications/statement-of-changes-to-the-immigration-rules-hc-584-3-september-2026</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Chester MSc Advanced Computer Science 2026/27: £15,500 (کف قیمت انگلستان)</t>
+          <t>بریتانیا – Skilled Worker نرخ شغل SOC 2134 £54,700</t>
         </is>
       </c>
       <c r="B139" s="20" t="inlineStr">
         <is>
-          <t>https://www.chester.ac.uk/study/course-search/advanced-computer-science-msc/</t>
+          <t>https://withrowan.co.uk/guides/skilled-worker-software-engineers</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="4" t="inlineStr">
         <is>
-          <t>بریتانیا – Brunel MSc AI 2026/27 £24,795</t>
+          <t>بریتانیا – Earned Settlement (وضعیت سپتامبر ۲۰۲۶)</t>
         </is>
       </c>
       <c r="B140" s="20" t="inlineStr">
         <is>
-          <t>https://www.brunel.ac.uk/study/courses/artificial-intelligence-msc</t>
+          <t>https://www.ukimmigration.law/earned-settlement-ilr-uk-plans/</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
         <is>
-          <t>بریتانیا – عوارض £925 به ازای هر دانشجوی بین‌المللی (انگلستان، از 2028-29)</t>
+          <t>انگلستان – Teesside MSc Computer Science 2026-27: £17,000، 2:2، IELTS 6.0</t>
         </is>
       </c>
       <c r="B141" s="20" t="inlineStr">
         <is>
-          <t>https://www.researchprofessionalnews.com/rr-news-uk-politics-2025-11-international-levy-to-be-flat-fee-of-925-per-student/</t>
+          <t>https://www.tees.ac.uk/postgraduate_courses/computing_&amp;_cyber_security/msc_computer_science.cfm</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
         <is>
-          <t>بریتانیا – وضعیت VAC تهران</t>
+          <t>انگلستان – Northumbria MSc Advanced Computer Science 2026/27: £21,500، 2:2</t>
         </is>
       </c>
       <c r="B142" s="20" t="inlineStr">
         <is>
-          <t>https://livingintehran.com/2026/02/03/tehran-diplomatic-update-recent-embassy-reopenings-current-status-feb-2026/</t>
+          <t>https://www.northumbria.ac.uk/study-at-northumbria/courses/msc-advanced-computer-science-dtfava6/</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
         <is>
-          <t>QS WUR 2027 – TU Dresden</t>
+          <t>انگلستان – Leicester MSc Advanced Computer Science سپتامبر ۲۰۲۶: £24,250، 2:1</t>
         </is>
       </c>
       <c r="B143" s="20" t="inlineStr">
         <is>
-          <t>https://tu-dresden.de/tu-dresden/newsportal/news/qs-ranking-2027-tud-gehoert-erneut-zu-den-zehn-besten-universitaeten-deutschlands-und-baut-internationalen-erfolg-weiter-aus</t>
+          <t>https://le.ac.uk/courses/advanced-computer-science-msc/2026</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="4" t="inlineStr">
         <is>
-          <t>QS WUR 2027 – Stuttgart</t>
+          <t>انگلستان – Essex MSc Advanced Computer Science 2026: £24,675، 2:2 (شامل Computer Engineering)</t>
         </is>
       </c>
       <c r="B144" s="20" t="inlineStr">
         <is>
-          <t>https://www.uni-stuttgart.de/en/university/news/all/QS-World-University-Rankings-2027-The-University-of-Stuttgart-is-recognized-for-its-strong-research-performance-and-commitment-to-sustainability/</t>
+          <t>https://www.essex.ac.uk/courses/pg00435/1/msc-advanced-computer-science</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
         <is>
-          <t>QS WUR 2027 – Newcastle 149</t>
+          <t>انگلستان – York MSc Advanced Computer Science 2026/27: £32,900، 2:2، IELTS 6.5</t>
         </is>
       </c>
       <c r="B145" s="20" t="inlineStr">
         <is>
-          <t>https://www.ncl.ac.uk/press/articles/latest/2026/06/qs2027/</t>
+          <t>https://www.york.ac.uk/study/postgraduate-taught/courses/msc-advanced-computer-science/</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
         <is>
-          <t>QS WUR 2027 – York =158</t>
+          <t>انگلستان – Chester MSc Advanced Computer Science 2026/27: £15,500 (کف قیمت انگلستان)</t>
         </is>
       </c>
       <c r="B146" s="20" t="inlineStr">
         <is>
-          <t>https://www.york.ac.uk/about/rankings/</t>
+          <t>https://www.chester.ac.uk/study/course-search/advanced-computer-science-msc/</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
         <is>
-          <t>QS WUR 2027 – Leicester =314</t>
+          <t>بریتانیا – Brunel MSc AI 2026/27 £24,795</t>
         </is>
       </c>
       <c r="B147" s="20" t="inlineStr">
         <is>
-          <t>https://www.topuniversities.com/universities/university-leicester</t>
+          <t>https://www.brunel.ac.uk/study/courses/artificial-intelligence-msc</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
         <is>
-          <t>QS WUR 2027 – Essex =438</t>
+          <t>بریتانیا – عوارض £925 به ازای هر دانشجوی بین‌المللی (انگلستان، از 2028-29)</t>
         </is>
       </c>
       <c r="B148" s="20" t="inlineStr">
         <is>
-          <t>https://www.topuniversities.com/universities/essex-university</t>
+          <t>https://www.researchprofessionalnews.com/rr-news-uk-politics-2025-11-international-levy-to-be-flat-fee-of-925-per-student/</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
         <is>
-          <t>QS WUR 2027 – Northumbria =528</t>
+          <t>بریتانیا – وضعیت VAC تهران</t>
         </is>
       </c>
       <c r="B149" s="20" t="inlineStr">
         <is>
-          <t>https://www.topuniversities.com/universities/northumbria-university-newcastle</t>
+          <t>https://livingintehran.com/2026/02/03/tehran-diplomatic-update-recent-embassy-reopenings-current-status-feb-2026/</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
         <is>
-          <t>QS WUR 2027 – Brunel</t>
+          <t>QS WUR 2027 – TU Dresden</t>
         </is>
       </c>
       <c r="B150" s="20" t="inlineStr">
         <is>
-          <t>https://students.brunel.ac.uk/campus-news/brunel-climbs-global-qs-rankings-after-strong-year-for-research-and-graduate-outcomes</t>
+          <t>https://tu-dresden.de/tu-dresden/newsportal/news/qs-ranking-2027-tud-gehoert-erneut-zu-den-zehn-besten-universitaeten-deutschlands-und-baut-internationalen-erfolg-weiter-aus</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
         <is>
-          <t>QS WUR 2027 – سایر</t>
+          <t>QS WUR 2027 – Stuttgart</t>
         </is>
       </c>
       <c r="B151" s="20" t="inlineStr">
         <is>
-          <t>https://www.topuniversities.com/world-university-rankings</t>
+          <t>https://www.uni-stuttgart.de/en/university/news/all/QS-World-University-Rankings-2027-The-University-of-Stuttgart-is-recognized-for-its-strong-research-performance-and-commitment-to-sustainability/</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="4" t="inlineStr">
         <is>
-          <t>حداقل دستمزد ۲۰۲۶ هلند (€14.71)</t>
+          <t>QS WUR 2027 – Newcastle 149</t>
         </is>
       </c>
       <c r="B152" s="20" t="inlineStr">
         <is>
-          <t>https://arlettipartners.com/new-increase-in-the-dutch-minimum-hourly-wage-from-january-1st-2026/</t>
+          <t>https://www.ncl.ac.uk/press/articles/latest/2026/06/qs2027/</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
         <is>
-          <t>نرخ ارز (xe.com، ۲۷ سپتامبر ۲۰۲۶)</t>
+          <t>QS WUR 2027 – York =158</t>
         </is>
       </c>
       <c r="B153" s="20" t="inlineStr">
         <is>
-          <t>https://www.xe.com/</t>
+          <t>https://www.york.ac.uk/about/rankings/</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
         <is>
-          <t>بازار کار – LinkedIn/WEF ژانویه ۲۰۲۶: ۱.۳ میلیون شغل جدید AI؛ AI Engineer سریع‌ترین‌رشد</t>
+          <t>QS WUR 2027 – Leicester =314</t>
         </is>
       </c>
       <c r="B154" s="20" t="inlineStr">
         <is>
-          <t>https://www.weforum.org/stories/jobs-and-the-future-of-work/ai-has-already-added-1-3-million-new-jobs-according-to-linkedin-data/</t>
+          <t>https://www.topuniversities.com/universities/university-leicester</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
         <is>
-          <t>بازار کار – Bitkom 2025: ۱۰۹ هزار جای خالی IT در آلمان، ۷.۷ ماه زمان پرکردن</t>
+          <t>QS WUR 2027 – Essex =438</t>
         </is>
       </c>
       <c r="B155" s="20" t="inlineStr">
         <is>
-          <t>https://www.bitkom.org/Bitkom/Publikationen/Der-Arbeitsmarkt-fuer-IT-Fachkraefte</t>
+          <t>https://www.topuniversities.com/universities/essex-university</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
         <is>
-          <t>بازار کار – ISC2 Cybersecurity Workforce Study 2024/2025 (حذف عدد کمبود؛ کمبود بودجه دلیل اول؛ ۳۱٪ تیم‌ها بدون جونیور)</t>
+          <t>QS WUR 2027 – Northumbria =528</t>
         </is>
       </c>
       <c r="B156" s="20" t="inlineStr">
         <is>
-          <t>https://www.isc2.org/research</t>
+          <t>https://www.topuniversities.com/universities/northumbria-university-newcastle</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
         <is>
-          <t>بازار کار – اخراج‌های صنعت بازی ۲۰۲۲–۲۰۲۶ (≈۴۵ هزار؛ افت حقوق Unity)</t>
+          <t>QS WUR 2027 – Brunel</t>
         </is>
       </c>
       <c r="B157" s="20" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/2022%E2%80%932026_video_game_industry_layoffs</t>
+          <t>https://students.brunel.ac.uk/campus-news/brunel-climbs-global-qs-rankings-after-strong-year-for-research-and-graduate-outcomes</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
         <is>
-          <t>بازار کار – آگهی‌های UX/UXR (Indeed تا Q4 2025)</t>
+          <t>QS WUR 2027 – سایر</t>
         </is>
       </c>
       <c r="B158" s="20" t="inlineStr">
         <is>
-          <t>https://www.thevoiceofuser.com/everyone-knows-the-uxr-hiring-market-is-bad-how-bad-is-it-though/</t>
+          <t>https://www.topuniversities.com/world-university-rankings</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
         <is>
-          <t>بازار کار – اشباع جونیور علم داده ۲۰۲۶</t>
+          <t>حداقل دستمزد ۲۰۲۶ هلند (€14.71)</t>
         </is>
       </c>
       <c r="B159" s="20" t="inlineStr">
         <is>
-          <t>https://research.com/advice/are-too-many-students-choosing-data-science-oversaturation-competition-hiring-reality</t>
+          <t>https://arlettipartners.com/new-increase-in-the-dutch-minimum-hourly-wage-from-january-1st-2026/</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
         <is>
-          <t>آلمان – Saarland MSc Cybersecurity (C1، بدون شهریه)</t>
+          <t>نرخ ارز (xe.com، ۲۷ سپتامبر ۲۰۲۶)</t>
         </is>
       </c>
       <c r="B160" s="20" t="inlineStr">
         <is>
-          <t>https://www.uni-saarland.de/en/study/programmes/master/cybersecurity.html</t>
+          <t>https://www.xe.com/</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
         <is>
-          <t>آلمان – Passau MSc AI Engineering (B2، معدل ≤ 2.7، A1 آلمانی سال اول)</t>
+          <t>بازار کار – LinkedIn/WEF ژانویه ۲۰۲۶: ۱.۳ میلیون شغل جدید AI؛ AI Engineer سریع‌ترین‌رشد</t>
         </is>
       </c>
       <c r="B161" s="20" t="inlineStr">
         <is>
-          <t>https://www.uni-passau.de/en/msc-ai-eng</t>
+          <t>https://www.weforum.org/stories/jobs-and-the-future-of-work/ai-has-already-added-1-3-million-new-jobs-according-to-linkedin-data/</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
         <is>
-          <t>آلمان – Cologne Game Lab MA Game Development &amp; Research (€2,500/ترم غیر-EU)</t>
+          <t>بازار کار – Bitkom 2025: ۱۰۹ هزار جای خالی IT در آلمان، ۷.۷ ماه زمان پرکردن</t>
         </is>
       </c>
       <c r="B162" s="20" t="inlineStr">
         <is>
-          <t>https://colognegamelab.de/study-programs/post-graduate-programs/game-development-research-ma/faqs/</t>
+          <t>https://www.bitkom.org/Bitkom/Publikationen/Der-Arbeitsmarkt-fuer-IT-Fachkraefte</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
         <is>
-          <t>آلمان – Siegen MSc HCI (DAAD)</t>
+          <t>بازار کار – ISC2 Cybersecurity Workforce Study 2024/2025 (حذف عدد کمبود؛ کمبود بودجه دلیل اول؛ ۳۱٪ تیم‌ها بدون جونیور)</t>
         </is>
       </c>
       <c r="B163" s="20" t="inlineStr">
         <is>
-          <t>https://www2.daad.de/deutschland/studienangebote/international-programmes/en/detail/4686/</t>
+          <t>https://www.isc2.org/research</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
         <is>
-          <t>آلمان – H-BRS MSc Autonomous Systems (B2+)</t>
+          <t>بازار کار – اخراج‌های صنعت بازی ۲۰۲۲–۲۰۲۶ (≈۴۵ هزار؛ افت حقوق Unity)</t>
         </is>
       </c>
       <c r="B164" s="20" t="inlineStr">
         <is>
-          <t>https://www.h-brs.de/en/inf/admission-application-master-autonomous-systems</t>
+          <t>https://en.wikipedia.org/wiki/2022%E2%80%932026_video_game_industry_layoffs</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
         <is>
-          <t>آلمان – RWTH MSc Software Systems Engineering</t>
+          <t>بازار کار – آگهی‌های UX/UXR (Indeed تا Q4 2025)</t>
         </is>
       </c>
       <c r="B165" s="20" t="inlineStr">
         <is>
-          <t>https://sc.informatik.rwth-aachen.de/en/studium/master/sse/</t>
+          <t>https://www.thevoiceofuser.com/everyone-knows-the-uxr-hiring-market-is-bad-how-bad-is-it-though/</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
         <is>
-          <t>آلمان – Tübingen MSc Machine Learning (IELTS 7، €1,500/ترم)</t>
+          <t>بازار کار – اشباع جونیور علم داده ۲۰۲۶</t>
         </is>
       </c>
       <c r="B166" s="20" t="inlineStr">
         <is>
-          <t>https://uni-tuebingen.de/fakultaeten/mathematisch-naturwissenschaftliche-fakultaet/fachbereiche/informatik/studium/studierende/lehre-studienorganisation/studiengaenge/machine-learning/admission-and-application/</t>
+          <t>https://research.com/advice/are-too-many-students-choosing-data-science-oversaturation-competition-hiring-reality</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
         <is>
-          <t>آلمان – TUM Informatics: €6,000 در ترم برای غیر-EU</t>
+          <t>آلمان – Saarland MSc Cybersecurity (C1، بدون شهریه)</t>
         </is>
       </c>
       <c r="B167" s="20" t="inlineStr">
         <is>
-          <t>https://www.tum.de/en/studies/degree-programs/detail/informatics-master-of-science-msc</t>
+          <t>https://www.uni-saarland.de/en/study/programmes/master/cybersecurity.html</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="4" t="inlineStr">
         <is>
-          <t>آلمان – FAU Autonomy Technologies (B2، IELTS 6.0)</t>
+          <t>آلمان – Passau MSc AI Engineering (B2، معدل ≤ 2.7، A1 آلمانی سال اول)</t>
         </is>
       </c>
       <c r="B168" s="20" t="inlineStr">
         <is>
-          <t>https://www.fau.eu/degree-program/autonomy-technologies-m-sc/</t>
+          <t>https://www.uni-passau.de/en/msc-ai-eng</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
         <is>
-          <t>هلند – Twente Embedded Systems 2026/27: €21,700</t>
+          <t>آلمان – Cologne Game Lab MA Game Development &amp; Research (€2,500/ترم غیر-EU)</t>
         </is>
       </c>
       <c r="B169" s="20" t="inlineStr">
         <is>
-          <t>https://www.utwente.nl/en/education/master/programmes/embedded-systems/finance/</t>
+          <t>https://colognegamelab.de/study-programs/post-graduate-programs/game-development-research-ma/faqs/</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="4" t="inlineStr">
         <is>
-          <t>هلند – Leiden CS 2026/27: €22,500</t>
+          <t>آلمان – Siegen MSc HCI (DAAD)</t>
         </is>
       </c>
       <c r="B170" s="20" t="inlineStr">
         <is>
-          <t>https://www.universiteitleiden.nl/en/education/study-programmes/master/computer-science/artificial-intelligence/admission-and-application/tuition-fees</t>
+          <t>https://www2.daad.de/deutschland/studienangebote/international-programmes/en/detail/4686/</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
         <is>
-          <t>هلند – Groningen AI 2026/27: €24,900</t>
+          <t>آلمان – H-BRS MSc Autonomous Systems (B2+)</t>
         </is>
       </c>
       <c r="B171" s="20" t="inlineStr">
         <is>
-          <t>https://www.rug.nl/masters/artificial-intelligence/?lang=en</t>
+          <t>https://www.h-brs.de/en/inf/admission-application-master-autonomous-systems</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
         <is>
-          <t>هلند – Utrecht Game &amp; Media Technology 2026/27: €25,306</t>
+          <t>آلمان – RWTH MSc Software Systems Engineering</t>
         </is>
       </c>
       <c r="B172" s="20" t="inlineStr">
         <is>
-          <t>https://www.uu.nl/en/masters/game-and-media-technology</t>
+          <t>https://sc.informatik.rwth-aachen.de/en/studium/master/sse/</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
         <is>
-          <t>هلند – QS 2027 فهرست دانشگاه‌های هلند</t>
+          <t>آلمان – Tübingen MSc Machine Learning (IELTS 7، €1,500/ترم)</t>
         </is>
       </c>
       <c r="B173" s="20" t="inlineStr">
         <is>
-          <t>https://dub.uu.nl/en/news/dutch-universities-fall-global-qs-rankings</t>
+          <t>https://uni-tuebingen.de/fakultaeten/mathematisch-naturwissenschaftliche-fakultaet/fachbereiche/informatik/studium/studierende/lehre-studienorganisation/studiengaenge/machine-learning/admission-and-application/</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
         <is>
-          <t>سوئد – Gothenburg Game Design &amp; Technology: SEK 290,000 کل</t>
+          <t>آلمان – TUM Informatics: €6,000 در ترم برای غیر-EU</t>
         </is>
       </c>
       <c r="B174" s="20" t="inlineStr">
         <is>
-          <t>https://www.gu.se/en/study-gothenburg/game-design-technology-masters-programme-n2gdt</t>
+          <t>https://www.tum.de/en/studies/degree-programs/detail/informatics-master-of-science-msc</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
         <is>
-          <t>سوئد – KTH Machine Learning: ≈ SEK 180,000–190,000 (کل دوره 360k طبق راهنمای ۲۰۲۶؛ kth.se رقم را فقط در سامانه نشان می‌دهد)</t>
+          <t>آلمان – FAU Autonomy Technologies (B2، IELTS 6.0)</t>
         </is>
       </c>
       <c r="B175" s="20" t="inlineStr">
         <is>
-          <t>https://www.kth.se/en/studies/master/machine-learning</t>
+          <t>https://www.fau.eu/degree-program/autonomy-technologies-m-sc/</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="4" t="inlineStr">
         <is>
-          <t>سوئد – Umeå AI: SEK 152,300</t>
+          <t>هلند – Twente Embedded Systems 2026/27: €21,700</t>
         </is>
       </c>
       <c r="B176" s="20" t="inlineStr">
         <is>
-          <t>https://www.umu.se/en/education/master/masters-programme-in-artificial-intelligence/</t>
+          <t>https://www.utwente.nl/en/education/master/programmes/embedded-systems/finance/</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
         <is>
-          <t>سوئد – QS 2027 فهرست دانشگاه‌های سوئد</t>
+          <t>هلند – Leiden CS 2026/27: €22,500</t>
         </is>
       </c>
       <c r="B177" s="20" t="inlineStr">
         <is>
-          <t>https://www.study.eu/best-universities/sweden</t>
+          <t>https://www.universiteitleiden.nl/en/education/study-programmes/master/computer-science/artificial-intelligence/admission-and-application/tuition-fees</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
         <is>
-          <t>دانمارک – ITU شهریهٔ رسمی ورودی ۲۰۲۶: €8,250 در ترم = €16,500 در سال (رقم قدیمی €6,700 منسوخ)</t>
+          <t>هلند – Groningen AI 2026/27: €24,900</t>
         </is>
       </c>
       <c r="B178" s="20" t="inlineStr">
         <is>
-          <t>https://en.itu.dk/Programmes/MSc-Programmes/Applying-to-a-MSc-programme/Non-EU-EOES</t>
+          <t>https://www.rug.nl/masters/artificial-intelligence/?lang=en</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
         <is>
-          <t>دانمارک – AAU Cyber Security / Medialogy €7,455 در ترم</t>
+          <t>هلند – Utrecht Game &amp; Media Technology 2026/27: €25,306</t>
         </is>
       </c>
       <c r="B179" s="20" t="inlineStr">
         <is>
-          <t>https://studyindenmark.dk/portal/aalborg-university-aau/copenhagen/cyber-security-msc-in-engineering</t>
+          <t>https://www.uu.nl/en/masters/game-and-media-technology</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="4" t="inlineStr">
         <is>
-          <t>دانمارک – DTU €15,000 (Human-Centered AI / Autonomous Systems)</t>
+          <t>هلند – QS 2027 فهرست دانشگاه‌های هلند</t>
         </is>
       </c>
       <c r="B180" s="20" t="inlineStr">
         <is>
-          <t>https://www.dtu.dk/english/education/graduate/msc-programmes/autonomous-systems/prerequisites</t>
+          <t>https://dub.uu.nl/en/news/dutch-universities-fall-global-qs-rankings</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
         <is>
-          <t>دانمارک – Aarhus CS €17,300</t>
+          <t>سوئد – Gothenburg Game Design &amp; Technology: SEK 290,000 کل</t>
         </is>
       </c>
       <c r="B181" s="20" t="inlineStr">
         <is>
-          <t>https://masters.au.dk/computerscience</t>
+          <t>https://www.gu.se/en/study-gothenburg/game-design-technology-masters-programme-n2gdt</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
         <is>
-          <t>دانمارک – QS 2027 فهرست دانشگاه‌های دانمارک</t>
+          <t>سوئد – KTH Machine Learning: ≈ SEK 180,000–190,000 (کل دوره 360k طبق راهنمای ۲۰۲۶؛ kth.se رقم را فقط در سامانه نشان می‌دهد)</t>
         </is>
       </c>
       <c r="B182" s="20" t="inlineStr">
         <is>
-          <t>https://leapscholar.com/blog/top-universities-in-denmark/</t>
+          <t>https://www.kth.se/en/studies/master/machine-learning</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Goldsmiths MSc Computer Games Programming £22,000</t>
+          <t>سوئد – Umeå AI: SEK 152,300</t>
         </is>
       </c>
       <c r="B183" s="20" t="inlineStr">
         <is>
-          <t>https://www.gold.ac.uk/pg/msc-computer-games-programming/</t>
+          <t>https://www.umu.se/en/education/master/masters-programme-in-artificial-intelligence/</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Royal Holloway MSc Information &amp; Cyber Security £25,500</t>
+          <t>سوئد – QS 2027 فهرست دانشگاه‌های سوئد</t>
         </is>
       </c>
       <c r="B184" s="20" t="inlineStr">
         <is>
-          <t>https://www.royalholloway.ac.uk/studying-here/postgraduate/information-security/information-and-cyber-security/</t>
+          <t>https://www.study.eu/best-universities/sweden</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Kent MSc Cyber Security (NCSC)</t>
+          <t>دانمارک – ITU شهریهٔ رسمی ورودی ۲۰۲۶: €8,250 در ترم = €16,500 در سال (رقم قدیمی €6,700 منسوخ)</t>
         </is>
       </c>
       <c r="B185" s="20" t="inlineStr">
         <is>
-          <t>https://www.kent.ac.uk/courses/postgraduate/1225/cyber-security</t>
+          <t>https://en.itu.dk/Programmes/MSc-Programmes/Applying-to-a-MSc-programme/Non-EU-EOES</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – MMU MSc Cyber Security £21,000</t>
+          <t>دانمارک – AAU Cyber Security / Medialogy €7,455 در ترم</t>
         </is>
       </c>
       <c r="B186" s="20" t="inlineStr">
         <is>
-          <t>https://www.mmu.ac.uk/study/postgraduate/course/msc-cyber-security</t>
+          <t>https://studyindenmark.dk/portal/aalborg-university-aau/copenhagen/cyber-security-msc-in-engineering</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – York MSc Human-Centred Interactive Technologies £32,900</t>
+          <t>دانمارک – DTU €15,000 (Human-Centered AI / Autonomous Systems)</t>
         </is>
       </c>
       <c r="B187" s="20" t="inlineStr">
         <is>
-          <t>https://www.york.ac.uk/study/postgraduate-taught/courses/msc-human-centred-interactive-technologies/</t>
+          <t>https://www.dtu.dk/english/education/graduate/msc-programmes/autonomous-systems/prerequisites</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Lancaster MSc Cyber Security £30,000</t>
+          <t>دانمارک – Aarhus CS €17,300</t>
         </is>
       </c>
       <c r="B188" s="20" t="inlineStr">
         <is>
-          <t>https://www.lancaster.ac.uk/study/postgraduate/postgraduate-courses/cyber-security-msc/2026/</t>
+          <t>https://masters.au.dk/computerscience</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – NTU QS 2027 =639</t>
+          <t>دانمارک – QS 2027 فهرست دانشگاه‌های دانمارک</t>
         </is>
       </c>
       <c r="B189" s="20" t="inlineStr">
         <is>
-          <t>https://collegedunia.com/uk/university/862-nottingham-trent-university-nottingham/ranking</t>
+          <t>https://leapscholar.com/blog/top-universities-in-denmark/</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
         <is>
-          <t>آلمان – FAU: شهریهٔ غیر-EU از ترم تابستان ۲۰۲۷ (AI/CS €4,000، Autonomy Tech €2,000 در ترم؛ BayHIG §13)</t>
+          <t>انگلستان – Goldsmiths MSc Computer Games Programming £22,000</t>
         </is>
       </c>
       <c r="B190" s="20" t="inlineStr">
         <is>
-          <t>https://www.fau.eu/studying/international-students/application-and-enrollment-for-international-applicants/tuition-fees-for-students-from-non-eu-states/</t>
+          <t>https://www.gold.ac.uk/pg/msc-computer-games-programming/</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
         <is>
-          <t>آلمان – Passau: «فعلاً» بدون شهریه برای غیر-EU (اعلام رسمی)</t>
+          <t>انگلستان – Royal Holloway MSc Information &amp; Cyber Security £25,500</t>
         </is>
       </c>
       <c r="B191" s="20" t="inlineStr">
         <is>
-          <t>https://www.uni-passau.de/en/study/news/news/no-tuition-fees-for-international-students-at-the-university-of-passau</t>
+          <t>https://www.royalholloway.ac.uk/studying-here/postgraduate/information-security/information-and-cyber-security/</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
         <is>
-          <t>دانمارک – Aarhus نرخ رسمی 2026/27: Computer Science / Data Science / Computer Engineering €17,300</t>
+          <t>انگلستان – Kent MSc Cyber Security (NCSC)</t>
         </is>
       </c>
       <c r="B192" s="20" t="inlineStr">
         <is>
-          <t>https://masters.au.dk/tuitionfees/current-tuition-fee-rates</t>
+          <t>https://www.kent.ac.uk/courses/postgraduate/1225/cyber-security</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="4" t="inlineStr">
         <is>
-          <t>دانمارک – AAU Computer Science (IT): شرط رسمی ≥ ۱۵۰ ECTS دروس CS؛ معیار رتبه‌بندی ۲۰۲۷ شامل سابقهٔ کار</t>
+          <t>انگلستان – MMU MSc Cyber Security £21,000</t>
         </is>
       </c>
       <c r="B193" s="20" t="inlineStr">
         <is>
-          <t>https://www.en.aau.dk/education/master/computer-science-it</t>
+          <t>https://www.mmu.ac.uk/study/postgraduate/course/msc-cyber-security</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="4" t="inlineStr">
         <is>
-          <t>سوئد – Chalmers شهریهٔ استاندارد 2026/27 ≈ SEK 175,000 (collegedunia به نقل از صفحهٔ شهریهٔ Chalmers)</t>
+          <t>انگلستان – York MSc Human-Centred Interactive Technologies £32,900</t>
         </is>
       </c>
       <c r="B194" s="20" t="inlineStr">
         <is>
-          <t>https://collegedunia.com/sweden/university/769-chalmers-university-of-technology-gothenburg/programs?stream_id=48&amp;degree_type=Master</t>
+          <t>https://www.york.ac.uk/study/postgraduate-taught/courses/msc-human-centred-interactive-technologies/</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Surrey MSc Cyber Security ورودی ۲۰۲۷: £25,900 (فوریه) / £26,900 (سپتامبر)</t>
+          <t>انگلستان – Lancaster MSc Cyber Security £30,000</t>
         </is>
       </c>
       <c r="B195" s="20" t="inlineStr">
         <is>
-          <t>https://www.surrey.ac.uk/postgraduate/cyber-security-msc</t>
+          <t>https://www.lancaster.ac.uk/study/postgraduate/postgraduate-courses/cyber-security-msc/2026/</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
         <is>
-          <t>انگلستان – Newcastle MSc Computer Game Engineering £32,300، شرط 2:2 (QS TopUniversities)</t>
+          <t>انگلستان – NTU QS 2027 =639</t>
         </is>
       </c>
       <c r="B196" s="20" t="inlineStr">
         <is>
-          <t>https://www.topuniversities.com/universities/newcastle-university/postgrad/msc-computer-game-engineering</t>
+          <t>https://collegedunia.com/uk/university/862-nottingham-trent-university-nottingham/ranking</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
         <is>
-          <t>هلند – TU/e شهریهٔ رسمی 2026/27 €21,700 (2027/28: €22,400)</t>
+          <t>آلمان – FAU: شهریهٔ غیر-EU از ترم تابستان ۲۰۲۷ (AI/CS €4,000، Autonomy Tech €2,000 در ترم؛ BayHIG §13)</t>
         </is>
       </c>
       <c r="B197" s="20" t="inlineStr">
         <is>
-          <t>https://www.tue.nl/en/education/become-a-tue-student/tuition-fees</t>
+          <t>https://www.fau.eu/studying/international-students/application-and-enrollment-for-international-applicants/tuition-fees-for-students-from-non-eu-states/</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="4" t="inlineStr">
         <is>
-          <t>ایران – توقف برگزاری IELTS در ایران از ۳۱ ژانویه ۲۰۲۶ (اعلام IDP)</t>
+          <t>آلمان – Passau: «فعلاً» بدون شهریه برای غیر-EU (اعلام رسمی)</t>
         </is>
       </c>
       <c r="B198" s="20" t="inlineStr">
         <is>
-          <t>https://wanaen.com/ielts-testing-to-be-suspended-in-iran/</t>
+          <t>https://www.uni-passau.de/en/study/news/news/no-tuition-fees-for-international-students-at-the-university-of-passau</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="4" t="inlineStr">
         <is>
-          <t>ایران – وضعیت IELTS شهریور ۱۴۰۵: در ایران برگزار نمی‌شود؛ آزمون در کشور دیگر</t>
+          <t>دانمارک – Aarhus نرخ رسمی 2026/27: Computer Science / Data Science / Computer Engineering €17,300</t>
         </is>
       </c>
       <c r="B199" s="20" t="inlineStr">
         <is>
-          <t>https://www.jahantahsil.com/%D8%A2%D8%B2%D9%85%D9%88%D9%86-%D8%A2%DB%8C%D9%84%D8%AA%D8%B3-ielts-%DA%86%DB%8C%D8%B3%D8%AA-%D9%88-%DA%A9%D8%AC%D8%A7-%D8%A8%D8%B1%DA%AF%D8%B2%D8%A7%D8%B1-%D9%85%DB%8C%D8%B4%D9%88%D8%AF/</t>
+          <t>https://masters.au.dk/tuitionfees/current-tuition-fee-rates</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="4" t="inlineStr">
         <is>
-          <t>ایران – توقف TOEFL در ایران (وضعیت شهریور ۱۴۰۵)</t>
+          <t>دانمارک – AAU Computer Science (IT): شرط رسمی ≥ ۱۵۰ ECTS دروس CS؛ معیار رتبه‌بندی ۲۰۲۷ شامل سابقهٔ کار</t>
         </is>
       </c>
       <c r="B200" s="20" t="inlineStr">
         <is>
-          <t>https://zandienglish.ir/toefl-in-iran/</t>
+          <t>https://www.en.aau.dk/education/master/computer-science-it</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="4" t="inlineStr">
         <is>
-          <t>ایران – وثیقهٔ خروج تحصیلی مشمولان ۲۰۰ میلیون تومان (سامانهٔ سخا، تیر ۱۴۰۵)</t>
+          <t>سوئد – Chalmers شهریهٔ استاندارد 2026/27 ≈ SEK 175,000 (collegedunia به نقل از صفحهٔ شهریهٔ Chalmers)</t>
         </is>
       </c>
       <c r="B201" s="20" t="inlineStr">
         <is>
-          <t>https://www.zoomit.ir/iran-news/464136-exit-permit-bond-sakha-1405/</t>
+          <t>https://collegedunia.com/sweden/university/769-chalmers-university-of-technology-gothenburg/programs?stream_id=48&amp;degree_type=Master</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="4" t="inlineStr">
         <is>
-          <t>سوئد – تاریخ‌های کلیدی ورودی پاییز ۲۰۲۷ (۱۶ اکتبر – ۱۵ ژانویه؛ مدارک ۱ فوریه؛ دور دوم ۱۵ آوریل)</t>
+          <t>انگلستان – Surrey MSc Cyber Security ورودی ۲۰۲۷: £25,900 (فوریه) / £26,900 (سپتامبر)</t>
         </is>
       </c>
       <c r="B202" s="20" t="inlineStr">
         <is>
-          <t>https://www.umu.se/en/education/application-and-admission/key-dates-and-deadlines/</t>
+          <t>https://www.surrey.ac.uk/postgraduate/cyber-security-msc</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="4" t="inlineStr">
         <is>
-          <t>آلمان – Stuttgart MSc CS: بازهٔ اپلای ترم زمستان ۱۵ نوامبر – ۱۵ ژانویه؛ انگلیسی C1</t>
+          <t>انگلستان – Newcastle MSc Computer Game Engineering £32,300، شرط 2:2 (QS TopUniversities)</t>
         </is>
       </c>
       <c r="B203" s="20" t="inlineStr">
         <is>
-          <t>https://www.uni-stuttgart.de/en/study/study-programs/Computer-Science-M.Sc.-00001/</t>
+          <t>https://www.topuniversities.com/universities/newcastle-university/postgrad/msc-computer-game-engineering</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="4" t="inlineStr">
         <is>
-          <t>آلمان – Passau: بازهٔ اپلای AI Engineering ۱ آوریل – ۳۱ می</t>
+          <t>هلند – TU/e شهریهٔ رسمی 2026/27 €21,700 (2027/28: €22,400)</t>
         </is>
       </c>
       <c r="B204" s="20" t="inlineStr">
         <is>
-          <t>https://www.uni-passau.de/en/apply/apply-with-intl-qualifications</t>
+          <t>https://www.tue.nl/en/education/become-a-tue-student/tuition-fees</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="4" t="inlineStr">
         <is>
-          <t>دانمارک – AAU: مهلت شهریه‌پردازها ۱۵ ژانویه (EU: ۱ مارس)؛ پورتال از اواسط دسامبر</t>
+          <t>ایران – توقف برگزاری IELTS در ایران از ۳۱ ژانویه ۲۰۲۶ (اعلام IDP)</t>
         </is>
       </c>
       <c r="B205" s="20" t="inlineStr">
         <is>
-          <t>https://www.en.aau.dk/education/apply/master/how-and-when-to-apply</t>
+          <t>https://wanaen.com/ielts-testing-to-be-suspended-in-iran/</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="4" t="inlineStr">
         <is>
-          <t>دانمارک – SDU Computer Science: مهلت غیر-EU ۱ فوریه؛ شهریه یک سال پیش‌پرداخت</t>
+          <t>ایران – وضعیت IELTS شهریور ۱۴۰۵: در ایران برگزار نمی‌شود؛ آزمون در کشور دیگر</t>
         </is>
       </c>
       <c r="B206" s="20" t="inlineStr">
         <is>
-          <t>https://www.sdu.dk/en/uddannelse/kandidat/datalogi</t>
+          <t>https://www.jahantahsil.com/%D8%A2%D8%B2%D9%85%D9%88%D9%86-%D8%A2%DB%8C%D9%84%D8%AA%D8%B3-ielts-%DA%86%DB%8C%D8%B3%D8%AA-%D9%88-%DA%A9%D8%AC%D8%A7-%D8%A8%D8%B1%DA%AF%D8%B2%D8%A7%D8%B1-%D9%85%DB%8C%D8%B4%D9%88%D8%AF/</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="4" t="inlineStr">
         <is>
-          <t>هلند – Radboud: مهلت غیر-EU ۱ آوریل، بورس ۳۱ ژانویه، ثبت‌نام ۱ ژوئن</t>
+          <t>ایران – توقف TOEFL در ایران (وضعیت شهریور ۱۴۰۵)</t>
         </is>
       </c>
       <c r="B207" s="20" t="inlineStr">
         <is>
-          <t>https://www.ru.nl/en/education/application-and-admission/application-procedure-masters/deadlines</t>
+          <t>https://zandienglish.ir/toefl-in-iran/</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="4" t="inlineStr">
         <is>
+          <t>ایران – وثیقهٔ خروج تحصیلی مشمولان ۲۰۰ میلیون تومان (سامانهٔ سخا، تیر ۱۴۰۵)</t>
+        </is>
+      </c>
+      <c r="B208" s="20" t="inlineStr">
+        <is>
+          <t>https://www.zoomit.ir/iran-news/464136-exit-permit-bond-sakha-1405/</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="4" t="inlineStr">
+        <is>
+          <t>سوئد – تاریخ‌های کلیدی ورودی پاییز ۲۰۲۷ (۱۶ اکتبر – ۱۵ ژانویه؛ مدارک ۱ فوریه؛ دور دوم ۱۵ آوریل)</t>
+        </is>
+      </c>
+      <c r="B209" s="20" t="inlineStr">
+        <is>
+          <t>https://www.umu.se/en/education/application-and-admission/key-dates-and-deadlines/</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="4" t="inlineStr">
+        <is>
+          <t>آلمان – Stuttgart MSc CS: بازهٔ اپلای ترم زمستان ۱۵ نوامبر – ۱۵ ژانویه؛ انگلیسی C1</t>
+        </is>
+      </c>
+      <c r="B210" s="20" t="inlineStr">
+        <is>
+          <t>https://www.uni-stuttgart.de/en/study/study-programs/Computer-Science-M.Sc.-00001/</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="4" t="inlineStr">
+        <is>
+          <t>آلمان – Passau: بازهٔ اپلای AI Engineering ۱ آوریل – ۳۱ می</t>
+        </is>
+      </c>
+      <c r="B211" s="20" t="inlineStr">
+        <is>
+          <t>https://www.uni-passau.de/en/apply/apply-with-intl-qualifications</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="4" t="inlineStr">
+        <is>
+          <t>دانمارک – AAU: مهلت شهریه‌پردازها ۱۵ ژانویه (EU: ۱ مارس)؛ پورتال از اواسط دسامبر</t>
+        </is>
+      </c>
+      <c r="B212" s="20" t="inlineStr">
+        <is>
+          <t>https://www.en.aau.dk/education/apply/master/how-and-when-to-apply</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="4" t="inlineStr">
+        <is>
+          <t>دانمارک – SDU Computer Science: مهلت غیر-EU ۱ فوریه؛ شهریه یک سال پیش‌پرداخت</t>
+        </is>
+      </c>
+      <c r="B213" s="20" t="inlineStr">
+        <is>
+          <t>https://www.sdu.dk/en/uddannelse/kandidat/datalogi</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="4" t="inlineStr">
+        <is>
+          <t>هلند – Radboud: مهلت غیر-EU ۱ آوریل، بورس ۳۱ ژانویه، ثبت‌نام ۱ ژوئن</t>
+        </is>
+      </c>
+      <c r="B214" s="20" t="inlineStr">
+        <is>
+          <t>https://www.ru.nl/en/education/application-and-admission/application-procedure-masters/deadlines</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="4" t="inlineStr">
+        <is>
           <t>هلند – Twente: مهلت غیر-EEA ۱ می ۲۰۲۷؛ بورس UTS ۱۵ اکتبر ۲۰۲۶ – ۱ آوریل ۲۰۲۷</t>
         </is>
       </c>
-      <c r="B208" s="20" t="inlineStr">
+      <c r="B215" s="20" t="inlineStr">
         <is>
           <t>https://collegedunia.com/netherlands/university/749-university-of-twente-enschede/admission</t>
         </is>
@@ -20526,6 +21369,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B206" r:id="rId205"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B207" r:id="rId206"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B208" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B209" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B210" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B211" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B212" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B213" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B214" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B215" r:id="rId214"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Summary sheet: Switzerland fully integrated in every comparative row with exact figures + new 'Switzerland at a glance' row (28-row digest); fields sheet: Switzerland added to all 8 fields; footer/date updates
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Table_final.xlsx
+++ b/Table_final.xlsx
@@ -883,7 +883,7 @@
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>نرخ تبدیل ۲۷ سپتامبر ۲۰۲۶: €1 = $1.14 · £1 = $1.325 · $1 ≈ SEK 9.9 · $1 ≈ DKK 6.55 · CHF 1 = $1.21</t>
+          <t>نرخ تبدیل ۲۷ سپتامبر ۲۰۲۶: €1 = $1.14 · £1 = $1.325 · $1 ≈ SEK 9.9 · $1 ≈ DKK 6.55 · CHF 1 = $1.21 (۲۸ سپتامبر: EUR/USD 1.137، GBP/USD 1.321، USD/CHF 0.829 — انحراف &lt; ۰.۵٪). سوئیس (هر ترم، غیرمقیم، رسمی 2026/27): ETH CHF 2,190 + ≈74 · EPFL 2,240 · USI 4,000 · HSLU 1,300 · ZHAW 1,220 + 60 · Fribourg 985 · UZH 879 · Basel 850 · Neuchâtel 790 · Bern 2,609 (از پاییز ۲۰۲۶)؛ ⚠️ ETH/EPFL ممکن است با EP27 از ۲۰۲۷ دوباره افزایش یابند.</t>
         </is>
       </c>
     </row>
@@ -2066,7 +2066,7 @@
     <row r="32">
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>تاریخ راستی‌آزمایی: ۲۷ سپتامبر ۲۰۲۶ (۵ مهر ۱۴۰۵). نرخ تبدیل ۲۷ سپتامبر ۲۰۲۶: €1 = $1.14 · £1 = $1.325 · $1 ≈ SEK 9.9 · $1 ≈ DKK 6.55 · CHF 1 = $1.21</t>
+          <t>تاریخ راستی‌آزمایی: ۲۷–۲۸ سپتامبر ۲۰۲۶ (۵–۶ مهر ۱۴۰۵). نرخ تبدیل ۲۷ سپتامبر ۲۰۲۶: €1 = $1.14 · £1 = $1.325 · $1 ≈ SEK 9.9 · $1 ≈ DKK 6.55 · CHF 1 = $1.21 (۲۸ سپتامبر: EUR/USD 1.137، GBP/USD 1.321، USD/CHF 0.829 — انحراف &lt; ۰.۵٪). سوئیس (هر ترم، غیرمقیم، رسمی 2026/27): ETH CHF 2,190 + ≈74 · EPFL 2,240 · USI 4,000 · HSLU 1,300 · ZHAW 1,220 + 60 · Fribourg 985 · UZH 879 · Basel 850 · Neuchâtel 790 · Bern 2,609 (از پاییز ۲۰۲۶)؛ ⚠️ ETH/EPFL ممکن است با EP27 از ۲۰۲۷ دوباره افزایش یابند.</t>
         </is>
       </c>
     </row>
@@ -2087,7 +2087,7 @@
     <row r="35">
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>شیت «برنامه‌ها»: ≈۱۰۰ برنامهٔ انگلیسی‌زبان در ۸ حوزهٔ کامپیوتری (نه فقط CS) برای هر ۶ کشور؛ شیت «حوزه‌ها و بازار کار»: کدام حوزه برای شما بازار و پذیرش بهتری دارد.</t>
+          <t>شیت «برنامه‌ها»: ۱۱۰ برنامهٔ انگلیسی‌زبان در ۸ حوزهٔ کامپیوتری (نه فقط CS) برای هر ۶ کشور (سوئیس ۱۴)؛ شیت «حوزه‌ها و بازار کار»: کدام حوزه برای شما بازار و پذیرش بهتری دارد.</t>
         </is>
       </c>
     </row>
@@ -11468,7 +11468,7 @@
     <row r="114" ht="34" customHeight="1">
       <c r="B114" s="13" t="inlineStr">
         <is>
-          <t>شهریهٔ دلاری با نرخ نرخ تبدیل ۲۷ سپتامبر ۲۰۲۶: €1 = $1.14 · £1 = $1.325 · $1 ≈ SEK 9.9 · $1 ≈ DKK 6.55 · CHF 1 = $1.21 و گرد شده به $100. برای ورودی سپتامبر ۲۰۲۷ نرخ 2027/28 ملاک است (تا بهار ۲۰۲۷ منتشر می‌شود؛ فعلاً +۳–۵٪؛ TU/e و Surrey و Gothenburg همین حالا رسمی‌اند). آلمان: عدد فقط سهم ترم (Semesterbeitrag) است که بلیت حمل‌ونقل را هم شامل می‌شود.</t>
+          <t>شهریهٔ دلاری با نرخ نرخ تبدیل ۲۷ سپتامبر ۲۰۲۶: €1 = $1.14 · £1 = $1.325 · $1 ≈ SEK 9.9 · $1 ≈ DKK 6.55 · CHF 1 = $1.21 (۲۸ سپتامبر: EUR/USD 1.137، GBP/USD 1.321، USD/CHF 0.829 — انحراف &lt; ۰.۵٪). سوئیس (هر ترم، غیرمقیم، رسمی 2026/27): ETH CHF 2,190 + ≈74 · EPFL 2,240 · USI 4,000 · HSLU 1,300 · ZHAW 1,220 + 60 · Fribourg 985 · UZH 879 · Basel 850 · Neuchâtel 790 · Bern 2,609 (از پاییز ۲۰۲۶)؛ ⚠️ ETH/EPFL ممکن است با EP27 از ۲۰۲۷ دوباره افزایش یابند. و گرد شده به $100. برای ورودی سپتامبر ۲۰۲۷ نرخ 2027/28 ملاک است (تا بهار ۲۰۲۷ منتشر می‌شود؛ فعلاً +۳–۵٪؛ TU/e و Surrey و Gothenburg همین حالا رسمی‌اند). آلمان: عدد فقط سهم ترم (Semesterbeitrag) است که بلیت حمل‌ونقل را هم شامل می‌شود.</t>
         </is>
       </c>
     </row>
@@ -11694,12 +11694,12 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>بالاتر (+۱۰ تا +۲۵٪؛ در آلمان €52–60k، انگلستان £35–45k خارج لندن)</t>
+          <t>بالاتر (+۱۰ تا +۲۵٪؛ آلمان €52–60k، انگلستان £35–45k خارج لندن، سوئیس ≈ CHF 95–120k در زوریخ)</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>بسیار خوب — تیم‌های AI/ML در همهٔ ۶ کشور انگلیسی‌زبان‌اند</t>
+          <t>بسیار خوب — تیم‌های AI/ML در همهٔ ۶ کشور انگلیسی‌زبان‌اند؛ زوریخ (Google، ETH AI Center، آزمایشگاه‌های AI) یکی از قطب‌های اروپاست و کاملاً انگلیسی</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -11805,7 +11805,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>بالاتر از توسعه‌دهندهٔ عمومی (+۵ تا +۱۵٪)؛ DevOps/SRE در دانمارک و سوئد پرتقاضا</t>
+          <t>بالاتر از توسعه‌دهندهٔ عمومی (+۵ تا +۱۵٪)؛ DevOps/SRE در دانمارک و سوئد پرتقاضا؛ سوئیس: بانک‌ها/بیمه‌ها و Google زوریخ (≈ CHF 90–110k)</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -11852,7 +11852,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>متوسط: مدرک‌های ارزان و Safe زیاد است (HSLU Lucerne ≈ CHF 3,150/سال، Skövde، Brunel، ITU €16.5k) ولی رقابت جونیور بالاست؛ اگر می‌روید، Data Engineering را انتخاب کنید</t>
+          <t>متوسط: مدرک‌های ارزان و Safe زیاد است (HSLU Lucerne ≈ CHF 3,150/سال، USI Software &amp; Data Eng CHF 8,000/سال، Skövde، Brunel، ITU €16.5k؛ EPFL Data Science فقط Reach) ولی رقابت جونیور بالاست؛ اگر می‌روید، Data Engineering را انتخاب کنید</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -11889,7 +11889,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>خوب از نظر پیش‌زمینه (Computer Engineering)؛ گزینه‌ها: Twente ES، Stuttgart INFOTECH، H-BRS Autonomous Systems، FAU Autonomy Tech، Halmstad، MDU، SDU Robot Systems، DTU Autonomous Systems</t>
+          <t>خوب از نظر پیش‌زمینه (Computer Engineering)؛ گزینه‌ها: Twente ES، Stuttgart INFOTECH، H-BRS Autonomous Systems، FAU Autonomy Tech، Halmstad، MDU، SDU Robot Systems، DTU Autonomous Systems؛ سوئیس: ETH Robotics فقط Reach، ZHAW MSE گرایش مهندسی (آلمانی‌محور)</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -11926,7 +11926,7 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>ضعیف برای هدف «حقوق شروع بالا»؛ فقط اگر واقعاً به طراحی علاقه دارید (Siegen رایگان، Twente I-Tech، York HCIT، Chalmers IxD، AAU Medialogy)</t>
+          <t>ضعیف برای هدف «حقوق شروع بالا»؛ فقط اگر واقعاً به طراحی علاقه دارید (Siegen رایگان، Twente I-Tech، York HCIT، Chalmers IxD، AAU Medialogy؛ سوئیس برنامهٔ انگلیسی مناسب ندارد — ZHdK آلمانی)</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -11958,7 +11958,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>خوب (استودیوهای بزرگ انگلیسی‌زبان: لندن، Guildford، Stockholm، Malmö، Copenhagen، Cologne)</t>
+          <t>خوب (استودیوهای بزرگ انگلیسی‌زبان: لندن، Guildford، Stockholm، Malmö، Copenhagen، Cologne؛ سوئیس صنعت بازی کوچکی دارد — Zürich: Giants Software — و ارشد انگلیسی بازی ندارد)</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -17645,7 +17645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -17672,7 +17672,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>آلمان $27–36k  &lt;  انگلستان $38–65k (۱ سال)  &lt;  سوئد $54–65k  &lt;  دانمارک $63–76k  &lt;  هلند $75–90k. سوئیس گسترده‌ترین بازه را دارد: $35–84k — Neuchâtel/Fribourg (۱.۵ سال) $35–47k کنار انگلستان، Bern $39–51k، UZH $45–58k، HSLU $53–64k، USI/EPFL $60–75k، ETH $66–84k کنار هلند</t>
+          <t>به ترتیب هزینهٔ کل تا مدرک (میانهٔ بازه): آلمان $27–36k (۲ سال) ‹ سوئیس–Neuchâtel/Fribourg $35–47k (۱.۵ سال) ‹ انگلستان $38–65k (۱ سال) ‹ سوئیس–UZH $45–58k ‹ سوئیس–HSLU $53–64k ≈ سوئد $54–65k ‹ سوئیس–USI/EPFL $60–75k ‹ دانمارک $63–76k ‹ سوئیس–ETH $66–84k ‹ هلند $75–90k. سوئیس بسته به دانشگاه از رتبهٔ ۲ تا ۹ را می‌گیرد: شهریه‌اش بعد از آلمان کمترین است ($1,900–9,700/سال) ولی زندگی‌اش گران‌ترین جدول (CHF 1,350–2,500/ماه) — و چون ۶ ماه اول کار دانشجویی ممنوع است، سال اول تماماً از جیب می‌رود.</t>
         </is>
       </c>
     </row>
@@ -17684,7 +17684,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>انگلستان کامل؛ هلند و سوئد برای زندگی/کار خوب ولی برای اقامت دائم/تابعیت زبان می‌خواهند (هلند B1 در راه، سوئد آزمون تابعیت)؛ سوئیس: تحصیل و Big Tech زوریخ انگلیسی، ولی اداری به زبان کانتون و PR/تابعیت با A2–B1 زبان محلی (۱۰ سال)؛ دانمارک و آلمان بدون زبان محلی هم بازار کار و هم PR محدود.</t>
+          <t>انگلستان کامل؛ هلند و سوئد برای زندگی/کار خوب ولی برای اقامت دائم/تابعیت زبان می‌خواهند (هلند B1 در راه، سوئد آزمون تابعیت)؛ سوئیس (امتیاز انگلیسی ۶/۱۰): تحصیل ۱۰۰٪ انگلیسی؛ Big Tech، بانک‌ها و استارتاپ‌های زوریخ انگلیسی، ولی حدود نیمی از آگهی‌های SMEها آلمانی/فرانسه می‌خواهند؛ همهٔ امور اداری به زبان کانتون (DE/FR/IT)؛ اجازهٔ C بعد از ۱۰ سال با A2 شفاهی/A1 کتبی و تابعیت با B1/A2 — یعنی برای «کار» بهتر از آلمان/دانمارک، برای «اقامت دائم» بدتر از هلند/سوئد؛ دانمارک و آلمان بدون زبان محلی هم بازار کار و هم PR محدود.</t>
         </is>
       </c>
     </row>
@@ -17696,7 +17696,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>حقوق ناخالص: سوئیس (CHF 85–105k) ≫ دانمارک &gt; آلمان &gt; هلند ≈ سوئد &gt; انگلستان. دسترسی برای جونیورِ فقط‌انگلیسی: هلند &gt; آلمان ≈ سوئیس (فقط شرکت‌های بزرگ، ۶ ماه فرصت) &gt; سوئد ≈ دانمارک ≈ انگلستان.</t>
+          <t>حقوق ناخالص جونیور: سوئیس CHF 85–105k (≈ $103–127k؛ میانهٔ زوریخ CHF 92k) ≫ دانمارک DKK 500–540k &gt; آلمان €48–55k &gt; هلند €40–50k ≈ سوئد SEK 420–540k &gt; انگلستان £28–35k. خالص ماهانه: سوئیس CHF 5,700–6,700 (بیمهٔ درمانی CHF 350–450 جدا) &gt; دانمارک €3,300–3,700 &gt; هلند/آلمان €2,700–3,100 &gt; سوئد €2,500–2,900 &gt; انگلستان £2,000–2,500. دسترسی برای جونیورِ فقط‌انگلیسی: هلند &gt; آلمان ≈ سوئیس (فقط شرکت‌های بزرگ زوریخ؛ فقط ۶ ماه مجوز L برای کاریابی؛ سهمیهٔ غیر-EU ۸,۵۰۰ در ۲۰۲۶؛ بیکاری ICT ۳.۲٪ و استخدام ۲۰۲۶ گزینشی) &gt; سوئد ≈ دانمارک ≈ انگلستان. کار حین تحصیل: سوئیس ۶ ماه اول صفر، بعد ۱۵ ساعت/هفته — ضعیف‌ترین جدول در سال اول.</t>
         </is>
       </c>
     </row>
@@ -17708,53 +17708,65 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>آلمان ۲۲ › سوئد ۱۹ = انگلستان ۱۹ › هلند ۱۸ = سوئیس ۱۸ › دانمارک ۱۶.  با حذف ایرلند، هیچ کشوری هر سه معیار را با هم نمی‌دهد: آلمان ارزان‌ترین (ولی آلمانی)، انگلستان تنها گزینهٔ کاملاً انگلیسی (ولی گران و بازار جونیور ضعیف)، سوئیس بالاترین حقوق (ولی گران‌ترین زندگی، ۶ ماه فرصت کار، زبان محلی برای PR). پیشنهاد: ۲ برنامه آلمان (Stuttgart + Passau/Saarland) + ۲ برنامه سوئیس با شانس واقعی (USI Lugano + HSLU یا Joint MSc CS در Neuchâtel/Fribourg) + ۱–۲ گزینهٔ ارزان انگلستان (Teesside/Northumbria) به‌عنوان مسیر تماماً انگلیسی؛ ETH/EPFL فقط اگر حاضرید CHF 150 را برای یک شانس کم خرج کنید. تصمیم نهایی با پذیرش/بورس و وضعیت سفارت‌ها در بهار ۲۰۲۷.</t>
+          <t>آلمان ۲۲ › سوئد ۱۹ = انگلستان ۱۹ › هلند ۱۸ = سوئیس ۱۸ (هزینه ۵ / انگلیسی ۶ / بازار ۷) › دانمارک ۱۶.  با حذف ایرلند، هیچ کشوری هر سه معیار را با هم نمی‌دهد: آلمان ارزان‌ترین (ولی آلمانی)، انگلستان تنها گزینهٔ کاملاً انگلیسی (ولی گران و بازار جونیور ضعیف)، سوئیس بالاترین حقوق (ولی گران‌ترین زندگی، ۶ ماه فرصت کار، زبان محلی برای PR). پیشنهاد: ۲ برنامه آلمان (Stuttgart + Passau/Saarland) + ۲ برنامه سوئیس با شانس واقعی (USI Lugano + HSLU یا Joint MSc CS در Neuchâtel/Fribourg) + ۱–۲ گزینهٔ ارزان انگلستان (Teesside/Northumbria) به‌عنوان مسیر تماماً انگلیسی؛ ETH/EPFL فقط اگر حاضرید CHF 150 را برای یک شانس کم خرج کنید. تصمیم نهایی با پذیرش/بورس و وضعیت سفارت‌ها در بهار ۲۰۲۷.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>ریسک شماره یک</t>
+          <t>سوئیس در یک نگاه (جایگزین ایرلند — همهٔ ۲۸ ردیف در یک پاراگراف)</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>دسترسی به سفارت‌ها از داخل ایران (ردیف ۲۳): در سپتامبر ۲۰۲۶ فقط سوئیس (ویزای D با وقت قبلی) و تا حدی سوئد (آنلاین) از تهران قابل اقدام‌اند؛ آلمان، هلند، دانمارک و انگلستان خدمات عادی ندارند. برای سوئیس گلوگاه به‌جای سفارت، اثبات تمکن CHF 21,000 در بانک سوئیسی (کانتون زوریخ) است. از الان هزینه «برنامه B» (اقدام از ترکیه/ارمنستان/امارات) را در بودجه ببینید.</t>
+          <t>دانشگاه‌های واقع‌بینانه با معدل ۱۵.۷۷: USI Lugano (Informatics / AI / Software &amp; Data Eng؛ ورود با B2؛ CHF 4,000/ترم) · HSLU Applied Data Science &amp; AI (Safe/Target؛ CHF 1,300/ترم؛ مهلت ویزایی‌ها ۱ آوریل) · Swiss Joint MSc CS در Neuchâtel (CHF 790/ترم) یا Fribourg (CHF 985/ترم؛ ویزایی‌ها ۲۸ فوریه) — بدون آزمون زبان؛ Bern همان مدرک با CHF 2,609/ترم از پاییز ۲۰۲۶ · Basel MSc CS (CHF 850؛ Target/Reach) · ZHAW MSE (CHF 1,220 + 60؛ نمرهٔ A/B) · UZH / EPFL / ETH Reach (ETH فقط ۱–۳۰ نوامبر ۲۰۲۶؛ EPFL دور اول ۱۵ دسامبر). QS 2027: ETH 8 · EPFL 22 · UZH 98 · Basel 150 · Bern 191 · USI 456 · Fribourg 670 · ZHAW 851–900. طول دوره ۱.۵ سال (90 ECTS) یا ۲ سال (120 ECTS). زندگی: زوریخ CHF 1,900–2,500/ماه · لوزان 1,700–2,200 · برن/بازل/لوسرن 1,550–2,100 · لوگانو/فریبورگ/نوشاتل 1,350–1,800؛ تمکن رسمی CHF 21,000/سال (Basel 24,000). سال اول $23–42k؛ کل دوره $35–84k — فقط Neuchâtel/Fribourg در بودجهٔ $32k/سال. کار: ۶ ماه اول صفر، بعد ۱۵ ساعت/هفته (≈ CHF 1,300–1,800/ماه)؛ بعد از مدرک فقط ۶ ماه مجوز L؛ اجازهٔ کار بدون کف حقوق ولی داخل سهمیهٔ غیر-EU (۲۰۲۶: ۴,۵۰۰ B + ۴,۰۰۰ L). حقوق جونیور CHF 85–105k (میانهٔ زوریخ 92k)، خالص CHF 5,700–6,700/ماه، پس‌انداز CHF 1,500–3,000/ماه. اقامت: اجازهٔ C بعد از ۱۰ سال + A2 شفاهی/A1 کتبی؛ تابعیت ۱۰ سال + B1/A2 — طولانی‌ترین جدول. ویزا: سفارت تهران باز، ویزای D با وقت قبلی، تصمیم کانتون ۸–۱۲ هفته؛ زوریخ تمکن را فقط در بانک سوئیسی به نام خودتان یا با ضامن مقیم می‌پذیرد. IELTS: USI B2→C1 · HSLU C1 (B2 مشروط) · Joint MSc بدون آزمون · ZHAW B2–C1 · UZH/ETH 7.0 · EPFL بدون آزمون. بورس: عملاً هیچ (ETH/EPFL Excellence برای ۱۰٪ بالا؛ USI CHF 4,000 با ≥ ۸۰/۱۰۰ — مرزی). خوابگاه: هیچ‌جا تضمین ندارد؛ زوریخ ۳–۱۲ ماه صف (WOKO CHF 295–1,180)، لوزان زود پر می‌شود، لوگانو/فریبورگ/نوشاتل آسان (≈ CHF 450–800). ریسک سیاستی متوسط (ابتکار ۱۰ میلیونی رد شد؛ EP27؛ Bilaterals III). امتیاز ۱۸/۳۰ = هلند. یک جمله: اگر شغل بگیرید بالاترین درآمد جدول، اگر در ۶ ماه نگیرید باید بروید — گزینهٔ پربازده/پرریسک، نه گزینهٔ امن.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>برنامه زمانی ورودی سپتامبر ۲۰۲۷ (فشرده — جزئیات در شیت «برنامهٔ زمانی ۲۰۲۷»)</t>
+          <t>ریسک شماره یک</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>اکتبر ۲۰۲۶: نظام‌وظیفه + رزرو IELTS خارج از ایران + مدارک · ۱۶ اکتبر: باز شدن سوئد · ۱–۳۰ نوامبر: پنجرهٔ ETH (Reach) · نوامبر–دسامبر: IELTS + VPD uni-assist · ۱۵ دسامبر: دور اول EPFL · ۱۵ ژانویه ۲۰۲۷: مهلت سوئد / AAU / Stuttgart · ۱ فوریه: مدارک سوئد + SDU · ۲۸ فوریه: UZH و Fribourg (ویزایی‌ها) · فوریه–مارس: انگلستان + پرونده‌های سوئیس · ۱ آوریل: Radboud + HSLU (ویزایی‌ها) · ۳۰ آوریل: USI / Neuchâtel / Bern / Basel / ZHAW · ۱ می: Twente · ۳۱ می: Passau · می–ژوئن: پول (سوئیس CHF 21,000 + شهریه) + ویزا یا برنامهٔ B · اوت–اکتبر: شروع (سوئیس اواسط سپتامبر).</t>
+          <t>دسترسی به سفارت‌ها از داخل ایران (ردیف ۲۳): در سپتامبر ۲۰۲۶ فقط سوئیس (ویزای D با وقت قبلی) و تا حدی سوئد (آنلاین) از تهران قابل اقدام‌اند؛ آلمان، هلند، دانمارک و انگلستان خدمات عادی ندارند. برای سوئیس گلوگاه به‌جای سفارت، اثبات تمکن CHF 21,000 در بانک سوئیسی (کانتون زوریخ) است؛ کانتون‌های تیچینو/فریبورگ/نوشاتل/برن/لوسرن انعطاف‌پذیرترند — قبل از اقدام کتباً بپرسید. ریسک سیاستی سوئیس متوسط: ابتکار «سوئیس ۱۰ میلیونی» در ۱۴ ژوئن ۲۰۲۶ رد شد (۵۴.۸٪ نه)، ولی بستهٔ صرفه‌جویی EP27 می‌تواند شهریهٔ ETH/EPFL را دوباره بالا ببرد و طرح معافیت فارغ‌التحصیلان از سهمیه (22.067) متوقف است. از الان هزینه «برنامه B» (اقدام از ترکیه/ارمنستان/امارات) را در بودجه ببینید.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>سه پیش‌نیاز عملی ورودی ۲۰۲۷</t>
+          <t>برنامه زمانی ورودی سپتامبر ۲۰۲۷ (فشرده — جزئیات در شیت «برنامهٔ زمانی ۲۰۲۷»)</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>(۱) آزمون زبان: IELTS و TOEFL در ایران برگزار نمی‌شوند → سفر به ترکیه/ارمنستان/امارات/گرجستان تا دسامبر ۲۰۲۶. (۲) نظام‌وظیفه: بدون کارت/معافیت، خروج تحصیلی فقط با مجوز سخا + وثیقهٔ ۲۰۰ میلیون تومان + پذیرش از دانشگاه مورد تأیید وزارت علوم. (۳) نقدینگی: شهریه/تمکن سال اول باید تا می–ژوئن ۲۰۲۷ قابل انتقال باشد (SDU یک سال کامل پیش‌پرداخت). اگر یکی از این سه تا ژانویه ۲۰۲۷ حل نشود، هدف واقع‌بینانه سوئیس (USI/Bern/Basel/ZHAW تا ۳۰ آوریل)، انگلستان، هلند و آلمان با مهلت‌های بهار ۲۰۲۷ است — یا ورودی ۲۰۲۸. برای سوئیس علاوه بر این سه، «ضامن مقیم یا حساب بانکی قابل قبول کانتون» پیش‌نیاز چهارم است.</t>
+          <t>اکتبر ۲۰۲۶: نظام‌وظیفه + رزرو IELTS خارج از ایران + مدارک · ۱۶ اکتبر: باز شدن سوئد · ۱–۳۰ نوامبر: پنجرهٔ ETH (Reach) · نوامبر–دسامبر: IELTS + VPD uni-assist · ۱۵ دسامبر: دور اول EPFL · ۱۵ ژانویه ۲۰۲۷: مهلت سوئد / AAU / Stuttgart · ۱ فوریه: مدارک سوئد + SDU · ۲۸ فوریه: UZH و Fribourg (ویزایی‌ها) · فوریه–مارس: انگلستان + پرونده‌های سوئیس · ۱ آوریل: Radboud + HSLU (ویزایی‌ها) · ۳۰ آوریل: USI / Neuchâtel / Bern / Basel / ZHAW · ۱ می: Twente · ۳۱ می: Passau · می–ژوئن: پول (سوئیس CHF 21,000 + شهریه) + ویزا یا برنامهٔ B · اوت–اکتبر: شروع (سوئیس اواسط سپتامبر).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
+          <t>سه پیش‌نیاز عملی ورودی ۲۰۲۷</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>(۱) آزمون زبان: IELTS و TOEFL در ایران برگزار نمی‌شوند → سفر به ترکیه/ارمنستان/امارات/گرجستان تا دسامبر ۲۰۲۶. (۲) نظام‌وظیفه: بدون کارت/معافیت، خروج تحصیلی فقط با مجوز سخا + وثیقهٔ ۲۰۰ میلیون تومان + پذیرش از دانشگاه مورد تأیید وزارت علوم. (۳) نقدینگی: شهریه/تمکن سال اول باید تا می–ژوئن ۲۰۲۷ قابل انتقال باشد (SDU یک سال کامل پیش‌پرداخت). اگر یکی از این سه تا ژانویه ۲۰۲۷ حل نشود، هدف واقع‌بینانه سوئیس (USI/Bern/Basel/ZHAW تا ۳۰ آوریل)، انگلستان، هلند و آلمان با مهلت‌های بهار ۲۰۲۷ است — یا ورودی ۲۰۲۸. برای سوئیس علاوه بر این سه، «ضامن مقیم یا حساب بانکی قابل قبول کانتون» پیش‌نیاز چهارم است.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
           <t>تغییرات اصلی نسبت به جدول اول</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>• ردیف ۵ب (بورس/تخفیف شهریهٔ واقعاً در دسترس شما) اضافه شد — ۲۸ سپتامبر ۲۰۲۶؛ امتیازها را عوض نمی‌کند
 • هزینه کل دوره اضافه شد (هلند از «نیاز به تأمین سال دوم» به گران‌ترین گزینه تبدیل شد)
@@ -17768,39 +17780,39 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>چرا «انگلستان» و نه «بریتانیا»</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>به خواست شما فقط دانشگاه‌های انگلستان مقایسه شده‌اند. قوانین ویزا، کار و اقامت در کل بریتانیا یکسان است؛ سه تفاوت عملی: (۱) ارزان‌ترین گزینه‌های انگلستان (Teesside £17,000، Northumbria £21,500) از Swansea/Strathclyde ارزان‌ترند → کل دوره از $48–71k به $38–65k رسید؛ (۲) عوارض £925 به ازای هر دانشجو از اوت ۲۰۲۸ فقط دانشگاه‌های انگلستان را می‌گیرد — یعنی همهٔ گزینه‌های شما؛ (۳) بازار کار فناوری بریتانیا عملاً در انگلستان است (London، Manchester، Cambridge، Bristol، Leeds) — حذف اسکاتلند/ولز به فرصت شغلی لطمه نمی‌زند. برای شهریهٔ کمتر باید رتبهٔ پایین‌تر را بپذیرید: Teesside/Chester بدون رتبه QS، Northumbria ≈ ۵۲۸، Essex ≈ ۴۳۸؛ York (۱۵۸) و Newcastle (۱۴۹) تقریباً دوبرابر گران‌ترند.</t>
-        </is>
-      </c>
-    </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>نکته پروفایل</t>
+          <t>چرا «انگلستان» و نه «بریتانیا»</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>معدل (۱۵.۷۷ طبق جدول اول؛ ۱۵.۷۰ طبق نقد دوم — تفاوتی در نتیجه ندارد) برای همه برنامه‌های بالا بالاتر از حداقل است. مهم‌تر از معدل، تطابق ریزنمرات با پیش‌نیازها (ریاضی، الگوریتم، CS نظری) و SOP با تکیه بر ۲ سال سابقه کار + بازی‌سازی + پروژه‌های گیت‌هاب است.</t>
+          <t>به خواست شما فقط دانشگاه‌های انگلستان مقایسه شده‌اند. قوانین ویزا، کار و اقامت در کل بریتانیا یکسان است؛ سه تفاوت عملی: (۱) ارزان‌ترین گزینه‌های انگلستان (Teesside £17,000، Northumbria £21,500) از Swansea/Strathclyde ارزان‌ترند → کل دوره از $48–71k به $38–65k رسید؛ (۲) عوارض £925 به ازای هر دانشجو از اوت ۲۰۲۸ فقط دانشگاه‌های انگلستان را می‌گیرد — یعنی همهٔ گزینه‌های شما؛ (۳) بازار کار فناوری بریتانیا عملاً در انگلستان است (London، Manchester، Cambridge، Bristol، Leeds) — حذف اسکاتلند/ولز به فرصت شغلی لطمه نمی‌زند. برای شهریهٔ کمتر باید رتبهٔ پایین‌تر را بپذیرید: Teesside/Chester بدون رتبه QS، Northumbria ≈ ۵۲۸، Essex ≈ ۴۳۸؛ York (۱۵۸) و Newcastle (۱۴۹) تقریباً دوبرابر گران‌ترند.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
+          <t>نکته پروفایل</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>معدل (۱۵.۷۷ طبق جدول اول؛ ۱۵.۷۰ طبق نقد دوم — تفاوتی در نتیجه ندارد) برای همه برنامه‌های بالا بالاتر از حداقل است. مهم‌تر از معدل، تطابق ریزنمرات با پیش‌نیازها (ریاضی، الگوریتم، CS نظری) و SOP با تکیه بر ۲ سال سابقه کار + بازی‌سازی + پروژه‌های گیت‌هاب است. سوئیس: معدل شما در مقیاس ۶ ≈ ۵.۲ — USI (بررسی موردی) و Joint MSc CS در Neuchâtel/Fribourg/Bern (ممکن است تا ۶۰ ECTS تکمیلی بخواهد که گاهی به آلمانی/فرانسه است) واقع‌بینانه‌اند؛ ZHAW نمرهٔ ECTS A/B (یک‌سوم بالای کلاس) می‌خواهد؛ ETH/EPFL «۱۰٪ بالای کلاس» → Reach؛ نامهٔ رتبهٔ کلاسی از دانشگاه سمنان اینجا بیشترین اثر را دارد.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
           <t>اعداد را چگونه بخوانم</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>مبالغ سطح 2026/27 هستند؛ نرخ 2027/28 (سال ورود شما) بین اکتبر ۲۰۲۶ تا بهار ۲۰۲۷ منتشر می‌شود — جایی که رسمی بود (TU/e €22,400، Surrey £26,900، Gothenburg SEK 294k کل) در جدول آمده؛ برای بقیه فعلاً ۳–۵٪ اضافه کنید. نرخ تبدیل ۲۷ سپتامبر ۲۰۲۶: €1 = $1.14 · £1 = $1.325 · $1 ≈ SEK 9.9 · $1 ≈ DKK 6.55 · CHF 1 = $1.21</t>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>مبالغ سطح 2026/27 هستند؛ نرخ 2027/28 (سال ورود شما) بین اکتبر ۲۰۲۶ تا بهار ۲۰۲۷ منتشر می‌شود — جایی که رسمی بود (TU/e €22,400، Surrey £26,900، Gothenburg SEK 294k کل) در جدول آمده؛ برای بقیه فعلاً ۳–۵٪ اضافه کنید. نرخ تبدیل ۲۷ سپتامبر ۲۰۲۶: €1 = $1.14 · £1 = $1.325 · $1 ≈ SEK 9.9 · $1 ≈ DKK 6.55 · CHF 1 = $1.21 (۲۸ سپتامبر: EUR/USD 1.137، GBP/USD 1.321، USD/CHF 0.829 — انحراف &lt; ۰.۵٪). سوئیس (هر ترم، غیرمقیم، رسمی 2026/27): ETH CHF 2,190 + ≈74 · EPFL 2,240 · USI 4,000 · HSLU 1,300 · ZHAW 1,220 + 60 · Fribourg 985 · UZH 879 · Basel 850 · Neuchâtel 790 · Bern 2,609 (از پاییز ۲۰۲۶)؛ ⚠️ ETH/EPFL ممکن است با EP27 از ۲۰۲۷ دوباره افزایش یابند.</t>
         </is>
       </c>
     </row>
@@ -18588,7 +18600,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>لینک (بازدید ۲۷ سپتامبر ۲۰۲۶)</t>
+          <t>لینک (بازدید ۲۷–۲۸ سپتامبر ۲۰۲۶)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Budget USD 40k/yr + equal weights for job-finding and salary (v3.1)
- Weights job 27.5 = salary 27.5 / English 30 / cost 15 -> CH 66.8 > NL 62.8 > DE 60 > EN 59.5 > SE 57.8 > DK 57
- CH job-finding sub-score 4 -> 5 (Art. 21(3) AIG: Swiss graduates exempt from priority test; quotas remain)
- Row 9 (budget fit) and decision-sheet budget row rewritten for USD 40,000/yr
- Decision sheet re-ordered CH, NL, DE, EN, SE, DK; weight block, sensitivity, gates, verdict, next steps updated
- Shortlist re-ordered: + Basel MSc CS, - Teesside; summary line, audit row, source; MD section 20

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Table_final.xlsx
+++ b/Table_final.xlsx
@@ -199,13 +199,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="2"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -635,14 +635,14 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>تصمیم در یک صفحه — شایان، ورودی سپتامبر ۲۰۲۷، بودجه $32,000 در سال</t>
+          <t>تصمیم در یک صفحه — شایان، ورودی سپتامبر ۲۰۲۷، بودجه $40,000 در سال (قبلاً $32,000)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="52" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>همهٔ مبالغ این فایل به دلار آمریکا تبدیل شده‌اند تا لازم نباشد چیزی را خودتان تبدیل کنید. نرخ‌های ۲۸ سپتامبر ۲۰۲۶: ۱ یورو = ۱.۱۴ دلار · ۱ پوند = ۱.۳۲۵ دلار · ۱ فرانک سوئیس = ۱.۲۱ دلار · ۱ کرون سوئد = ۰.۱۰ دلار · ۱ کرون دانمارک = ۰.۱۵ دلار. اعداد گرد شده‌اند (زیر ۱۰ هزار به ۱۰ دلار، بالاتر به ۱۰۰ دلار)؛ رقم رسمی به ارز محلی فقط در شیت «راستی‌آزمایی» داخل پرانتز آمده است. شهریه‌ها سطح 2026/27 هستند (Bristol 2027/28)؛ نرخ سال ورود شما (2027/28) بین اکتبر ۲۰۲۶ تا بهار ۲۰۲۷ منتشر می‌شود — ۳ تا ۵ درصد بالاتر بگیرید؛ ⚠️ ETH/EPFL ممکن است با بستهٔ EP27 از ۲۰۲۷ دوباره گران شوند. ترتیب کشورها و امتیازها در این شیت بر اساس وزن‌هایی است که ۲۸ سپتامبر گفتید: کار پیدا کردن، حقوق و انگلیسی مهم‌تر از هزینه.</t>
+          <t>همهٔ مبالغ این فایل به دلار آمریکا تبدیل شده‌اند تا لازم نباشد چیزی را خودتان تبدیل کنید. نرخ‌های ۲۸ سپتامبر ۲۰۲۶: ۱ یورو = ۱.۱۴ دلار · ۱ پوند = ۱.۳۲۵ دلار · ۱ فرانک سوئیس = ۱.۲۱ دلار · ۱ کرون سوئد = ۰.۱۰ دلار · ۱ کرون دانمارک = ۰.۱۵ دلار. اعداد گرد شده‌اند (زیر ۱۰ هزار به ۱۰ دلار، بالاتر به ۱۰۰ دلار)؛ رقم رسمی به ارز محلی فقط در شیت «راستی‌آزمایی» داخل پرانتز آمده است. شهریه‌ها سطح 2026/27 هستند (Bristol 2027/28)؛ نرخ سال ورود شما (2027/28) بین اکتبر ۲۰۲۶ تا بهار ۲۰۲۷ منتشر می‌شود — ۳ تا ۵ درصد بالاتر بگیرید؛ ⚠️ ETH/EPFL ممکن است با بستهٔ EP27 از ۲۰۲۷ دوباره گران شوند. ترتیب کشورها و امتیازها در این شیت بر اساس وزن‌هایی است که ۲۸ سپتامبر گفتید: کار پیدا کردن و حقوق هم‌وزن، انگلیسی مهم‌تر از هزینه؛ بودجه $40,000 در سال.</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>الف) شش کشور در یک نگاه — به ترتیب امتیاز با وزن‌های شما: کار پیدا کردن، حقوق و انگلیسی سنگین‌تر از هزینه (چپ به راست بدتر می‌شود)</t>
+          <t>الف) شش کشور در یک نگاه — به ترتیب امتیاز با وزن‌های شما: کار پیدا کردن = حقوق (۲۷.۵٪ هر کدام)، انگلیسی ۳۰٪، هزینه ۱۵٪ (چپ به راست بدتر می‌شود)</t>
         </is>
       </c>
     </row>
@@ -662,12 +662,12 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
+          <t>🇨🇭 سوئیس</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
           <t>🇳🇱 هلند</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>🇨🇭 سوئیس</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -699,12 +699,12 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
+          <t>۱.۵ یا ۲ سال</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
           <t>۲ سال</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>۱.۵ یا ۲ سال</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
@@ -736,15 +736,15 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>$22,500–24,700</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
           <t>$1,900–9,700
 (Neuchâtel $1,900 · USI $9,700)</t>
         </is>
       </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>$22,500–24,700</t>
+        </is>
+      </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
           <t>$350–900
@@ -776,15 +776,15 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>$1,250–1,700</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
           <t>$1,650–2,200
 (زوریخ تا $3,000)</t>
         </is>
       </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>$1,250–1,700</t>
+        </is>
+      </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
           <t>$1,100–1,400</t>
@@ -815,12 +815,12 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
+          <t>$23,000–42,000</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
           <t>$37,500–45,000</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>$23,000–42,000</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -852,15 +852,15 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>$75,000–90,000</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
           <t>$35,000–84,000
 (Neuchâtel/Fribourg $35–47k)</t>
         </is>
       </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>$75,000–90,000</t>
+        </is>
+      </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
           <t>$27,000–36,000
@@ -886,17 +886,18 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>با بودجهٔ $32,000 در سال جور درمی‌آید؟</t>
+          <t>با بودجهٔ جدید $40,000 در سال جور درمی‌آید؟
+(فرض: $40k برای هر سال تحصیل)</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>❌ کسری $5–13k در هر سال</t>
+          <t>✅ HSLU / USI / Joint MSc / Basel / UZH راحت؛ ETH/EPFL مرزی</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>⚠️ فقط Neuchâtel/Fribourg (و با صرفه‌جویی Lucerne/Lugano)</t>
+          <t>✅ مرزی — Radboud ✓؛ Twente ۰ تا −$5k کل دوره؛ UvA یک‌ساله فقط با خرج بودجهٔ دو سال در یک سال</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -906,17 +907,17 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>❌ فقط Teesside/Northumbria، با کسری $6–16k</t>
+          <t>⚠️ Teesside ✓؛ Northumbria/Essex کسری $4–14k؛ Russell Group ❌ (مگر بودجهٔ دو سال در یک سال)</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>✅ بله (مرزی)</t>
+          <t>✅ بله، راحت (حتی LiU)</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>⚠️ AAU مرزی؛ SDU کسری ≈ $6k</t>
+          <t>✅ AAU/SDU در بودجه — ولی ویزا</t>
         </is>
       </c>
     </row>
@@ -929,13 +930,13 @@
       <c r="B12" s="6" t="inlineStr">
         <is>
           <t>متوسط
+(USI/HSLU/Joint MSc Target؛ ETH/EPFL/UZH بعید)</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>متوسط
 (Twente/Radboud Target)</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>متوسط
-(USI/HSLU/Joint MSc Target؛ ETH/EPFL/UZH بعید)</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -971,15 +972,15 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>NL Scholarship $5,700 (یک‌بار)</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
           <t>USI $4,850 (مرزی)
 بقیه هیچ</t>
         </is>
       </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>NL Scholarship $5,700 (یک‌بار)</t>
+        </is>
+      </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
           <t>تقریباً هیچ
@@ -1012,16 +1013,16 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
+          <t>۶ ماه اول: صفر
+بعد $1,550–2,200</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
           <t>تا $1,150
 (۱۶ ساعت؛ مجوز TWV)</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>۶ ماه اول: صفر
-بعد $1,550–2,200</t>
-        </is>
-      </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
           <t>$1,150–1,800
@@ -1055,12 +1056,12 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
+          <t>۶</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
           <t>۸</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>۶</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -1092,12 +1093,12 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
+          <t>۶ ماه ⚠️</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
           <t>۱۲ ماه</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>۶ ماه ⚠️</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -1129,12 +1130,12 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
+          <t>$103,000–127,000</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
           <t>$46,000–57,000</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>$103,000–127,000</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -1167,15 +1168,15 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>$3,100–3,550</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
           <t>$6,900–8,100
 (منهای بیمهٔ درمانی $420–540)</t>
         </is>
       </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>$3,100–3,550</t>
+        </is>
+      </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
           <t>$3,100–3,400</t>
@@ -1205,12 +1206,12 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
+          <t>$1,800–3,600</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
           <t>$800–1,350</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>$1,800–3,600</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -1242,12 +1243,12 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
+          <t>۵</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
           <t>۸</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>۴</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -1279,12 +1280,12 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
+          <t>ممکن (سفارت باز؛ ویزای D با نوبت)</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
           <t>سخت (از باکو)</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>ممکن (سفارت باز؛ ویزای D با نوبت)</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -1312,19 +1313,19 @@
       <c r="A22" s="7" t="inlineStr">
         <is>
           <t>★ امتیاز با وزن‌های شما (از ۱۰۰)
-کار ۳۰ / حقوق ۲۵ / انگلیسی ۳۰ / هزینه ۱۵</t>
+کار ۲۷.۵ = حقوق ۲۷.۵ / انگلیسی ۳۰ / هزینه ۱۵</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>۶۳.۵
+          <t>۶۶.۸
+(۵ / ۱۰ / ۶ / ۵)</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>۶۲.۸
 (۸ / ۵ / ۸ / ۲)</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>۶۲.۵
-(۴ / ۱۰ / ۶ / ۵)</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
@@ -1335,19 +1336,19 @@
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>۶۰
+          <t>۵۹.۵
 (۵ / ۳ / ۱۰ / ۵)</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
-          <t>۵۷.۵
+          <t>۵۷.۸
 (۴ / ۵ / ۸ / ۶)</t>
         </is>
       </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
-          <t>۵۶.۵
+          <t>۵۷
 (۵ / ۷ / ۶ / ۴)</t>
         </is>
       </c>
@@ -1397,22 +1398,22 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>اول با وزن‌های شما — به شرط جور کردن ≈ $10–20k بیشتر از بودجه</t>
+          <t>اول با وزن‌های جدید — حقوق ۱۰/۱۰، معاف از اولویت نیروی داخلی؛ ریسک: ۶ ماه + سهمیهٔ کانتونی</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>دوم — بالاترین حقوق؛ ولی «کار پیدا کردن» در ۶ ماه پرریسک‌ترین</t>
+          <t>دوم (۴ امتیاز کمتر) — احتمال ماندن بالاتر، حقوق پایین‌تر؛ با $40k/سال در بودجه</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>سوم — امن‌ترین و ارزان‌ترین پشتوانه؛ ضعفش آلمانی برای نیمی از بازار کار</t>
+          <t>سوم — پشتوانهٔ امن و ارزان؛ ضعفش آلمانی برای نیمی از بازار کار</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>انگلیسیِ کامل، ولی همان «کار» و «حقوق» که برایتان مهم‌اند ضعیف‌ترین‌اند؛ فقط برای ۱ سال + پذیرش قطعی</t>
+          <t>انگلیسیِ کامل، ولی «کار» و «حقوق» ضعیف‌ترین؛ فقط پذیرش قطعیِ یک‌ساله (Essex)</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
@@ -1447,12 +1448,12 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
+          <t>🇨🇭 سوئیس</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
           <t>🇳🇱 هلند</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>🇨🇭 سوئیس</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
@@ -1483,13 +1484,13 @@
         </is>
       </c>
       <c r="B28" s="9" t="n">
-        <v>30</v>
+        <v>27.5</v>
       </c>
       <c r="C28" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D28" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="D28" s="6" t="n">
-        <v>4</v>
       </c>
       <c r="E28" s="6" t="n">
         <v>6</v>
@@ -1511,13 +1512,13 @@
         </is>
       </c>
       <c r="B29" s="9" t="n">
-        <v>25</v>
+        <v>27.5</v>
       </c>
       <c r="C29" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D29" s="6" t="n">
         <v>5</v>
-      </c>
-      <c r="D29" s="6" t="n">
-        <v>10</v>
       </c>
       <c r="E29" s="6" t="n">
         <v>6</v>
@@ -1542,10 +1543,10 @@
         <v>30</v>
       </c>
       <c r="C30" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D30" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="D30" s="6" t="n">
-        <v>6</v>
       </c>
       <c r="E30" s="6" t="n">
         <v>4</v>
@@ -1570,10 +1571,10 @@
         <v>15</v>
       </c>
       <c r="C31" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D31" s="6" t="n">
         <v>2</v>
-      </c>
-      <c r="D31" s="6" t="n">
-        <v>5</v>
       </c>
       <c r="E31" s="6" t="n">
         <v>10</v>
@@ -1633,22 +1634,22 @@
         <v>100</v>
       </c>
       <c r="C33" s="8" t="n">
-        <v>63.5</v>
+        <v>66.8</v>
       </c>
       <c r="D33" s="8" t="n">
-        <v>62.5</v>
+        <v>62.8</v>
       </c>
       <c r="E33" s="8" t="n">
         <v>60</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>60</v>
+        <v>59.5</v>
       </c>
       <c r="G33" s="8" t="n">
-        <v>57.5</v>
+        <v>57.8</v>
       </c>
       <c r="H33" s="8" t="n">
-        <v>56.5</v>
+        <v>57</v>
       </c>
     </row>
     <row r="34">
@@ -1668,7 +1669,7 @@
         <v>3</v>
       </c>
       <c r="F34" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G34" s="6" t="n">
         <v>5</v>
@@ -1703,24 +1704,24 @@
         <v>16</v>
       </c>
     </row>
-    <row r="36" ht="64" customHeight="1">
+    <row r="36" ht="78" customHeight="1">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>چرا این زیرامتیازها؟ کار: هلند ۸ (انگلیسی‌دوست‌ترین بازار قاره، کف HSM فارغ‌التحصیل $3,560/ماه که یک جونیور می‌گیرد، ۱۲ ماه zoekjaar) · آلمان ۶ (۱۰۹ هزار جای خالی IT و ۱۸ ماه، ولی نیمی از آگهی‌ها آلمانی می‌خواهند) · انگلستان ۵ (۱۰۰٪ انگلیسی و ۱۸ ماه Graduate visa، ولی بازار جونیور اشباع و اسپانسری $50,700+ برای جونیور نادر) · دانمارک ۵ (۳ سال اقامت، ولی بدون دانمارکی و خارج کپنهاگ سخت) · سوئد ۴ (بازار ۲۰۲۴–۲۶ ضعیف، شبکهٔ محلی) · سوئیس ۴ (فقط ۶ ماه مجوز L، سهمیهٔ غیر-EU، رقابت با ETH/EPFL). حقوق: سوئیس ۱۰ ($103–127k) · دانمارک ۷ ($76–82k) · آلمان ۶ ($55–63k) · هلند ۵ ($46–57k) · سوئد ۵ ($42–55k) · انگلستان ۳ ($37–46k). انگلیسی و هزینه: همان ردیف ۲۸ جدول اصلی.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="48" customHeight="1">
+          <t>چرا این زیرامتیازها؟ کار: هلند ۸ (انگلیسی‌دوست‌ترین بازار قاره، کف HSM فارغ‌التحصیل $3,560/ماه که یک جونیور می‌گیرد، ۱۲ ماه zoekjaar) · آلمان ۶ (۱۰۹ هزار جای خالی IT و ۱۸ ماه، ولی نیمی از آگهی‌ها آلمانی می‌خواهند) · انگلستان ۵ (۱۰۰٪ انگلیسی و ۱۸ ماه Graduate visa، ولی بازار جونیور اشباع و اسپانسری $50,700+ برای جونیور نادر) · دانمارک ۵ (۳ سال اقامت، ولی بدون دانمارکی و خارج کپنهاگ سخت) · سوئد ۴ (بازار ۲۰۲۴–۲۶ ضعیف، شبکهٔ محلی) · سوئیس ۵ (قبلاً ۴: فارغ‌التحصیلان دانشگاه‌های سوئیس طبق مادهٔ ۲۱(۳) AIG از «اولویت نیروی داخلی» معاف‌اند و تا ۱۲ ماه بعد از مدرک برای کار مرتبط اعتبار دارد؛ ولی مجوز کاریابی فقط ۶ ماه است و مجوز کار همچنان از سهمیهٔ کانتونی کم می‌شود — زوریخ ۲۰۲۵: ۳۹۹ مجوز L + ۲۴۹ مجوز B برای همهٔ رشته‌ها؛ رقابت با ETH/EPFL). حقوق: سوئیس ۱۰ ($103–127k) · دانمارک ۷ ($76–82k) · آلمان ۶ ($55–63k) · هلند ۵ ($46–57k) · سوئد ۵ ($42–55k) · انگلستان ۳ ($37–46k). انگلیسی و هزینه: همان ردیف ۲۸ جدول اصلی (هزینه نسبی است؛ بودجهٔ جدید فقط ردیف «جور درمی‌آید؟» را عوض می‌کند).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="64" customHeight="1">
       <c r="A37" s="11" t="inlineStr">
         <is>
-          <t>حساسیت: اگر هزینه را صفر کنید (کار ۳۵ / حقوق ۳۰ / انگلیسی ۳۵): هلند ۷۱ › سوئیس ۶۵ › انگلستان ۶۱.۵ › دانمارک ۵۹.۵ › سوئد ۵۷ › آلمان ۵۳. اگر حقوق را سنگین‌تر کنید (کار ۳۰ / حقوق ۳۵ / انگلیسی ۲۵ / هزینه ۱۰): سوئیس ۶۷ › هلند ۶۳.۵ › آلمان ۵۹ › دانمارک ۵۸.۵ › انگلستان ۵۵.۵ = سوئد ۵۵.۵. در هر سه حالت هلند و سوئیس بالا هستند و انگلستان با وجود انگلیسیِ کامل بالا نمی‌آید. فاصله‌ها کم است — این امتیازها قضاوت‌اند، نه اندازه‌گیری.</t>
+          <t>حساسیت: (۱) همین وزن‌ها ولی «کار» سوئیس = ۴ (مثل نسخهٔ قبل): سوئیس ۶۴ › هلند ۶۲.۸ › آلمان ۶۰ › انگلستان ۵۹.۵ › سوئد ۵۷.۸ › دانمارک ۵۷. (۲) کار ۳۰ / حقوق ۳۰ / انگلیسی ۳۰ / هزینه ۱۰ (هزینه سبک‌تر چون بودجه بالا رفت): سوئیس ۶۸ › هلند ۶۵ › انگلستان ۵۹ › آلمان ۵۸ = دانمارک ۵۸ › سوئد ۵۷. (۳) وزن‌های نسخهٔ قبل (کار ۳۰ / حقوق ۲۵ / انگلیسی ۳۰ / هزینه ۱۵) با «کار» سوئیس = ۵: سوئیس ۶۵.۵ › هلند ۶۳.۵ › آلمان ۶۰ = انگلستان ۶۰. در همهٔ حالت‌ها سوئیس و هلند دو فینالیست‌اند و اختلافشان ۱ تا ۴ امتیاز است — این امتیازها قضاوت‌اند، نه اندازه‌گیری؛ تصمیم بین این دو با ریسک‌پذیری شما و پذیرش‌ها گرفته می‌شود، نه با اعشار.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="48" customHeight="1">
       <c r="A38" s="11" t="inlineStr">
         <is>
-          <t>سه فیلتری که امتیاز نمی‌بیند: (۱) پول — Twente/Radboud ≈ $10–20k بیشتر از بودجهٔ دو سال شما ($64k) می‌خواهند؛ UvA یک‌ساله ≈ $57–62k؛ HSLU ($53–64k) در بودجه، USI ($60–72k) کمی بالاتر. (۲) ویزا از تهران — هلند از باکو، سوئیس سفارت تهران باز، دانمارک عملاً بسته. (۳) پذیرش — همهٔ گزینه‌های هلند و سوئیس Target هستند، نه Safe؛ پس یک Safe (Essex یا Passau) کنار آن‌ها لازم است.</t>
+          <t>سه فیلتری که امتیاز نمی‌بیند: (۱) پول — با $40,000 در سال: HSLU ($53–64k)، USI ($60–72k)، Joint MSc ($32–41k)، Basel ($38–49k) و Radboud ($74–82k) در بودجه؛ Twente ($77–85k) مرزی (NL Scholarship $5,700 جبران می‌کند)؛ UvA یک‌ساله ($57–62k) و Russell Group فقط اگر بودجهٔ دو سال را در یک سال خرج کنید. (۲) ویزا از تهران — سوئیس سفارت تهران باز، هلند از باکو، دانمارک عملاً بسته. (۳) پذیرش — همهٔ گزینه‌های سوئیس و هلند Target هستند، نه Safe؛ پس یک Safe (Essex یا Passau) کنارشان لازم است.</t>
         </is>
       </c>
     </row>
@@ -1795,12 +1796,12 @@
       </c>
       <c r="B42" s="12" t="inlineStr">
         <is>
-          <t>University of Twente (UT) – Enschede</t>
+          <t>Hochschule Luzern (HSLU) – Lucerne / Luzern</t>
         </is>
       </c>
       <c r="C42" s="12" t="inlineStr">
         <is>
-          <t>MSc Computer Science (گرایش‌ها: Cyber Security، Data Science، Software Tech، ...)</t>
+          <t>MSc Applied Data Science and AI (نام جدید از اوت ۲۰۲۶؛ قبلاً Applied Information and Data Science)</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
@@ -1810,37 +1811,37 @@
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>$49,500</t>
+          <t>$7,620</t>
         </is>
       </c>
       <c r="F42" s="12" t="inlineStr">
         <is>
-          <t>$27–36k</t>
+          <t>$45–57k</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>$77–85k</t>
+          <t>$53–64k</t>
         </is>
       </c>
       <c r="H42" s="12" t="inlineStr">
         <is>
-          <t>۱ می ۲۰۲۷ (غیر-EEA)</t>
+          <t>۱ آوریل ۲۰۲۷</t>
         </is>
       </c>
       <c r="I42" s="13" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Safe/Target</t>
         </is>
       </c>
       <c r="J42" s="12" t="inlineStr">
         <is>
-          <t>⚠️ Roomspot، اول‌آمده‌اول‌گرفته؛ $340–910</t>
+          <t>✅ نسبتاً آسان؛ $605–970</t>
         </is>
       </c>
       <c r="K42" s="12" t="inlineStr">
         <is>
-          <t>انگلیسی‌دوست‌ترین بازار کار؛ حداقل رسمی ایران ۱۵/۲۰ ✓؛ کسری بودجه ≈ $13–21k در کل دوره (NL Scholarship $5,700 + کار ۱۶ ساعت کمش می‌کند)</t>
+          <t>بالاترین حقوق‌ها ۴۵ دقیقه آن‌طرف‌تر (زوریخ)؛ راحت در بودجهٔ جدید؛ هر کارشناسی را می‌پذیرد؛ ریسک: فقط ۶ ماه مجوز L بعد از مدرک</t>
         </is>
       </c>
     </row>
@@ -1850,12 +1851,12 @@
       </c>
       <c r="B43" s="12" t="inlineStr">
         <is>
-          <t>Radboud University – Nijmegen</t>
+          <t>USI – Università della Svizzera italiana – Lugano</t>
         </is>
       </c>
       <c r="C43" s="12" t="inlineStr">
         <is>
-          <t>MSc Computing Science (گرایش‌ها: Cyber Security، Data Science، Software Science)</t>
+          <t>MSc Artificial Intelligence (با IDSIA)</t>
         </is>
       </c>
       <c r="D43" s="12" t="inlineStr">
@@ -1865,37 +1866,37 @@
       </c>
       <c r="E43" s="12" t="inlineStr">
         <is>
-          <t>$44,900</t>
+          <t>$19,400</t>
         </is>
       </c>
       <c r="F43" s="12" t="inlineStr">
         <is>
-          <t>$29–37k</t>
+          <t>$41–52k</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>$74–82k</t>
+          <t>$60–72k</t>
         </is>
       </c>
       <c r="H43" s="12" t="inlineStr">
         <is>
-          <t>۱ آوریل ۲۰۲۷</t>
-        </is>
-      </c>
-      <c r="I43" s="13" t="inlineStr">
+          <t>۳۰ آوریل ۲۰۲۷</t>
+        </is>
+      </c>
+      <c r="I43" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
       <c r="J43" s="12" t="inlineStr">
         <is>
-          <t>⚠️ فرم PAS تا ۱ ژوئن؛ اتاق $420–740؛ بدون تضمین</t>
+          <t>✅ آسان؛ $545–845</t>
         </is>
       </c>
       <c r="K43" s="12" t="inlineStr">
         <is>
-          <t>Nijmegen ارزان‌تر؛ کسری ≈ $10–18k در کل دوره؛ بورس Radboud فقط Reach</t>
+          <t>AI با IDSIA؛ ورود با B2؛ بورس $4,840 مرزی؛ در بودجهٔ جدید؛ همان ریسک ۶ ماه</t>
         </is>
       </c>
     </row>
@@ -1905,52 +1906,52 @@
       </c>
       <c r="B44" s="12" t="inlineStr">
         <is>
-          <t>University of Amsterdam (UvA) – Amsterdam</t>
+          <t>University of Basel – Basel</t>
         </is>
       </c>
       <c r="C44" s="12" t="inlineStr">
         <is>
-          <t>MSc Software Engineering (۱ ساله!)</t>
+          <t>MSc Computer Science</t>
         </is>
       </c>
       <c r="D44" s="12" t="inlineStr">
         <is>
-          <t>۱ سال</t>
+          <t>۱.۵ سال</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>$39,100</t>
+          <t>$3,090</t>
         </is>
       </c>
       <c r="F44" s="12" t="inlineStr">
         <is>
-          <t>$18–23k</t>
+          <t>$35–46k</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>$57–62k</t>
+          <t>$38–49k</t>
         </is>
       </c>
       <c r="H44" s="12" t="inlineStr">
         <is>
-          <t>≈ ۱ آوریل ۲۰۲۷ (غیر-EU؛ چک شود)</t>
-        </is>
-      </c>
-      <c r="I44" s="14" t="inlineStr">
+          <t>۳۰ آوریل ۲۰۲۷</t>
+        </is>
+      </c>
+      <c r="I44" s="15" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
       </c>
       <c r="J44" s="12" t="inlineStr">
         <is>
-          <t>❌ بحرانی‌ترین شهر؛ اتاق $1,030–1,480</t>
+          <t>✅ نسبتاً آسان؛ $605–970</t>
         </is>
       </c>
       <c r="K44" s="12" t="inlineStr">
         <is>
-          <t>۱ سال در بهترین بازار انگلیسی‌زبان اروپا؛ شهریه $39,100 رسمی 2026/27؛ Target/Reach؛ کل یک سال ≈ بودجهٔ دو سال</t>
+          <t>رتبهٔ ۱۵۰، ۹۰ واحد انگلیسی، شهریه ناچیز؛ Basel = Roche/Novartis/IT و ۱ ساعت تا زوریخ؛ Target/Reach؛ تمکن کانتون $29,000</t>
         </is>
       </c>
     </row>
@@ -1960,52 +1961,52 @@
       </c>
       <c r="B45" s="12" t="inlineStr">
         <is>
-          <t>Hochschule Luzern (HSLU) – Lucerne / Luzern</t>
+          <t>University of Neuchâtel – Neuchâtel</t>
         </is>
       </c>
       <c r="C45" s="12" t="inlineStr">
         <is>
-          <t>MSc Applied Data Science and AI (نام جدید از اوت ۲۰۲۶؛ قبلاً Applied Information and Data Science)</t>
+          <t>Swiss Joint MSc Computer Science (ثبت‌نام در Neuchâtel)</t>
         </is>
       </c>
       <c r="D45" s="12" t="inlineStr">
         <is>
-          <t>۲ سال</t>
+          <t>۱.۵ سال</t>
         </is>
       </c>
       <c r="E45" s="12" t="inlineStr">
         <is>
-          <t>$7,620</t>
+          <t>$2,870</t>
         </is>
       </c>
       <c r="F45" s="12" t="inlineStr">
         <is>
-          <t>$45–57k</t>
+          <t>$29–38k</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>$53–64k</t>
+          <t>$32–41k</t>
         </is>
       </c>
       <c r="H45" s="12" t="inlineStr">
         <is>
-          <t>۱ آوریل ۲۰۲۷</t>
-        </is>
-      </c>
-      <c r="I45" s="15" t="inlineStr">
-        <is>
-          <t>Safe/Target</t>
+          <t>۳۱ مارس ۲۰۲۷ (خارجی‌ها)</t>
+        </is>
+      </c>
+      <c r="I45" s="14" t="inlineStr">
+        <is>
+          <t>Target</t>
         </is>
       </c>
       <c r="J45" s="12" t="inlineStr">
         <is>
-          <t>✅ نسبتاً آسان؛ $605–970</t>
+          <t>✅ آسان؛ $545–970</t>
         </is>
       </c>
       <c r="K45" s="12" t="inlineStr">
         <is>
-          <t>بالاترین حقوق‌ها ۴۵ دقیقه آن‌طرف‌تر (زوریخ)؛ در بودجه؛ هر کارشناسی را می‌پذیرد؛ ریسک: فقط ۶ ماه مجوز L بعد از مدرک</t>
+          <t>ارزان‌ترین سوئیس و بدون آزمون زبان؛ Safe-ترِ سوئیس؛ ولی منطقهٔ فرانسه‌زبان و پیوند ضعیف‌تر با بازار زوریخ</t>
         </is>
       </c>
     </row>
@@ -2015,12 +2016,12 @@
       </c>
       <c r="B46" s="12" t="inlineStr">
         <is>
-          <t>USI – Università della Svizzera italiana – Lugano</t>
+          <t>University of Twente (UT) – Enschede</t>
         </is>
       </c>
       <c r="C46" s="12" t="inlineStr">
         <is>
-          <t>MSc Artificial Intelligence (با IDSIA)</t>
+          <t>MSc Computer Science (گرایش‌ها: Cyber Security، Data Science، Software Tech، ...)</t>
         </is>
       </c>
       <c r="D46" s="12" t="inlineStr">
@@ -2030,37 +2031,37 @@
       </c>
       <c r="E46" s="12" t="inlineStr">
         <is>
-          <t>$19,400</t>
+          <t>$49,500</t>
         </is>
       </c>
       <c r="F46" s="12" t="inlineStr">
         <is>
-          <t>$41–52k</t>
+          <t>$27–36k</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>$60–72k</t>
+          <t>$77–85k</t>
         </is>
       </c>
       <c r="H46" s="12" t="inlineStr">
         <is>
-          <t>۳۰ آوریل ۲۰۲۷</t>
-        </is>
-      </c>
-      <c r="I46" s="13" t="inlineStr">
+          <t>۱ می ۲۰۲۷ (غیر-EEA)</t>
+        </is>
+      </c>
+      <c r="I46" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
       <c r="J46" s="12" t="inlineStr">
         <is>
-          <t>✅ آسان؛ $545–845</t>
+          <t>⚠️ Roomspot، اول‌آمده‌اول‌گرفته؛ $340–910</t>
         </is>
       </c>
       <c r="K46" s="12" t="inlineStr">
         <is>
-          <t>AI با IDSIA؛ ورود با B2؛ بورس $4,840 مرزی؛ کمی بالاتر از بودجه؛ همان ریسک ۶ ماه</t>
+          <t>انگلیسی‌دوست‌ترین بازار کار؛ حداقل رسمی ایران ۱۵/۲۰ ✓؛ با بودجهٔ جدید مرزی (۰ تا −$5k در کل دوره؛ NL Scholarship $5,700 جبران می‌کند)</t>
         </is>
       </c>
     </row>
@@ -2070,12 +2071,12 @@
       </c>
       <c r="B47" s="12" t="inlineStr">
         <is>
-          <t>Universität Stuttgart – Stuttgart</t>
+          <t>Radboud University – Nijmegen</t>
         </is>
       </c>
       <c r="C47" s="12" t="inlineStr">
         <is>
-          <t>M.Sc. Computer Science (انگلیسی، بدون NC)</t>
+          <t>MSc Computing Science (گرایش‌ها: Cyber Security، Data Science، Software Science)</t>
         </is>
       </c>
       <c r="D47" s="12" t="inlineStr">
@@ -2085,37 +2086,37 @@
       </c>
       <c r="E47" s="12" t="inlineStr">
         <is>
-          <t>$7,750</t>
+          <t>$44,900</t>
         </is>
       </c>
       <c r="F47" s="12" t="inlineStr">
         <is>
-          <t>$30–37k</t>
+          <t>$29–37k</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>$38–45k</t>
+          <t>$74–82k</t>
         </is>
       </c>
       <c r="H47" s="12" t="inlineStr">
         <is>
-          <t>۱۵ ژانویه ۲۰۲۷</t>
-        </is>
-      </c>
-      <c r="I47" s="13" t="inlineStr">
+          <t>۱ آوریل ۲۰۲۷</t>
+        </is>
+      </c>
+      <c r="I47" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
       <c r="J47" s="12" t="inlineStr">
         <is>
-          <t>❌ صف ۶–۸ ماه؛ اتاق WG خصوصی $545–685</t>
+          <t>⚠️ فرم PAS تا ۱ ژوئن؛ اتاق $420–740؛ بدون تضمین</t>
         </is>
       </c>
       <c r="K47" s="12" t="inlineStr">
         <is>
-          <t>پشتوانهٔ امن و ارزان؛ حقوق $55–63k؛ ۱۸ ماه؛ Bosch / Mercedes / Porsche؛ ضعف: آلمانی برای نیمی از بازار</t>
+          <t>Nijmegen ارزان‌تر؛ با بودجهٔ جدید در بودجه (تا −$2k)؛ بورس Radboud فقط Reach</t>
         </is>
       </c>
     </row>
@@ -2125,52 +2126,52 @@
       </c>
       <c r="B48" s="12" t="inlineStr">
         <is>
-          <t>TU Darmstadt – Darmstadt</t>
+          <t>University of Amsterdam (UvA) – Amsterdam</t>
         </is>
       </c>
       <c r="C48" s="12" t="inlineStr">
         <is>
-          <t>M.Sc. Distributed Software Systems (انگلیسی)</t>
+          <t>MSc Software Engineering (۱ ساله!)</t>
         </is>
       </c>
       <c r="D48" s="12" t="inlineStr">
         <is>
-          <t>۲ سال</t>
+          <t>۱ سال</t>
         </is>
       </c>
       <c r="E48" s="12" t="inlineStr">
         <is>
-          <t>$1,370</t>
+          <t>$39,100</t>
         </is>
       </c>
       <c r="F48" s="12" t="inlineStr">
         <is>
-          <t>$29–36k</t>
+          <t>$18–23k</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>$30–37k</t>
+          <t>$57–62k</t>
         </is>
       </c>
       <c r="H48" s="12" t="inlineStr">
         <is>
-          <t>≈ ۱۵ می – ۱۵ ژوئیه ۲۰۲۷ (چک شود)</t>
-        </is>
-      </c>
-      <c r="I48" s="14" t="inlineStr">
+          <t>≈ ۱ آوریل ۲۰۲۷ (غیر-EU؛ چک شود)</t>
+        </is>
+      </c>
+      <c r="I48" s="15" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
       </c>
       <c r="J48" s="12" t="inlineStr">
         <is>
-          <t>❌ لیست انتظار؛ WG $515–625</t>
+          <t>❌ بحرانی‌ترین شهر؛ اتاق $1,030–1,480</t>
         </is>
       </c>
       <c r="K48" s="12" t="inlineStr">
         <is>
-          <t>تقریباً رایگان؛ ۲۵ دقیقه تا قطب مالی/IT فرانکفورت (شرکت‌های بین‌المللی انگلیسی‌زبان بیشتر)</t>
+          <t>۱ سال در بهترین بازار انگلیسی‌زبان اروپا؛ شهریه $39,100 رسمی 2026/27؛ Target/Reach؛ فقط اگر بودجهٔ دو سال را در یک سال خرج کنید</t>
         </is>
       </c>
     </row>
@@ -2180,12 +2181,12 @@
       </c>
       <c r="B49" s="12" t="inlineStr">
         <is>
-          <t>Saarland University (UdS) – Saarbrücken</t>
+          <t>Universität Stuttgart – Stuttgart</t>
         </is>
       </c>
       <c r="C49" s="12" t="inlineStr">
         <is>
-          <t>M.Sc. Data Science and Artificial Intelligence</t>
+          <t>M.Sc. Computer Science (انگلیسی، بدون NC)</t>
         </is>
       </c>
       <c r="D49" s="12" t="inlineStr">
@@ -2195,37 +2196,37 @@
       </c>
       <c r="E49" s="12" t="inlineStr">
         <is>
-          <t>$1,800</t>
+          <t>$7,750</t>
         </is>
       </c>
       <c r="F49" s="12" t="inlineStr">
         <is>
-          <t>$25–30k</t>
+          <t>$30–37k</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>$26–32k</t>
+          <t>$38–45k</t>
         </is>
       </c>
       <c r="H49" s="12" t="inlineStr">
         <is>
-          <t>≈ ۱۵ می – ۱۵ ژوئیه ۲۰۲۷ (چک شود)</t>
-        </is>
-      </c>
-      <c r="I49" s="13" t="inlineStr">
+          <t>۱۵ ژانویه ۲۰۲۷</t>
+        </is>
+      </c>
+      <c r="I49" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
       <c r="J49" s="12" t="inlineStr">
         <is>
-          <t>✅ نسبتاً آسان؛ خوابگاه $340–455</t>
+          <t>❌ صف ۶–۸ ماه؛ اتاق WG خصوصی $545–685</t>
         </is>
       </c>
       <c r="K49" s="12" t="inlineStr">
         <is>
-          <t>AI کنار CISPA/DFKI؛ ارزان؛ بدون NC</t>
+          <t>پشتوانهٔ امن و ارزان؛ حقوق $55–63k؛ ۱۸ ماه؛ Bosch / Mercedes / Porsche؛ ضعف: آلمانی برای نیمی از بازار</t>
         </is>
       </c>
     </row>
@@ -2235,52 +2236,52 @@
       </c>
       <c r="B50" s="12" t="inlineStr">
         <is>
-          <t>University of Neuchâtel – Neuchâtel</t>
+          <t>TU Darmstadt – Darmstadt</t>
         </is>
       </c>
       <c r="C50" s="12" t="inlineStr">
         <is>
-          <t>Swiss Joint MSc Computer Science (ثبت‌نام در Neuchâtel)</t>
+          <t>M.Sc. Distributed Software Systems (انگلیسی)</t>
         </is>
       </c>
       <c r="D50" s="12" t="inlineStr">
         <is>
-          <t>۱.۵ سال</t>
+          <t>۲ سال</t>
         </is>
       </c>
       <c r="E50" s="12" t="inlineStr">
         <is>
-          <t>$2,870</t>
+          <t>$1,370</t>
         </is>
       </c>
       <c r="F50" s="12" t="inlineStr">
         <is>
-          <t>$29–38k</t>
+          <t>$29–36k</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>$32–41k</t>
+          <t>$30–37k</t>
         </is>
       </c>
       <c r="H50" s="12" t="inlineStr">
         <is>
-          <t>۳۱ مارس ۲۰۲۷ (خارجی‌ها)</t>
-        </is>
-      </c>
-      <c r="I50" s="13" t="inlineStr">
-        <is>
-          <t>Target</t>
+          <t>≈ ۱۵ می – ۱۵ ژوئیه ۲۰۲۷ (چک شود)</t>
+        </is>
+      </c>
+      <c r="I50" s="15" t="inlineStr">
+        <is>
+          <t>Target/Reach</t>
         </is>
       </c>
       <c r="J50" s="12" t="inlineStr">
         <is>
-          <t>✅ آسان؛ $545–970</t>
+          <t>❌ لیست انتظار؛ WG $515–625</t>
         </is>
       </c>
       <c r="K50" s="12" t="inlineStr">
         <is>
-          <t>ارزان‌ترین سوئیس و بدون آزمون زبان؛ ولی منطقهٔ فرانسه‌زبان و پیوند ضعیف‌تر با بازار زوریخ — فقط اگر پول تعیین‌کننده شد</t>
+          <t>تقریباً رایگان؛ ۲۵ دقیقه تا قطب مالی/IT فرانکفورت (شرکت‌های بین‌المللی انگلیسی‌زبان بیشتر)</t>
         </is>
       </c>
     </row>
@@ -2290,52 +2291,52 @@
       </c>
       <c r="B51" s="12" t="inlineStr">
         <is>
-          <t>University of Essex – Colchester</t>
+          <t>Saarland University (UdS) – Saarbrücken</t>
         </is>
       </c>
       <c r="C51" s="12" t="inlineStr">
         <is>
-          <t>MSc Advanced Computer Science</t>
+          <t>M.Sc. Data Science and Artificial Intelligence</t>
         </is>
       </c>
       <c r="D51" s="12" t="inlineStr">
         <is>
-          <t>۱ سال</t>
+          <t>۲ سال</t>
         </is>
       </c>
       <c r="E51" s="12" t="inlineStr">
         <is>
-          <t>$32,700</t>
+          <t>$1,800</t>
         </is>
       </c>
       <c r="F51" s="12" t="inlineStr">
         <is>
-          <t>$16–21k</t>
+          <t>$25–30k</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>$49–54k</t>
+          <t>$26–32k</t>
         </is>
       </c>
       <c r="H51" s="12" t="inlineStr">
         <is>
-          <t>rolling — تا ژوئن ۲۰۲۷</t>
-        </is>
-      </c>
-      <c r="I51" s="15" t="inlineStr">
-        <is>
-          <t>Safe/Target</t>
+          <t>≈ ۱۵ می – ۱۵ ژوئیه ۲۰۲۷ (چک شود)</t>
+        </is>
+      </c>
+      <c r="I51" s="14" t="inlineStr">
+        <is>
+          <t>Target</t>
         </is>
       </c>
       <c r="J51" s="12" t="inlineStr">
         <is>
-          <t>✅ تضمین برای کل دوره؛ $225–265/هفته</t>
+          <t>✅ نسبتاً آسان؛ خوابگاه $340–455</t>
         </is>
       </c>
       <c r="K51" s="12" t="inlineStr">
         <is>
-          <t>پذیرش قطعیِ ۱۰۰٪ انگلیسی و ۱ ساله؛ بورس خودکار $5,960 برای ایران؛ ولی بازار جونیور و حقوق ضعیف</t>
+          <t>AI کنار CISPA/DFKI؛ ارزان؛ بدون NC</t>
         </is>
       </c>
     </row>
@@ -2345,7 +2346,7 @@
       </c>
       <c r="B52" s="12" t="inlineStr">
         <is>
-          <t>Northumbria University – Newcastle upon Tyne</t>
+          <t>University of Essex – Colchester</t>
         </is>
       </c>
       <c r="C52" s="12" t="inlineStr">
@@ -2360,17 +2361,17 @@
       </c>
       <c r="E52" s="12" t="inlineStr">
         <is>
-          <t>$28,500</t>
+          <t>$32,700</t>
         </is>
       </c>
       <c r="F52" s="12" t="inlineStr">
         <is>
-          <t>$15–20k</t>
+          <t>$16–21k</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>$44–48k</t>
+          <t>$49–54k</t>
         </is>
       </c>
       <c r="H52" s="12" t="inlineStr">
@@ -2378,19 +2379,19 @@
           <t>rolling — تا ژوئن ۲۰۲۷</t>
         </is>
       </c>
-      <c r="I52" s="16" t="inlineStr">
-        <is>
-          <t>Safe</t>
+      <c r="I52" s="13" t="inlineStr">
+        <is>
+          <t>Safe/Target</t>
         </is>
       </c>
       <c r="J52" s="12" t="inlineStr">
         <is>
-          <t>✅ احتمالاً (تأیید نشده)؛ $125–210/هفته</t>
+          <t>✅ تضمین برای کل دوره؛ $225–265/هفته</t>
         </is>
       </c>
       <c r="K52" s="12" t="inlineStr">
         <is>
-          <t>ارزان‌ترِ انگلستان با رتبهٔ قابل قبول؛ همان ضعف بازار/حقوق</t>
+          <t>پذیرش قطعیِ ۱۰۰٪ انگلیسی و ۱ ساله؛ بورس خودکار $5,960 برای ایران؛ کسری $3–8k نسبت به $40k یک‌ساله؛ بازار جونیور و حقوق ضعیف</t>
         </is>
       </c>
     </row>
@@ -2400,12 +2401,12 @@
       </c>
       <c r="B53" s="12" t="inlineStr">
         <is>
-          <t>Teesside University – Middlesbrough</t>
+          <t>Northumbria University – Newcastle upon Tyne</t>
         </is>
       </c>
       <c r="C53" s="12" t="inlineStr">
         <is>
-          <t>MSc Computer Science</t>
+          <t>MSc Advanced Computer Science</t>
         </is>
       </c>
       <c r="D53" s="12" t="inlineStr">
@@ -2415,17 +2416,17 @@
       </c>
       <c r="E53" s="12" t="inlineStr">
         <is>
-          <t>$22,500</t>
+          <t>$28,500</t>
         </is>
       </c>
       <c r="F53" s="12" t="inlineStr">
         <is>
-          <t>$15–18k</t>
+          <t>$15–20k</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>$38–41k</t>
+          <t>$44–48k</t>
         </is>
       </c>
       <c r="H53" s="12" t="inlineStr">
@@ -2440,12 +2441,12 @@
       </c>
       <c r="J53" s="12" t="inlineStr">
         <is>
-          <t>✅ احتمالاً (تأیید نشده)؛ $115–210/هفته</t>
+          <t>✅ احتمالاً (تأیید نشده)؛ $125–210/هفته</t>
         </is>
       </c>
       <c r="K53" s="12" t="inlineStr">
         <is>
-          <t>ارزان‌ترین انگلستان؛ Middlesbrough بازار محلی کوچک</t>
+          <t>ارزان‌ترِ انگلستان با رتبهٔ قابل قبول؛ کسری $4–8k؛ همان ضعف بازار/حقوق</t>
         </is>
       </c>
     </row>
@@ -2543,7 +2544,7 @@
           <t>۱۵ ژانویه ۲۰۲۷</t>
         </is>
       </c>
-      <c r="I55" s="15" t="inlineStr">
+      <c r="I55" s="13" t="inlineStr">
         <is>
           <t>Safe/Target</t>
         </is>
@@ -2598,7 +2599,7 @@
           <t>۱۵ ژانویه ۲۰۲۷</t>
         </is>
       </c>
-      <c r="I56" s="13" t="inlineStr">
+      <c r="I56" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -2610,7 +2611,7 @@
       </c>
       <c r="K56" s="17" t="inlineStr">
         <is>
-          <t>برای مقایسه: ۳ سال اجازهٔ کاریابی و حقوق بالا — ولی ویزا از تهران تقریباً غیرممکن</t>
+          <t>برای مقایسه: ۳ سال اجازهٔ کاریابی و حقوق بالا؛ حالا در بودجه — ولی ویزا از تهران تقریباً غیرممکن</t>
         </is>
       </c>
     </row>
@@ -2632,35 +2633,35 @@
     <row r="60" ht="40" customHeight="1">
       <c r="A60" s="11" t="inlineStr">
         <is>
-          <t>۱) با وزن‌های شما (کار ۳۰ / حقوق ۲۵ / انگلیسی ۳۰ / هزینه ۱۵) ترتیب عوض می‌شود: هلند ۶۳.۵ › سوئیس ۶۲.۵ › آلمان ۶۰ = انگلستان ۶۰ › سوئد ۵۷.۵ › دانمارک ۵۶.۵. فاصله‌ها کم است — این امتیازها قضاوت‌اند، نه اندازه‌گیری؛ در بخش «ب» وزن‌ها را خودتان عوض کنید و ببینید چه می‌شود.</t>
+          <t>۱) با وزن‌های جدید شما (کار پیدا کردن ۲۷.۵ = حقوق ۲۷.۵ / انگلیسی ۳۰ / هزینه ۱۵) و بودجهٔ $40,000 در سال: سوئیس ۶۶.۸ › هلند ۶۲.۸ › آلمان ۶۰ › انگلستان ۵۹.۵ › سوئد ۵۷.۸ › دانمارک ۵۷. برابر شدن وزن حقوق با کار، سوئیس را به صدر می‌برد؛ حتی اگر «کار» سوئیس را مثل قبل ۴ بگذارید باز سوئیس ۶۴ › هلند ۶۲.۸ است. ولی اختلاف ۱ تا ۴ امتیاز است — دو فینالیست دارید، نه یک برنده.</t>
         </is>
       </c>
     </row>
     <row r="61" ht="40" customHeight="1">
       <c r="A61" s="11" t="inlineStr">
         <is>
-          <t>۲) هلند اول می‌شود چون هر سه چیزی که برایتان مهم است را با هم دارد: انگلیسی‌دوست‌ترین بازار کار اروپا، کف حقوق HSM برای فارغ‌التحصیلان ($3,560/ماه) که یک جونیور می‌گیرد، و ۱۲ ماه zoekjaar. مشکلش فقط پول است: Twente/Radboud ≈ $10–20k بیشتر از بودجهٔ دو سال شما ($64k)؛ UvA یک‌ساله ≈ $57–62k. اگر این کسری با NL Scholarship ($5,700) + کار دانشجویی + کمک خانواده جور می‌شود، هلند انتخاب اول است.</t>
+          <t>۲) سوئیس: حقوق ۱۰/۱۰ ($103–127k ناخالص، خالص $6,900–8,110، پس‌انداز $1,820–3,630 در ماه) و با $40k/سال همهٔ گزینه‌های واقعی (HSLU، USI، Joint MSc، Basel، حتی UZH) در بودجه‌اند. «کار» را از ۴ به ۵ بردم چون فارغ‌التحصیلان دانشگاه‌های سوئیس طبق مادهٔ ۲۱(۳) قانون خارجیان از «اولویت نیروی داخلی» معاف‌اند؛ ولی مجوز کاریابی فقط ۶ ماه است و مجوز کار از سهمیهٔ کانتونی کم می‌شود (زوریخ ۲۰۲۵: ۳۹۹ L + ۲۴۹ B برای همهٔ رشته‌ها). یعنی ریسکِ «بعد از ۶ ماه شاید مجبور به ترک شوید» هنوز واقعی است.</t>
         </is>
       </c>
     </row>
     <row r="62" ht="40" customHeight="1">
       <c r="A62" s="11" t="inlineStr">
         <is>
-          <t>۳) سوئیس دوم است فقط به‌خاطر حقوق ($103–127k؛ خالص $6,900–8,110). ولی «کار پیدا کردن» که برایتان مهم‌تر است، در سوئیس ضعیف‌ترین حلقه است: ۶ ماه مجوز L، سهمیهٔ غیر-EU، رقابت با ETH/EPFL. HSLU (در بودجه) و USI (کمی بالاتر) گزینه‌های واقعی‌اند — به شرط پذیرفتن این ریسک که بعد از ۶ ماه شاید مجبور به ترک شوید.</t>
+          <t>۳) هلند: با $40k/سال، Radboud ($74–82k) در بودجه و Twente ($77–85k) مرزی است؛ UvA یک‌ساله ($57–62k) فقط اگر بودجهٔ دو سال را در یک سال خرج کنید. مزیت هلند نسبت به سوئیس: احتمال بالاتر ماندن (۱۲ ماه zoekjaar، کف HSM فارغ‌التحصیل $3,560/ماه که یک جونیور می‌گیرد، بازار انگلیسی‌زبان)؛ ضعفش: حقوق ۵/۱۰ و مسکن.</t>
         </is>
       </c>
     </row>
     <row r="63" ht="40" customHeight="1">
       <c r="A63" s="11" t="inlineStr">
         <is>
-          <t>۴) آلمان از اول به سوم می‌رود ولی همچنان امن‌ترین پشتوانه است: ارزان، حقوق $55–63k، ۱۸ ماه، بازار بزرگ؛ فقط نیمی از آگهی‌ها بدون آلمانی بسته‌اند. انگلستان با انگلیسیِ کامل هم بالا نمی‌آید، چون همان «کار» و «حقوق» در آن ضعیف‌ترین‌اند (بازار جونیور اشباع، اسپانسری $50,700+ نادر، حقوق $37–46k). سوئد (بازار ضعیف) و دانمارک (ویزا) کنار می‌روند.</t>
+          <t>۴) آلمان (۶۰) و انگلستان (۵۹.۵) دیگر رقیب صدر نیستند: آلمان پشتوانهٔ امن (ارزان، ۱۸ ماه، حقوق $55–63k، ولی آلمانی برای نیمی از بازار)؛ انگلستان با بودجهٔ جدید فقط Teesside/Northumbria/Essex را می‌گیرد (Russell Group $62–87k مگر با خرج دو سال در یک سال) و بازار جونیورش ضعیف است. سوئد و دانمارک حذف.</t>
         </is>
       </c>
     </row>
     <row r="64" ht="40" customHeight="1">
       <c r="A64" s="11" t="inlineStr">
         <is>
-          <t>۵) توصیهٔ نهایی با وزن‌های شما: ۸ درخواست — ۳ هلند (Twente، Radboud، UvA SE) + ۲ سوئیس (HSLU، USI) + ۲ آلمان (Stuttgart، Darmstadt یا Saarland) + ۱ انگلستان (Essex) به‌عنوان پذیرش قطعیِ ۱۰۰٪ انگلیسی. دو سؤالی که فقط شما می‌توانید جواب دهید: (۱) $10–20k بالاتر از بودجه برای هلند شدنی است؟ (۲) ریسک ۶ ماههٔ سوئیس را می‌پذیرید؟ اگر هر دو «نه» → آلمان (Stuttgart/Darmstadt) + Essex.</t>
+          <t>۵) توصیه: ۹ درخواست — ۳ سوئیس (HSLU، USI، Basel یا Neuchâtel) + ۳ هلند (Twente، Radboud، UvA SE) + ۲ آلمان (Stuttgart، Darmstadt یا Saarland) + ۱ انگلستان (Essex؛ پذیرش قطعی). انتخاب نهایی بین سوئیس و هلند را در می–ژوئن ۲۰۲۷ با پذیرش‌ها، بورس و مسکن بگیرید: اگر پذیرش HSLU/USI آمد و ریسک ۶ ماه را می‌پذیرید → سوئیس؛ اگر نه → Radboud/Twente؛ اگر هیچ‌کدام → Stuttgart/Darmstadt + Essex.</t>
         </is>
       </c>
     </row>
@@ -2675,28 +2676,28 @@
     <row r="67" ht="34" customHeight="1">
       <c r="A67" s="11" t="inlineStr">
         <is>
-          <t>اکتبر – دسامبر ۲۰۲۶: تکلیف نظام‌وظیفه · رزرو IELTS Academic خارج از ایران (استانبول / ایروان / دبی؛ هدف ۷.۰ — برای هلند ۶.۵ کافی است) و گرفتن آن تا دسامبر · ترجمهٔ رسمی ریزنمرات و دانشنامه · شرایط NL Scholarship را در Twente / Radboud / UvA چک کنید.</t>
+          <t>اکتبر – دسامبر ۲۰۲۶: تکلیف نظام‌وظیفه · رزرو IELTS Academic خارج از ایران (استانبول / ایروان / دبی؛ هدف ۷.۰ — هلند ۶.۵، USI B2 کافی است) و گرفتن آن تا دسامبر · ترجمهٔ رسمی ریزنمرات و دانشنامه · گواهی رتبهٔ کلاسی از سمنان (برای سوئیس مفید است) · شرایط NL Scholarship را در Twente / Radboud / UvA چک کنید.</t>
         </is>
       </c>
     </row>
     <row r="68" ht="34" customHeight="1">
       <c r="A68" s="11" t="inlineStr">
         <is>
-          <t>۱۵ ژانویه ۲۰۲۷: مهلت Stuttgart (و BTH اگر پشتوانهٔ سوئد را خواستید).</t>
+          <t>۱۵ ژانویه ۲۰۲۷: مهلت Stuttgart (و BTH اگر پشتوانهٔ سوئد را خواستید) · ۲۸ فوریه: UZH فقط اگر خواستید یک شانس کم (Reach، $180) بخرید.</t>
         </is>
       </c>
     </row>
     <row r="69" ht="34" customHeight="1">
       <c r="A69" s="11" t="inlineStr">
         <is>
-          <t>۱ فوریه – ۱ می ۲۰۲۷: NL Scholarship (۱ فوریه یا ۱ می، بسته به دانشگاه) · Radboud و UvA (≈ ۱ آوریل) · HSLU (۱ آوریل) · USI (۳۰ آوریل) · Twente (۱ می) · Darmstadt / Saarland (می – ژوئیه) · Essex rolling.</t>
+          <t>۱ فوریه – ۱ می ۲۰۲۷: NL Scholarship (۱ فوریه یا ۱ می، بسته به دانشگاه) · Neuchâtel (۳۱ مارس) · HSLU، Radboud و UvA (۱ آوریل) · USI و Basel (۳۰ آوریل) · Twente (۱ می) · Darmstadt / Saarland (می – ژوئیه) · Essex rolling.</t>
         </is>
       </c>
     </row>
     <row r="70" ht="34" customHeight="1">
       <c r="A70" s="11" t="inlineStr">
         <is>
-          <t>می – ژوئیه ۲۰۲۷: پول سال اول نقد و قابل انتقال (هلند: شهریه + $15,500 زندگی به حساب دانشگاه · سوئیس $25,400 · آلمان حساب مسدود $13,600) → ویزا (هلند از باکو؛ سوئیس سفارت تهران؛ آلمان سفارت فقط اضطراری → برنامهٔ B از ترکیه / ارمنستان).</t>
+          <t>می – ژوئیه ۲۰۲۷: پول سال اول نقد و قابل انتقال (سوئیس $25,400 در بانک سوئیسی — Basel $29,000 · هلند: شهریه + $15,500 زندگی به حساب دانشگاه · آلمان حساب مسدود $13,600) → ویزا (سوئیس سفارت تهران؛ هلند از باکو؛ آلمان سفارت فقط اضطراری → برنامهٔ B از ترکیه / ارمنستان).</t>
         </is>
       </c>
     </row>
@@ -3323,7 +3324,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>سازگاری با بودجه $32,000 در سال</t>
+          <t>سازگاری با بودجهٔ جدید $40,000 در سال (از ۲۸ سپتامبر؛ قبلاً $32,000)</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
@@ -3333,32 +3334,32 @@
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>❌ کسری $5,500–13,000 در هر سال</t>
+          <t>✅ مرزی — Radboud ($74–82k کل دوره) در بودجهٔ دو سال ($80k)؛ Twente ($77–85k) ۰ تا −$5k در کل دوره (NL Scholarship $5,700 جبران می‌کند)؛ Amsterdam/Delft/Utrecht کسری $5–10k؛ UvA یک‌ساله ($57–62k) فقط اگر بودجهٔ دو سال را در یک سال خرج کنید</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>✅ (Linköping دقیقاً مرزی)</t>
+          <t>✅ راحت (حتی Linköping)</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>⚠️ مرزی؛ AAU تقریباً در بودجه، SDU کسری تا ≈ $6,000 در سال</t>
+          <t>✅ AAU و SDU در بودجه — ولی مشکل ویزا (ردیف ۲۳) سر جایش است</t>
         </is>
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>⚠️ فقط Neuchâtel/Fribourg (و با صرفه‌جویی Lucerne/Lugano) در بودجه؛ Zürich/Lausanne کسری $1,000–10,000 در سال؛ کار دانشجویی در ۶ ماه اول ممنوع → سال اول تماماً از جیب</t>
+          <t>✅ HSLU / USI / Joint MSc / Basel / UZH / Bern راحت؛ ETH / EPFL مرزی (تا −$2k در سال)؛ کار دانشجویی در ۶ ماه اول ممنوع → سال اول تماماً از جیب</t>
         </is>
       </c>
       <c r="H11" s="12" t="inlineStr">
         <is>
-          <t>❌ کسری $6,000–33,000 (کمترین: Teesside ≈ $6–10k؛ Northumbria ≈ $12–16k)</t>
+          <t>⚠️ برنامهٔ یک‌ساله = یک سال بودجه ($40k): Teesside ✓ ($38–41k)؛ Northumbria کسری $4–8k؛ Essex کسری $9–14k (با بورس $6k → $3–8k)؛ Russell Group ($62–87k) ❌ — مگر بودجهٔ دو سال را در یک سال خرج کنید (آن‌وقت همه به‌جز London/Imperial)</t>
         </is>
       </c>
       <c r="I11" s="18" t="inlineStr">
         <is>
-          <t>محاسبه از ردیف ۷</t>
+          <t>محاسبه از ردیف‌های ۷ و ۸؛ فرض: $40k برای هر سال تحصیل</t>
         </is>
       </c>
     </row>
@@ -4271,42 +4272,42 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>امتیاز با وزن‌های شما (۲۸ سپتامبر): کار پیدا کردن ۳۰٪ / حقوق ۲۵٪ / فقط انگلیسی ۳۰٪ / هزینهٔ کل ۱۵٪ — از ۱۰۰ (زیرامتیازها از ۱۰)</t>
+          <t>امتیاز با وزن‌های شما (۲۸ سپتامبر، نسخهٔ دوم): کار پیدا کردن ۲۷.۵٪ = حقوق ۲۷.۵٪ / فقط انگلیسی ۳۰٪ / هزینهٔ کل ۱۵٪ — از ۱۰۰ (زیرامتیازها از ۱۰)؛ بودجهٔ جدید $40,000 در سال</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">
         <is>
-          <t>کار ۶ · حقوق ۶ · انگلیسی ۴ · هزینه ۱۰ → ۶۰ (سوم، برابر با انگلستان)</t>
+          <t>کار ۶ · حقوق ۶ · انگلیسی ۴ · هزینه ۱۰ → ۶۰ (سوم)</t>
         </is>
       </c>
       <c r="D31" s="12" t="inlineStr">
         <is>
-          <t>کار ۸ · حقوق ۵ · انگلیسی ۸ · هزینه ۲ → ۶۳.۵ (اول)</t>
+          <t>کار ۸ · حقوق ۵ · انگلیسی ۸ · هزینه ۲ → ۶۲.۸ (دوم)</t>
         </is>
       </c>
       <c r="E31" s="12" t="inlineStr">
         <is>
-          <t>کار ۴ · حقوق ۵ · انگلیسی ۸ · هزینه ۶ → ۵۷.۵ (پنجم)</t>
+          <t>کار ۴ · حقوق ۵ · انگلیسی ۸ · هزینه ۶ → ۵۷.۸ (پنجم)</t>
         </is>
       </c>
       <c r="F31" s="12" t="inlineStr">
         <is>
-          <t>کار ۵ · حقوق ۷ · انگلیسی ۶ · هزینه ۴ → ۵۶.۵ (ششم؛ ویزا از تهران عملاً بسته)</t>
+          <t>کار ۵ · حقوق ۷ · انگلیسی ۶ · هزینه ۴ → ۵۷ (ششم؛ ویزا از تهران عملاً بسته)</t>
         </is>
       </c>
       <c r="G31" s="12" t="inlineStr">
         <is>
-          <t>کار ۴ · حقوق ۱۰ · انگلیسی ۶ · هزینه ۵ → ۶۲.۵ (دوم)</t>
+          <t>کار ۵ · حقوق ۱۰ · انگلیسی ۶ · هزینه ۵ → ۶۶.۸ (اول)</t>
         </is>
       </c>
       <c r="H31" s="12" t="inlineStr">
         <is>
-          <t>کار ۵ · حقوق ۳ · انگلیسی ۱۰ · هزینه ۵ → ۶۰ (سوم، برابر با آلمان)</t>
+          <t>کار ۵ · حقوق ۳ · انگلیسی ۱۰ · هزینه ۵ → ۵۹.۵ (چهارم)</t>
         </is>
       </c>
       <c r="I31" s="18" t="inlineStr">
         <is>
-          <t>ارزیابی من با وزن‌هایی که گفتید (کار، حقوق و انگلیسی سنگین‌تر از هزینه). «کار» = بازار جونیورِ فقط‌انگلیسی (ردیف ۲۶) + مدت اقامت کاریابی (ردیف ۱۵) + دست‌یافتنی بودن کف اسپانسری (ردیف ۱۶ در برابر ۱۷)؛ «حقوق» = ردیف‌های ۱۷–۱۹؛ «انگلیسی» و «هزینه» همان ردیف ۲۸. فاصله‌ها کم است (۵۶.۵ تا ۶۳.۵) — امتیازها قضاوت‌اند؛ در شیت «تصمیم» وزن‌ها را خودتان عوض کنید. با حذف هزینه: هلند ۷۱ › سوئیس ۶۵ › انگلستان ۶۱.۵ › دانمارک ۵۹.۵ › سوئد ۵۷ › آلمان ۵۳؛ با حقوق سنگین‌تر (۳۰/۳۵/۲۵/۱۰): سوئیس ۶۷ › هلند ۶۳.۵ › آلمان ۵۹.</t>
+          <t>ارزیابی من با وزن‌های شما: کار پیدا کردن و حقوق برابر (۲۷.۵٪ هر کدام)، انگلیسی ۳۰٪، هزینه ۱۵٪. «کار» = بازار جونیورِ فقط‌انگلیسی (ردیف ۲۶) + مدت اقامت کاریابی (ردیف ۱۵) + دست‌یافتنی بودن کف اسپانسری (ردیف ۱۶ در برابر ۱۷)؛ «حقوق» = ردیف‌های ۱۷–۱۹. تغییر نسبت به نسخهٔ قبل: «کار» سوئیس از ۴ به ۵، چون فارغ‌التحصیلان دانشگاه‌های سوئیس طبق مادهٔ ۲۱(۳) قانون خارجیان (AIG) از «اولویت نیروی داخلی» معاف‌اند (سهمیهٔ کانتونی و پنجرهٔ ۶ ماهه باقی است). حتی با «کار» سوئیس = ۴ هم با این وزن‌ها سوئیس ۶۴ › هلند ۶۲.۸ می‌شود. حساسیت: کار ۳۰ / حقوق ۳۰ / انگلیسی ۳۰ / هزینه ۱۰ → سوئیس ۶۸ › هلند ۶۵ › انگلستان ۵۹ › آلمان ۵۸ = دانمارک ۵۸ › سوئد ۵۷. در همهٔ حالت‌ها سوئیس و هلند دو فینالیست‌اند (اختلاف ۱–۴ امتیاز)؛ امتیازها قضاوت‌اند و در شیت «تصمیم» وزن‌ها قابل تغییرند.</t>
         </is>
       </c>
     </row>
@@ -5249,7 +5250,7 @@
         <f>438</f>
         <v/>
       </c>
-      <c r="O10" s="15" t="inlineStr">
+      <c r="O10" s="13" t="inlineStr">
         <is>
           <t>Safe/Target</t>
         </is>
@@ -5338,7 +5339,7 @@
         <f>438</f>
         <v/>
       </c>
-      <c r="O11" s="15" t="inlineStr">
+      <c r="O11" s="13" t="inlineStr">
         <is>
           <t>Safe/Target</t>
         </is>
@@ -5427,7 +5428,7 @@
         <f>314</f>
         <v/>
       </c>
-      <c r="O12" s="13" t="inlineStr">
+      <c r="O12" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -5516,7 +5517,7 @@
         <f>314</f>
         <v/>
       </c>
-      <c r="O13" s="13" t="inlineStr">
+      <c r="O13" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -5601,7 +5602,7 @@
         <f>314</f>
         <v/>
       </c>
-      <c r="O14" s="13" t="inlineStr">
+      <c r="O14" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -5691,7 +5692,7 @@
           <t>353</t>
         </is>
       </c>
-      <c r="O15" s="15" t="inlineStr">
+      <c r="O15" s="13" t="inlineStr">
         <is>
           <t>Safe/Target</t>
         </is>
@@ -5781,7 +5782,7 @@
           <t>353</t>
         </is>
       </c>
-      <c r="O16" s="15" t="inlineStr">
+      <c r="O16" s="13" t="inlineStr">
         <is>
           <t>Safe/Target</t>
         </is>
@@ -5867,7 +5868,7 @@
           <t>415</t>
         </is>
       </c>
-      <c r="O17" s="13" t="inlineStr">
+      <c r="O17" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -5956,7 +5957,7 @@
         <f>485</f>
         <v/>
       </c>
-      <c r="O18" s="13" t="inlineStr">
+      <c r="O18" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -6046,7 +6047,7 @@
           <t>≈ 800–1000</t>
         </is>
       </c>
-      <c r="O19" s="15" t="inlineStr">
+      <c r="O19" s="13" t="inlineStr">
         <is>
           <t>Safe/Target</t>
         </is>
@@ -6135,7 +6136,7 @@
         <f>246</f>
         <v/>
       </c>
-      <c r="O20" s="13" t="inlineStr">
+      <c r="O20" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -6224,7 +6225,7 @@
         <f>246</f>
         <v/>
       </c>
-      <c r="O21" s="13" t="inlineStr">
+      <c r="O21" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -6313,7 +6314,7 @@
         <f>158</f>
         <v/>
       </c>
-      <c r="O22" s="14" t="inlineStr">
+      <c r="O22" s="15" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
@@ -6402,7 +6403,7 @@
         <f>158</f>
         <v/>
       </c>
-      <c r="O23" s="13" t="inlineStr">
+      <c r="O23" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -6492,7 +6493,7 @@
           <t>149</t>
         </is>
       </c>
-      <c r="O24" s="14" t="inlineStr">
+      <c r="O24" s="15" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
@@ -7028,7 +7029,7 @@
         <f>69</f>
         <v/>
       </c>
-      <c r="O30" s="14" t="inlineStr">
+      <c r="O30" s="15" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
@@ -7206,7 +7207,7 @@
         <f>94</f>
         <v/>
       </c>
-      <c r="O32" s="13" t="inlineStr">
+      <c r="O32" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -7295,7 +7296,7 @@
         <f>456</f>
         <v/>
       </c>
-      <c r="O33" s="13" t="inlineStr">
+      <c r="O33" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -7384,7 +7385,7 @@
         <f>456</f>
         <v/>
       </c>
-      <c r="O34" s="13" t="inlineStr">
+      <c r="O34" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -7473,7 +7474,7 @@
         <f>456</f>
         <v/>
       </c>
-      <c r="O35" s="13" t="inlineStr">
+      <c r="O35" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -7563,7 +7564,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O36" s="15" t="inlineStr">
+      <c r="O36" s="13" t="inlineStr">
         <is>
           <t>Safe/Target</t>
         </is>
@@ -7652,7 +7653,7 @@
         <f>191</f>
         <v/>
       </c>
-      <c r="O37" s="13" t="inlineStr">
+      <c r="O37" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -7742,7 +7743,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O38" s="13" t="inlineStr">
+      <c r="O38" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -7831,7 +7832,7 @@
         <f>670</f>
         <v/>
       </c>
-      <c r="O39" s="13" t="inlineStr">
+      <c r="O39" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -7920,7 +7921,7 @@
         <f>150</f>
         <v/>
       </c>
-      <c r="O40" s="14" t="inlineStr">
+      <c r="O40" s="15" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
@@ -8099,7 +8100,7 @@
           <t>851–900</t>
         </is>
       </c>
-      <c r="O42" s="14" t="inlineStr">
+      <c r="O42" s="15" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
@@ -8545,7 +8546,7 @@
           <t>318</t>
         </is>
       </c>
-      <c r="O47" s="13" t="inlineStr">
+      <c r="O47" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -8635,7 +8636,7 @@
           <t>318</t>
         </is>
       </c>
-      <c r="O48" s="13" t="inlineStr">
+      <c r="O48" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -8725,7 +8726,7 @@
           <t>218</t>
         </is>
       </c>
-      <c r="O49" s="13" t="inlineStr">
+      <c r="O49" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -8815,7 +8816,7 @@
           <t>218</t>
         </is>
       </c>
-      <c r="O50" s="13" t="inlineStr">
+      <c r="O50" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -8905,7 +8906,7 @@
           <t>250</t>
         </is>
       </c>
-      <c r="O51" s="14" t="inlineStr">
+      <c r="O51" s="15" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
@@ -9084,7 +9085,7 @@
         <f>588 (CS ≈ 251)</f>
         <v/>
       </c>
-      <c r="O53" s="13" t="inlineStr">
+      <c r="O53" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -9173,7 +9174,7 @@
         <f>588 (CS ≈ 251)</f>
         <v/>
       </c>
-      <c r="O54" s="13" t="inlineStr">
+      <c r="O54" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -9443,7 +9444,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O57" s="15" t="inlineStr">
+      <c r="O57" s="13" t="inlineStr">
         <is>
           <t>Safe/Target</t>
         </is>
@@ -9529,7 +9530,7 @@
           <t>— (UAS)</t>
         </is>
       </c>
-      <c r="O58" s="13" t="inlineStr">
+      <c r="O58" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -9709,7 +9710,7 @@
           <t>— (UAS)</t>
         </is>
       </c>
-      <c r="O60" s="13" t="inlineStr">
+      <c r="O60" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -10068,7 +10069,7 @@
           <t>223</t>
         </is>
       </c>
-      <c r="O64" s="13" t="inlineStr">
+      <c r="O64" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -10158,7 +10159,7 @@
           <t>223</t>
         </is>
       </c>
-      <c r="O65" s="13" t="inlineStr">
+      <c r="O65" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -10248,7 +10249,7 @@
           <t>223</t>
         </is>
       </c>
-      <c r="O66" s="13" t="inlineStr">
+      <c r="O66" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -10338,7 +10339,7 @@
           <t>283</t>
         </is>
       </c>
-      <c r="O67" s="13" t="inlineStr">
+      <c r="O67" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -10428,7 +10429,7 @@
           <t>283</t>
         </is>
       </c>
-      <c r="O68" s="13" t="inlineStr">
+      <c r="O68" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -10518,7 +10519,7 @@
           <t>119</t>
         </is>
       </c>
-      <c r="O69" s="14" t="inlineStr">
+      <c r="O69" s="15" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
@@ -10608,7 +10609,7 @@
           <t>157</t>
         </is>
       </c>
-      <c r="O70" s="14" t="inlineStr">
+      <c r="O70" s="15" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
@@ -10698,7 +10699,7 @@
           <t>157</t>
         </is>
       </c>
-      <c r="O71" s="13" t="inlineStr">
+      <c r="O71" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -10964,7 +10965,7 @@
           <t>60</t>
         </is>
       </c>
-      <c r="O74" s="14" t="inlineStr">
+      <c r="O74" s="15" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
@@ -11410,7 +11411,7 @@
           <t>— (UAS)</t>
         </is>
       </c>
-      <c r="O79" s="15" t="inlineStr">
+      <c r="O79" s="13" t="inlineStr">
         <is>
           <t>Safe/Target</t>
         </is>
@@ -11500,7 +11501,7 @@
           <t>308</t>
         </is>
       </c>
-      <c r="O80" s="13" t="inlineStr">
+      <c r="O80" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -11590,7 +11591,7 @@
           <t>308</t>
         </is>
       </c>
-      <c r="O81" s="13" t="inlineStr">
+      <c r="O81" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -11766,7 +11767,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O83" s="15" t="inlineStr">
+      <c r="O83" s="13" t="inlineStr">
         <is>
           <t>Safe/Target</t>
         </is>
@@ -12032,7 +12033,7 @@
           <t>82</t>
         </is>
       </c>
-      <c r="O86" s="14" t="inlineStr">
+      <c r="O86" s="15" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
@@ -12122,7 +12123,7 @@
           <t>174</t>
         </is>
       </c>
-      <c r="O87" s="14" t="inlineStr">
+      <c r="O87" s="15" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
@@ -12212,7 +12213,7 @@
           <t>174</t>
         </is>
       </c>
-      <c r="O88" s="13" t="inlineStr">
+      <c r="O88" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -12298,7 +12299,7 @@
           <t>174</t>
         </is>
       </c>
-      <c r="O89" s="13" t="inlineStr">
+      <c r="O89" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -12384,7 +12385,7 @@
           <t>225</t>
         </is>
       </c>
-      <c r="O90" s="13" t="inlineStr">
+      <c r="O90" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -12474,7 +12475,7 @@
           <t>87</t>
         </is>
       </c>
-      <c r="O91" s="14" t="inlineStr">
+      <c r="O91" s="15" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
@@ -12564,7 +12565,7 @@
           <t>438</t>
         </is>
       </c>
-      <c r="O92" s="13" t="inlineStr">
+      <c r="O92" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -12919,7 +12920,7 @@
         <f>329</f>
         <v/>
       </c>
-      <c r="O96" s="13" t="inlineStr">
+      <c r="O96" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -13008,7 +13009,7 @@
         <f>329</f>
         <v/>
       </c>
-      <c r="O97" s="13" t="inlineStr">
+      <c r="O97" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -13093,7 +13094,7 @@
         <f>329</f>
         <v/>
       </c>
-      <c r="O98" s="13" t="inlineStr">
+      <c r="O98" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -13182,7 +13183,7 @@
         <f>329</f>
         <v/>
       </c>
-      <c r="O99" s="13" t="inlineStr">
+      <c r="O99" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -13271,7 +13272,7 @@
         <f>283</f>
         <v/>
       </c>
-      <c r="O100" s="13" t="inlineStr">
+      <c r="O100" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -13360,7 +13361,7 @@
         <f>283</f>
         <v/>
       </c>
-      <c r="O101" s="13" t="inlineStr">
+      <c r="O101" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -13449,7 +13450,7 @@
         <f>283</f>
         <v/>
       </c>
-      <c r="O102" s="13" t="inlineStr">
+      <c r="O102" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -13538,7 +13539,7 @@
         <f>283</f>
         <v/>
       </c>
-      <c r="O103" s="13" t="inlineStr">
+      <c r="O103" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -13627,7 +13628,7 @@
         <f>283</f>
         <v/>
       </c>
-      <c r="O104" s="13" t="inlineStr">
+      <c r="O104" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -13713,7 +13714,7 @@
           <t>— (تخصصی)</t>
         </is>
       </c>
-      <c r="O105" s="13" t="inlineStr">
+      <c r="O105" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -13803,7 +13804,7 @@
           <t>— (تخصصی)</t>
         </is>
       </c>
-      <c r="O106" s="13" t="inlineStr">
+      <c r="O106" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -13893,7 +13894,7 @@
           <t>— (تخصصی)</t>
         </is>
       </c>
-      <c r="O107" s="13" t="inlineStr">
+      <c r="O107" s="14" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -14241,7 +14242,7 @@
           <t>128</t>
         </is>
       </c>
-      <c r="O111" s="14" t="inlineStr">
+      <c r="O111" s="15" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
@@ -20514,12 +20515,12 @@
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>نتیجه با وزن‌های شما (کار ۳۰ / حقوق ۲۵ / انگلیسی ۳۰ / هزینه ۱۵) — ۲۸ سپتامبر</t>
+          <t>نتیجه با وزن‌های شما (کار ۲۷.۵ = حقوق ۲۷.۵ / انگلیسی ۳۰ / هزینه ۱۵) و بودجهٔ $40,000 در سال — ۲۸ سپتامبر</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>هلند ۶۳.۵ › سوئیس ۶۲.۵ › آلمان ۶۰ = انگلستان ۶۰ › سوئد ۵۷.۵ › دانمارک ۵۶.۵ (ردیف ۲۸ب). وقتی «کار پیدا کردن»، «حقوق» و «انگلیسی» را سنگین‌تر از هزینه می‌کنید، هلند و سوئیس بالا می‌آیند و آلمان به سوم می‌رود؛ انگلستان با وجود انگلیسیِ کامل بالا نمی‌آید، چون همان دو معیار «کار» (بازار جونیور اشباع، اسپانسری $50,700+ نادر) و «حقوق» ($37–46k) در آن ضعیف‌ترین‌اند. هلند: انگلیسی‌دوست‌ترین بازار، کف HSM فارغ‌التحصیل $3,560/ماه دست‌یافتنی، ۱۲ ماه zoekjaar — مشکل فقط پول است (Twente/Radboud ≈ $10–20k بالاتر از بودجهٔ دو سال؛ UvA یک‌ساله $39,100 شهریه + Amsterdam). سوئیس: حقوق ۱۰/۱۰ ولی «کار» ۴/۱۰ (۶ ماه مجوز L، سهمیه، رقابت با ETH/EPFL) — HSLU در بودجه، USI کمی بالاتر. توصیه با این وزن‌ها: ۳ هلند (Twente، Radboud، UvA SE) + ۲ سوئیس (HSLU، USI) + ۲ آلمان (Stuttgart، Darmstadt/Saarland) + ۱ انگلستان (Essex) — و دو سؤال که فقط شما جواب می‌دهید: کسری $10–20k برای هلند شدنی است؟ ریسک ۶ ماههٔ سوئیس را می‌پذیرید؟ اگر هر دو نه → آلمان.</t>
+          <t>سوئیس ۶۶.۸ › هلند ۶۲.۸ › آلمان ۶۰ › انگلستان ۵۹.۵ › سوئد ۵۷.۸ › دانمارک ۵۷ (ردیف ۲۸ب). وقتی حقوق هم‌وزن کار می‌شود، سوئیس (حقوق ۱۰/۱۰؛ $103–127k ناخالص، خالص $6,900–8,110) به صدر می‌رود و با بودجهٔ $40k/سال همهٔ گزینه‌های واقعی‌اش (HSLU $53–64k، USI $60–72k، Joint MSc $32–41k، Basel، UZH) در بودجه‌اند؛ ریسک اصلی همچنان پنجرهٔ ۶ ماههٔ کاریابی و سهمیهٔ کانتونی است (اولویت نیروی داخلی برای فارغ‌التحصیلان سوئیس طبق مادهٔ ۲۱(۳) AIG برداشته شده). هلند دوم است (۴ امتیاز کمتر): احتمال ماندن بالاتر (۱۲ ماه zoekjaar، کف HSM فارغ‌التحصیل $3,560/ماه، بازار انگلیسی‌زبان) ولی حقوق ۵/۱۰؛ با $40k/سال Radboud در بودجه و Twente مرزی است. آلمان ۶۰ پشتوانهٔ امن؛ انگلستان ۵۹.۵ فقط پذیرش قطعی یک‌ساله (Essex)؛ سوئد و دانمارک حذف. توصیه: ۹ درخواست — ۳ سوئیس (HSLU، USI، Basel یا Neuchâtel) + ۳ هلند (Twente، Radboud، UvA SE) + ۲ آلمان (Stuttgart، Darmstadt/Saarland) + ۱ انگلستان (Essex). انتخاب نهایی سوئیس/هلند در می–ژوئن ۲۰۲۷ با پذیرش‌ها: اگر HSLU/USI پذیرفتند و ریسک ۶ ماه را می‌پذیرید → سوئیس؛ اگر نه → Radboud/Twente.</t>
         </is>
       </c>
     </row>
@@ -20650,7 +20651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -21432,30 +21433,62 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
+          <t>بودجه و وزن‌ها – نسخهٔ دوم (۲۸ سپتامبر)</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>بودجه $32,000 → $40,000 در سال؛ وزن‌ها کار ۲۷.۵ = حقوق ۲۷.۵ / انگلیسی ۳۰ / هزینه ۱۵؛ «کار» سوئیس ۴ → ۵</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>گفتهٔ شما + مادهٔ ۲۱(۳) AIG (معافیت فارغ‌التحصیلان سوئیس از اولویت نیروی داخلی؛ سهمیه باقی است — SEM Weisungen §4.2)</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>قضاوت + قانون</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>۲۸ سپتامبر ۲۰۲۶</t>
+        </is>
+      </c>
+      <c r="F25" s="27" t="inlineStr">
+        <is>
+          <t>⚠️ نتیجه: سوئیس ۶۶.۸ › هلند ۶۲.۸ › آلمان ۶۰ › انگلستان ۵۹.۵ › سوئد ۵۷.۸ › دانمارک ۵۷؛ ردیف ۹ جدول اصلی با بودجهٔ جدید بازنویسی شد</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
           <t>کل فایل – وضعیت</t>
         </is>
       </c>
-      <c r="B25" s="12" t="inlineStr">
+      <c r="B26" s="12" t="inlineStr">
         <is>
           <t>≈ ۱,۶۰۰ سلول عددی؛ ≈ ۳۴۰ سلول با علامت ≈/برآورد</t>
         </is>
       </c>
-      <c r="C25" s="12" t="inlineStr">
+      <c r="C26" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D25" s="12" t="inlineStr">
+      <c r="D26" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E25" s="12" t="inlineStr">
+      <c r="E26" s="12" t="inlineStr">
         <is>
           <t>۲۸ سپتامبر ۲۰۲۶</t>
         </is>
       </c>
-      <c r="F25" s="12" t="inlineStr">
+      <c r="F26" s="12" t="inlineStr">
         <is>
           <t>خلاصه: تصمیم‌سازها (شهریه، ویزا، تمکن، مهلت، تطبیق نمره، بورس‌های اصلی، خوابگاه‌های اصلی) رسمی‌اند؛ حقوق، هزینهٔ زندگی، شانس خوابگاه و اجاره‌های شهرهای فرعی برآوردند و همان‌طور علامت خورده‌اند</t>
         </is>
@@ -21472,7 +21505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B217"/>
+  <dimension ref="A1:B218"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -24050,34 +24083,46 @@
     <row r="215">
       <c r="A215" s="12" t="inlineStr">
         <is>
-          <t>هلند – UvA شهریهٔ نهادی 2026/27 (دانشکدهٔ علوم، غیر-EEA: ارشد یک‌ساله €34,300، دوساله €26,000، CS مشترک با VU €24,150)</t>
+          <t>سوئیس – Art. 21 Abs. 3 AIG: فارغ‌التحصیلان سوئیس معاف از اولویت نیروی داخلی؛ سهمیه باقی است (SEM Weisungen §4.2؛ زوریخ ۲۰۲۵: ۳۹۹ L + ۲۴۹ B)</t>
         </is>
       </c>
       <c r="B215" s="30" t="inlineStr">
         <is>
-          <t>https://www.uva.nl/en/education/fees-and-funding/tuition-fees/tuition-fees.html</t>
+          <t>https://www.fedlex.admin.ch/eli/cc/2007/758/en#art_21</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="12" t="inlineStr">
         <is>
-          <t>هلند – UvA MSc Software Engineering: 60 ECTS، ۱۲ ماه، انگلیسی</t>
+          <t>هلند – UvA شهریهٔ نهادی 2026/27 (دانشکدهٔ علوم، غیر-EEA: ارشد یک‌ساله €34,300، دوساله €26,000، CS مشترک با VU €24,150)</t>
         </is>
       </c>
       <c r="B216" s="30" t="inlineStr">
         <is>
-          <t>https://www.uva.nl/en/programmes/masters/software-engineering/software-engineering.html</t>
+          <t>https://www.uva.nl/en/education/fees-and-funding/tuition-fees/tuition-fees.html</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="12" t="inlineStr">
         <is>
+          <t>هلند – UvA MSc Software Engineering: 60 ECTS، ۱۲ ماه، انگلیسی</t>
+        </is>
+      </c>
+      <c r="B217" s="30" t="inlineStr">
+        <is>
+          <t>https://www.uva.nl/en/programmes/masters/software-engineering/software-engineering.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="12" t="inlineStr">
+        <is>
           <t>هلند – Twente: مهلت غیر-EEA ۱ می ۲۰۲۷؛ بورس UTS ۱۵ اکتبر ۲۰۲۶ – ۱ آوریل ۲۰۲۷</t>
         </is>
       </c>
-      <c r="B217" s="30" t="inlineStr">
+      <c r="B218" s="30" t="inlineStr">
         <is>
           <t>https://collegedunia.com/netherlands/university/749-university-of-twente-enschede/admission</t>
         </is>
@@ -24301,6 +24346,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B215" r:id="rId214"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B216" r:id="rId215"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B217" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B218" r:id="rId217"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Budget model: tuition + first months' living, then student work (v3.3)
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Table_final.xlsx
+++ b/Table_final.xlsx
@@ -209,22 +209,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="2"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -638,7 +638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O79"/>
+  <dimension ref="A1:O86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -661,14 +661,14 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>تصمیم در یک صفحه — شایان، ورودی سپتامبر ۲۰۲۷، بودجه $40,000 برای کل دوره</t>
+          <t>تصمیم در یک صفحه — شایان، ورودی سپتامبر ۲۰۲۷، بودجه $40,000 = شهریه + زندگی تا پیدا شدن کار دانشجویی</t>
         </is>
       </c>
     </row>
     <row r="2" ht="52" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>همهٔ مبالغ این فایل به دلار آمریکا تبدیل شده‌اند تا لازم نباشد چیزی را خودتان تبدیل کنید. نرخ‌های ۲۸ سپتامبر ۲۰۲۶: ۱ یورو = ۱.۱۴ دلار · ۱ پوند = ۱.۳۲۵ دلار · ۱ فرانک سوئیس = ۱.۲۱ دلار · ۱ کرون سوئد = ۰.۱۰ دلار · ۱ کرون دانمارک = ۰.۱۵ دلار. اعداد گرد شده‌اند (زیر ۱۰ هزار به ۱۰ دلار، بالاتر به ۱۰۰ دلار)؛ رقم رسمی به ارز محلی فقط در شیت «راستی‌آزمایی» داخل پرانتز آمده است. شهریه‌ها سطح 2026/27 هستند (Bristol 2027/28)؛ نرخ سال ورود شما (2027/28) بین اکتبر ۲۰۲۶ تا بهار ۲۰۲۷ منتشر می‌شود — ۳ تا ۵ درصد بالاتر بگیرید؛ ⚠️ ETH/EPFL ممکن است با بستهٔ EP27 از ۲۰۲۷ دوباره گران شوند. وزن‌ها: کار پیدا کردن = حقوق (۲۷.۵٪)، انگلیسی ۳۰٪، هزینه ۱۵٪ — بودجه $40,000 برای کل دوره (گفتهٔ شما، ۲۸ سپتامبر).</t>
+          <t>همهٔ مبالغ این فایل به دلار آمریکا تبدیل شده‌اند تا لازم نباشد چیزی را خودتان تبدیل کنید. نرخ‌های ۲۸ سپتامبر ۲۰۲۶: ۱ یورو = ۱.۱۴ دلار · ۱ پوند = ۱.۳۲۵ دلار · ۱ فرانک سوئیس = ۱.۲۱ دلار · ۱ کرون سوئد = ۰.۱۰ دلار · ۱ کرون دانمارک = ۰.۱۵ دلار. اعداد گرد شده‌اند (زیر ۱۰ هزار به ۱۰ دلار، بالاتر به ۱۰۰ دلار)؛ رقم رسمی به ارز محلی فقط در شیت «راستی‌آزمایی» داخل پرانتز آمده است. شهریه‌ها سطح 2026/27 هستند (Bristol 2027/28)؛ نرخ سال ورود شما (2027/28) بین اکتبر ۲۰۲۶ تا بهار ۲۰۲۷ منتشر می‌شود — ۳ تا ۵ درصد بالاتر بگیرید؛ ⚠️ ETH/EPFL ممکن است با بستهٔ EP27 از ۲۰۲۷ دوباره گران شوند. وزن‌ها: کار پیدا کردن = حقوق (۲۷.۵٪)، انگلیسی ۳۰٪، هزینه ۱۵٪ — بودجه $40,000 = کل شهریه + زندگی تا پیدا شدن کار دانشجویی (تعریف شما، ۲۸ سپتامبر).</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>الف) شش کشور در یک نگاه — اول سه کشوری که برنامه‌ای در بودجهٔ $40,000 کل دارند (به ترتیب امتیاز شما: کار = حقوق ۲۷.۵٪، انگلیسی ۳۰٪، هزینه ۱۵٪)، بعد سه کشور خارج از بودجه</t>
+          <t>الف) شش کشور در یک نگاه — اول کشورهایی که با مدل «$40,000 = شهریه + زندگی تا کار» جا می‌شوند (سوئیس، آلمان، انگلستان — به ترتیب امتیاز شما: کار = حقوق ۲۷.۵٪، انگلیسی ۳۰٪، هزینه ۱۵٪)، بعد سوئد (فقط با بورس)، هلند و دانمارک (❌)</t>
         </is>
       </c>
     </row>
@@ -703,12 +703,12 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
+          <t>🇸🇪 سوئد</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
           <t>🇳🇱 هلند</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>🇸🇪 سوئد</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -780,12 +780,12 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
+          <t>$14,100–16,800</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
           <t>$22,500–24,700</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>$14,100–16,800</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -819,12 +819,12 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
+          <t>$1,100–1,300</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
           <t>$1,250–1,700</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>$1,100–1,300</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -856,12 +856,12 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
+          <t>$27,000–32,500</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
           <t>$37,500–45,000</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>$27,000–32,500</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
@@ -895,12 +895,12 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
+          <t>$54,000–65,000</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
           <t>$75,000–90,000</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>$54,000–65,000</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
@@ -912,37 +912,38 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>با بودجهٔ $40,000 برای کل دوره جور درمی‌آید؟</t>
+          <t>با $40,000 = شهریه + زندگی تا کار جور درمی‌آید؟
+(ماه‌های پوشش بعد از شهریه)</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>⚠️ فقط Joint MSc Neuchâtel / Fribourg ($32–43k) و Basel با کار؛ HSLU / USI / UZH / ETH ❌</t>
+          <t>⚠️ ۶ ماه اول کار ممنوع، بعد ۱۵ ساعت: Neuchâtel / Fribourg ۱۸ ماه ✅، Basel ۱۶–۱۷ ماه ✅، HSLU ۱۵ ماه → ≈ $1,000/ماه ⚠️، USI ۱۰–۱۱ ماه ⚠️ پرریسک؛ اثبات $25,400</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>✅ Darmstadt / Saarland / Passau راحت؛ Stuttgart با Werkstudent</t>
+          <t>✅ حتی بدون کار: Darmstadt / Saarland / Passau ۲۴ ماه + اضافه؛ Stuttgart ۲۳ ماه</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>⚠️ Teesside مرزی؛ Northumbria / Essex فقط با ۲۰ ساعت کار؛ Russell Group ❌</t>
+          <t>✅ با ۲۰ ساعت کار (≈ $1,450/ماه): Teesside ۱۲ ماه بدون کار؛ Northumbria / Essex / MMU ۸ ماه → ≈ $500/ماه؛ Russell Group ❌</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>❌ $74–90k (کسری $34–50k)؛ فقط با بورس Reach</t>
+          <t>⚠️ LiU ۵–۶ ماه، BTH/MDU ۱۱ ماه → بقیه از کار بدون سوئدی سخت؛ فقط با بورس</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>❌ $51–65k (فقط با بورس ۵۰–۱۰۰٪)</t>
+          <t>❌ شهریهٔ دو سال $45–50k به‌تنهایی › $40k؛ UvA یک‌ساله $900 برای زندگی</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>❌ $63–76k + ویزا</t>
+          <t>❌ AAU ۴ ماه پوشش + ویزا</t>
         </is>
       </c>
     </row>
@@ -972,16 +973,16 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
+          <t>خوب
+(BTH/Halmstad راحت؛ LiU Target)</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
           <t>متوسط
 (Twente/Radboud Target)</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>خوب
-(BTH/Halmstad راحت؛ LiU Target)</t>
-        </is>
-      </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
           <t>متوسط
@@ -1015,15 +1016,15 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>NL Scholarship $5,700 (یک‌بار)</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
           <t>Halmstad ۲۵–۵۰٪ · MDU تا ۱۰۰٪
 (LiU ۵۰٪ فقط با معدل بالاتر)</t>
         </is>
       </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>NL Scholarship $5,700 (یک‌بار)</t>
+        </is>
+      </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
           <t>≈ ۱۵ بورس AAU (بعید)</t>
@@ -1056,16 +1057,16 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
+          <t>$350–900
+(۱۵ ساعت؛ کمیاب)</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
           <t>تا $1,150
 (۱۶ ساعت؛ مجوز TWV)</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>$350–900
-(۱۵ ساعت؛ کمیاب)</t>
-        </is>
-      </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
           <t>$1,200–1,850
@@ -1171,12 +1172,12 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
+          <t>$42,000–55,000</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
           <t>$46,000–57,000</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>$42,000–55,000</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
@@ -1209,12 +1210,12 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
+          <t>$2,850–3,300</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
           <t>$3,100–3,550</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>$2,850–3,300</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1246,12 +1247,12 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
+          <t>$1,050–1,600</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
           <t>$800–1,350</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>$1,050–1,600</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
@@ -1283,12 +1284,12 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
+          <t>۴</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
           <t>۸</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>۴</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
@@ -1320,12 +1321,12 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
+          <t>ممکن (آنلاین، بدون بیومتریک)</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
           <t>سخت (از باکو)</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>ممکن (آنلاین، بدون بیومتریک)</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
@@ -1361,16 +1362,16 @@
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
+          <t>۵۷.۸
+(۴ / ۵ / ۸ / ۶)</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
           <t>۶۲.۸
 (۸ / ۵ / ۸ / ۲)</t>
         </is>
       </c>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>۵۷.۸
-(۴ / ۵ / ۸ / ۶)</t>
-        </is>
-      </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
           <t>۵۷
@@ -1401,12 +1402,12 @@
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
+          <t>۱۹</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
           <t>۱۸</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="inlineStr">
-        <is>
-          <t>۱۹</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
@@ -1423,27 +1424,27 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>اول در امتیاز — ولی فقط Joint MSc / Basel، روی لبهٔ بودجه؛ شرط‌بندی حساب‌شده با پاداش $103–127k</t>
+          <t>اول در امتیاز (حقوق ۱۰/۱۰) — Neuchâtel / Basel / HSLU شدنی؛ ولی ۶ ماه بدون درآمد، اثبات $25,400 و ۶ ماه بعد از مدرک = ریسک</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>دوم در امتیاز، اول در امنیت — تنها کشوری که با $40k کل راحت جا می‌شود و بهترین شانس استخدام (Werkstudent → کار)؛ بهایش آلمانی B1</t>
+          <t>امن‌ترین — بدون نیاز به کار جا می‌شود و Werkstudent بهترین راه استخدام است؛ بهایش آلمانی B1</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>سوم — فقط Teesside / Northumbria / Essex با ۲۰ ساعت کار؛ بازار جونیور و اسپانسری ضعیف</t>
+          <t>انگلیسیِ کامل، کار دانشجویی آسان، ۱ ساله — ولی بازار جونیور و حقوق ضعیف‌ترین</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>❌ خارج از بودجه ($74–90k)؛ فقط با بورس Reach</t>
+          <t>فقط با بورس؛ بازار و کار دانشجویی بدون سوئدی ضعیف</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>❌ خارج از بودجه (و بازار ضعیف)</t>
+          <t>❌ شهریه به‌تنهایی بودجه را می‌خورد؛ فقط با بورس Reach</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
@@ -1488,12 +1489,12 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
+          <t>🇸🇪 سوئد</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
           <t>🇳🇱 هلند</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>🇸🇪 سوئد</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
@@ -1521,10 +1522,10 @@
         <v>5</v>
       </c>
       <c r="F28" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G28" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="G28" s="6" t="n">
-        <v>4</v>
       </c>
       <c r="H28" s="6" t="n">
         <v>5</v>
@@ -1605,10 +1606,10 @@
         <v>5</v>
       </c>
       <c r="F31" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="G31" s="6" t="n">
         <v>2</v>
-      </c>
-      <c r="G31" s="6" t="n">
-        <v>6</v>
       </c>
       <c r="H31" s="6" t="n">
         <v>4</v>
@@ -1668,10 +1669,10 @@
         <v>59.5</v>
       </c>
       <c r="F33" s="8" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="G33" s="8" t="n">
         <v>62.8</v>
-      </c>
-      <c r="G33" s="8" t="n">
-        <v>57.8</v>
       </c>
       <c r="H33" s="8" t="n">
         <v>57</v>
@@ -1694,10 +1695,10 @@
         <v>4</v>
       </c>
       <c r="F34" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G34" s="6" t="n">
         <v>2</v>
-      </c>
-      <c r="G34" s="6" t="n">
-        <v>5</v>
       </c>
       <c r="H34" s="6" t="n">
         <v>6</v>
@@ -1720,10 +1721,10 @@
         <v>19</v>
       </c>
       <c r="F35" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="G35" s="6" t="n">
         <v>18</v>
-      </c>
-      <c r="G35" s="6" t="n">
-        <v>19</v>
       </c>
       <c r="H35" s="6" t="n">
         <v>16</v>
@@ -1732,38 +1733,38 @@
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>در بودجهٔ $40,000 کل؟</t>
+          <t>با $40,000 = شهریه + زندگی تا کار؟</t>
         </is>
       </c>
       <c r="B36" s="9" t="inlineStr"/>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>⚠️ فقط Joint MSc / Basel</t>
+          <t>⚠️ ۶ ماه بدون کار؛ Neuchâtel/Basel/HSLU</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>✅ حتی بدون کار</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>⚠️ فقط با کار</t>
+          <t>✅ با ۲۰ ساعت کار</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>❌</t>
+          <t>⚠️ فقط با بورس</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>❌</t>
+          <t>❌ شهریه به‌تنهایی</t>
         </is>
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>❌</t>
+          <t>❌ + ویزا</t>
         </is>
       </c>
     </row>
@@ -1774,17 +1775,17 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="64" customHeight="1">
+    <row r="38" ht="72" customHeight="1">
       <c r="A38" s="11" t="inlineStr">
         <is>
-          <t>حساسیت: (۱) همین وزن‌ها ولی «کار» سوئیس = ۴ (مثل نسخهٔ قبل): سوئیس ۶۴ › هلند ۶۲.۸ › آلمان ۶۰ › انگلستان ۵۹.۵ › سوئد ۵۷.۸ › دانمارک ۵۷. (۲) کار ۳۰ / حقوق ۳۰ / انگلیسی ۳۰ / هزینه ۱۰ (هزینه سبک‌تر چون بودجه بالا رفت): سوئیس ۶۸ › هلند ۶۵ › انگلستان ۵۹ › آلمان ۵۸ = دانمارک ۵۸ › سوئد ۵۷. (۳) وزن‌های نسخهٔ قبل (کار ۳۰ / حقوق ۲۵ / انگلیسی ۳۰ / هزینه ۱۵) با «کار» سوئیس = ۵: سوئیس ۶۵.۵ › هلند ۶۳.۵ › آلمان ۶۰ = انگلستان ۶۰. در همهٔ حالت‌ها سوئیس و هلند دو فینالیست‌اند و اختلافشان ۱ تا ۴ امتیاز است — این امتیازها قضاوت‌اند، نه اندازه‌گیری؛ تصمیم بین این دو با ریسک‌پذیری شما و پذیرش‌ها گرفته می‌شود، نه با اعشار.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="48" customHeight="1">
+          <t>حساسیت: (۱) همین وزن‌ها ولی «کار» سوئیس = ۴ (مثل نسخهٔ قبل): سوئیس ۶۴ › هلند ۶۲.۸ › آلمان ۶۰ › انگلستان ۵۹.۵ › سوئد ۵۷.۸ › دانمارک ۵۷. (۲) کار ۳۰ / حقوق ۳۰ / انگلیسی ۳۰ / هزینه ۱۰ (هزینه سبک‌تر چون بودجه بالا رفت): سوئیس ۶۸ › هلند ۶۵ › انگلستان ۵۹ › آلمان ۵۸ = دانمارک ۵۸ › سوئد ۵۷. (۳) وزن‌های نسخهٔ قبل (کار ۳۰ / حقوق ۲۵ / انگلیسی ۳۰ / هزینه ۱۵) با «کار» سوئیس = ۵: سوئیس ۶۵.۵ › هلند ۶۳.۵ › آلمان ۶۰ = انگلستان ۶۰. در همهٔ حالت‌ها سوئیس و هلند دو فینالیست‌اند و اختلافشان ۱ تا ۴ امتیاز است — این امتیازها قضاوت‌اند، نه اندازه‌گیری؛ تصمیم بین این دو با ریسک‌پذیری شما و پذیرش‌ها گرفته می‌شود، نه با اعشار. ⚠️ ولی با بودجهٔ شما (شهریه + زندگی تا کار) هلند عملاً بسته است (شهریهٔ دو سال $45–50k) — پس فینالیست‌های واقعی سوئیس و آلمان‌اند، با انگلستان به‌عنوان گزینهٔ ۱۰۰٪ انگلیسی.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="56" customHeight="1">
       <c r="A39" s="11" t="inlineStr">
         <is>
-          <t>سه فیلتری که امتیاز نمی‌بیند: (۱) پول — بودجه $40,000 برای کل دوره: هلند، سوئد و دانمارک بیرون؛ سوئیس فقط Joint MSc (Neuchâtel/Fribourg) و Basel با کار؛ آلمان راحت (Stuttgart با Werkstudent)؛ انگلستان فقط با ۲۰ ساعت کار. (۲) ویزا از تهران — سوئیس سفارت تهران باز، آلمان فقط اضطراری (برنامهٔ B از ترکیه/ارمنستان)، انگلستان VAC متغیر. (۳) پذیرش — سوئیس و Stuttgart/Darmstadt Target هستند؛ Saarland/Passau/Essex/Northumbria امن‌ترند.</t>
+          <t>سه فیلتری که امتیاز نمی‌بیند: (۱) پول با مدل شما ($40,000 = شهریه + زندگی تا کار): هلند و دانمارک بیرون؛ سوئد فقط با بورس؛ سوئیس فقط اگر ۶ ماه اول را بدون درآمد بگذرانید (Neuchâtel/Fribourg/Basel تقریباً بدون کار جا می‌شوند، HSLU از ماه ۷ ≈ $1,000/ماه می‌خواهد، USI ≈ $1,450)؛ آلمان بدون کار؛ انگلستان با ۲۰ ساعت کار. (۲) اثبات تمکن قبل از ویزا (از همان پول، ولی یک‌جا): آلمان $13,600 · سوئیس $25,400 (زوریخ فقط بانک سوئیسی به نام خودتان؛ انتقال پول از ایران به بانک سوئیسی سخت است — از International Office دانشگاه بپرسید) · انگلستان شهریه + $14,300 (حساب خانواده مجاز). (۳) پذیرش — سوئیس و Stuttgart/Darmstadt Target؛ Saarland/Passau/Essex/Northumbria امن‌تر.</t>
         </is>
       </c>
     </row>
@@ -1792,7 +1793,7 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>پ) برنامه‌هایی که در بودجهٔ $40,000 کل جا می‌شوند (یا با کار دانشجویی نزدیک‌اند) — با امتیاز وزنی شما؛ ۱ = بالاترین امتیاز</t>
+          <t>پ) برنامه‌هایی که با «$40,000 = شهریه + زندگی تا پیدا شدن کار دانشجویی» شدنی‌اند — با امتیاز وزنی شما؛ ۱ = بالاترین امتیاز (ستون «شدنی؟» را حتماً کنار امتیاز بخوانید)</t>
         </is>
       </c>
     </row>
@@ -1819,17 +1820,17 @@
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>★ کل تا مدرک</t>
+          <t>★ کل تا مدرک (بدون کار)</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>در $40,000 کل جا می‌شود؟</t>
+          <t>با $40,000 = شهریه + زندگی تا کار؟ (ماه‌های پوشش بعد از شهریه / درآمد لازم از کار)</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>زیرامتیازها: کار / حقوق / انگلیسی / هزینه → امتیاز</t>
+          <t>زیرامتیازها: کار / حقوق / انگلیسی / بودجه → امتیاز</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
@@ -1877,21 +1878,21 @@
           <t>$38–49k</t>
         </is>
       </c>
-      <c r="F43" s="13" t="inlineStr">
-        <is>
-          <t>⚠️ فقط با اتاق ارزان + کار ۱۵ ساعت بعد از ماه ۶؛ کانتون تمکن $29,000 می‌خواهد</t>
+      <c r="F43" s="12" t="inlineStr">
+        <is>
+          <t>✅ بعد از شهریه $36.9k = ۱۶–۱۷ ماه از ۱۸؛ کسری ≈ $3.4k → از ماه ۷ حدود $300/ماه (۱۵ ساعت ≈ $1,550–2,200)؛ اثبات $29,000</t>
         </is>
       </c>
       <c r="G43" s="6" t="inlineStr">
         <is>
-          <t>5 / 10 / 6 / 5 → 66.8</t>
-        </is>
-      </c>
-      <c r="H43" s="14">
+          <t>5 / 10 / 6 / 8 → 71.3</t>
+        </is>
+      </c>
+      <c r="H43" s="13">
         <f>ROUND(($B$28*L43+$B$29*M43+$B$30*N43+$B$31*O43)/SUM($B$28:$B$31)*10,1)</f>
         <v/>
       </c>
-      <c r="I43" s="15" t="inlineStr">
+      <c r="I43" s="14" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
@@ -1903,7 +1904,7 @@
       </c>
       <c r="K43" s="12" t="inlineStr">
         <is>
-          <t>Roche / Novartis / IT و ۱ ساعت تا زوریخ؛ آلمانی‌زبان؛ پذیرش سخت‌تر؛ ۶ ماه مجوز L</t>
+          <t>Roche / Novartis / IT و ۱ ساعت تا زوریخ؛ آلمانی‌زبان؛ پذیرش سخت‌تر؛ ۶ ماه مجوز L بعد از مدرک</t>
         </is>
       </c>
       <c r="L43" t="n">
@@ -1916,7 +1917,7 @@
         <v>6</v>
       </c>
       <c r="O43" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="44">
@@ -1925,64 +1926,64 @@
       </c>
       <c r="B44" s="12" t="inlineStr">
         <is>
-          <t>University of Neuchâtel – Neuchâtel</t>
+          <t>Hochschule Luzern (HSLU) – Lucerne / Luzern</t>
         </is>
       </c>
       <c r="C44" s="12" t="inlineStr">
         <is>
-          <t>Swiss Joint MSc Computer Science (ثبت‌نام در Neuchâtel)</t>
+          <t>MSc Applied Data Science and AI (نام جدید از اوت ۲۰۲۶؛ قبلاً Applied Information and Data Science)</t>
         </is>
       </c>
       <c r="D44" s="12" t="inlineStr">
         <is>
-          <t>۱.۵ سال</t>
+          <t>۲ سال</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>$32–41k</t>
-        </is>
-      </c>
-      <c r="F44" s="12" t="inlineStr">
-        <is>
-          <t>✅ مرزی — با زندگی صرفه‌جویانه (≈ $1,650/ماه) ≈ $33–35k؛ کار بعد از ماه ۶ حاشیه می‌سازد</t>
+          <t>$53–64k</t>
+        </is>
+      </c>
+      <c r="F44" s="15" t="inlineStr">
+        <is>
+          <t>⚠️ شدنی: بعد از شهریه $32.4k = ۱۵ ماه از ۲۴؛ کسری ≈ $18k → از ماه ۷ حدود $1,000/ماه خالص از ۱۵ ساعت کار — به شرط پیدا شدن کار تا ماه ۹؛ اثبات $25,400</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
-          <t>4 / 10 / 5 / 8 → 65.5</t>
-        </is>
-      </c>
-      <c r="H44" s="14">
+          <t>5 / 10 / 6 / 6 → 68.3</t>
+        </is>
+      </c>
+      <c r="H44" s="13">
         <f>ROUND(($B$28*L44+$B$29*M44+$B$30*N44+$B$31*O44)/SUM($B$28:$B$31)*10,1)</f>
         <v/>
       </c>
       <c r="I44" s="16" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Safe/Target</t>
         </is>
       </c>
       <c r="J44" s="12" t="inlineStr">
         <is>
-          <t>۳۱ مارس ۲۰۲۷</t>
+          <t>۱ آوریل ۲۰۲۷</t>
         </is>
       </c>
       <c r="K44" s="12" t="inlineStr">
         <is>
-          <t>ارزان‌ترین سوئیس؛ بدون مدرک زبان؛ فرانسه‌زبان در زندگی روزمره؛ بازار کار ملی ولی رقابت با ETH/EPFL؛ ۶ ماه مجوز L</t>
+          <t>۴۵ دقیقه تا زوریخ/زوگ؛ هر کارشناسی را می‌پذیرد (Safe/Target)؛ کار دانشجویی IT به انگلیسی هست ولی کمتر از زوریخ؛ ۶ ماه مجوز L</t>
         </is>
       </c>
       <c r="L44" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M44" t="n">
         <v>10</v>
       </c>
       <c r="N44" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O44" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="45">
@@ -1991,12 +1992,12 @@
       </c>
       <c r="B45" s="12" t="inlineStr">
         <is>
-          <t>University of Fribourg – Fribourg</t>
+          <t>University of Neuchâtel – Neuchâtel</t>
         </is>
       </c>
       <c r="C45" s="12" t="inlineStr">
         <is>
-          <t>Swiss Joint MSc Computer Science (ثبت‌نام در Fribourg)</t>
+          <t>Swiss Joint MSc Computer Science (ثبت‌نام در Neuchâtel)</t>
         </is>
       </c>
       <c r="D45" s="12" t="inlineStr">
@@ -2006,36 +2007,36 @@
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>$35–43k</t>
-        </is>
-      </c>
-      <c r="F45" s="13" t="inlineStr">
-        <is>
-          <t>⚠️ مرزی — با کار بعد از ماه ۶</t>
+          <t>$32–41k</t>
+        </is>
+      </c>
+      <c r="F45" s="12" t="inlineStr">
+        <is>
+          <t>✅ بعد از شهریه $37.1k = تمام ۱۸ ماه (+ ≈ $3k)؛ کار فقط حاشیهٔ امن</t>
         </is>
       </c>
       <c r="G45" s="6" t="inlineStr">
         <is>
-          <t>4 / 10 / 5 / 7 → 64.0</t>
-        </is>
-      </c>
-      <c r="H45" s="14">
+          <t>4 / 10 / 5 / 9 → 67.0</t>
+        </is>
+      </c>
+      <c r="H45" s="13">
         <f>ROUND(($B$28*L45+$B$29*M45+$B$30*N45+$B$31*O45)/SUM($B$28:$B$31)*10,1)</f>
         <v/>
       </c>
-      <c r="I45" s="16" t="inlineStr">
+      <c r="I45" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
       <c r="J45" s="12" t="inlineStr">
         <is>
-          <t>۲۸ فوریه ۲۰۲۷ (ویزایی‌ها)</t>
+          <t>۳۱ مارس ۲۰۲۷</t>
         </is>
       </c>
       <c r="K45" s="12" t="inlineStr">
         <is>
-          <t>همان مدرک مشترک؛ شهر دوزبانه (فرانسه/آلمانی)؛ ۲۰ دقیقه تا برن</t>
+          <t>ارزان‌ترین سوئیس؛ بدون مدرک زبان؛ فرانسه‌زبان در زندگی روزمره؛ بازار ملی ولی رقابت با ETH/EPFL؛ ۶ ماه مجوز L</t>
         </is>
       </c>
       <c r="L45" t="n">
@@ -2048,7 +2049,7 @@
         <v>5</v>
       </c>
       <c r="O45" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="46">
@@ -2057,64 +2058,64 @@
       </c>
       <c r="B46" s="12" t="inlineStr">
         <is>
-          <t>Universität Stuttgart – Stuttgart</t>
+          <t>University of Fribourg – Fribourg</t>
         </is>
       </c>
       <c r="C46" s="12" t="inlineStr">
         <is>
-          <t>M.Sc. Computer Science (انگلیسی، بدون NC)</t>
+          <t>Swiss Joint MSc Computer Science (ثبت‌نام در Fribourg)</t>
         </is>
       </c>
       <c r="D46" s="12" t="inlineStr">
         <is>
-          <t>۲ سال</t>
+          <t>۱.۵ سال</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>$38–45k</t>
-        </is>
-      </c>
-      <c r="F46" s="13" t="inlineStr">
-        <is>
-          <t>⚠️ مرزی — با Werkstudent از ترم اول جا می‌شود</t>
+          <t>$35–43k</t>
+        </is>
+      </c>
+      <c r="F46" s="12" t="inlineStr">
+        <is>
+          <t>✅ بعد از شهریه $36.4k = تمام ۱۸ ماه (مرزی)</t>
         </is>
       </c>
       <c r="G46" s="6" t="inlineStr">
         <is>
-          <t>7 / 7 / 4 / 6 → 59.5</t>
-        </is>
-      </c>
-      <c r="H46" s="14">
+          <t>4 / 10 / 5 / 8 → 65.5</t>
+        </is>
+      </c>
+      <c r="H46" s="13">
         <f>ROUND(($B$28*L46+$B$29*M46+$B$30*N46+$B$31*O46)/SUM($B$28:$B$31)*10,1)</f>
         <v/>
       </c>
-      <c r="I46" s="16" t="inlineStr">
+      <c r="I46" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
       <c r="J46" s="12" t="inlineStr">
         <is>
-          <t>۱۵ ژانویه ۲۰۲۷</t>
+          <t>۲۸ فوریه ۲۰۲۷ (ویزایی‌ها)</t>
         </is>
       </c>
       <c r="K46" s="12" t="inlineStr">
         <is>
-          <t>بزرگ‌ترین بازار مهندسی/IT (Bosch، Mercedes، Porsche)؛ حقوق BW بالاتر؛ ۱۸ ماه؛ IELTS 7؛ آلمانی برای نیمی از بازار؛ صف خوابگاه ۶–۸ ماه</t>
+          <t>همان مدرک مشترک؛ شهر دوزبانه (فرانسه/آلمانی)؛ ۲۰ دقیقه تا برن</t>
         </is>
       </c>
       <c r="L46" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M46" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="N46" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O46" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="47">
@@ -2123,12 +2124,12 @@
       </c>
       <c r="B47" s="12" t="inlineStr">
         <is>
-          <t>TU Darmstadt – Darmstadt</t>
+          <t>Universität Stuttgart – Stuttgart</t>
         </is>
       </c>
       <c r="C47" s="12" t="inlineStr">
         <is>
-          <t>M.Sc. Distributed Software Systems (انگلیسی)</t>
+          <t>M.Sc. Computer Science (انگلیسی، بدون NC)</t>
         </is>
       </c>
       <c r="D47" s="12" t="inlineStr">
@@ -2138,43 +2139,43 @@
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>$30–37k</t>
+          <t>$38–45k</t>
         </is>
       </c>
       <c r="F47" s="12" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>✅ بعد از شهریه $32.3k = ۲۳ ماه از ۲۴؛ کسری ≈ $1.4k → Werkstudent ۲۰ ساعت ($1,140–1,710) از روز اول مجاز؛ اثبات $13,600</t>
         </is>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
-          <t>6 / 6 / 4 / 9 → 58.5</t>
-        </is>
-      </c>
-      <c r="H47" s="14">
+          <t>7 / 7 / 4 / 9 → 64.0</t>
+        </is>
+      </c>
+      <c r="H47" s="13">
         <f>ROUND(($B$28*L47+$B$29*M47+$B$30*N47+$B$31*O47)/SUM($B$28:$B$31)*10,1)</f>
         <v/>
       </c>
-      <c r="I47" s="15" t="inlineStr">
-        <is>
-          <t>Target/Reach</t>
+      <c r="I47" s="17" t="inlineStr">
+        <is>
+          <t>Target</t>
         </is>
       </c>
       <c r="J47" s="12" t="inlineStr">
         <is>
-          <t>≈ ۱۵ می – ۱۵ ژوئیه ۲۰۲۷ (چک شود)</t>
+          <t>۱۵ ژانویه ۲۰۲۷</t>
         </is>
       </c>
       <c r="K47" s="12" t="inlineStr">
         <is>
-          <t>۲۵ دقیقه تا فرانکفورت (شرکت‌های بین‌المللی انگلیسی‌زبان)؛ تقریباً رایگان؛ لیست انتظار خوابگاه</t>
+          <t>بزرگ‌ترین بازار مهندسی/IT (Bosch، Mercedes، Porsche)؛ حقوق BW بالاتر؛ ۱۸ ماه؛ IELTS 7؛ آلمانی برای نیمی از بازار؛ صف خوابگاه ۶–۸ ماه</t>
         </is>
       </c>
       <c r="L47" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M47" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N47" t="n">
         <v>4</v>
@@ -2189,64 +2190,64 @@
       </c>
       <c r="B48" s="12" t="inlineStr">
         <is>
-          <t>Saarland University (UdS) – Saarbrücken</t>
+          <t>Manchester Metropolitan University (MMU) – Manchester</t>
         </is>
       </c>
       <c r="C48" s="12" t="inlineStr">
         <is>
-          <t>M.Sc. Data Science and Artificial Intelligence</t>
+          <t>MSc Cyber Security</t>
         </is>
       </c>
       <c r="D48" s="12" t="inlineStr">
         <is>
-          <t>۲ سال</t>
+          <t>۱ سال</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>$26–32k</t>
+          <t>$45–49k</t>
         </is>
       </c>
       <c r="F48" s="12" t="inlineStr">
         <is>
-          <t>✅ راحت</t>
+          <t>✅ بعد از شهریه $12.2k = ۸ ماه؛ کسری ≈ $6.8k → ≈ $570/ماه؛ اثبات ≈ $42k</t>
         </is>
       </c>
       <c r="G48" s="6" t="inlineStr">
         <is>
-          <t>5 / 6 / 4 / 10 → 57.2</t>
-        </is>
-      </c>
-      <c r="H48" s="14">
+          <t>5 / 3 / 10 / 8 → 64.0</t>
+        </is>
+      </c>
+      <c r="H48" s="13">
         <f>ROUND(($B$28*L48+$B$29*M48+$B$30*N48+$B$31*O48)/SUM($B$28:$B$31)*10,1)</f>
         <v/>
       </c>
-      <c r="I48" s="16" t="inlineStr">
-        <is>
-          <t>Target</t>
+      <c r="I48" s="18" t="inlineStr">
+        <is>
+          <t>Safe</t>
         </is>
       </c>
       <c r="J48" s="12" t="inlineStr">
         <is>
-          <t>≈ ۱۵ می – ۱۵ ژوئیه ۲۰۲۷ (چک شود)</t>
+          <t>rolling — تا ژوئن ۲۰۲۷</t>
         </is>
       </c>
       <c r="K48" s="12" t="inlineStr">
         <is>
-          <t>AI کنار CISPA/DFKI؛ ارزان‌ترین زندگی؛ شهر کوچک (لوکزامبورگ ۱ ساعت)</t>
+          <t>منچستر = دومین قطب فناوری انگلستان (کار دانشجویی و جونیور بیشتر)؛ فقط Cyber Security در فهرست؛ Safe</t>
         </is>
       </c>
       <c r="L48" t="n">
         <v>5</v>
       </c>
       <c r="M48" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="N48" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="O48" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="49">
@@ -2275,19 +2276,19 @@
       </c>
       <c r="F49" s="12" t="inlineStr">
         <is>
-          <t>✅ مرزی</t>
+          <t>✅ بعد از شهریه $17.5k = تمام ۱۲ ماه بدون کار؛ اثبات تمکن ≈ $36.8k ✓</t>
         </is>
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
-          <t>3 / 3 / 10 / 7 → 57.0</t>
-        </is>
-      </c>
-      <c r="H49" s="14">
+          <t>3 / 3 / 10 / 10 → 61.5</t>
+        </is>
+      </c>
+      <c r="H49" s="13">
         <f>ROUND(($B$28*L49+$B$29*M49+$B$30*N49+$B$31*O49)/SUM($B$28:$B$31)*10,1)</f>
         <v/>
       </c>
-      <c r="I49" s="17" t="inlineStr">
+      <c r="I49" s="18" t="inlineStr">
         <is>
           <t>Safe</t>
         </is>
@@ -2312,7 +2313,7 @@
         <v>10</v>
       </c>
       <c r="O49" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="50">
@@ -2339,21 +2340,21 @@
           <t>$44–48k</t>
         </is>
       </c>
-      <c r="F50" s="13" t="inlineStr">
-        <is>
-          <t>⚠️ کسری $4–8k → فقط با ۲۰ ساعت کار ($8–12k در سال)</t>
+      <c r="F50" s="12" t="inlineStr">
+        <is>
+          <t>✅ بعد از شهریه $11.5k = ۸ ماه از ۱۲؛ کسری ≈ $5.8k → ≈ $500/ماه از ۲۰ ساعت کار ($16.8/ساعت ≈ $1,450/ماه)؛ اثبات ≈ $42.8k (≈ $3k موقتاً از خانواده)</t>
         </is>
       </c>
       <c r="G50" s="6" t="inlineStr">
         <is>
-          <t>4 / 3 / 10 / 4 → 55.2</t>
-        </is>
-      </c>
-      <c r="H50" s="14">
+          <t>4 / 3 / 10 / 8 → 61.3</t>
+        </is>
+      </c>
+      <c r="H50" s="13">
         <f>ROUND(($B$28*L50+$B$29*M50+$B$30*N50+$B$31*O50)/SUM($B$28:$B$31)*10,1)</f>
         <v/>
       </c>
-      <c r="I50" s="17" t="inlineStr">
+      <c r="I50" s="18" t="inlineStr">
         <is>
           <t>Safe</t>
         </is>
@@ -2378,7 +2379,7 @@
         <v>10</v>
       </c>
       <c r="O50" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="51">
@@ -2405,21 +2406,21 @@
           <t>$49–54k</t>
         </is>
       </c>
-      <c r="F51" s="13" t="inlineStr">
-        <is>
-          <t>⚠️ بعد از بورس $5,960 کسری $3–8k → فقط با ۲۰ ساعت کار</t>
+      <c r="F51" s="12" t="inlineStr">
+        <is>
+          <t>✅ بعد از شهریه و بورس $5,960: $13.3k = ۸–۹ ماه؛ کسری ≈ $5.5k → ≈ $460/ماه؛ اثبات ≈ $41k</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
-          <t>4 / 3 / 10 / 4 → 55.2</t>
-        </is>
-      </c>
-      <c r="H51" s="14">
+          <t>4 / 3 / 10 / 8 → 61.3</t>
+        </is>
+      </c>
+      <c r="H51" s="13">
         <f>ROUND(($B$28*L51+$B$29*M51+$B$30*N51+$B$31*O51)/SUM($B$28:$B$31)*10,1)</f>
         <v/>
       </c>
-      <c r="I51" s="18" t="inlineStr">
+      <c r="I51" s="16" t="inlineStr">
         <is>
           <t>Safe/Target</t>
         </is>
@@ -2444,7 +2445,7 @@
         <v>10</v>
       </c>
       <c r="O51" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="52">
@@ -2453,12 +2454,12 @@
       </c>
       <c r="B52" s="12" t="inlineStr">
         <is>
-          <t>Universität Passau – Passau</t>
+          <t>USI – Università della Svizzera italiana – Lugano</t>
         </is>
       </c>
       <c r="C52" s="12" t="inlineStr">
         <is>
-          <t>M.Sc. Artificial Intelligence Engineering</t>
+          <t>MSc Artificial Intelligence (با IDSIA)</t>
         </is>
       </c>
       <c r="D52" s="12" t="inlineStr">
@@ -2468,410 +2469,512 @@
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>$25–31k</t>
-        </is>
-      </c>
-      <c r="F52" s="12" t="inlineStr">
-        <is>
-          <t>✅ راحت</t>
+          <t>$60–72k</t>
+        </is>
+      </c>
+      <c r="F52" s="15" t="inlineStr">
+        <is>
+          <t>⚠️ پرریسک: بعد از شهریه $20.6k = ۱۰–۱۱ ماه از ۲۴؛ کسری ≈ $26k → از ماه ۷ حدود $1,450/ماه خالص از ۱۵ ساعت کار در لوگانو (ایتالیایی‌زبان)</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>4 / 6 / 3 / 10 → 51.5</t>
-        </is>
-      </c>
-      <c r="H52" s="14">
+          <t>4 / 10 / 5 / 5 → 61.0</t>
+        </is>
+      </c>
+      <c r="H52" s="13">
         <f>ROUND(($B$28*L52+$B$29*M52+$B$30*N52+$B$31*O52)/SUM($B$28:$B$31)*10,1)</f>
         <v/>
       </c>
       <c r="I52" s="17" t="inlineStr">
         <is>
-          <t>Safe</t>
+          <t>Target</t>
         </is>
       </c>
       <c r="J52" s="12" t="inlineStr">
         <is>
-          <t>۳۱ می ۲۰۲۷</t>
+          <t>۳۰ آوریل ۲۰۲۷</t>
         </is>
       </c>
       <c r="K52" s="12" t="inlineStr">
         <is>
-          <t>Safe آلمان (معدل ۲.۳ ≤ ۲.۷ ✓)؛ شهر کوچک؛ آلمانی A1 اجباری در سال اول؛ مونیخ ۲ ساعت</t>
+          <t>AI با IDSIA؛ ورود با B2؛ بورس $4,840 مرزی؛ همان ریسک ۶ ماه</t>
         </is>
       </c>
       <c r="L52" t="n">
         <v>4</v>
       </c>
       <c r="M52" t="n">
+        <v>10</v>
+      </c>
+      <c r="N52" t="n">
+        <v>5</v>
+      </c>
+      <c r="O52" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>TU Darmstadt – Darmstadt</t>
+        </is>
+      </c>
+      <c r="C53" s="12" t="inlineStr">
+        <is>
+          <t>M.Sc. Distributed Software Systems (انگلیسی)</t>
+        </is>
+      </c>
+      <c r="D53" s="12" t="inlineStr">
+        <is>
+          <t>۲ سال</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>$30–37k</t>
+        </is>
+      </c>
+      <c r="F53" s="12" t="inlineStr">
+        <is>
+          <t>✅ بعد از شهریه $38.6k = تمام ۲۴ ماه + ≈ $6k؛ کار = اضافه</t>
+        </is>
+      </c>
+      <c r="G53" s="6" t="inlineStr">
+        <is>
+          <t>6 / 6 / 4 / 10 → 60.0</t>
+        </is>
+      </c>
+      <c r="H53" s="13">
+        <f>ROUND(($B$28*L53+$B$29*M53+$B$30*N53+$B$31*O53)/SUM($B$28:$B$31)*10,1)</f>
+        <v/>
+      </c>
+      <c r="I53" s="14" t="inlineStr">
+        <is>
+          <t>Target/Reach</t>
+        </is>
+      </c>
+      <c r="J53" s="12" t="inlineStr">
+        <is>
+          <t>≈ ۱۵ می – ۱۵ ژوئیه ۲۰۲۷ (چک شود)</t>
+        </is>
+      </c>
+      <c r="K53" s="12" t="inlineStr">
+        <is>
+          <t>۲۵ دقیقه تا فرانکفورت (شرکت‌های بین‌المللی انگلیسی‌زبان)؛ تقریباً رایگان؛ لیست انتظار خوابگاه</t>
+        </is>
+      </c>
+      <c r="L53" t="n">
         <v>6</v>
       </c>
-      <c r="N52" t="n">
+      <c r="M53" t="n">
+        <v>6</v>
+      </c>
+      <c r="N53" t="n">
+        <v>4</v>
+      </c>
+      <c r="O53" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B54" s="12" t="inlineStr">
+        <is>
+          <t>University of Leicester – Leicester</t>
+        </is>
+      </c>
+      <c r="C54" s="12" t="inlineStr">
+        <is>
+          <t>MSc Advanced Computer Science</t>
+        </is>
+      </c>
+      <c r="D54" s="12" t="inlineStr">
+        <is>
+          <t>۱ سال</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>$48–53k</t>
+        </is>
+      </c>
+      <c r="F54" s="15" t="inlineStr">
+        <is>
+          <t>⚠️ بعد از شهریه $7.9k = ۵ ماه؛ کسری ≈ $10.4k → ≈ $870/ماه از ماه ۲؛ اثبات ≈ $46k</t>
+        </is>
+      </c>
+      <c r="G54" s="6" t="inlineStr">
+        <is>
+          <t>4 / 3 / 10 / 7 → 59.8</t>
+        </is>
+      </c>
+      <c r="H54" s="13">
+        <f>ROUND(($B$28*L54+$B$29*M54+$B$30*N54+$B$31*O54)/SUM($B$28:$B$31)*10,1)</f>
+        <v/>
+      </c>
+      <c r="I54" s="17" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="J54" s="12" t="inlineStr">
+        <is>
+          <t>rolling — تا ژوئن ۲۰۲۷</t>
+        </is>
+      </c>
+      <c r="K54" s="12" t="inlineStr">
+        <is>
+          <t>رتبهٔ بهتر از Teesside/Northumbria؛ ولی وابسته به پیدا کردن سریع کار</t>
+        </is>
+      </c>
+      <c r="L54" t="n">
+        <v>4</v>
+      </c>
+      <c r="M54" t="n">
         <v>3</v>
       </c>
-      <c r="O52" t="n">
+      <c r="N54" t="n">
         <v>10</v>
       </c>
-    </row>
-    <row r="53" ht="52" customHeight="1">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>زیرامتیازها (از ۱۰) برای همان برنامه/شهر: «کار» = بازار جونیورِ فقط‌انگلیسی همان شهر + مدت اقامت کاریابی + کار دانشجویی به‌عنوان راه استخدام؛ «حقوق» = حقوق شروع همان کشور/منطقه؛ «انگلیسی» = تحصیل + زندگی روزمره همان شهر؛ «هزینه» = فاصله تا سقف $40,000 کل (۱۰ = زیر $32k راحت … ۴ = فقط با کار). ستون «امتیاز (فرمول)» از وزن‌های سبز بخش ب می‌خواند؛ عدد داخل ستون کناری همان امتیاز با وزن‌های پیش‌فرض است. ستون «کل تا مدرک» = شهریه × طول دوره + زندگی همان شهر × ماه‌ها، بدون بورس/بلیت/ویزا/ودیعه.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54"/>
+      <c r="O54" t="n">
+        <v>7</v>
+      </c>
+    </row>
     <row r="55">
-      <c r="A55" s="3" t="inlineStr">
-        <is>
-          <t>پ-۲) برای مقایسه: برنامه‌های خوب که با $40,000 کل جور درنمی‌آیند (فقط با بورس Reach یا کار پرریسک)</t>
-        </is>
+      <c r="A55" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>Saarland University (UdS) – Saarbrücken</t>
+        </is>
+      </c>
+      <c r="C55" s="12" t="inlineStr">
+        <is>
+          <t>M.Sc. Data Science and Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="D55" s="12" t="inlineStr">
+        <is>
+          <t>۲ سال</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>$26–32k</t>
+        </is>
+      </c>
+      <c r="F55" s="12" t="inlineStr">
+        <is>
+          <t>✅ بعد از شهریه $38.2k = تمام ۲۴ ماه + ≈ $11k</t>
+        </is>
+      </c>
+      <c r="G55" s="6" t="inlineStr">
+        <is>
+          <t>5 / 6 / 4 / 10 → 57.3</t>
+        </is>
+      </c>
+      <c r="H55" s="13">
+        <f>ROUND(($B$28*L55+$B$29*M55+$B$30*N55+$B$31*O55)/SUM($B$28:$B$31)*10,1)</f>
+        <v/>
+      </c>
+      <c r="I55" s="17" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="J55" s="12" t="inlineStr">
+        <is>
+          <t>≈ ۱۵ می – ۱۵ ژوئیه ۲۰۲۷ (چک شود)</t>
+        </is>
+      </c>
+      <c r="K55" s="12" t="inlineStr">
+        <is>
+          <t>AI کنار CISPA/DFKI؛ ارزان‌ترین زندگی؛ شهر کوچک (لوکزامبورگ ۱ ساعت)</t>
+        </is>
+      </c>
+      <c r="L55" t="n">
+        <v>5</v>
+      </c>
+      <c r="M55" t="n">
+        <v>6</v>
+      </c>
+      <c r="N55" t="n">
+        <v>4</v>
+      </c>
+      <c r="O55" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="4" t="inlineStr">
+      <c r="A56" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B56" s="12" t="inlineStr">
+        <is>
+          <t>Blekinge Institute of Technology (BTH) – Karlskrona</t>
+        </is>
+      </c>
+      <c r="C56" s="12" t="inlineStr">
+        <is>
+          <t>MSc Software Engineering (120 cr)</t>
+        </is>
+      </c>
+      <c r="D56" s="12" t="inlineStr">
+        <is>
+          <t>۲ سال</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>$51–56k</t>
+        </is>
+      </c>
+      <c r="F56" s="15" t="inlineStr">
+        <is>
+          <t>⚠️ بعد از شهریه $11.7k = ۱۱ ماه از ۲۴؛ کسری ≈ $14k → ≈ $630/ماه — بدون سوئدی سخت ($350–900)؛ اثبات $10,800 سال اول</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>3 / 5 / 8 / 6 → 55.0</t>
+        </is>
+      </c>
+      <c r="H56" s="13">
+        <f>ROUND(($B$28*L56+$B$29*M56+$B$30*N56+$B$31*O56)/SUM($B$28:$B$31)*10,1)</f>
+        <v/>
+      </c>
+      <c r="I56" s="16" t="inlineStr">
+        <is>
+          <t>Safe/Target</t>
+        </is>
+      </c>
+      <c r="J56" s="12" t="inlineStr">
+        <is>
+          <t>۱۵ ژانویه ۲۰۲۷</t>
+        </is>
+      </c>
+      <c r="K56" s="12" t="inlineStr">
+        <is>
+          <t>پشتوانهٔ ارزانِ ۱۰۰٪ انگلیسی؛ Ericsson در شهر؛ ولی بازار سوئد ضعیف</t>
+        </is>
+      </c>
+      <c r="L56" t="n">
+        <v>3</v>
+      </c>
+      <c r="M56" t="n">
+        <v>5</v>
+      </c>
+      <c r="N56" t="n">
+        <v>8</v>
+      </c>
+      <c r="O56" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B57" s="12" t="inlineStr">
+        <is>
+          <t>Mälardalen University (MDU) – Västerås</t>
+        </is>
+      </c>
+      <c r="C57" s="12" t="inlineStr">
+        <is>
+          <t>MSc Software Engineering</t>
+        </is>
+      </c>
+      <c r="D57" s="12" t="inlineStr">
+        <is>
+          <t>۲ سال</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>$52–56k</t>
+        </is>
+      </c>
+      <c r="F57" s="15" t="inlineStr">
+        <is>
+          <t>⚠️ بعد از شهریه $12.7k = ۱۱–۱۲ ماه؛ ≈ $640/ماه از کار — با بورس MDU (تا ۱۰۰٪) ✅</t>
+        </is>
+      </c>
+      <c r="G57" s="6" t="inlineStr">
+        <is>
+          <t>3 / 5 / 8 / 6 → 55.0</t>
+        </is>
+      </c>
+      <c r="H57" s="13">
+        <f>ROUND(($B$28*L57+$B$29*M57+$B$30*N57+$B$31*O57)/SUM($B$28:$B$31)*10,1)</f>
+        <v/>
+      </c>
+      <c r="I57" s="18" t="inlineStr">
+        <is>
+          <t>Safe</t>
+        </is>
+      </c>
+      <c r="J57" s="12" t="inlineStr">
+        <is>
+          <t>۱۵ ژانویه ۲۰۲۷</t>
+        </is>
+      </c>
+      <c r="K57" s="12" t="inlineStr">
+        <is>
+          <t>Västerås (ABB)؛ خوابگاه تضمینی؛ بورس سخاوتمند ولی رقابتی</t>
+        </is>
+      </c>
+      <c r="L57" t="n">
+        <v>3</v>
+      </c>
+      <c r="M57" t="n">
+        <v>5</v>
+      </c>
+      <c r="N57" t="n">
+        <v>8</v>
+      </c>
+      <c r="O57" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="B58" s="12" t="inlineStr">
+        <is>
+          <t>Universität Passau – Passau</t>
+        </is>
+      </c>
+      <c r="C58" s="12" t="inlineStr">
+        <is>
+          <t>M.Sc. Artificial Intelligence Engineering</t>
+        </is>
+      </c>
+      <c r="D58" s="12" t="inlineStr">
+        <is>
+          <t>۲ سال</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>$25–31k</t>
+        </is>
+      </c>
+      <c r="F58" s="12" t="inlineStr">
+        <is>
+          <t>✅ بعد از شهریه $39.3k = تمام ۲۴ ماه + ≈ $12k</t>
+        </is>
+      </c>
+      <c r="G58" s="6" t="inlineStr">
+        <is>
+          <t>4 / 6 / 3 / 10 → 51.5</t>
+        </is>
+      </c>
+      <c r="H58" s="13">
+        <f>ROUND(($B$28*L58+$B$29*M58+$B$30*N58+$B$31*O58)/SUM($B$28:$B$31)*10,1)</f>
+        <v/>
+      </c>
+      <c r="I58" s="18" t="inlineStr">
+        <is>
+          <t>Safe</t>
+        </is>
+      </c>
+      <c r="J58" s="12" t="inlineStr">
+        <is>
+          <t>۳۱ می ۲۰۲۷</t>
+        </is>
+      </c>
+      <c r="K58" s="12" t="inlineStr">
+        <is>
+          <t>Safe آلمان (معدل ۲.۳ ≤ ۲.۷ ✓)؛ شهر کوچک؛ آلمانی A1 اجباری در سال اول؛ مونیخ ۲ ساعت</t>
+        </is>
+      </c>
+      <c r="L58" t="n">
+        <v>4</v>
+      </c>
+      <c r="M58" t="n">
+        <v>6</v>
+      </c>
+      <c r="N58" t="n">
+        <v>3</v>
+      </c>
+      <c r="O58" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="59" ht="64" customHeight="1">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>محاسبهٔ ستون «شدنی؟»: (۴۰,۰۰۰ − شهریهٔ کل دوره) ÷ میانهٔ زندگی ماهانهٔ همان شهر = ماه‌های پوشش‌داده‌شده؛ بقیهٔ ماه‌ها باید از کار دانشجویی دربیاید (سقف قانونی: آلمان و انگلستان ۲۰ ساعت از روز اول؛ سوئیس صفر تا ماه ۶، بعد ۱۵ ساعت؛ سوئد بدون سقف ولی بدون سوئدی کم). زیرامتیازها (از ۱۰) برای همان برنامه/شهر: «کار» = بازار جونیورِ فقط‌انگلیسی + اقامت کاریابی + کار دانشجویی به‌عنوان راه استخدام؛ «حقوق» = حقوق شروع همان کشور/منطقه؛ «انگلیسی» = تحصیل + زندگی روزمرهٔ همان شهر؛ «بودجه» = ۱۰ بدون نیاز به کار با اضافه … ۸ کمتر از $500/ماه از کار … ۶ حدود $1,000/ماه … ۵ بیش از $1,400/ماه. ستون «امتیاز (فرمول)» از وزن‌های سبز بخش ب می‌خواند؛ عدد داخل ستون کناری همان امتیاز با وزن‌های پیش‌فرض است. «کل تا مدرک» = شهریه × طول دوره + زندگی همان شهر × ماه‌ها، بدون بورس/بلیت/ویزا/ودیعه.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60"/>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>پ-۲) برای مقایسه: برنامه‌هایی که با این مدل هم جور درنمی‌آیند (شهریه به‌تنهایی › $40k یا ماه‌های پوشش خیلی کم)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="B56" s="4" t="inlineStr">
+      <c r="B62" s="4" t="inlineStr">
         <is>
           <t>دانشگاه – شهر</t>
         </is>
       </c>
-      <c r="C56" s="4" t="inlineStr">
+      <c r="C62" s="4" t="inlineStr">
         <is>
           <t>برنامه</t>
         </is>
       </c>
-      <c r="D56" s="4" t="inlineStr">
+      <c r="D62" s="4" t="inlineStr">
         <is>
           <t>طول</t>
         </is>
       </c>
-      <c r="E56" s="4" t="inlineStr">
+      <c r="E62" s="4" t="inlineStr">
         <is>
           <t>★ کل تا مدرک</t>
         </is>
       </c>
-      <c r="F56" s="4" t="inlineStr">
-        <is>
-          <t>فاصله تا $40,000</t>
-        </is>
-      </c>
-      <c r="G56" s="4" t="inlineStr">
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>چرا جور درنمی‌آید</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="inlineStr">
         <is>
           <t>چه چیزی می‌توانست ببندد؟</t>
         </is>
       </c>
-      <c r="H56" s="4" t="inlineStr"/>
-      <c r="I56" s="4" t="inlineStr">
+      <c r="H62" s="4" t="inlineStr"/>
+      <c r="I62" s="4" t="inlineStr">
         <is>
           <t>شانس</t>
         </is>
       </c>
-      <c r="J56" s="4" t="inlineStr">
+      <c r="J62" s="4" t="inlineStr">
         <is>
           <t>مهلت</t>
         </is>
       </c>
-      <c r="K56" s="4" t="inlineStr">
+      <c r="K62" s="4" t="inlineStr">
         <is>
           <t>چرا جذاب بود</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B57" s="20" t="inlineStr">
-        <is>
-          <t>University of Twente (UT) – Enschede</t>
-        </is>
-      </c>
-      <c r="C57" s="20" t="inlineStr">
-        <is>
-          <t>MSc Computer Science (گرایش‌ها: Cyber Security، Data Science، Software Tech، ...)</t>
-        </is>
-      </c>
-      <c r="D57" s="20" t="inlineStr">
-        <is>
-          <t>۲ سال</t>
-        </is>
-      </c>
-      <c r="E57" s="20" t="inlineStr">
-        <is>
-          <t>$77–85k</t>
-        </is>
-      </c>
-      <c r="F57" s="21" t="inlineStr">
-        <is>
-          <t>❌ کسری $37–45k</t>
-        </is>
-      </c>
-      <c r="G57" s="20" t="inlineStr">
-        <is>
-          <t>فقط بورس UTS (تا ≈ $25k/سال؛ Reach)؛ NL Scholarship $5,700 کافی نیست</t>
-        </is>
-      </c>
-      <c r="H57" s="20" t="inlineStr"/>
-      <c r="I57" s="19" t="inlineStr">
-        <is>
-          <t>Target</t>
-        </is>
-      </c>
-      <c r="J57" s="20" t="inlineStr"/>
-      <c r="K57" s="20" t="inlineStr">
-        <is>
-          <t>انگلیسی‌دوست‌ترین بازار کار؛ ۱۲ ماه zoekjaar</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B58" s="20" t="inlineStr">
-        <is>
-          <t>Radboud University – Nijmegen</t>
-        </is>
-      </c>
-      <c r="C58" s="20" t="inlineStr">
-        <is>
-          <t>MSc Computing Science (گرایش‌ها: Cyber Security، Data Science، Software Science)</t>
-        </is>
-      </c>
-      <c r="D58" s="20" t="inlineStr">
-        <is>
-          <t>۲ سال</t>
-        </is>
-      </c>
-      <c r="E58" s="20" t="inlineStr">
-        <is>
-          <t>$74–82k</t>
-        </is>
-      </c>
-      <c r="F58" s="21" t="inlineStr">
-        <is>
-          <t>❌ کسری $34–42k</t>
-        </is>
-      </c>
-      <c r="G58" s="20" t="inlineStr">
-        <is>
-          <t>فقط Radboud Scholarship (Reach)</t>
-        </is>
-      </c>
-      <c r="H58" s="20" t="inlineStr"/>
-      <c r="I58" s="19" t="inlineStr">
-        <is>
-          <t>Target</t>
-        </is>
-      </c>
-      <c r="J58" s="20" t="inlineStr"/>
-      <c r="K58" s="20" t="inlineStr">
-        <is>
-          <t>ارزان‌ترِ هلند</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B59" s="20" t="inlineStr">
-        <is>
-          <t>University of Amsterdam (UvA) – Amsterdam</t>
-        </is>
-      </c>
-      <c r="C59" s="20" t="inlineStr">
-        <is>
-          <t>MSc Software Engineering (۱ ساله!)</t>
-        </is>
-      </c>
-      <c r="D59" s="20" t="inlineStr">
-        <is>
-          <t>۱ سال</t>
-        </is>
-      </c>
-      <c r="E59" s="20" t="inlineStr">
-        <is>
-          <t>$57–62k</t>
-        </is>
-      </c>
-      <c r="F59" s="21" t="inlineStr">
-        <is>
-          <t>❌ کسری $17–22k</t>
-        </is>
-      </c>
-      <c r="G59" s="20" t="inlineStr">
-        <is>
-          <t>بورس قابل اتکایی ندارد</t>
-        </is>
-      </c>
-      <c r="H59" s="20" t="inlineStr"/>
-      <c r="I59" s="19" t="inlineStr">
-        <is>
-          <t>Target/Reach</t>
-        </is>
-      </c>
-      <c r="J59" s="20" t="inlineStr"/>
-      <c r="K59" s="20" t="inlineStr">
-        <is>
-          <t>۱ ساله در بهترین بازار انگلیسی‌زبان</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B60" s="20" t="inlineStr">
-        <is>
-          <t>Hochschule Luzern (HSLU) – Lucerne / Luzern</t>
-        </is>
-      </c>
-      <c r="C60" s="20" t="inlineStr">
-        <is>
-          <t>MSc Applied Data Science and AI (نام جدید از اوت ۲۰۲۶؛ قبلاً Applied Information and Data Science)</t>
-        </is>
-      </c>
-      <c r="D60" s="20" t="inlineStr">
-        <is>
-          <t>۲ سال</t>
-        </is>
-      </c>
-      <c r="E60" s="20" t="inlineStr">
-        <is>
-          <t>$53–64k</t>
-        </is>
-      </c>
-      <c r="F60" s="21" t="inlineStr">
-        <is>
-          <t>❌ کسری $13–24k</t>
-        </is>
-      </c>
-      <c r="G60" s="20" t="inlineStr">
-        <is>
-          <t>فقط با ۱۵ ساعت کار در ۱۸ ماه ($1,570–2,180/ماه) — پرریسک، معمولاً آلمانی می‌خواهد</t>
-        </is>
-      </c>
-      <c r="H60" s="20" t="inlineStr"/>
-      <c r="I60" s="19" t="inlineStr">
-        <is>
-          <t>Safe/Target</t>
-        </is>
-      </c>
-      <c r="J60" s="20" t="inlineStr"/>
-      <c r="K60" s="20" t="inlineStr">
-        <is>
-          <t>۴۵ دقیقه تا زوریخ؛ هر کارشناسی را می‌پذیرد</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B61" s="20" t="inlineStr">
-        <is>
-          <t>USI – Università della Svizzera italiana – Lugano</t>
-        </is>
-      </c>
-      <c r="C61" s="20" t="inlineStr">
-        <is>
-          <t>MSc Artificial Intelligence (با IDSIA)</t>
-        </is>
-      </c>
-      <c r="D61" s="20" t="inlineStr">
-        <is>
-          <t>۲ سال</t>
-        </is>
-      </c>
-      <c r="E61" s="20" t="inlineStr">
-        <is>
-          <t>$60–72k</t>
-        </is>
-      </c>
-      <c r="F61" s="21" t="inlineStr">
-        <is>
-          <t>❌ کسری $20–32k</t>
-        </is>
-      </c>
-      <c r="G61" s="20" t="inlineStr">
-        <is>
-          <t>بورس $4,840 + کار — نمی‌بندد</t>
-        </is>
-      </c>
-      <c r="H61" s="20" t="inlineStr"/>
-      <c r="I61" s="19" t="inlineStr">
-        <is>
-          <t>Target</t>
-        </is>
-      </c>
-      <c r="J61" s="20" t="inlineStr"/>
-      <c r="K61" s="20" t="inlineStr">
-        <is>
-          <t>AI با IDSIA؛ ورود با B2</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B62" s="20" t="inlineStr">
-        <is>
-          <t>Linköping University (LiU) – Linköping</t>
-        </is>
-      </c>
-      <c r="C62" s="20" t="inlineStr">
-        <is>
-          <t>MSc Computer Science</t>
-        </is>
-      </c>
-      <c r="D62" s="20" t="inlineStr">
-        <is>
-          <t>۲ سال</t>
-        </is>
-      </c>
-      <c r="E62" s="20" t="inlineStr">
-        <is>
-          <t>$59–64k</t>
-        </is>
-      </c>
-      <c r="F62" s="21" t="inlineStr">
-        <is>
-          <t>❌ کسری $19–24k</t>
-        </is>
-      </c>
-      <c r="G62" s="20" t="inlineStr">
-        <is>
-          <t>بورس ۵۰٪ LiU → $40–48k (معدل ۳.۵/۴؛ Reach)</t>
-        </is>
-      </c>
-      <c r="H62" s="20" t="inlineStr"/>
-      <c r="I62" s="19" t="inlineStr">
-        <is>
-          <t>Target</t>
-        </is>
-      </c>
-      <c r="J62" s="20" t="inlineStr"/>
-      <c r="K62" s="20" t="inlineStr">
-        <is>
-          <t>خوابگاه تضمینی؛ ولی بازار سوئد ضعیف</t>
         </is>
       </c>
     </row>
@@ -2883,12 +2986,12 @@
       </c>
       <c r="B63" s="20" t="inlineStr">
         <is>
-          <t>Aalborg University (AAU) – Aalborg</t>
+          <t>University of Twente (UT) – Enschede</t>
         </is>
       </c>
       <c r="C63" s="20" t="inlineStr">
         <is>
-          <t>MSc Computer Science (IT)</t>
+          <t>MSc Computer Science (گرایش‌ها: Cyber Security، Data Science، Software Tech، ...)</t>
         </is>
       </c>
       <c r="D63" s="20" t="inlineStr">
@@ -2898,17 +3001,17 @@
       </c>
       <c r="E63" s="20" t="inlineStr">
         <is>
-          <t>$63–70k</t>
+          <t>$77–85k</t>
         </is>
       </c>
       <c r="F63" s="21" t="inlineStr">
         <is>
-          <t>❌ کسری $23–30k</t>
+          <t>❌ شهریهٔ دو سال $49,500 › $40,000</t>
         </is>
       </c>
       <c r="G63" s="20" t="inlineStr">
         <is>
-          <t>≈ ۱۵ بورس AAU (بعید) + ویزا از تهران</t>
+          <t>فقط بورس UTS (تا ≈ $25k/سال؛ Reach)</t>
         </is>
       </c>
       <c r="H63" s="20" t="inlineStr"/>
@@ -2920,50 +3023,350 @@
       <c r="J63" s="20" t="inlineStr"/>
       <c r="K63" s="20" t="inlineStr">
         <is>
+          <t>انگلیسی‌دوست‌ترین بازار کار؛ ۱۲ ماه zoekjaar</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B64" s="20" t="inlineStr">
+        <is>
+          <t>Radboud University – Nijmegen</t>
+        </is>
+      </c>
+      <c r="C64" s="20" t="inlineStr">
+        <is>
+          <t>MSc Computing Science (گرایش‌ها: Cyber Security، Data Science، Software Science)</t>
+        </is>
+      </c>
+      <c r="D64" s="20" t="inlineStr">
+        <is>
+          <t>۲ سال</t>
+        </is>
+      </c>
+      <c r="E64" s="20" t="inlineStr">
+        <is>
+          <t>$74–82k</t>
+        </is>
+      </c>
+      <c r="F64" s="21" t="inlineStr">
+        <is>
+          <t>❌ شهریهٔ دو سال $44,900 › $40,000</t>
+        </is>
+      </c>
+      <c r="G64" s="20" t="inlineStr">
+        <is>
+          <t>فقط Radboud Scholarship (Reach)</t>
+        </is>
+      </c>
+      <c r="H64" s="20" t="inlineStr"/>
+      <c r="I64" s="19" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="J64" s="20" t="inlineStr"/>
+      <c r="K64" s="20" t="inlineStr">
+        <is>
+          <t>ارزان‌ترِ هلند</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B65" s="20" t="inlineStr">
+        <is>
+          <t>University of Amsterdam (UvA) – Amsterdam</t>
+        </is>
+      </c>
+      <c r="C65" s="20" t="inlineStr">
+        <is>
+          <t>MSc Software Engineering (۱ ساله!)</t>
+        </is>
+      </c>
+      <c r="D65" s="20" t="inlineStr">
+        <is>
+          <t>۱ سال</t>
+        </is>
+      </c>
+      <c r="E65" s="20" t="inlineStr">
+        <is>
+          <t>$57–62k</t>
+        </is>
+      </c>
+      <c r="F65" s="21" t="inlineStr">
+        <is>
+          <t>❌ شهریه $39,100 → $900 برای زندگی؛ کار ۱۶ ساعت + TWV ≤ $1,150</t>
+        </is>
+      </c>
+      <c r="G65" s="20" t="inlineStr">
+        <is>
+          <t>هیچ</t>
+        </is>
+      </c>
+      <c r="H65" s="20" t="inlineStr"/>
+      <c r="I65" s="19" t="inlineStr">
+        <is>
+          <t>Target/Reach</t>
+        </is>
+      </c>
+      <c r="J65" s="20" t="inlineStr"/>
+      <c r="K65" s="20" t="inlineStr">
+        <is>
+          <t>۱ ساله در بهترین بازار انگلیسی‌زبان</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B66" s="20" t="inlineStr">
+        <is>
+          <t>Linköping University (LiU) – Linköping</t>
+        </is>
+      </c>
+      <c r="C66" s="20" t="inlineStr">
+        <is>
+          <t>MSc Computer Science</t>
+        </is>
+      </c>
+      <c r="D66" s="20" t="inlineStr">
+        <is>
+          <t>۲ سال</t>
+        </is>
+      </c>
+      <c r="E66" s="20" t="inlineStr">
+        <is>
+          <t>$59–64k</t>
+        </is>
+      </c>
+      <c r="F66" s="21" t="inlineStr">
+        <is>
+          <t>❌ بعد از شهریه $6,500 = ۵–۶ ماه؛ ۱۸ ماه × $1,160 از کار بدون سوئدی غیرواقعی</t>
+        </is>
+      </c>
+      <c r="G66" s="20" t="inlineStr">
+        <is>
+          <t>بورس ۵۰٪ LiU → ۲۰ ماه پوشش ✅ (معدل ۳.۵/۴؛ Reach)</t>
+        </is>
+      </c>
+      <c r="H66" s="20" t="inlineStr"/>
+      <c r="I66" s="19" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="J66" s="20" t="inlineStr"/>
+      <c r="K66" s="20" t="inlineStr">
+        <is>
+          <t>خوابگاه تضمینی؛ Saab/Ericsson</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B67" s="20" t="inlineStr">
+        <is>
+          <t>Aalborg University (AAU) – Aalborg</t>
+        </is>
+      </c>
+      <c r="C67" s="20" t="inlineStr">
+        <is>
+          <t>MSc Computer Science (IT)</t>
+        </is>
+      </c>
+      <c r="D67" s="20" t="inlineStr">
+        <is>
+          <t>۲ سال</t>
+        </is>
+      </c>
+      <c r="E67" s="20" t="inlineStr">
+        <is>
+          <t>$63–70k</t>
+        </is>
+      </c>
+      <c r="F67" s="21" t="inlineStr">
+        <is>
+          <t>❌ بعد از شهریه $5,500 = ۴ ماه؛ ۲۰ ماه × $1,335 از کار (معمولاً دانمارکی)</t>
+        </is>
+      </c>
+      <c r="G67" s="20" t="inlineStr">
+        <is>
+          <t>≈ ۱۵ بورس AAU (بعید) + ویزا از تهران</t>
+        </is>
+      </c>
+      <c r="H67" s="20" t="inlineStr"/>
+      <c r="I67" s="19" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="J67" s="20" t="inlineStr"/>
+      <c r="K67" s="20" t="inlineStr">
+        <is>
           <t>۳ سال اقامت کاریابی؛ حقوق بالا</t>
         </is>
       </c>
     </row>
-    <row r="64"/>
-    <row r="65">
-      <c r="A65" s="3" t="inlineStr">
-        <is>
-          <t>ت) نتیجه در ۵ خط</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="40" customHeight="1">
-      <c r="A66" s="11" t="inlineStr">
-        <is>
-          <t>۱) اصلاح مهم: بودجهٔ شما $40,000 برای کل دوره است (نه در سال). این عدد بازی را عوض می‌کند: هلند ($74–90k)، سوئد ($51–65k) و دانمارک ($63–76k) کلاً بیرون‌اند؛ از سوئیس فقط Joint MSc در Neuchâtel/Fribourg ($32–43k) و با کار دانشجویی Basel ($38–49k) می‌مانند (HSLU/USI/UZH/ETH نه)؛ آلمان ($25–37k) تنها کشوری است که راحت جا می‌شود؛ انگلستان فقط Teesside/Northumbria/Essex، آن هم با ۲۰ ساعت کار در هفته.</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="40" customHeight="1">
-      <c r="A67" s="11" t="inlineStr">
-        <is>
-          <t>۲) با وزن‌های شما (کار = حقوق ۲۷.۵ / انگلیسی ۳۰ / هزینه ۱۵) بین همین برنامه‌ها: Basel ۶۶.۸ › Neuchâtel ۶۵.۵ › Fribourg ۶۴ › Stuttgart ۵۹.۵ › Darmstadt ۵۸.۵ › Saarland ۵۷.۳ › Teesside ۵۷ › Northumbria = Essex ۵۵.۳ › Passau ۵۱.۵. سوئیسِ ارزان روی کاغذ برنده است چون حقوق ۱۰/۱۰ دارد و شهریه‌اش ناچیز است.</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="40" customHeight="1">
-      <c r="A68" s="11" t="inlineStr">
-        <is>
-          <t>۳) ولی هر سه گزینهٔ سوئیس روی لبهٔ بودجه‌اند: ۶ ماه اول حق کار ندارید و بعد فقط ۱۵ ساعت؛ کانتون برای مجوز اقامت $25,400 در سال (Basel $29,000) در بانک سوئیسی به نام خودتان می‌خواهد؛ زندگی روزمره فرانسه (Neuchâtel/Fribourg) یا آلمانی (Basel)؛ و بعد از مدرک فقط ۶ ماه برای کاری که از سهمیهٔ کانتونی کم می‌شود. اگر پذیرش بگیرید، $40k را نشان دهید و کار دانشجویی پیدا کنید، پاداشش حقوق $103–127k است — این یک شرط‌بندی حساب‌شده است، نه برنامهٔ امن.</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" ht="40" customHeight="1">
-      <c r="A69" s="11" t="inlineStr">
-        <is>
-          <t>۴) آلمان برنامهٔ امن با بهترین شانس استخدام در این بودجه است: Darmstadt/Saarland ($26–37k) راحت، Stuttgart ($38–45k) با Werkstudent؛ ۲۰ ساعت کار دانشجویی ($1,140–1,820/ماه) که هم پول است و هم راه استاندارد استخدام؛ ۱۸ ماه بعد از مدرک؛ حقوق $55–63k. بهایش: آلمانی B1 در این دو سال برای زندگی روزمره و نیمی از آگهی‌ها. انگلستان با ۱۰۰٪ انگلیسی فقط اگر ۲۰ ساعت کار کنید و بازار جونیور ضعیف و اسپانسری $50,700+ را بپذیرید.</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="40" customHeight="1">
-      <c r="A70" s="11" t="inlineStr">
-        <is>
-          <t>۵) توصیه با بودجهٔ $40k کل: ۷ درخواست — ۲ سوئیس (Neuchâtel، Basel؛ Fribourg هم اگر خواستید، همان مدرک) + ۳ آلمان (Stuttgart، Darmstadt، Saarland) + ۱–۲ انگلستان (Essex یا Northumbria) به‌عنوان پذیرش قطعیِ انگلیسی. پذیرش سوئیس + شرط‌های خط ۳ → سوئیس (با وزن‌های شما)؛ وگرنه آلمان. هلند را فقط با بورس Reach (UTS Twente / Radboud Scholarship) دنبال کنید — بدون آن دیگر گزینه نیست.</t>
+    <row r="68">
+      <c r="A68" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B68" s="20" t="inlineStr">
+        <is>
+          <t>University of Southern Denmark (SDU) – Odense</t>
+        </is>
+      </c>
+      <c r="C68" s="20" t="inlineStr">
+        <is>
+          <t>MSc Computer Science</t>
+        </is>
+      </c>
+      <c r="D68" s="20" t="inlineStr">
+        <is>
+          <t>۲ سال</t>
+        </is>
+      </c>
+      <c r="E68" s="20" t="inlineStr">
+        <is>
+          <t>$69–76k</t>
+        </is>
+      </c>
+      <c r="F68" s="21" t="inlineStr">
+        <is>
+          <t>❌ شهریه $39,400 → $600 برای زندگی</t>
+        </is>
+      </c>
+      <c r="G68" s="20" t="inlineStr">
+        <is>
+          <t>هیچ</t>
+        </is>
+      </c>
+      <c r="H68" s="20" t="inlineStr"/>
+      <c r="I68" s="19" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="J68" s="20" t="inlineStr"/>
+      <c r="K68" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B69" s="20" t="inlineStr">
+        <is>
+          <t>Durham University (Russell Group) – Durham</t>
+        </is>
+      </c>
+      <c r="C69" s="20" t="inlineStr">
+        <is>
+          <t>MSc Advanced Computer Science (و MSc Data Science)</t>
+        </is>
+      </c>
+      <c r="D69" s="20" t="inlineStr">
+        <is>
+          <t>۱ سال</t>
+        </is>
+      </c>
+      <c r="E69" s="20" t="inlineStr">
+        <is>
+          <t>$61–65k</t>
+        </is>
+      </c>
+      <c r="F69" s="21" t="inlineStr">
+        <is>
+          <t>❌ شهریه $45,700 › $40,000 (Russell Group: $43–50k)</t>
+        </is>
+      </c>
+      <c r="G69" s="20" t="inlineStr">
+        <is>
+          <t>هیچ بورس قابل اتکایی برای ایران</t>
+        </is>
+      </c>
+      <c r="H69" s="20" t="inlineStr"/>
+      <c r="I69" s="19" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="J69" s="20" t="inlineStr"/>
+      <c r="K69" s="20" t="inlineStr">
+        <is>
+          <t>برند Russell Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B70" s="20" t="inlineStr">
+        <is>
+          <t>ETH Zürich – Zürich</t>
+        </is>
+      </c>
+      <c r="C70" s="20" t="inlineStr">
+        <is>
+          <t>MSc Computer Science</t>
+        </is>
+      </c>
+      <c r="D70" s="20" t="inlineStr">
+        <is>
+          <t>۲ سال</t>
+        </is>
+      </c>
+      <c r="E70" s="20" t="inlineStr">
+        <is>
+          <t>$66–84k</t>
+        </is>
+      </c>
+      <c r="F70" s="21" t="inlineStr">
+        <is>
+          <t>❌ بعد از شهریه $29k = ۱۱ ماه زوریخ؛ ۱۳ ماه × $2,665 با ۱۵ ساعت کار کنار ETH غیرواقعی</t>
+        </is>
+      </c>
+      <c r="G70" s="20" t="inlineStr">
+        <is>
+          <t>ESOP (بسیار Reach)</t>
+        </is>
+      </c>
+      <c r="H70" s="20" t="inlineStr"/>
+      <c r="I70" s="19" t="inlineStr">
+        <is>
+          <t>Reach</t>
+        </is>
+      </c>
+      <c r="J70" s="20" t="inlineStr"/>
+      <c r="K70" s="20" t="inlineStr">
+        <is>
+          <t>رتبهٔ ۸ جهان؛ Reach برای معدل ۱۵.۷۷</t>
         </is>
       </c>
     </row>
@@ -2971,48 +3374,91 @@
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
+          <t>ت) نتیجه در ۵ خط</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="40" customHeight="1">
+      <c r="A73" s="11" t="inlineStr">
+        <is>
+          <t>۱) تعریف شما: $40,000 = کل شهریه + زندگیِ ماه‌های اول تا پیدا شدن کار دانشجویی. پس فیلتر واقعی این است: بعد از پرداخت شهریه چند ماه زندگی می‌ماند و بقیه را قانوناً و عملاً می‌توانید با کار دربیاورید؟ نتیجه: آلمان حتی بدون کار جا می‌شود؛ انگلستان با ۲۰ ساعت کار (ساده‌ترین کار دانشجویی، $16.8/ساعت ≈ $1,450/ماه)؛ سوئیس فقط اگر ۶ ماه اول را بدون درآمد بگذرانید؛ سوئد فقط با بورس؛ هلند (شهریهٔ دو سال $45–50k به‌تنهایی) و دانمارک (۴ ماه پوشش + ویزا) بیرون.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="40" customHeight="1">
+      <c r="A74" s="11" t="inlineStr">
+        <is>
+          <t>۲) با وزن‌های شما (کار = حقوق ۲۷.۵ / انگلیسی ۳۰ / هزینه ۱۵): Basel ۷۱.۳ › HSLU ۶۸.۳ › Neuchâtel ۶۷ › Fribourg ۶۵.۵ › Stuttgart ۶۴ = Manchester Met ۶۴ › Teesside ۶۱.۵ › Northumbria = Essex ۶۱.۳ › USI ۶۱ › Darmstadt ۶۰ › Leicester ۵۹.۸ › Saarland ۵۷.۳ › BTH = MDU ۵۵ › Passau ۵۱.۵. سوئیس بالاست چون حقوق ۱۰/۱۰ دارد و شهریه‌اش ناچیز است؛ HSLU و USI با این مدل برمی‌گردند، ولی فقط با کار از ماه ۷.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="40" customHeight="1">
+      <c r="A75" s="11" t="inlineStr">
+        <is>
+          <t>۳) ریسک سوئیس را با عدد ببینید: ۶ ماه اول حق کار ندارید (Neuchâtel/Fribourg/Basel این ۶ ماه را از خودِ $40k رد می‌کنند و تقریباً بی‌نیاز از کارند؛ HSLU از ماه ۷ حدود $1,000/ماه و USI حدود $1,450/ماه از ۱۵ ساعت کار می‌خواهد)؛ کانتون $25,400 (Basel 24,000) را در بانک می‌خواهد — انتقال پول از ایران به بانک سوئیسی سخت است و زوریخ فقط حساب سوئیسی به نام خودتان را می‌پذیرد؛ بعد از مدرک ۶ ماه برای کاری که از سهمیهٔ کانتونی کم می‌شود. پاداش: حقوق $103–127k.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="40" customHeight="1">
+      <c r="A76" s="11" t="inlineStr">
+        <is>
+          <t>۴) آلمان امن‌ترین است: Darmstadt/Saarland/Passau بعد از شهریه تمام ۲۴ ماه + $6–12k اضافه دارند، Stuttgart ۲۳ ماه؛ Werkstudent ۲۰ ساعت از روز اول ($1,140–1,710 خالص) هم پول است و هم راه استاندارد استخدام؛ ۱۸ ماه بعد از مدرک؛ حقوق $55–63k؛ بهایش آلمانی B1. انگلستان انگلیسیِ کامل و کار دانشجویی آسان دارد (Teesside حتی بدون کار)، ولی همان دو معیار «کار جونیور» و «حقوق» در آن ضعیف‌ترین‌اند و اثبات تمکن Northumbria/Essex/MMU ≈ $1–3k بیشتر از $40k است (موقتاً از حساب خانواده).</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="40" customHeight="1">
+      <c r="A77" s="11" t="inlineStr">
+        <is>
+          <t>۵) توصیه: ۸ درخواست — ۳ سوئیس (HSLU، Basel، Neuchâtel؛ USI فقط اگر ریسک بیشتر می‌پذیرید) + ۳ آلمان (Stuttgart، Darmstadt، Saarland) + ۲ انگلستان (Northumbria یا Manchester Met، Essex). قاعدهٔ تصمیم در می–ژوئن ۲۰۲۷: پذیرش سوئیس + راهی برای نشان دادن $25,400 + پذیرفتن ۶ ماه بدون درآمد و ۶ ماه بعد از مدرک → سوئیس (با وزن‌های شما)؛ وگرنه آلمان (Stuttgart اگر Werkstudent، وگرنه Darmstadt/Saarland)؛ انگلستان فقط اگر ۱۰۰٪ انگلیسی و ۱ ساله برایتان از حقوق و بازار مهم‌تر شد.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78"/>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
           <t>ث) چهار قدم بعدی</t>
         </is>
       </c>
     </row>
-    <row r="73" ht="34" customHeight="1">
-      <c r="A73" s="11" t="inlineStr">
-        <is>
-          <t>اکتبر – دسامبر ۲۰۲۶: نظام‌وظیفه · IELTS Academic خارج از ایران تا دسامبر (Joint MSc سوئیس مدرک زبان نمی‌خواهد؛ Stuttgart / Saarland / Darmstadt IELTS 7؛ Basel B2–C1؛ Passau B2؛ انگلستان 6.0–6.5) · ترجمهٔ رسمی مدارک · گواهی رتبهٔ کلاسی از سمنان · شروع آلمانی A1–A2 (برای آلمان لازم می‌شود).</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="34" customHeight="1">
-      <c r="A74" s="11" t="inlineStr">
-        <is>
-          <t>۱۵ ژانویه ۲۰۲۷: Stuttgart · ۲۸ فوریه: Fribourg (ویزایی‌ها) · ۳۱ مارس: Neuchâtel · ۳۰ آوریل: Basel · ۳۱ می: Passau · می – ژوئیه: Darmstadt / Saarland · Essex / Northumbria rolling.</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="34" customHeight="1">
-      <c r="A75" s="11" t="inlineStr">
-        <is>
-          <t>با هر پذیرش، تمکن مالی را چک کنید: سوئیس $25,400 (Basel $29,000) در بانک سوئیسی به نام خودتان قبل از ویزا · آلمان حساب مسدود $13,600 (ماهی $1,130 آزاد می‌شود) · انگلستان شهریهٔ سال + ۹ × $1,590 به مدت ۲۸ روز. همهٔ این‌ها از همان $40k است، «اضافه» نیست — ولی باید یک‌جا نشان داده شود.</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="34" customHeight="1">
-      <c r="A76" s="11" t="inlineStr">
-        <is>
-          <t>می – ژوئیه ۲۰۲۷: ویزا (سوئیس: سفارت تهران با وقت قبلی · آلمان: سفارت فقط اضطراری → برنامهٔ B از ترکیه / ارمنستان · انگلستان: VAC تهران متغیر) · مسکن را همان روز پذیرش شروع کنید (Stuttgart صف ۶–۸ ماه؛ Essex تضمینی؛ سوئیس WOKO/خوابگاه دانشگاه).</t>
-        </is>
-      </c>
-    </row>
-    <row r="77"/>
-    <row r="78">
-      <c r="A78" s="3" t="inlineStr">
+    <row r="80" ht="34" customHeight="1">
+      <c r="A80" s="11" t="inlineStr">
+        <is>
+          <t>اکتبر – دسامبر ۲۰۲۶: نظام‌وظیفه · IELTS Academic خارج از ایران تا دسامبر (Joint MSc سوئیس مدرک زبان نمی‌خواهد؛ Stuttgart / Saarland / Darmstadt IELTS 7؛ HSLU / Basel B2–C1؛ Passau B2؛ انگلستان 6.0–6.5) · ترجمهٔ رسمی مدارک · گواهی رتبهٔ کلاسی از سمنان · شروع آلمانی A1–A2 · از International Office دانشگاه‌های سوئیس بپرسید اثبات $25,400 را برای متقاضی ایرانی چطور می‌پذیرند (بانک سوئیسی / ضمانت‌نامه / حساب خانواده).</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="34" customHeight="1">
+      <c r="A81" s="11" t="inlineStr">
+        <is>
+          <t>۱۵ ژانویه ۲۰۲۷: Stuttgart (و BTH/MDU اگر پشتوانهٔ سوئد را خواستید) · ۲۸ فوریه: Fribourg (ویزایی‌ها) · ۳۱ مارس: Neuchâtel · ۱ آوریل: HSLU · ۳۰ آوریل: Basel، USI · ۳۱ می: Passau · می – ژوئیه: Darmstadt / Saarland · Essex / Northumbria / Manchester Met rolling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="34" customHeight="1">
+      <c r="A82" s="11" t="inlineStr">
+        <is>
+          <t>با هر پذیرش، تمکن مالی را همان روز بررسی کنید: سوئیس $25,400 (Basel $29,000) در بانک قبل از ویزا · آلمان حساب مسدود $13,600 (ماهی $1,130 آزاد می‌شود) · انگلستان شهریهٔ سال + ۹ × $1,590 به مدت ۲۸ روز (حساب والدین با رضایت‌نامه مجاز). همهٔ این‌ها از همان $40k است، ولی باید یک‌جا نشان داده شود — و انتقال پول از ایران زمان و کارمزد دارد.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="34" customHeight="1">
+      <c r="A83" s="11" t="inlineStr">
+        <is>
+          <t>می – ژوئیه ۲۰۲۷: ویزا (سوئیس: سفارت تهران با وقت قبلی · آلمان: سفارت فقط اضطراری → برنامهٔ B از ترکیه / ارمنستان · انگلستان: VAC تهران متغیر) · مسکن را همان روز پذیرش شروع کنید (Stuttgart صف ۶–۸ ماه؛ Essex تضمینی؛ سوئیس خوابگاه دانشگاه/WOKO) · از هفتهٔ اول دنبال کار دانشجویی بروید (آلمان/انگلستان) یا برای ماه ۷ آماده شوید (سوئیس).</t>
+        </is>
+      </c>
+    </row>
+    <row r="84"/>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
         <is>
           <t>ج) بقیهٔ فایل</t>
         </is>
       </c>
     </row>
-    <row r="79" ht="44" customHeight="1">
-      <c r="A79" s="11" t="inlineStr">
+    <row r="86" ht="44" customHeight="1">
+      <c r="A86" s="11" t="inlineStr">
         <is>
           <t>بقیهٔ شیت‌ها پیوست‌اند و فقط برای جزئیات: «جدول نهایی ۲۰۲۶» (۲۸ معیار)، «برنامه‌ها» (۱۱۰ برنامه، هر کدام با ستون «کل هزینهٔ دوره»)، «حوزه‌ها و بازار کار»، «برنامهٔ زمانی ۲۰۲۷»، «خوابگاه و مسکن»، «جمع‌بندی»، «راستی‌آزمایی» (تنها جایی که رقم رسمی به ارز محلی هم داخل پرانتز آمده) و «منابع». همهٔ آن‌ها هم به دلار هستند.</t>
         </is>
@@ -3020,29 +3466,29 @@
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="A83:K83"/>
     <mergeCell ref="A39:K39"/>
+    <mergeCell ref="A77:K77"/>
+    <mergeCell ref="A59:K59"/>
+    <mergeCell ref="A82:K82"/>
     <mergeCell ref="A73:K73"/>
     <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A70:K70"/>
     <mergeCell ref="A79:K79"/>
-    <mergeCell ref="A69:K69"/>
-    <mergeCell ref="A78:K78"/>
-    <mergeCell ref="A65:K65"/>
+    <mergeCell ref="A61:K61"/>
     <mergeCell ref="A41:K41"/>
-    <mergeCell ref="A66:K66"/>
+    <mergeCell ref="A80:K80"/>
+    <mergeCell ref="A75:K75"/>
     <mergeCell ref="A37:K37"/>
-    <mergeCell ref="A75:K75"/>
     <mergeCell ref="A74:K74"/>
     <mergeCell ref="A26:K26"/>
-    <mergeCell ref="A55:K55"/>
+    <mergeCell ref="A86:K86"/>
     <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A85:K85"/>
     <mergeCell ref="A76:K76"/>
-    <mergeCell ref="A53:K53"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A72:K72"/>
+    <mergeCell ref="A81:K81"/>
     <mergeCell ref="A38:K38"/>
-    <mergeCell ref="A68:K68"/>
-    <mergeCell ref="A67:K67"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3627,42 +4073,42 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>سازگاری با بودجهٔ $40,000 برای کل دوره (اصلاح ۲۸ سپتامبر: بودجه «کل تحصیل» است، نه سالانه — همهٔ برداشت‌های قبلی منسوخ)</t>
+          <t>سازگاری با بودجهٔ $40,000 = کل شهریه + زندگیِ ماه‌های اول تا پیدا شدن کار دانشجویی (تعریف شما، ۲۸ سپتامبر). محاسبه: (۴۰,۰۰۰ − شهریهٔ کل دوره) ÷ زندگی ماهانهٔ همان شهر = ماه‌های پوشش‌داده‌شده؛ بقیهٔ ماه‌ها باید از کار دانشجویی دربیاید</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>✅ Darmstadt $30–37k · Saarland $26–32k · Passau $25–31k راحت؛ Stuttgart $38–45k مرزی (با Werkstudent از ترم اول جا می‌شود)</t>
+          <t>✅ حتی بدون کار جا می‌شود: Darmstadt / Saarland / Passau بعد از شهریه $38–39k می‌ماند = تمام ۲۴ ماه + $6–12k اضافه؛ Stuttgart $32k = ۲۳ ماه (کسری ≈ $1.4k). کار: ۲۰ ساعت از روز اول، Werkstudent $1,140–1,710 خالص = راه استاندارد استخدام. اثبات برای ویزا: حساب مسدود $13,600</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>❌ کل دوره $74–90k → کسری $34–50k؛ NL Scholarship $5,700 نمی‌بندد؛ فقط با بورس Reach (UTS Twente تا ≈ $25k/سال، Radboud Scholarship)</t>
+          <t>❌ شهریه به‌تنهایی بودجه را می‌خورد: Twente $49,500 و Radboud $44,900 برای دو سال؛ UvA یک‌ساله $39,100 → فقط $900 برای زندگی؛ کار ۱۶ ساعت (با مجوز TWV، حداکثر ≈ $1,150) هم جبران نمی‌کند</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>❌ $51–65k → کسری $11–25k؛ فقط با بورس ۵۰٪ LiU ($40–48k؛ معدل ۳.۵/۴ لازم) یا ۱۰۰٪ MDU (قرعه)</t>
+          <t>⚠️ فقط با بورس یا شانس: LiU بعد از شهریه $6,500 = ۵–۶ ماه، ۱۸ ماه باقی ≈ $970/ماه از کار — بدون سوئدی غیرواقعی ($350–900)؛ BTH $11,700 = ۱۱ ماه → ≈ $630/ماه ⚠️؛ MDU $12,700 = ۱۱–۱۲ ماه → ≈ $640/ماه ⚠️؛ با بورس ۵۰٪ LiU یا ۲۵–۱۰۰٪ MDU/Halmstad ✓. اثبات: $1,080 × ۱۰ ماه</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>❌ $63–76k → کسری $23–36k؛ به‌علاوه ویزا از تهران</t>
+          <t>❌ AAU بعد از شهریه $5,500 = ۴ ماه؛ ۲۰ ماه باقی ≈ $1,200/ماه از کار (۲۰ ساعت، معمولاً دانمارکی)؛ SDU $600؛ به‌علاوه ویزا از تهران</t>
         </is>
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>⚠️ فقط Joint MSc: Neuchâtel $32–41k / Fribourg $35–43k (زندگی صرفه‌جویانه ≈ $1,650/ماه + کار ۱۵ ساعت بعد از ماه ۶) و Basel $38–49k فقط با کار؛ HSLU $53–64k، USI $60–72k، UZH $45–58k، ETH/EPFL $60–84k ❌؛ کانتون تمکن $25,400/سال (Basel $29,000) را باید در بانک ببیند</t>
+          <t>⚠️ قانون: ۶ ماه اول کار ممنوع، بعد حداکثر ۱۵ ساعت ($24–36/ساعت ≈ $1,550–2,200 در ماه). Neuchâtel/Fribourg بعد از شهریه $36–37k = تمام ۱۸ ماه ✅ · Basel $37k = ۱۶–۱۷ ماه از ۱۸ ✅ · HSLU $32k = ۱۵ ماه از ۲۴ → از ماه ۷ حدود $1,000/ماه لازم ⚠️ شدنی · USI $21k = ۱۰–۱۱ ماه از ۲۴ → ≈ $1,450/ماه ⚠️ پرریسک · UZH $37k = ۱۴ ماه زوریخ (Reach) · ETH ❌. اثبات: $25,400 در سال (زوریخ: فقط بانک سوئیسی به نام خودتان؛ Basel $29,000)</t>
         </is>
       </c>
       <c r="H11" s="12" t="inlineStr">
         <is>
-          <t>⚠️ برنامهٔ یک‌ساله: Teesside $38–41k مرزی؛ Northumbria $44–48k و Essex $43–48k (بعد از بورس $5,960) فقط با ۲۰ ساعت کار ($8–12k در سال)؛ Russell Group $62–87k ❌</t>
+          <t>✅ با ۲۰ ساعت کار (حداقل دستمزد $16.8/ساعت از آوریل ۲۰۲۶ → ≈ $1,450 در ماه؛ کار پیدا کردن آسان‌ترین در بین این کشورها): Teesside بعد از شهریه $17.5k = تمام ۱۲ ماه بدون کار ✅ · Northumbria $11.5k = ۸ ماه → ≈ $500/ماه ✅ · Manchester Met $12.2k = ۸ ماه ✅ · Essex بعد از بورس $13.3k = ۸–۹ ماه ✅ · Leicester $7.9k = ۵ ماه → ≈ $870/ماه ⚠️ · لندن (Brunel: ۳ ماه) ❌ · Russell Group (شهریه $43–50k) ❌. اثبات: شهریه + ۹ × $1,590 = برای Northumbria/Essex/MMU ≈ $41–43k، یعنی $1–3k بیشتر از بودجه (موقتاً از حساب خانواده مجاز است)</t>
         </is>
       </c>
       <c r="I11" s="22" t="inlineStr">
         <is>
-          <t>محاسبه از ستون «کل هزینهٔ دوره» شیت «برنامه‌ها» (شهریه × طول دوره + زندگی همان شهر × ماه‌ها)؛ بدون بلیت/ویزا/ودیعه</t>
+          <t>محاسبه از شیت «برنامه‌ها» (شهریهٔ کل دوره؛ زندگی = میانهٔ بازهٔ همان شهر). سقف قانونی کار دانشجویی: آلمان ۲۰ ساعت (۱۴۰ روز/سال) · هلند ۱۶ ساعت + TWV · سوئد بدون سقف · دانمارک ۲۰ ساعت · سوئیس ۰ تا ماه ۶، بعد ۱۵ ساعت · انگلستان ۲۰ ساعت در ترم. درآمدها خالص برآوردی (ردیف کار دانشجویی)</t>
         </is>
       </c>
     </row>
@@ -4575,42 +5021,42 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>امتیاز با وزن‌های شما (۲۸ سپتامبر): کار پیدا کردن ۲۷.۵٪ = حقوق ۲۷.۵٪ / فقط انگلیسی ۳۰٪ / هزینهٔ کل ۱۵٪ — از ۱۰۰ (زیرامتیازها از ۱۰)؛ ⚠️ فیلتر بودجهٔ $40,000 کل (ردیف ۹) جداگانه اعمال می‌شود</t>
+          <t>امتیاز با وزن‌های شما (۲۸ سپتامبر): کار پیدا کردن ۲۷.۵٪ = حقوق ۲۷.۵٪ / فقط انگلیسی ۳۰٪ / هزینهٔ کل ۱۵٪ — از ۱۰۰ (زیرامتیازها از ۱۰)؛ ⚠️ فیلتر بودجه (ردیف ۹: $40,000 = شهریه + زندگی تا کار) جداگانه اعمال می‌شود</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">
         <is>
-          <t>کار ۶ · حقوق ۶ · انگلیسی ۴ · هزینه ۱۰ → ۶۰ — در بودجه ✅ (بهترین شانس کار در این بودجه)</t>
+          <t>کار ۶ · حقوق ۶ · انگلیسی ۴ · هزینه ۱۰ → ۶۰ — ✅ حتی بدون کار جا می‌شود</t>
         </is>
       </c>
       <c r="D31" s="12" t="inlineStr">
         <is>
-          <t>کار ۸ · حقوق ۵ · انگلیسی ۸ · هزینه ۲ → ۶۲.۸ — ❌ خارج از بودجهٔ $40k کل</t>
+          <t>کار ۸ · حقوق ۵ · انگلیسی ۸ · هزینه ۲ → ۶۲.۸ — ❌ شهریه به‌تنهایی بیش از $40k</t>
         </is>
       </c>
       <c r="E31" s="12" t="inlineStr">
         <is>
-          <t>کار ۴ · حقوق ۵ · انگلیسی ۸ · هزینه ۶ → ۵۷.۸ — ❌ خارج از بودجه</t>
+          <t>کار ۴ · حقوق ۵ · انگلیسی ۸ · هزینه ۶ → ۵۷.۸ — ⚠️ فقط با بورس</t>
         </is>
       </c>
       <c r="F31" s="12" t="inlineStr">
         <is>
-          <t>کار ۵ · حقوق ۷ · انگلیسی ۶ · هزینه ۴ → ۵۷ — ❌ خارج از بودجه + ویزا</t>
+          <t>کار ۵ · حقوق ۷ · انگلیسی ۶ · هزینه ۴ → ۵۷ — ❌ بودجه + ویزا</t>
         </is>
       </c>
       <c r="G31" s="12" t="inlineStr">
         <is>
-          <t>کار ۵ · حقوق ۱۰ · انگلیسی ۶ · هزینه ۵ → ۶۶.۸ — فقط Joint MSc Neuchâtel/Fribourg و Basel در بودجه ⚠️</t>
+          <t>کار ۵ · حقوق ۱۰ · انگلیسی ۶ · هزینه ۵ → ۶۶.۸ — ✅ Neuchâtel/Fribourg/Basel؛ ⚠️ HSLU با کار از ماه ۷؛ USI پرریسک</t>
         </is>
       </c>
       <c r="H31" s="12" t="inlineStr">
         <is>
-          <t>کار ۵ · حقوق ۳ · انگلیسی ۱۰ · هزینه ۵ → ۵۹.۵ — فقط Teesside/Northumbria/Essex با ۲۰ ساعت کار ⚠️</t>
+          <t>کار ۵ · حقوق ۳ · انگلیسی ۱۰ · هزینه ۵ → ۵۹.۵ — ✅ Teesside بدون کار؛ Northumbria/Essex/MMU با ≈ $500/ماه کار</t>
         </is>
       </c>
       <c r="I31" s="22" t="inlineStr">
         <is>
-          <t>امتیاز کشوری با وزن‌های شما (کار و حقوق برابر). «کار» = ردیف‌های ۱۵، ۱۶/۱۷، ۲۶؛ «حقوق» = ۱۷–۱۹؛ «کار» سوئیس ۵ چون فارغ‌التحصیلان سوئیس طبق مادهٔ ۲۱(۳) AIG از اولویت نیروی داخلی معاف‌اند (سهمیه و ۶ ماه باقی است). با بودجهٔ $40,000 برای کل دوره، فقط سه کشور برنامه‌ای در بودجه دارند: سوئیس (Joint MSc/Basel)، آلمان، انگلستان (ارزان‌ها با کار). امتیاز برنامه‌به‌برنامه در شیت «تصمیم» بخش پ: Basel ۶۶.۸ › Neuchâtel ۶۵.۵ › Fribourg ۶۴ › Stuttgart ۵۹.۵ › Darmstadt ۵۸.۵ › Saarland ۵۷.۳ › Teesside ۵۷ › Northumbria = Essex ۵۵.۳ › Passau ۵۱.۵. امتیازها قضاوت‌اند؛ وزن‌ها در شیت «تصمیم» قابل تغییرند.</t>
+          <t>امتیاز کشوری با وزن‌های شما (کار و حقوق برابر). «کار» = ردیف‌های ۱۵، ۱۶/۱۷، ۲۶؛ «حقوق» = ۱۷–۱۹؛ «کار» سوئیس ۵ چون فارغ‌التحصیلان سوئیس طبق مادهٔ ۲۱(۳) AIG از اولویت نیروی داخلی معاف‌اند (سهمیه و ۶ ماه باقی است). امتیاز برنامه‌به‌برنامه با مدل بودجهٔ «شهریه + زندگی تا کار» در شیت «تصمیم» بخش پ: Basel ۷۱.۳ › HSLU ۶۸.۳ › Neuchâtel ۶۷ › Fribourg ۶۵.۵ › Stuttgart ۶۴ = Manchester Met ۶۴ › Teesside ۶۱.۵ › Northumbria = Essex ۶۱.۳ › USI ۶۱ › Darmstadt ۶۰ › Leicester ۵۹.۸ › Saarland ۵۷.۳ › BTH = MDU ۵۵ › Passau ۵۱.۵. امتیازها قضاوت‌اند؛ وزن‌ها در شیت «تصمیم» قابل تغییرند.</t>
         </is>
       </c>
     </row>
@@ -4838,7 +5284,7 @@
           <t>— (THE 601–800)</t>
         </is>
       </c>
-      <c r="O2" s="17" t="inlineStr">
+      <c r="O2" s="18" t="inlineStr">
         <is>
           <t>Safe</t>
         </is>
@@ -4928,7 +5374,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O3" s="17" t="inlineStr">
+      <c r="O3" s="18" t="inlineStr">
         <is>
           <t>Safe</t>
         </is>
@@ -5018,7 +5464,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O4" s="17" t="inlineStr">
+      <c r="O4" s="18" t="inlineStr">
         <is>
           <t>Safe</t>
         </is>
@@ -5107,7 +5553,7 @@
         <f>528</f>
         <v/>
       </c>
-      <c r="O5" s="17" t="inlineStr">
+      <c r="O5" s="18" t="inlineStr">
         <is>
           <t>Safe</t>
         </is>
@@ -5196,7 +5642,7 @@
         <f>528</f>
         <v/>
       </c>
-      <c r="O6" s="17" t="inlineStr">
+      <c r="O6" s="18" t="inlineStr">
         <is>
           <t>Safe</t>
         </is>
@@ -5285,7 +5731,7 @@
         <f>639</f>
         <v/>
       </c>
-      <c r="O7" s="17" t="inlineStr">
+      <c r="O7" s="18" t="inlineStr">
         <is>
           <t>Safe</t>
         </is>
@@ -5374,7 +5820,7 @@
         <f>639</f>
         <v/>
       </c>
-      <c r="O8" s="17" t="inlineStr">
+      <c r="O8" s="18" t="inlineStr">
         <is>
           <t>Safe</t>
         </is>
@@ -5464,7 +5910,7 @@
           <t>≈ 600–650</t>
         </is>
       </c>
-      <c r="O9" s="17" t="inlineStr">
+      <c r="O9" s="18" t="inlineStr">
         <is>
           <t>Safe</t>
         </is>
@@ -5553,7 +5999,7 @@
         <f>438</f>
         <v/>
       </c>
-      <c r="O10" s="18" t="inlineStr">
+      <c r="O10" s="16" t="inlineStr">
         <is>
           <t>Safe/Target</t>
         </is>
@@ -5642,7 +6088,7 @@
         <f>438</f>
         <v/>
       </c>
-      <c r="O11" s="18" t="inlineStr">
+      <c r="O11" s="16" t="inlineStr">
         <is>
           <t>Safe/Target</t>
         </is>
@@ -5731,7 +6177,7 @@
         <f>314</f>
         <v/>
       </c>
-      <c r="O12" s="16" t="inlineStr">
+      <c r="O12" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -5820,7 +6266,7 @@
         <f>314</f>
         <v/>
       </c>
-      <c r="O13" s="16" t="inlineStr">
+      <c r="O13" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -5905,7 +6351,7 @@
         <f>314</f>
         <v/>
       </c>
-      <c r="O14" s="16" t="inlineStr">
+      <c r="O14" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -5995,7 +6441,7 @@
           <t>353</t>
         </is>
       </c>
-      <c r="O15" s="18" t="inlineStr">
+      <c r="O15" s="16" t="inlineStr">
         <is>
           <t>Safe/Target</t>
         </is>
@@ -6085,7 +6531,7 @@
           <t>353</t>
         </is>
       </c>
-      <c r="O16" s="18" t="inlineStr">
+      <c r="O16" s="16" t="inlineStr">
         <is>
           <t>Safe/Target</t>
         </is>
@@ -6171,7 +6617,7 @@
           <t>415</t>
         </is>
       </c>
-      <c r="O17" s="16" t="inlineStr">
+      <c r="O17" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -6260,7 +6706,7 @@
         <f>485</f>
         <v/>
       </c>
-      <c r="O18" s="16" t="inlineStr">
+      <c r="O18" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -6350,7 +6796,7 @@
           <t>≈ 800–1000</t>
         </is>
       </c>
-      <c r="O19" s="18" t="inlineStr">
+      <c r="O19" s="16" t="inlineStr">
         <is>
           <t>Safe/Target</t>
         </is>
@@ -6439,7 +6885,7 @@
         <f>246</f>
         <v/>
       </c>
-      <c r="O20" s="16" t="inlineStr">
+      <c r="O20" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -6528,7 +6974,7 @@
         <f>246</f>
         <v/>
       </c>
-      <c r="O21" s="16" t="inlineStr">
+      <c r="O21" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -6617,7 +7063,7 @@
         <f>158</f>
         <v/>
       </c>
-      <c r="O22" s="15" t="inlineStr">
+      <c r="O22" s="14" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
@@ -6706,7 +7152,7 @@
         <f>158</f>
         <v/>
       </c>
-      <c r="O23" s="16" t="inlineStr">
+      <c r="O23" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -6796,7 +7242,7 @@
           <t>149</t>
         </is>
       </c>
-      <c r="O24" s="15" t="inlineStr">
+      <c r="O24" s="14" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
@@ -7332,7 +7778,7 @@
         <f>69</f>
         <v/>
       </c>
-      <c r="O30" s="15" t="inlineStr">
+      <c r="O30" s="14" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
@@ -7510,7 +7956,7 @@
         <f>94</f>
         <v/>
       </c>
-      <c r="O32" s="16" t="inlineStr">
+      <c r="O32" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -7599,7 +8045,7 @@
         <f>456</f>
         <v/>
       </c>
-      <c r="O33" s="16" t="inlineStr">
+      <c r="O33" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -7688,7 +8134,7 @@
         <f>456</f>
         <v/>
       </c>
-      <c r="O34" s="16" t="inlineStr">
+      <c r="O34" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -7777,7 +8223,7 @@
         <f>456</f>
         <v/>
       </c>
-      <c r="O35" s="16" t="inlineStr">
+      <c r="O35" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -7867,7 +8313,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O36" s="18" t="inlineStr">
+      <c r="O36" s="16" t="inlineStr">
         <is>
           <t>Safe/Target</t>
         </is>
@@ -7956,7 +8402,7 @@
         <f>191</f>
         <v/>
       </c>
-      <c r="O37" s="16" t="inlineStr">
+      <c r="O37" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -8046,7 +8492,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O38" s="16" t="inlineStr">
+      <c r="O38" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -8135,7 +8581,7 @@
         <f>670</f>
         <v/>
       </c>
-      <c r="O39" s="16" t="inlineStr">
+      <c r="O39" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -8224,7 +8670,7 @@
         <f>150</f>
         <v/>
       </c>
-      <c r="O40" s="15" t="inlineStr">
+      <c r="O40" s="14" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
@@ -8403,7 +8849,7 @@
           <t>851–900</t>
         </is>
       </c>
-      <c r="O42" s="15" t="inlineStr">
+      <c r="O42" s="14" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
@@ -8849,7 +9295,7 @@
           <t>318</t>
         </is>
       </c>
-      <c r="O47" s="16" t="inlineStr">
+      <c r="O47" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -8939,7 +9385,7 @@
           <t>318</t>
         </is>
       </c>
-      <c r="O48" s="16" t="inlineStr">
+      <c r="O48" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -9029,7 +9475,7 @@
           <t>218</t>
         </is>
       </c>
-      <c r="O49" s="16" t="inlineStr">
+      <c r="O49" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -9119,7 +9565,7 @@
           <t>218</t>
         </is>
       </c>
-      <c r="O50" s="16" t="inlineStr">
+      <c r="O50" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -9209,7 +9655,7 @@
           <t>250</t>
         </is>
       </c>
-      <c r="O51" s="15" t="inlineStr">
+      <c r="O51" s="14" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
@@ -9388,7 +9834,7 @@
         <f>588 (CS ≈ 251)</f>
         <v/>
       </c>
-      <c r="O53" s="16" t="inlineStr">
+      <c r="O53" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -9477,7 +9923,7 @@
         <f>588 (CS ≈ 251)</f>
         <v/>
       </c>
-      <c r="O54" s="16" t="inlineStr">
+      <c r="O54" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -9567,7 +10013,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O55" s="17" t="inlineStr">
+      <c r="O55" s="18" t="inlineStr">
         <is>
           <t>Safe</t>
         </is>
@@ -9657,7 +10103,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O56" s="17" t="inlineStr">
+      <c r="O56" s="18" t="inlineStr">
         <is>
           <t>Safe</t>
         </is>
@@ -9747,7 +10193,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O57" s="18" t="inlineStr">
+      <c r="O57" s="16" t="inlineStr">
         <is>
           <t>Safe/Target</t>
         </is>
@@ -9833,7 +10279,7 @@
           <t>— (UAS)</t>
         </is>
       </c>
-      <c r="O58" s="16" t="inlineStr">
+      <c r="O58" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -9923,7 +10369,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O59" s="17" t="inlineStr">
+      <c r="O59" s="18" t="inlineStr">
         <is>
           <t>Safe</t>
         </is>
@@ -10013,7 +10459,7 @@
           <t>— (UAS)</t>
         </is>
       </c>
-      <c r="O60" s="16" t="inlineStr">
+      <c r="O60" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -10372,7 +10818,7 @@
           <t>223</t>
         </is>
       </c>
-      <c r="O64" s="16" t="inlineStr">
+      <c r="O64" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -10462,7 +10908,7 @@
           <t>223</t>
         </is>
       </c>
-      <c r="O65" s="16" t="inlineStr">
+      <c r="O65" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -10552,7 +10998,7 @@
           <t>223</t>
         </is>
       </c>
-      <c r="O66" s="16" t="inlineStr">
+      <c r="O66" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -10642,7 +11088,7 @@
           <t>283</t>
         </is>
       </c>
-      <c r="O67" s="16" t="inlineStr">
+      <c r="O67" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -10732,7 +11178,7 @@
           <t>283</t>
         </is>
       </c>
-      <c r="O68" s="16" t="inlineStr">
+      <c r="O68" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -10822,7 +11268,7 @@
           <t>119</t>
         </is>
       </c>
-      <c r="O69" s="15" t="inlineStr">
+      <c r="O69" s="14" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
@@ -10912,7 +11358,7 @@
           <t>157</t>
         </is>
       </c>
-      <c r="O70" s="15" t="inlineStr">
+      <c r="O70" s="14" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
@@ -11002,7 +11448,7 @@
           <t>157</t>
         </is>
       </c>
-      <c r="O71" s="16" t="inlineStr">
+      <c r="O71" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -11268,7 +11714,7 @@
           <t>60</t>
         </is>
       </c>
-      <c r="O74" s="15" t="inlineStr">
+      <c r="O74" s="14" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
@@ -11714,7 +12160,7 @@
           <t>— (UAS)</t>
         </is>
       </c>
-      <c r="O79" s="18" t="inlineStr">
+      <c r="O79" s="16" t="inlineStr">
         <is>
           <t>Safe/Target</t>
         </is>
@@ -11804,7 +12250,7 @@
           <t>308</t>
         </is>
       </c>
-      <c r="O80" s="16" t="inlineStr">
+      <c r="O80" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -11894,7 +12340,7 @@
           <t>308</t>
         </is>
       </c>
-      <c r="O81" s="16" t="inlineStr">
+      <c r="O81" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -11980,7 +12426,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O82" s="17" t="inlineStr">
+      <c r="O82" s="18" t="inlineStr">
         <is>
           <t>Safe</t>
         </is>
@@ -12070,7 +12516,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O83" s="18" t="inlineStr">
+      <c r="O83" s="16" t="inlineStr">
         <is>
           <t>Safe/Target</t>
         </is>
@@ -12336,7 +12782,7 @@
           <t>82</t>
         </is>
       </c>
-      <c r="O86" s="15" t="inlineStr">
+      <c r="O86" s="14" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
@@ -12426,7 +12872,7 @@
           <t>174</t>
         </is>
       </c>
-      <c r="O87" s="15" t="inlineStr">
+      <c r="O87" s="14" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
@@ -12516,7 +12962,7 @@
           <t>174</t>
         </is>
       </c>
-      <c r="O88" s="16" t="inlineStr">
+      <c r="O88" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -12602,7 +13048,7 @@
           <t>174</t>
         </is>
       </c>
-      <c r="O89" s="16" t="inlineStr">
+      <c r="O89" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -12688,7 +13134,7 @@
           <t>225</t>
         </is>
       </c>
-      <c r="O90" s="16" t="inlineStr">
+      <c r="O90" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -12778,7 +13224,7 @@
           <t>87</t>
         </is>
       </c>
-      <c r="O91" s="15" t="inlineStr">
+      <c r="O91" s="14" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
@@ -12868,7 +13314,7 @@
           <t>438</t>
         </is>
       </c>
-      <c r="O92" s="16" t="inlineStr">
+      <c r="O92" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -12958,7 +13404,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O93" s="17" t="inlineStr">
+      <c r="O93" s="18" t="inlineStr">
         <is>
           <t>Safe</t>
         </is>
@@ -13048,7 +13494,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O94" s="17" t="inlineStr">
+      <c r="O94" s="18" t="inlineStr">
         <is>
           <t>Safe</t>
         </is>
@@ -13138,7 +13584,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O95" s="17" t="inlineStr">
+      <c r="O95" s="18" t="inlineStr">
         <is>
           <t>Safe</t>
         </is>
@@ -13223,7 +13669,7 @@
         <f>329</f>
         <v/>
       </c>
-      <c r="O96" s="16" t="inlineStr">
+      <c r="O96" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -13312,7 +13758,7 @@
         <f>329</f>
         <v/>
       </c>
-      <c r="O97" s="16" t="inlineStr">
+      <c r="O97" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -13397,7 +13843,7 @@
         <f>329</f>
         <v/>
       </c>
-      <c r="O98" s="16" t="inlineStr">
+      <c r="O98" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -13486,7 +13932,7 @@
         <f>329</f>
         <v/>
       </c>
-      <c r="O99" s="16" t="inlineStr">
+      <c r="O99" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -13575,7 +14021,7 @@
         <f>283</f>
         <v/>
       </c>
-      <c r="O100" s="16" t="inlineStr">
+      <c r="O100" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -13664,7 +14110,7 @@
         <f>283</f>
         <v/>
       </c>
-      <c r="O101" s="16" t="inlineStr">
+      <c r="O101" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -13753,7 +14199,7 @@
         <f>283</f>
         <v/>
       </c>
-      <c r="O102" s="16" t="inlineStr">
+      <c r="O102" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -13842,7 +14288,7 @@
         <f>283</f>
         <v/>
       </c>
-      <c r="O103" s="16" t="inlineStr">
+      <c r="O103" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -13931,7 +14377,7 @@
         <f>283</f>
         <v/>
       </c>
-      <c r="O104" s="16" t="inlineStr">
+      <c r="O104" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -14017,7 +14463,7 @@
           <t>— (تخصصی)</t>
         </is>
       </c>
-      <c r="O105" s="16" t="inlineStr">
+      <c r="O105" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -14107,7 +14553,7 @@
           <t>— (تخصصی)</t>
         </is>
       </c>
-      <c r="O106" s="16" t="inlineStr">
+      <c r="O106" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -14197,7 +14643,7 @@
           <t>— (تخصصی)</t>
         </is>
       </c>
-      <c r="O107" s="16" t="inlineStr">
+      <c r="O107" s="17" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
@@ -14545,7 +14991,7 @@
           <t>128</t>
         </is>
       </c>
-      <c r="O111" s="15" t="inlineStr">
+      <c r="O111" s="14" t="inlineStr">
         <is>
           <t>Target/Reach</t>
         </is>
@@ -20818,12 +21264,12 @@
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>نتیجه با وزن‌های شما (کار ۲۷.۵ = حقوق ۲۷.۵ / انگلیسی ۳۰ / هزینه ۱۵) و بودجهٔ $40,000 برای کل دوره — ۲۸ سپتامبر</t>
+          <t>نتیجه با وزن‌های شما (کار ۲۷.۵ = حقوق ۲۷.۵ / انگلیسی ۳۰ / هزینه ۱۵) و بودجهٔ $40,000 = شهریه + زندگی تا پیدا شدن کار دانشجویی — ۲۸ سپتامبر</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>بودجه $40,000 برای کل تحصیل است (نه در سال) و این عدد بازی را عوض می‌کند: هلند ($74–90k)، سوئد ($51–65k) و دانمارک ($63–76k) کلاً بیرون‌اند؛ از سوئیس فقط Joint MSc در Neuchâtel/Fribourg ($32–43k) و با کار دانشجویی Basel ($38–49k) می‌مانند (HSLU/USI/UZH/ETH نه)؛ آلمان ($25–37k؛ Stuttgart $38–45k با Werkstudent) تنها کشوری است که راحت جا می‌شود؛ انگلستان فقط Teesside/Northumbria/Essex با ۲۰ ساعت کار. امتیاز برنامه‌به‌برنامه با وزن‌های شما: Basel ۶۶.۸ › Neuchâtel ۶۵.۵ › Fribourg ۶۴ › Stuttgart ۵۹.۵ › Darmstadt ۵۸.۵ › Saarland ۵۷.۳ › Teesside ۵۷ › Northumbria = Essex ۵۵.۳ › Passau ۵۱.۵ — سوئیسِ ارزان روی کاغذ برنده است (حقوق $103–127k، شهریهٔ ناچیز)، ولی روی لبهٔ بودجه: ۶ ماه اول بدون حق کار، بعد ۱۵ ساعت؛ تمکن $25,400/سال در بانک سوئیسی؛ زندگی روزمره فرانسه/آلمانی؛ ۶ ماه برای کار بعد از مدرک. آلمان برنامهٔ امن با بهترین شانس استخدام (Werkstudent → استخدام، ۱۸ ماه، $55–63k) به بهای آلمانی B1. توصیه: ۷ درخواست — ۲ سوئیس (Neuchâtel، Basel) + ۳ آلمان (Stuttgart، Darmstadt، Saarland) + ۱–۲ انگلستان (Essex/Northumbria). پذیرش سوئیس + اثبات $40k + کار دانشجویی → سوئیس (با وزن‌های شما)؛ وگرنه آلمان. هلند فقط با بورس Reach.</t>
+          <t>با این تعریف، فیلتر بودجه = (۴۰,۰۰۰ − شهریهٔ کل) ÷ زندگی ماهانه = ماه‌های پوشش‌داده‌شده؛ بقیه از کار دانشجویی. نتیجه: آلمان حتی بدون کار جا می‌شود (Darmstadt/Saarland/Passau تمام ۲۴ ماه + $6–12k؛ Stuttgart ۲۳ ماه). انگلستان با ۲۰ ساعت کار ($16.8/ساعت ≈ $1,450/ماه؛ آسان‌ترین کار دانشجویی) ✅: Teesside بدون کار، Northumbria/Essex/Manchester Met با ≈ $500/ماه، Leicester ⚠️، لندن و Russell Group ❌. سوئیس: ۶ ماه اول کار ممنوع و بعد ۱۵ ساعت (ولی $24–36/ساعت) → Neuchâtel/Fribourg/Basel ✅ (تقریباً بدون نیاز به کار)، HSLU ⚠️ شدنی (۱۵ ماه پوشش، از ماه ۷ ≈ $1,000/ماه)، USI ⚠️ پرریسک (۱۰–۱۱ ماه پوشش، ≈ $1,450/ماه)، UZH/ETH ❌؛ اثبات $25,400/سال در بانک. سوئد فقط با بورس (بدون سوئدی کار دانشجویی $350–900). هلند ❌ (شهریهٔ دو سال $45–50k به‌تنهایی)؛ دانمارک ❌ (۴ ماه پوشش + ویزا). امتیاز برنامه‌به‌برنامه: Basel ۷۱.۳ › HSLU ۶۸.۳ › Neuchâtel ۶۷ › Fribourg ۶۵.۵ › Stuttgart ۶۴ = Manchester Met ۶۴ › Teesside ۶۱.۵ › Northumbria = Essex ۶۱.۳ › USI ۶۱ › Darmstadt ۶۰ › Leicester ۵۹.۸ › Saarland ۵۷.۳. توصیه: ۸ درخواست — ۳ سوئیس (HSLU، Basel، Neuchâtel) + ۳ آلمان (Stuttgart، Darmstadt، Saarland) + ۲ انگلستان (Northumbria یا Manchester Met، Essex). سوئیس فقط اگر «۶ ماه بدون درآمد + اثبات $25,400 + ریسک ۶ ماه بعد از مدرک» را می‌پذیرید؛ آلمان امن‌ترین؛ انگلستان انگلیسیِ کامل با بازار ضعیف.</t>
         </is>
       </c>
     </row>
@@ -20847,7 +21293,7 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>دانشگاه‌های واقع‌بینانه با معدل ۱۵.۷۷: USI Lugano (Informatics / AI / Software &amp; Data Eng؛ ورود با B2؛ $4,840/ترم) · HSLU Applied Data Science &amp; AI (Safe/Target؛ $1,570/ترم؛ مهلت ویزایی‌ها ۱ آوریل) · Swiss Joint MSc CS در Neuchâtel ($955/ترم) یا Fribourg ($1,190/ترم؛ ویزایی‌ها ۲۸ فوریه) — بدون آزمون زبان؛ Bern همان مدرک با $3,160/ترم از پاییز ۲۰۲۶ · Basel MSc CS ($1,030؛ Target/Reach) · ZHAW MSE ($1,550؛ نمرهٔ A/B) · UZH / EPFL / ETH Reach (ETH فقط ۱–۳۰ نوامبر ۲۰۲۶؛ EPFL دور اول ۱۵ دسامبر). QS 2027: ETH 8 · EPFL 22 · UZH 98 · Basel 150 · Bern 191 · USI 456 · Fribourg 670 · ZHAW 851–900. طول دوره ۱.۵ سال (90 ECTS) یا ۲ سال (120 ECTS). زندگی: زوریخ $2,300–3,030/ماه · لوزان $2,060–2,660 · برن/بازل/لوسرن $1,880–2,540 · لوگانو/فریبورگ/نوشاتل $1,630–2,180؛ تمکن رسمی $25,400/سال (Basel $29,000). سال اول $23–42k؛ کل دوره $35–84k — فقط Joint MSc Neuchâtel/Fribourg (و Basel با کار) در بودجهٔ $40k کل. کار: ۶ ماه اول صفر، بعد ۱۵ ساعت/هفته (≈ $1,570–2,180/ماه)؛ بعد از مدرک فقط ۶ ماه مجوز L؛ اجازهٔ کار بدون کف حقوق ولی داخل سهمیهٔ غیر-EU (۲۰۲۶: ۴,۵۰۰ B + ۴,۰۰۰ L). حقوق جونیور $103–127k (میانهٔ زوریخ $111k)، خالص $6,900–8,110/ماه، پس‌انداز $1,820–3,630/ماه. اقامت: اجازهٔ C بعد از ۱۰ سال + A2 شفاهی/A1 کتبی؛ تابعیت ۱۰ سال + B1/A2 — طولانی‌ترین جدول. ویزا: سفارت تهران باز، ویزای D با وقت قبلی، تصمیم کانتون ۸–۱۲ هفته؛ زوریخ تمکن را فقط در بانک سوئیسی به نام خودتان یا با ضامن مقیم می‌پذیرد. IELTS: USI B2→C1 · HSLU C1 (B2 مشروط) · Joint MSc بدون آزمون · ZHAW B2–C1 · UZH/ETH 7.0 · EPFL بدون آزمون. بورس: عملاً هیچ (ETH/EPFL Excellence برای ۱۰٪ بالا؛ USI $4,840 با ≥ ۸۰/۱۰۰ — مرزی). خوابگاه: هیچ‌جا تضمین ندارد؛ زوریخ ۳–۱۲ ماه صف (WOKO $355–1,430)، لوزان زود پر می‌شود، لوگانو/فریبورگ/نوشاتل آسان (≈ $545–970). ریسک سیاستی متوسط (ابتکار ۱۰ میلیونی رد شد؛ EP27؛ Bilaterals III). امتیاز ۱۸/۳۰ = هلند. یک جمله: اگر شغل بگیرید بالاترین درآمد جدول، اگر در ۶ ماه نگیرید باید بروید — گزینهٔ پربازده/پرریسک، نه گزینهٔ امن.</t>
+          <t>دانشگاه‌های واقع‌بینانه با معدل ۱۵.۷۷: USI Lugano (Informatics / AI / Software &amp; Data Eng؛ ورود با B2؛ $4,840/ترم) · HSLU Applied Data Science &amp; AI (Safe/Target؛ $1,570/ترم؛ مهلت ویزایی‌ها ۱ آوریل) · Swiss Joint MSc CS در Neuchâtel ($955/ترم) یا Fribourg ($1,190/ترم؛ ویزایی‌ها ۲۸ فوریه) — بدون آزمون زبان؛ Bern همان مدرک با $3,160/ترم از پاییز ۲۰۲۶ · Basel MSc CS ($1,030؛ Target/Reach) · ZHAW MSE ($1,550؛ نمرهٔ A/B) · UZH / EPFL / ETH Reach (ETH فقط ۱–۳۰ نوامبر ۲۰۲۶؛ EPFL دور اول ۱۵ دسامبر). QS 2027: ETH 8 · EPFL 22 · UZH 98 · Basel 150 · Bern 191 · USI 456 · Fribourg 670 · ZHAW 851–900. طول دوره ۱.۵ سال (90 ECTS) یا ۲ سال (120 ECTS). زندگی: زوریخ $2,300–3,030/ماه · لوزان $2,060–2,660 · برن/بازل/لوسرن $1,880–2,540 · لوگانو/فریبورگ/نوشاتل $1,630–2,180؛ تمکن رسمی $25,400/سال (Basel $29,000). سال اول $23–42k؛ کل دوره $35–84k — با مدل «شهریه + زندگی تا پیدا شدن کار»: Neuchâtel/Fribourg/Basel ✅، HSLU ⚠️ شدنی (از ماه ۷ ≈ $1,000/ماه کار)، USI ⚠️ پرریسک، UZH/ETH ❌. کار: ۶ ماه اول صفر، بعد ۱۵ ساعت/هفته (≈ $1,570–2,180/ماه)؛ بعد از مدرک فقط ۶ ماه مجوز L؛ اجازهٔ کار بدون کف حقوق ولی داخل سهمیهٔ غیر-EU (۲۰۲۶: ۴,۵۰۰ B + ۴,۰۰۰ L). حقوق جونیور $103–127k (میانهٔ زوریخ $111k)، خالص $6,900–8,110/ماه، پس‌انداز $1,820–3,630/ماه. اقامت: اجازهٔ C بعد از ۱۰ سال + A2 شفاهی/A1 کتبی؛ تابعیت ۱۰ سال + B1/A2 — طولانی‌ترین جدول. ویزا: سفارت تهران باز، ویزای D با وقت قبلی، تصمیم کانتون ۸–۱۲ هفته؛ زوریخ تمکن را فقط در بانک سوئیسی به نام خودتان یا با ضامن مقیم می‌پذیرد. IELTS: USI B2→C1 · HSLU C1 (B2 مشروط) · Joint MSc بدون آزمون · ZHAW B2–C1 · UZH/ETH 7.0 · EPFL بدون آزمون. بورس: عملاً هیچ (ETH/EPFL Excellence برای ۱۰٪ بالا؛ USI $4,840 با ≥ ۸۰/۱۰۰ — مرزی). خوابگاه: هیچ‌جا تضمین ندارد؛ زوریخ ۳–۱۲ ماه صف (WOKO $355–1,430)، لوزان زود پر می‌شود، لوگانو/فریبورگ/نوشاتل آسان (≈ $545–970). ریسک سیاستی متوسط (ابتکار ۱۰ میلیونی رد شد؛ EP27؛ Bilaterals III). امتیاز ۱۸/۳۰ = هلند. یک جمله: اگر شغل بگیرید بالاترین درآمد جدول، اگر در ۶ ماه نگیرید باید بروید — گزینهٔ پربازده/پرریسک، نه گزینهٔ امن.</t>
         </is>
       </c>
     </row>
@@ -20954,7 +21400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -21800,30 +22246,62 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
+          <t>بودجه – تعریف نهایی (۲۸ سپتامبر)</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>$40,000 = کل شهریه + زندگی تا پیدا شدن کار دانشجویی</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>گفتهٔ شما؛ سقف ساعت کار از منابع رسمی (SEM، BAMF، UKVI، IND)؛ حداقل دستمزد انگلستان $16.8 (£12.71) (gov.uk، ۱ آوریل ۲۰۲۶)</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>قانون + برآورد درآمد</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="inlineStr">
+        <is>
+          <t>۲۸ سپتامبر ۲۰۲۶</t>
+        </is>
+      </c>
+      <c r="F27" s="31" t="inlineStr">
+        <is>
+          <t>⚠️ ردیف ۹، شیت «تصمیم» و بخش ۲۲ گزارش با این مدل بازنویسی شد؛ ماه‌های پوشش = (۴۰,۰۰۰ − شهریه) ÷ میانهٔ زندگی شهر</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
           <t>کل فایل – وضعیت</t>
         </is>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B28" s="12" t="inlineStr">
         <is>
           <t>≈ ۱,۶۰۰ سلول عددی؛ ≈ ۳۴۰ سلول با علامت ≈/برآورد</t>
         </is>
       </c>
-      <c r="C27" s="12" t="inlineStr">
+      <c r="C28" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D27" s="12" t="inlineStr">
+      <c r="D28" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E27" s="12" t="inlineStr">
+      <c r="E28" s="12" t="inlineStr">
         <is>
           <t>۲۸ سپتامبر ۲۰۲۶</t>
         </is>
       </c>
-      <c r="F27" s="12" t="inlineStr">
+      <c r="F28" s="12" t="inlineStr">
         <is>
           <t>خلاصه: تصمیم‌سازها (شهریه، ویزا، تمکن، مهلت، تطبیق نمره، بورس‌های اصلی، خوابگاه‌های اصلی) رسمی‌اند؛ حقوق، هزینهٔ زندگی، شانس خوابگاه و اجاره‌های شهرهای فرعی برآوردند و همان‌طور علامت خورده‌اند</t>
         </is>
@@ -21840,7 +22318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B218"/>
+  <dimension ref="A1:B219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -24418,46 +24896,58 @@
     <row r="215">
       <c r="A215" s="12" t="inlineStr">
         <is>
-          <t>سوئیس – Art. 21 Abs. 3 AIG: فارغ‌التحصیلان سوئیس معاف از اولویت نیروی داخلی؛ سهمیه باقی است (SEM Weisungen §4.2؛ زوریخ ۲۰۲۵: ۳۹۹ L + ۲۴۹ B)</t>
+          <t>انگلستان – National Living Wage £12.71 از ۱ آوریل ۲۰۲۶ (Low Pay Commission)</t>
         </is>
       </c>
       <c r="B215" s="34" t="inlineStr">
         <is>
-          <t>https://www.fedlex.admin.ch/eli/cc/2007/758/en#art_21</t>
+          <t>https://www.gov.uk/government/news/national-living-wage-increases-to-1271-per-hour</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="12" t="inlineStr">
         <is>
-          <t>هلند – UvA شهریهٔ نهادی 2026/27 (دانشکدهٔ علوم، غیر-EEA: ارشد یک‌ساله €34,300، دوساله €26,000، CS مشترک با VU €24,150)</t>
+          <t>سوئیس – Art. 21 Abs. 3 AIG: فارغ‌التحصیلان سوئیس معاف از اولویت نیروی داخلی؛ سهمیه باقی است (SEM Weisungen §4.2؛ زوریخ ۲۰۲۵: ۳۹۹ L + ۲۴۹ B)</t>
         </is>
       </c>
       <c r="B216" s="34" t="inlineStr">
         <is>
-          <t>https://www.uva.nl/en/education/fees-and-funding/tuition-fees/tuition-fees.html</t>
+          <t>https://www.fedlex.admin.ch/eli/cc/2007/758/en#art_21</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="12" t="inlineStr">
         <is>
-          <t>هلند – UvA MSc Software Engineering: 60 ECTS، ۱۲ ماه، انگلیسی</t>
+          <t>هلند – UvA شهریهٔ نهادی 2026/27 (دانشکدهٔ علوم، غیر-EEA: ارشد یک‌ساله €34,300، دوساله €26,000، CS مشترک با VU €24,150)</t>
         </is>
       </c>
       <c r="B217" s="34" t="inlineStr">
         <is>
-          <t>https://www.uva.nl/en/programmes/masters/software-engineering/software-engineering.html</t>
+          <t>https://www.uva.nl/en/education/fees-and-funding/tuition-fees/tuition-fees.html</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="12" t="inlineStr">
         <is>
+          <t>هلند – UvA MSc Software Engineering: 60 ECTS، ۱۲ ماه، انگلیسی</t>
+        </is>
+      </c>
+      <c r="B218" s="34" t="inlineStr">
+        <is>
+          <t>https://www.uva.nl/en/programmes/masters/software-engineering/software-engineering.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="12" t="inlineStr">
+        <is>
           <t>هلند – Twente: مهلت غیر-EEA ۱ می ۲۰۲۷؛ بورس UTS ۱۵ اکتبر ۲۰۲۶ – ۱ آوریل ۲۰۲۷</t>
         </is>
       </c>
-      <c r="B218" s="34" t="inlineStr">
+      <c r="B219" s="34" t="inlineStr">
         <is>
           <t>https://collegedunia.com/netherlands/university/749-university-of-twente-enschede/admission</t>
         </is>
@@ -24682,6 +25172,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B216" r:id="rId215"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B217" r:id="rId216"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B218" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B219" r:id="rId218"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Audit: which numbers are official vs estimated vs due to change before 2027; audit row for independence-model assumptions (v3.6.1)
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Table_final.xlsx
+++ b/Table_final.xlsx
@@ -22380,7 +22380,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -23258,30 +23258,62 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
+          <t>شیت تصمیم – پ-۳ استقلال مالی (نسخهٔ ۳.۶)</t>
+        </is>
+      </c>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>ساعت لازم در هفته = میانهٔ زندگی شهر ÷ (دستمزد خالص ساعتی × ۴.۳۳)؛ سقف قانونی: آلمان ۲۰ ساعت از ماه ۱ · انگلستان ۲۰ (میانگین سالانه ۲۲.۳ با کار تمام‌وقت کریسمس/ایستر) · سوئیس ۱۵ از ماه ۷ (میانگین ۲۱.۷۵ با تعطیلات ترم) · سوئد بدون سقف (۲۰ فرض)؛ کف دستمزد: $16.6 (€14.60) (ژانویهٔ ۲۰۲۷) · $16.8 (£12.71) (آوریل ۲۰۲۶) · $26.9 (CHF 22.20) Basel-Stadt / 22.00 شهر لوسرن / 21.35 Neuchâtel / 22 فرض Fribourg · $15 (SEK 150) فرض؛ نرخ کار IT دانشجویی: $19 (€17) · $19 (£14) · $34 (CHF 28) · $17 (SEK 170)؛ ضریب خالص: ۰.۹۰۵ · ۰.۹۸۶ · ۰.۹۱ · ۰.۸۶؛ ماه‌های کاریابی: ۲ · ۱ · ۱ (پس از ماه ۶) · ۴</t>
+        </is>
+      </c>
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>سقف ساعت و کف دستمزد: §16b AufenthG/BMAS، gov.uk (NLW)، SEM + قوانین کانتونی، Migrationsverket؛ نرخ IT: آگهی‌های Werkstudent (StepStone/Indeed)، Indeed UK، jobs.ch؛ ضریب خالص: محاسبهٔ خودم (Werkstudentenprivileg، Personal Allowance، AHV/ALV/کسر مالیات در مبدأ، jobbskatteavdrag)</t>
+        </is>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
+        <is>
+          <t>قانون (رسمی) + برآورد (نرخ IT، ضریب خالص، ماه‌های کاریابی، میانگین سالانه)</t>
+        </is>
+      </c>
+      <c r="E28" s="13" t="inlineStr">
+        <is>
+          <t>۲۸ سپتامبر ۲۰۲۶</t>
+        </is>
+      </c>
+      <c r="F28" s="36" t="inlineStr">
+        <is>
+          <t>✅ سقف‌ها و کف‌های دستمزد رسمی‌اند؛ ⚠️ نرخ IT، ضریب خالص، ماه‌های کاریابی و «میانگین سالانه با کار تمام‌وقت در تعطیلات» فرض‌اند (خطای محتمل ±۵–۱۰٪)؛ حکم‌های سر مرز با ±۵٪ تغییر اجاره یا دستمزد جابه‌جا می‌شوند: Newcastle ۹۹٪، Darmstadt ۹۷٪، Manchester (میانگین) ۱۰۱٪، Västerås ۱۰۲٪، Basel (میانگین) ۱۰۳٪، Middlesbrough ۱۰۳٪؛ پایدار: Saarbrücken/Passau ۱۱۴٪، Luzern (میانگین) ۱۰۸٪، Karlskrona ۱۰۶٪</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
           <t>کل فایل – وضعیت</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>≈ ۱,۶۰۰ سلول عددی؛ ≈ ۳۴۰ سلول با علامت ≈/برآورد</t>
         </is>
       </c>
-      <c r="C28" s="13" t="inlineStr">
+      <c r="C29" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D28" s="13" t="inlineStr">
+      <c r="D29" s="13" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E28" s="13" t="inlineStr">
+      <c r="E29" s="13" t="inlineStr">
         <is>
           <t>۲۸ سپتامبر ۲۰۲۶</t>
         </is>
       </c>
-      <c r="F28" s="13" t="inlineStr">
+      <c r="F29" s="13" t="inlineStr">
         <is>
           <t>خلاصه: تصمیم‌سازها (شهریه، ویزا، تمکن، مهلت، تطبیق نمره، بورس‌های اصلی، خوابگاه‌های اصلی) رسمی‌اند؛ حقوق، هزینهٔ زندگی، شانس خوابگاه و اجاره‌های شهرهای فرعی برآوردند و همان‌طور علامت خورده‌اند</t>
         </is>

</xml_diff>